<commit_message>
Document sequencer bridge protocol
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBABCF57-02F9-4BF2-804E-6FB406024E22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5E4F78-A1C7-4759-B290-A9B1BA735748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -21,6 +21,7 @@
     <sheet name="bus" sheetId="5" r:id="rId6"/>
     <sheet name="cycle" sheetId="9" r:id="rId7"/>
     <sheet name="memory" sheetId="11" r:id="rId8"/>
+    <sheet name="seq-brg protocol" sheetId="14" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="201">
   <si>
     <t>MODE B</t>
   </si>
@@ -590,13 +591,70 @@
   </si>
   <si>
     <t>value [0..2]</t>
+  </si>
+  <si>
+    <t>No action</t>
+  </si>
+  <si>
+    <t>Step Instruction</t>
+  </si>
+  <si>
+    <t>Step Cycle</t>
+  </si>
+  <si>
+    <t>Reset</t>
+  </si>
+  <si>
+    <t>Stopped</t>
+  </si>
+  <si>
+    <t>Running</t>
+  </si>
+  <si>
+    <t>Halted</t>
+  </si>
+  <si>
+    <t>OPERATING STATE</t>
+  </si>
+  <si>
+    <t>undefined</t>
+  </si>
+  <si>
+    <t>BRIDGE   →   SEQUENCER</t>
+  </si>
+  <si>
+    <t>SEQUENCER   →   BRIDGE</t>
+  </si>
+  <si>
+    <t>CYCLE STATE</t>
+  </si>
+  <si>
+    <t>DIRECTION</t>
+  </si>
+  <si>
+    <t>BIT</t>
+  </si>
+  <si>
+    <t>SEQUENCER COMMAND</t>
+  </si>
+  <si>
+    <t>INDEX</t>
+  </si>
+  <si>
+    <t>Continue</t>
+  </si>
+  <si>
+    <t>RESPOND (1 = send packet to bridge)</t>
+  </si>
+  <si>
+    <t>ENABLE (0 = STOP, 1 = RUNNING)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -606,6 +664,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -685,7 +751,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="65">
+  <borders count="69">
     <border>
       <left/>
       <right/>
@@ -1481,11 +1547,67 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="273">
+  <cellXfs count="295">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2005,6 +2127,42 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2044,94 +2202,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2140,19 +2244,43 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2191,9 +2319,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2254,12 +2379,67 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2280,7 +2460,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2597,15 +2777,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F30110-9AA6-4607-84AE-181659F51D05}">
   <dimension ref="B1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="6" width="4.73046875" style="1" customWidth="1"/>
-    <col min="7" max="9" width="9.1328125" customWidth="1"/>
-    <col min="10" max="10" width="34.265625" customWidth="1"/>
+    <col min="3" max="6" width="4.7109375" style="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" customWidth="1"/>
+    <col min="10" max="10" width="34.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="181" t="s">
         <v>15</v>
       </c>
@@ -2622,7 +2802,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="57" t="s">
         <v>16</v>
       </c>
@@ -2649,7 +2829,7 @@
       </c>
       <c r="J3" s="185"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="107">
         <v>0</v>
       </c>
@@ -2682,7 +2862,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -2715,7 +2895,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -2748,7 +2928,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -2781,7 +2961,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -2814,7 +2994,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -2847,7 +3027,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -2880,7 +3060,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -2913,7 +3093,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="13">
         <v>8</v>
       </c>
@@ -2944,7 +3124,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="13">
         <v>9</v>
       </c>
@@ -2973,7 +3153,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="19">
         <v>10</v>
       </c>
@@ -2998,7 +3178,7 @@
       <c r="I14" s="116"/>
       <c r="J14" s="32"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="22">
         <v>11</v>
       </c>
@@ -3029,7 +3209,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="13">
         <v>12</v>
       </c>
@@ -3054,7 +3234,7 @@
       <c r="I16" s="115"/>
       <c r="J16" s="31"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="13">
         <v>13</v>
       </c>
@@ -3079,7 +3259,7 @@
       <c r="I17" s="115"/>
       <c r="J17" s="31"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="19">
         <v>14</v>
       </c>
@@ -3104,7 +3284,7 @@
       <c r="I18" s="116"/>
       <c r="J18" s="32"/>
     </row>
-    <row r="19" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="16">
         <v>15</v>
       </c>
@@ -3143,13 +3323,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE0A35C-77D4-4A92-BE06-765002DB2402}">
   <dimension ref="B1:AH8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="34" width="7.73046875" customWidth="1"/>
+    <col min="3" max="34" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="2">
         <v>31</v>
       </c>
@@ -3247,74 +3427,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C3" s="211" t="s">
+    <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="198" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="212"/>
-      <c r="E3" s="212"/>
-      <c r="F3" s="212"/>
-      <c r="G3" s="213"/>
-      <c r="H3" s="208" t="s">
+      <c r="D3" s="199"/>
+      <c r="E3" s="199"/>
+      <c r="F3" s="199"/>
+      <c r="G3" s="200"/>
+      <c r="H3" s="195" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="209"/>
-      <c r="J3" s="210"/>
-      <c r="K3" s="208" t="s">
+      <c r="I3" s="196"/>
+      <c r="J3" s="197"/>
+      <c r="K3" s="195" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="209"/>
-      <c r="M3" s="209"/>
-      <c r="N3" s="195" t="s">
+      <c r="L3" s="196"/>
+      <c r="M3" s="196"/>
+      <c r="N3" s="207" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="196"/>
-      <c r="P3" s="197"/>
+      <c r="O3" s="208"/>
+      <c r="P3" s="209"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="189" t="s">
+      <c r="S3" s="201" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="190"/>
-      <c r="U3" s="190"/>
-      <c r="V3" s="190"/>
-      <c r="W3" s="190"/>
-      <c r="X3" s="190"/>
-      <c r="Y3" s="190"/>
-      <c r="Z3" s="191"/>
-      <c r="AA3" s="192" t="s">
+      <c r="T3" s="202"/>
+      <c r="U3" s="202"/>
+      <c r="V3" s="202"/>
+      <c r="W3" s="202"/>
+      <c r="X3" s="202"/>
+      <c r="Y3" s="202"/>
+      <c r="Z3" s="203"/>
+      <c r="AA3" s="204" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="193"/>
-      <c r="AC3" s="193"/>
-      <c r="AD3" s="193"/>
-      <c r="AE3" s="193"/>
-      <c r="AF3" s="193"/>
-      <c r="AG3" s="193"/>
-      <c r="AH3" s="194"/>
-    </row>
-    <row r="4" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="5" spans="2:34" x14ac:dyDescent="0.45">
-      <c r="B5" s="200" t="s">
+      <c r="AB3" s="205"/>
+      <c r="AC3" s="205"/>
+      <c r="AD3" s="205"/>
+      <c r="AE3" s="205"/>
+      <c r="AF3" s="205"/>
+      <c r="AG3" s="205"/>
+      <c r="AH3" s="206"/>
+    </row>
+    <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:34" x14ac:dyDescent="0.25">
+      <c r="B5" s="212" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="198" t="s">
+      <c r="C5" s="210" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="198"/>
-      <c r="E5" s="198"/>
-      <c r="F5" s="198"/>
-      <c r="G5" s="198"/>
-      <c r="H5" s="198"/>
-      <c r="I5" s="198"/>
-      <c r="J5" s="199"/>
-    </row>
-    <row r="6" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="201"/>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="210"/>
+      <c r="H5" s="210"/>
+      <c r="I5" s="210"/>
+      <c r="J5" s="211"/>
+    </row>
+    <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="213"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3340,22 +3520,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:34" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="202" t="s">
+      <c r="C7" s="189" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="203"/>
-      <c r="E7" s="203"/>
-      <c r="F7" s="203"/>
-      <c r="G7" s="203"/>
-      <c r="H7" s="203"/>
-      <c r="I7" s="203"/>
-      <c r="J7" s="204"/>
-    </row>
-    <row r="8" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D7" s="190"/>
+      <c r="E7" s="190"/>
+      <c r="F7" s="190"/>
+      <c r="G7" s="190"/>
+      <c r="H7" s="190"/>
+      <c r="I7" s="190"/>
+      <c r="J7" s="191"/>
+    </row>
+    <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
         <v>1</v>
       </c>
@@ -3363,25 +3543,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="205" t="s">
+      <c r="G8" s="192" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="206"/>
-      <c r="I8" s="206"/>
-      <c r="J8" s="207"/>
+      <c r="H8" s="193"/>
+      <c r="I8" s="193"/>
+      <c r="J8" s="194"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="S3:Z3"/>
+    <mergeCell ref="AA3:AH3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:J7"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="S3:Z3"/>
-    <mergeCell ref="AA3:AH3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3391,38 +3571,38 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B20B11-9266-4E5E-A2B3-3496A1A10C3B}">
   <dimension ref="B1:Q35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.1328125" style="1"/>
-    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.73046875" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.7109375" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="90.265625" customWidth="1"/>
+    <col min="14" max="14" width="90.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B2" s="235" t="s">
+    <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B2" s="214" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
-      <c r="F2" s="236"/>
-      <c r="G2" s="237"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="216"/>
       <c r="H2" s="184" t="s">
         <v>54</v>
       </c>
       <c r="I2" s="184" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="235" t="s">
+      <c r="J2" s="214" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="236"/>
-      <c r="L2" s="236"/>
+      <c r="K2" s="215"/>
+      <c r="L2" s="215"/>
       <c r="M2" s="184" t="s">
         <v>112</v>
       </c>
@@ -3430,7 +3610,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
         <v>16</v>
       </c>
@@ -3463,7 +3643,7 @@
       <c r="M3" s="185"/>
       <c r="N3" s="185"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="81">
         <v>0</v>
       </c>
@@ -3487,7 +3667,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="216" t="s">
+      <c r="H4" s="217" t="s">
         <v>45</v>
       </c>
       <c r="I4" s="68" t="s">
@@ -3509,7 +3689,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="83">
         <v>1</v>
       </c>
@@ -3533,7 +3713,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="215"/>
+      <c r="H5" s="218"/>
       <c r="I5" s="43" t="s">
         <v>3</v>
       </c>
@@ -3553,7 +3733,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="82">
         <v>2</v>
       </c>
@@ -3577,29 +3757,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="214" t="s">
+      <c r="H6" s="219" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="218" t="s">
+      <c r="J6" s="220" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="227" t="s">
+      <c r="K6" s="222" t="s">
         <v>69</v>
       </c>
       <c r="L6" s="224" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="229" t="s">
+      <c r="M6" s="232" t="s">
         <v>113</v>
       </c>
-      <c r="N6" s="232" t="s">
+      <c r="N6" s="226" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="82">
         <v>3</v>
       </c>
@@ -3623,17 +3803,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="214"/>
+      <c r="H7" s="219"/>
       <c r="I7" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="218"/>
-      <c r="K7" s="227"/>
+      <c r="J7" s="220"/>
+      <c r="K7" s="222"/>
       <c r="L7" s="224"/>
-      <c r="M7" s="230"/>
-      <c r="N7" s="232"/>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M7" s="233"/>
+      <c r="N7" s="226"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="82">
         <v>4</v>
       </c>
@@ -3657,17 +3837,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="214"/>
+      <c r="H8" s="219"/>
       <c r="I8" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="218"/>
-      <c r="K8" s="227"/>
+      <c r="J8" s="220"/>
+      <c r="K8" s="222"/>
       <c r="L8" s="224"/>
-      <c r="M8" s="230"/>
-      <c r="N8" s="232"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M8" s="233"/>
+      <c r="N8" s="226"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="82">
         <v>5</v>
       </c>
@@ -3691,17 +3871,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="214"/>
+      <c r="H9" s="219"/>
       <c r="I9" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="218"/>
-      <c r="K9" s="227"/>
+      <c r="J9" s="220"/>
+      <c r="K9" s="222"/>
       <c r="L9" s="224"/>
-      <c r="M9" s="230"/>
-      <c r="N9" s="232"/>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M9" s="233"/>
+      <c r="N9" s="226"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="82">
         <v>6</v>
       </c>
@@ -3725,17 +3905,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="214"/>
+      <c r="H10" s="219"/>
       <c r="I10" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="218"/>
-      <c r="K10" s="227"/>
+      <c r="J10" s="220"/>
+      <c r="K10" s="222"/>
       <c r="L10" s="224"/>
-      <c r="M10" s="230"/>
-      <c r="N10" s="232"/>
-    </row>
-    <row r="11" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M10" s="233"/>
+      <c r="N10" s="226"/>
+    </row>
+    <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="83">
         <v>7</v>
       </c>
@@ -3759,17 +3939,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="215"/>
+      <c r="H11" s="218"/>
       <c r="I11" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="219"/>
-      <c r="K11" s="228"/>
+      <c r="J11" s="221"/>
+      <c r="K11" s="223"/>
       <c r="L11" s="225"/>
-      <c r="M11" s="231"/>
-      <c r="N11" s="233"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M11" s="234"/>
+      <c r="N11" s="227"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="81">
         <v>8</v>
       </c>
@@ -3793,29 +3973,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="216" t="s">
+      <c r="H12" s="217" t="s">
         <v>55</v>
       </c>
       <c r="I12" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="217" t="s">
+      <c r="J12" s="228" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="226" t="s">
+      <c r="K12" s="229" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="223" t="s">
+      <c r="L12" s="230" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="216" t="s">
+      <c r="M12" s="217" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="234" t="s">
+      <c r="N12" s="231" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="82">
         <v>9</v>
       </c>
@@ -3839,17 +4019,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="214"/>
+      <c r="H13" s="219"/>
       <c r="I13" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="218"/>
-      <c r="K13" s="227"/>
+      <c r="J13" s="220"/>
+      <c r="K13" s="222"/>
       <c r="L13" s="224"/>
-      <c r="M13" s="214"/>
-      <c r="N13" s="232"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M13" s="219"/>
+      <c r="N13" s="226"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="82">
         <v>10</v>
       </c>
@@ -3873,17 +4053,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="214"/>
+      <c r="H14" s="219"/>
       <c r="I14" s="91" t="s">
         <v>102</v>
       </c>
-      <c r="J14" s="218"/>
-      <c r="K14" s="227"/>
+      <c r="J14" s="220"/>
+      <c r="K14" s="222"/>
       <c r="L14" s="224"/>
-      <c r="M14" s="214"/>
-      <c r="N14" s="232"/>
-    </row>
-    <row r="15" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M14" s="219"/>
+      <c r="N14" s="226"/>
+    </row>
+    <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="83">
         <v>11</v>
       </c>
@@ -3907,17 +4087,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="215"/>
+      <c r="H15" s="218"/>
       <c r="I15" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="219"/>
-      <c r="K15" s="228"/>
+      <c r="J15" s="221"/>
+      <c r="K15" s="223"/>
       <c r="L15" s="225"/>
-      <c r="M15" s="215"/>
-      <c r="N15" s="233"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M15" s="218"/>
+      <c r="N15" s="227"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="81">
         <v>12</v>
       </c>
@@ -3941,29 +4121,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="216" t="s">
+      <c r="H16" s="217" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="217" t="s">
+      <c r="J16" s="228" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="220" t="s">
+      <c r="K16" s="235" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="223" t="s">
+      <c r="L16" s="230" t="s">
         <v>66</v>
       </c>
-      <c r="M16" s="216" t="s">
+      <c r="M16" s="217" t="s">
         <v>114</v>
       </c>
       <c r="N16" s="76" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="82">
         <v>13</v>
       </c>
@@ -3987,19 +4167,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="214"/>
+      <c r="H17" s="219"/>
       <c r="I17" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="218"/>
-      <c r="K17" s="221"/>
+      <c r="J17" s="220"/>
+      <c r="K17" s="236"/>
       <c r="L17" s="224"/>
-      <c r="M17" s="214"/>
+      <c r="M17" s="219"/>
       <c r="N17" s="75" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="82">
         <v>14</v>
       </c>
@@ -4023,19 +4203,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="214"/>
+      <c r="H18" s="219"/>
       <c r="I18" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="218"/>
-      <c r="K18" s="221"/>
+      <c r="J18" s="220"/>
+      <c r="K18" s="236"/>
       <c r="L18" s="224"/>
-      <c r="M18" s="214"/>
+      <c r="M18" s="219"/>
       <c r="N18" s="75" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="83">
         <v>15</v>
       </c>
@@ -4059,20 +4239,20 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="215"/>
+      <c r="H19" s="218"/>
       <c r="I19" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="219"/>
-      <c r="K19" s="222"/>
+      <c r="J19" s="221"/>
+      <c r="K19" s="237"/>
       <c r="L19" s="225"/>
-      <c r="M19" s="215"/>
+      <c r="M19" s="218"/>
       <c r="N19" s="45" t="s">
         <v>108</v>
       </c>
       <c r="P19" s="1"/>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="81">
         <v>16</v>
       </c>
@@ -4096,29 +4276,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="216" t="s">
+      <c r="H20" s="217" t="s">
         <v>57</v>
       </c>
       <c r="I20" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="217" t="s">
+      <c r="J20" s="228" t="s">
         <v>16</v>
       </c>
-      <c r="K20" s="226" t="s">
+      <c r="K20" s="229" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="223" t="s">
+      <c r="L20" s="230" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="229" t="s">
+      <c r="M20" s="232" t="s">
         <v>113</v>
       </c>
       <c r="N20" s="42" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B21" s="82">
         <v>17</v>
       </c>
@@ -4142,19 +4322,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="214"/>
+      <c r="H21" s="219"/>
       <c r="I21" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="218"/>
-      <c r="K21" s="227"/>
+      <c r="J21" s="220"/>
+      <c r="K21" s="222"/>
       <c r="L21" s="224"/>
-      <c r="M21" s="230"/>
+      <c r="M21" s="233"/>
       <c r="N21" s="75" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B22" s="82">
         <v>18</v>
       </c>
@@ -4178,19 +4358,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="214"/>
+      <c r="H22" s="219"/>
       <c r="I22" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="218"/>
-      <c r="K22" s="227"/>
+      <c r="J22" s="220"/>
+      <c r="K22" s="222"/>
       <c r="L22" s="224"/>
-      <c r="M22" s="230"/>
+      <c r="M22" s="233"/>
       <c r="N22" s="75" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="82">
         <v>19</v>
       </c>
@@ -4214,19 +4394,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="215"/>
+      <c r="H23" s="218"/>
       <c r="I23" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="J23" s="219"/>
-      <c r="K23" s="228"/>
+      <c r="J23" s="221"/>
+      <c r="K23" s="223"/>
       <c r="L23" s="225"/>
-      <c r="M23" s="231"/>
+      <c r="M23" s="234"/>
       <c r="N23" s="42" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B24" s="81">
         <v>20</v>
       </c>
@@ -4250,7 +4430,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="216" t="s">
+      <c r="H24" s="217" t="s">
         <v>58</v>
       </c>
       <c r="I24" s="65" t="s">
@@ -4272,7 +4452,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B25" s="82">
         <v>21</v>
       </c>
@@ -4296,7 +4476,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="214"/>
+      <c r="H25" s="219"/>
       <c r="I25" s="71" t="s">
         <v>46</v>
       </c>
@@ -4316,7 +4496,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B26" s="82">
         <v>22</v>
       </c>
@@ -4340,7 +4520,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="214"/>
+      <c r="H26" s="219"/>
       <c r="I26" s="105"/>
       <c r="J26" s="139"/>
       <c r="K26" s="140"/>
@@ -4348,7 +4528,7 @@
       <c r="M26" s="106"/>
       <c r="N26" s="106"/>
     </row>
-    <row r="27" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="27" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="83">
         <v>23</v>
       </c>
@@ -4372,7 +4552,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="215"/>
+      <c r="H27" s="218"/>
       <c r="I27" s="98"/>
       <c r="J27" s="136"/>
       <c r="K27" s="137"/>
@@ -4380,7 +4560,7 @@
       <c r="M27" s="135"/>
       <c r="N27" s="135"/>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B28" s="81">
         <v>24</v>
       </c>
@@ -4404,7 +4584,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="216" t="s">
+      <c r="H28" s="217" t="s">
         <v>60</v>
       </c>
       <c r="I28" s="38" t="s">
@@ -4426,7 +4606,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B29" s="82">
         <v>25</v>
       </c>
@@ -4450,7 +4630,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="214"/>
+      <c r="H29" s="219"/>
       <c r="I29" s="71" t="s">
         <v>52</v>
       </c>
@@ -4470,7 +4650,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B30" s="82">
         <v>26</v>
       </c>
@@ -4494,7 +4674,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="214"/>
+      <c r="H30" s="219"/>
       <c r="I30" s="71" t="s">
         <v>53</v>
       </c>
@@ -4514,7 +4694,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="83">
         <v>27</v>
       </c>
@@ -4538,7 +4718,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="215"/>
+      <c r="H31" s="218"/>
       <c r="I31" s="92"/>
       <c r="J31" s="95"/>
       <c r="K31" s="96"/>
@@ -4546,7 +4726,7 @@
       <c r="M31" s="97"/>
       <c r="N31" s="94"/>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B32" s="82">
         <v>28</v>
       </c>
@@ -4570,7 +4750,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="214" t="s">
+      <c r="H32" s="219" t="s">
         <v>59</v>
       </c>
       <c r="I32" s="65" t="s">
@@ -4593,7 +4773,7 @@
       </c>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B33" s="82">
         <v>29</v>
       </c>
@@ -4617,7 +4797,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="214"/>
+      <c r="H33" s="219"/>
       <c r="I33" s="71" t="s">
         <v>24</v>
       </c>
@@ -4638,7 +4818,7 @@
       </c>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="82">
         <v>30</v>
       </c>
@@ -4662,7 +4842,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="215"/>
+      <c r="H34" s="218"/>
       <c r="I34" s="98"/>
       <c r="J34" s="95"/>
       <c r="K34" s="96"/>
@@ -4671,7 +4851,7 @@
       <c r="N34" s="94"/>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="84">
         <v>31</v>
       </c>
@@ -4719,17 +4899,19 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="J20:J23"/>
+    <mergeCell ref="K20:K23"/>
+    <mergeCell ref="L20:L23"/>
+    <mergeCell ref="M20:M23"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4738,19 +4920,17 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="J20:J23"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="M20:M23"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4760,42 +4940,42 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD788E61-AC5A-4E7F-9536-02553AF94143}">
   <dimension ref="B1:P35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="1"/>
-    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.73046875" customWidth="1"/>
-    <col min="13" max="13" width="90.265625" customWidth="1"/>
+    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.7109375" customWidth="1"/>
+    <col min="13" max="13" width="90.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B2" s="235" t="s">
+    <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="214" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="236"/>
-      <c r="F2" s="236"/>
-      <c r="G2" s="237"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
+      <c r="E2" s="215"/>
+      <c r="F2" s="215"/>
+      <c r="G2" s="216"/>
       <c r="H2" s="184" t="s">
         <v>54</v>
       </c>
       <c r="I2" s="184" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="235" t="s">
+      <c r="J2" s="214" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="236"/>
-      <c r="L2" s="236"/>
+      <c r="K2" s="215"/>
+      <c r="L2" s="215"/>
       <c r="M2" s="184" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="85" t="s">
         <v>16</v>
       </c>
@@ -4827,7 +5007,7 @@
       </c>
       <c r="M3" s="185"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="81">
         <v>0</v>
       </c>
@@ -4851,7 +5031,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="216" t="s">
+      <c r="H4" s="217" t="s">
         <v>45</v>
       </c>
       <c r="I4" s="68" t="s">
@@ -4870,7 +5050,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="83">
         <v>1</v>
       </c>
@@ -4894,7 +5074,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="215"/>
+      <c r="H5" s="218"/>
       <c r="I5" s="43" t="s">
         <v>3</v>
       </c>
@@ -4911,7 +5091,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="82">
         <v>2</v>
       </c>
@@ -4935,26 +5115,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="214" t="s">
+      <c r="H6" s="219" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="218" t="s">
+      <c r="J6" s="220" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="227" t="s">
+      <c r="K6" s="222" t="s">
         <v>69</v>
       </c>
       <c r="L6" s="224" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="232" t="s">
+      <c r="M6" s="226" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="82">
         <v>3</v>
       </c>
@@ -4978,14 +5158,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="214"/>
+      <c r="H7" s="219"/>
       <c r="I7" s="238"/>
-      <c r="J7" s="218"/>
-      <c r="K7" s="227"/>
+      <c r="J7" s="220"/>
+      <c r="K7" s="222"/>
       <c r="L7" s="224"/>
-      <c r="M7" s="232"/>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M7" s="226"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="82">
         <v>4</v>
       </c>
@@ -5009,14 +5189,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="214"/>
-      <c r="I8" s="251"/>
-      <c r="J8" s="218"/>
-      <c r="K8" s="227"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="239"/>
+      <c r="J8" s="220"/>
+      <c r="K8" s="222"/>
       <c r="L8" s="224"/>
-      <c r="M8" s="232"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M8" s="226"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="82">
         <v>5</v>
       </c>
@@ -5040,14 +5220,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="214"/>
-      <c r="I9" s="272"/>
-      <c r="J9" s="218"/>
-      <c r="K9" s="227"/>
+      <c r="H9" s="219"/>
+      <c r="I9" s="240"/>
+      <c r="J9" s="220"/>
+      <c r="K9" s="222"/>
       <c r="L9" s="224"/>
-      <c r="M9" s="232"/>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M9" s="226"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="82">
         <v>6</v>
       </c>
@@ -5071,16 +5251,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="214"/>
+      <c r="H10" s="219"/>
       <c r="I10" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="218"/>
-      <c r="K10" s="227"/>
+      <c r="J10" s="220"/>
+      <c r="K10" s="222"/>
       <c r="L10" s="224"/>
-      <c r="M10" s="232"/>
-    </row>
-    <row r="11" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M10" s="226"/>
+    </row>
+    <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="83">
         <v>7</v>
       </c>
@@ -5104,14 +5284,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="215"/>
+      <c r="H11" s="218"/>
       <c r="I11" s="105"/>
-      <c r="J11" s="219"/>
-      <c r="K11" s="228"/>
+      <c r="J11" s="221"/>
+      <c r="K11" s="223"/>
       <c r="L11" s="225"/>
-      <c r="M11" s="233"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M11" s="227"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="81">
         <v>8</v>
       </c>
@@ -5135,26 +5315,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="216" t="s">
+      <c r="H12" s="217" t="s">
         <v>55</v>
       </c>
       <c r="I12" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="217" t="s">
+      <c r="J12" s="228" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="226" t="s">
+      <c r="K12" s="229" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="223" t="s">
+      <c r="L12" s="230" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="234" t="s">
+      <c r="M12" s="231" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="82">
         <v>9</v>
       </c>
@@ -5178,14 +5358,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="214"/>
+      <c r="H13" s="219"/>
       <c r="I13" s="238"/>
-      <c r="J13" s="218"/>
-      <c r="K13" s="227"/>
+      <c r="J13" s="220"/>
+      <c r="K13" s="222"/>
       <c r="L13" s="224"/>
-      <c r="M13" s="232"/>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M13" s="226"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="82">
         <v>10</v>
       </c>
@@ -5209,14 +5389,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="214"/>
-      <c r="I14" s="251"/>
-      <c r="J14" s="218"/>
-      <c r="K14" s="227"/>
+      <c r="H14" s="219"/>
+      <c r="I14" s="239"/>
+      <c r="J14" s="220"/>
+      <c r="K14" s="222"/>
       <c r="L14" s="224"/>
-      <c r="M14" s="232"/>
-    </row>
-    <row r="15" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M14" s="226"/>
+    </row>
+    <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="83">
         <v>11</v>
       </c>
@@ -5240,14 +5420,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="215"/>
-      <c r="I15" s="239"/>
-      <c r="J15" s="219"/>
-      <c r="K15" s="228"/>
+      <c r="H15" s="218"/>
+      <c r="I15" s="241"/>
+      <c r="J15" s="221"/>
+      <c r="K15" s="223"/>
       <c r="L15" s="225"/>
-      <c r="M15" s="233"/>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M15" s="227"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="81">
         <v>12</v>
       </c>
@@ -5271,26 +5451,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="216" t="s">
+      <c r="H16" s="217" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="217" t="s">
+      <c r="J16" s="228" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="220" t="s">
+      <c r="K16" s="235" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="223" t="s">
+      <c r="L16" s="230" t="s">
         <v>66</v>
       </c>
       <c r="M16" s="76" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="82">
         <v>13</v>
       </c>
@@ -5314,18 +5494,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="214"/>
+      <c r="H17" s="219"/>
       <c r="I17" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="218"/>
-      <c r="K17" s="221"/>
+      <c r="J17" s="220"/>
+      <c r="K17" s="236"/>
       <c r="L17" s="224"/>
       <c r="M17" s="75" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="82">
         <v>14</v>
       </c>
@@ -5349,14 +5529,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="214"/>
+      <c r="H18" s="219"/>
       <c r="I18" s="238"/>
-      <c r="J18" s="218"/>
-      <c r="K18" s="221"/>
+      <c r="J18" s="220"/>
+      <c r="K18" s="236"/>
       <c r="L18" s="224"/>
       <c r="M18" s="238"/>
     </row>
-    <row r="19" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="83">
         <v>15</v>
       </c>
@@ -5380,15 +5560,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="215"/>
-      <c r="I19" s="239"/>
-      <c r="J19" s="219"/>
-      <c r="K19" s="222"/>
+      <c r="H19" s="218"/>
+      <c r="I19" s="241"/>
+      <c r="J19" s="221"/>
+      <c r="K19" s="237"/>
       <c r="L19" s="225"/>
-      <c r="M19" s="239"/>
+      <c r="M19" s="241"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="81">
         <v>16</v>
       </c>
@@ -5412,7 +5592,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="240" t="s">
+      <c r="H20" s="242" t="s">
         <v>179</v>
       </c>
       <c r="I20" s="180" t="s">
@@ -5431,7 +5611,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="82">
         <v>17</v>
       </c>
@@ -5455,14 +5635,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="241"/>
+      <c r="H21" s="243"/>
       <c r="I21" s="171"/>
       <c r="J21" s="173"/>
       <c r="K21" s="175"/>
       <c r="L21" s="177"/>
       <c r="M21" s="171"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="82">
         <v>18</v>
       </c>
@@ -5486,14 +5666,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="241"/>
+      <c r="H22" s="243"/>
       <c r="I22" s="171"/>
       <c r="J22" s="173"/>
       <c r="K22" s="175"/>
       <c r="L22" s="177"/>
       <c r="M22" s="171"/>
     </row>
-    <row r="23" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="82">
         <v>19</v>
       </c>
@@ -5517,14 +5697,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="242"/>
+      <c r="H23" s="244"/>
       <c r="I23" s="172"/>
       <c r="J23" s="174"/>
       <c r="K23" s="176"/>
       <c r="L23" s="178"/>
       <c r="M23" s="172"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="81">
         <v>20</v>
       </c>
@@ -5548,7 +5728,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="216" t="s">
+      <c r="H24" s="217" t="s">
         <v>58</v>
       </c>
       <c r="I24" s="65" t="s">
@@ -5567,7 +5747,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="82">
         <v>21</v>
       </c>
@@ -5591,7 +5771,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="214"/>
+      <c r="H25" s="219"/>
       <c r="I25" s="71" t="s">
         <v>46</v>
       </c>
@@ -5608,7 +5788,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="82">
         <v>22</v>
       </c>
@@ -5632,14 +5812,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="214"/>
+      <c r="H26" s="219"/>
       <c r="I26" s="238"/>
-      <c r="J26" s="243"/>
-      <c r="K26" s="245"/>
-      <c r="L26" s="247"/>
-      <c r="M26" s="249"/>
-    </row>
-    <row r="27" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J26" s="245"/>
+      <c r="K26" s="247"/>
+      <c r="L26" s="249"/>
+      <c r="M26" s="251"/>
+    </row>
+    <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="83">
         <v>23</v>
       </c>
@@ -5663,14 +5843,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="215"/>
-      <c r="I27" s="239"/>
-      <c r="J27" s="244"/>
-      <c r="K27" s="246"/>
-      <c r="L27" s="248"/>
-      <c r="M27" s="250"/>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="H27" s="218"/>
+      <c r="I27" s="241"/>
+      <c r="J27" s="246"/>
+      <c r="K27" s="248"/>
+      <c r="L27" s="250"/>
+      <c r="M27" s="252"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="81">
         <v>24</v>
       </c>
@@ -5694,7 +5874,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="216" t="s">
+      <c r="H28" s="217" t="s">
         <v>167</v>
       </c>
       <c r="I28" s="38" t="s">
@@ -5713,7 +5893,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" s="82">
         <v>25</v>
       </c>
@@ -5737,7 +5917,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="214"/>
+      <c r="H29" s="219"/>
       <c r="I29" s="71" t="s">
         <v>52</v>
       </c>
@@ -5754,7 +5934,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="82">
         <v>26</v>
       </c>
@@ -5778,7 +5958,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="214"/>
+      <c r="H30" s="219"/>
       <c r="I30" s="71" t="s">
         <v>53</v>
       </c>
@@ -5795,7 +5975,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="83">
         <v>27</v>
       </c>
@@ -5819,14 +5999,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="215"/>
+      <c r="H31" s="218"/>
       <c r="I31" s="92"/>
       <c r="J31" s="166"/>
       <c r="K31" s="167"/>
       <c r="L31" s="168"/>
       <c r="M31" s="94"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B32" s="82">
         <v>28</v>
       </c>
@@ -5850,7 +6030,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="214" t="s">
+      <c r="H32" s="219" t="s">
         <v>168</v>
       </c>
       <c r="I32" s="38" t="s">
@@ -5870,7 +6050,7 @@
       </c>
       <c r="P32" s="1"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B33" s="82">
         <v>29</v>
       </c>
@@ -5894,7 +6074,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="214"/>
+      <c r="H33" s="219"/>
       <c r="I33" s="71" t="s">
         <v>52</v>
       </c>
@@ -5912,7 +6092,7 @@
       </c>
       <c r="P33" s="1"/>
     </row>
-    <row r="34" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="82">
         <v>30</v>
       </c>
@@ -5936,7 +6116,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="215"/>
+      <c r="H34" s="218"/>
       <c r="I34" s="71" t="s">
         <v>53</v>
       </c>
@@ -5954,7 +6134,7 @@
       </c>
       <c r="P34" s="1"/>
     </row>
-    <row r="35" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="84">
         <v>31</v>
       </c>
@@ -5999,24 +6179,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6032,6 +6194,24 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6041,24 +6221,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4182B34D-1176-43D9-83DE-D8E7EA5C96ED}">
   <dimension ref="B1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="5" width="4.73046875" customWidth="1"/>
+    <col min="3" max="5" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B2" s="235" t="s">
+    <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="214" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="236"/>
-      <c r="D2" s="236"/>
-      <c r="E2" s="237"/>
+      <c r="C2" s="215"/>
+      <c r="D2" s="215"/>
+      <c r="E2" s="216"/>
       <c r="F2" s="184" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
@@ -6073,7 +6253,7 @@
       </c>
       <c r="F3" s="185"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="13">
         <v>0</v>
       </c>
@@ -6093,7 +6273,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -6113,7 +6293,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -6133,7 +6313,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -6153,7 +6333,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -6173,7 +6353,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -6193,7 +6373,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -6213,7 +6393,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -6245,36 +6425,36 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{197DCCAF-E75B-41F9-A939-BF94359E828F}">
   <dimension ref="B1:R9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.265625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" s="184" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="261" t="s">
+      <c r="C2" s="262" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="262"/>
-      <c r="E2" s="262"/>
-      <c r="F2" s="262"/>
-      <c r="G2" s="262"/>
-      <c r="H2" s="262"/>
-      <c r="I2" s="262"/>
-      <c r="J2" s="262"/>
-      <c r="K2" s="262"/>
-      <c r="L2" s="262"/>
-      <c r="M2" s="262"/>
-      <c r="N2" s="262"/>
-      <c r="O2" s="262"/>
-      <c r="P2" s="262"/>
-      <c r="Q2" s="262"/>
-      <c r="R2" s="263"/>
-    </row>
-    <row r="3" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D2" s="263"/>
+      <c r="E2" s="263"/>
+      <c r="F2" s="263"/>
+      <c r="G2" s="263"/>
+      <c r="H2" s="263"/>
+      <c r="I2" s="263"/>
+      <c r="J2" s="263"/>
+      <c r="K2" s="263"/>
+      <c r="L2" s="263"/>
+      <c r="M2" s="263"/>
+      <c r="N2" s="263"/>
+      <c r="O2" s="263"/>
+      <c r="P2" s="263"/>
+      <c r="Q2" s="263"/>
+      <c r="R2" s="264"/>
+    </row>
+    <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="185"/>
       <c r="C3" s="118">
         <v>15</v>
@@ -6325,7 +6505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="88" t="s">
         <v>82</v>
       </c>
@@ -6346,15 +6526,15 @@
       <c r="M4" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="255" t="s">
+      <c r="N4" s="256" t="s">
         <v>89</v>
       </c>
-      <c r="O4" s="255"/>
-      <c r="P4" s="255"/>
-      <c r="Q4" s="255"/>
-      <c r="R4" s="256"/>
-    </row>
-    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="O4" s="256"/>
+      <c r="P4" s="256"/>
+      <c r="Q4" s="256"/>
+      <c r="R4" s="257"/>
+    </row>
+    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="89" t="s">
         <v>3</v>
       </c>
@@ -6366,18 +6546,18 @@
       <c r="H5" s="157"/>
       <c r="I5" s="157"/>
       <c r="J5" s="158"/>
-      <c r="K5" s="257" t="s">
+      <c r="K5" s="258" t="s">
         <v>85</v>
       </c>
-      <c r="L5" s="253"/>
-      <c r="M5" s="253"/>
-      <c r="N5" s="253"/>
-      <c r="O5" s="253"/>
-      <c r="P5" s="253"/>
-      <c r="Q5" s="253"/>
-      <c r="R5" s="254"/>
-    </row>
-    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="L5" s="254"/>
+      <c r="M5" s="254"/>
+      <c r="N5" s="254"/>
+      <c r="O5" s="254"/>
+      <c r="P5" s="254"/>
+      <c r="Q5" s="254"/>
+      <c r="R5" s="255"/>
+    </row>
+    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="89" t="s">
         <v>2</v>
       </c>
@@ -6389,18 +6569,18 @@
       <c r="H6" s="157"/>
       <c r="I6" s="157"/>
       <c r="J6" s="158"/>
-      <c r="K6" s="257" t="s">
+      <c r="K6" s="258" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="253"/>
-      <c r="M6" s="253"/>
-      <c r="N6" s="253"/>
-      <c r="O6" s="253"/>
-      <c r="P6" s="253"/>
-      <c r="Q6" s="253"/>
-      <c r="R6" s="254"/>
-    </row>
-    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="L6" s="254"/>
+      <c r="M6" s="254"/>
+      <c r="N6" s="254"/>
+      <c r="O6" s="254"/>
+      <c r="P6" s="254"/>
+      <c r="Q6" s="254"/>
+      <c r="R6" s="255"/>
+    </row>
+    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="89" t="s">
         <v>83</v>
       </c>
@@ -6412,41 +6592,41 @@
       <c r="H7" s="159"/>
       <c r="I7" s="159"/>
       <c r="J7" s="159"/>
-      <c r="K7" s="258" t="s">
+      <c r="K7" s="259" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="259"/>
-      <c r="M7" s="259"/>
-      <c r="N7" s="259"/>
-      <c r="O7" s="259"/>
-      <c r="P7" s="259"/>
-      <c r="Q7" s="259"/>
-      <c r="R7" s="260"/>
-    </row>
-    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="L7" s="260"/>
+      <c r="M7" s="260"/>
+      <c r="N7" s="260"/>
+      <c r="O7" s="260"/>
+      <c r="P7" s="260"/>
+      <c r="Q7" s="260"/>
+      <c r="R7" s="261"/>
+    </row>
+    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="89" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="252" t="s">
+      <c r="C8" s="253" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="253"/>
-      <c r="E8" s="253"/>
-      <c r="F8" s="253"/>
-      <c r="G8" s="253"/>
-      <c r="H8" s="253"/>
-      <c r="I8" s="253"/>
-      <c r="J8" s="253"/>
-      <c r="K8" s="253"/>
-      <c r="L8" s="253"/>
-      <c r="M8" s="253"/>
-      <c r="N8" s="253"/>
-      <c r="O8" s="253"/>
-      <c r="P8" s="253"/>
-      <c r="Q8" s="253"/>
-      <c r="R8" s="254"/>
-    </row>
-    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D8" s="254"/>
+      <c r="E8" s="254"/>
+      <c r="F8" s="254"/>
+      <c r="G8" s="254"/>
+      <c r="H8" s="254"/>
+      <c r="I8" s="254"/>
+      <c r="J8" s="254"/>
+      <c r="K8" s="254"/>
+      <c r="L8" s="254"/>
+      <c r="M8" s="254"/>
+      <c r="N8" s="254"/>
+      <c r="O8" s="254"/>
+      <c r="P8" s="254"/>
+      <c r="Q8" s="254"/>
+      <c r="R8" s="255"/>
+    </row>
+    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="90" t="s">
         <v>90</v>
       </c>
@@ -6491,15 +6671,15 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
   <dimension ref="B1:D17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.1328125" customWidth="1"/>
-    <col min="3" max="3" width="82.265625" customWidth="1"/>
-    <col min="4" max="4" width="43.9296875" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="82.28515625" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="160" t="s">
         <v>152</v>
       </c>
@@ -6507,7 +6687,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="161" t="s">
         <v>118</v>
       </c>
@@ -6515,7 +6695,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="163" t="s">
         <v>119</v>
       </c>
@@ -6523,7 +6703,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="161" t="s">
         <v>125</v>
       </c>
@@ -6531,7 +6711,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="163" t="s">
         <v>120</v>
       </c>
@@ -6539,7 +6719,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="161" t="s">
         <v>121</v>
       </c>
@@ -6547,7 +6727,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="8" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="164" t="s">
         <v>46</v>
       </c>
@@ -6555,8 +6735,8 @@
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="11" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="10" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="160" t="s">
         <v>152</v>
       </c>
@@ -6567,7 +6747,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="163" t="s">
         <v>156</v>
       </c>
@@ -6578,7 +6758,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="161" t="s">
         <v>158</v>
       </c>
@@ -6589,7 +6769,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="163" t="s">
         <v>160</v>
       </c>
@@ -6600,7 +6780,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="163" t="s">
         <v>121</v>
       </c>
@@ -6611,7 +6791,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="161" t="s">
         <v>169</v>
       </c>
@@ -6622,7 +6802,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="17" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="164" t="s">
         <v>46</v>
       </c>
@@ -6641,20 +6821,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D036B2-790A-4A3D-BD75-883CE886D2D8}">
   <dimension ref="B1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="7.265625" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="264" t="s">
+    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="265" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="265"/>
+      <c r="C2" s="266"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="143" t="s">
         <v>139</v>
       </c>
@@ -6663,79 +6843,79 @@
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="93"/>
       <c r="C4" s="133" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="266" t="s">
+      <c r="D4" s="267" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="95"/>
       <c r="C5" s="134" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="267"/>
-    </row>
-    <row r="6" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D5" s="268"/>
+    </row>
+    <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="136"/>
       <c r="C6" s="64" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="268"/>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="D6" s="269"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="144" t="s">
         <v>143</v>
       </c>
       <c r="C7" s="145"/>
-      <c r="D7" s="269" t="s">
+      <c r="D7" s="270" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="41" t="s">
         <v>142</v>
       </c>
       <c r="C8" s="146"/>
-      <c r="D8" s="270"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="D8" s="271"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="41" t="s">
         <v>144</v>
       </c>
       <c r="C9" s="146"/>
-      <c r="D9" s="270"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="D9" s="271"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="147" t="s">
         <v>145</v>
       </c>
       <c r="C10" s="148" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="270"/>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="D10" s="271"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="41" t="s">
         <v>142</v>
       </c>
       <c r="C11" s="134" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="270"/>
+      <c r="D11" s="271"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="149" t="s">
         <v>146</v>
       </c>
       <c r="C12" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="D12" s="271"/>
+      <c r="D12" s="272"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6745,4 +6925,295 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{728A29D2-349C-45CC-BF5A-2F605D047162}">
+  <dimension ref="B1:D40"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="4" width="38.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="287" t="s">
+        <v>195</v>
+      </c>
+      <c r="C2" s="285" t="s">
+        <v>194</v>
+      </c>
+      <c r="D2" s="286"/>
+    </row>
+    <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="288"/>
+      <c r="C3" s="289" t="s">
+        <v>191</v>
+      </c>
+      <c r="D3" s="290" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="89">
+        <v>0</v>
+      </c>
+      <c r="C4" s="147" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" s="230" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="273">
+        <v>1</v>
+      </c>
+      <c r="C5" s="294" t="s">
+        <v>200</v>
+      </c>
+      <c r="D5" s="277"/>
+    </row>
+    <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="89">
+        <v>2</v>
+      </c>
+      <c r="C6" s="275" t="s">
+        <v>196</v>
+      </c>
+      <c r="D6" s="280" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="273">
+        <v>3</v>
+      </c>
+      <c r="C7" s="220"/>
+      <c r="D7" s="224"/>
+    </row>
+    <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="89">
+        <v>4</v>
+      </c>
+      <c r="C8" s="276"/>
+      <c r="D8" s="277"/>
+    </row>
+    <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="273">
+        <v>5</v>
+      </c>
+      <c r="C9" s="95"/>
+      <c r="D9" s="278"/>
+    </row>
+    <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="89">
+        <v>6</v>
+      </c>
+      <c r="C10" s="139"/>
+      <c r="D10" s="146"/>
+    </row>
+    <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="274">
+        <v>7</v>
+      </c>
+      <c r="C11" s="136"/>
+      <c r="D11" s="279"/>
+    </row>
+    <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="291" t="s">
+        <v>197</v>
+      </c>
+      <c r="C14" s="292" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="89">
+        <v>0</v>
+      </c>
+      <c r="C15" s="26" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="273">
+        <v>1</v>
+      </c>
+      <c r="C16" s="281" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="89">
+        <v>2</v>
+      </c>
+      <c r="C17" s="26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B18" s="273">
+        <v>3</v>
+      </c>
+      <c r="C18" s="281" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="89">
+        <v>4</v>
+      </c>
+      <c r="C19" s="26" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="273">
+        <v>5</v>
+      </c>
+      <c r="C20" s="281"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="89">
+        <v>6</v>
+      </c>
+      <c r="C21" s="26"/>
+    </row>
+    <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="274">
+        <v>7</v>
+      </c>
+      <c r="C22" s="284"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="291" t="s">
+        <v>197</v>
+      </c>
+      <c r="C25" s="292" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="89">
+        <v>0</v>
+      </c>
+      <c r="C26" s="26" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B27" s="273">
+        <v>1</v>
+      </c>
+      <c r="C27" s="281" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B28" s="89">
+        <v>2</v>
+      </c>
+      <c r="C28" s="26" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="282">
+        <v>3</v>
+      </c>
+      <c r="C29" s="283" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="291" t="s">
+        <v>197</v>
+      </c>
+      <c r="C32" s="292" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" s="89">
+        <v>0</v>
+      </c>
+      <c r="C33" s="26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B34" s="273">
+        <v>1</v>
+      </c>
+      <c r="C34" s="281" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B35" s="89">
+        <v>2</v>
+      </c>
+      <c r="C35" s="26" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B36" s="273">
+        <v>3</v>
+      </c>
+      <c r="C36" s="281" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B37" s="89">
+        <v>4</v>
+      </c>
+      <c r="C37" s="26" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B38" s="273">
+        <v>5</v>
+      </c>
+      <c r="C38" s="281" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B39" s="92">
+        <v>6</v>
+      </c>
+      <c r="C39" s="293" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="282">
+        <v>7</v>
+      </c>
+      <c r="C40" s="283" t="s">
+        <v>190</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:D2"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="C6:C8"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Small modifications to the bridge-sequencer protocol
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C5E4F78-A1C7-4759-B290-A9B1BA735748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEB2F67-9CC5-4F47-BB95-820EBA17111D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="202">
   <si>
     <t>MODE B</t>
   </si>
@@ -648,6 +648,9 @@
   </si>
   <si>
     <t>ENABLE (0 = STOP, 1 = RUNNING)</t>
+  </si>
+  <si>
+    <t>reason</t>
   </si>
 </sst>
 </file>
@@ -2103,6 +2106,40 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2127,6 +2164,45 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2163,44 +2239,68 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2211,76 +2311,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2319,6 +2350,12 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2379,62 +2416,28 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="180"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="64" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="65" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="63" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2786,19 +2789,19 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="181" t="s">
+      <c r="B2" s="195" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="182"/>
-      <c r="D2" s="182"/>
-      <c r="E2" s="182"/>
-      <c r="F2" s="183"/>
-      <c r="G2" s="186" t="s">
+      <c r="C2" s="196"/>
+      <c r="D2" s="196"/>
+      <c r="E2" s="196"/>
+      <c r="F2" s="197"/>
+      <c r="G2" s="200" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="187"/>
-      <c r="I2" s="188"/>
-      <c r="J2" s="184" t="s">
+      <c r="H2" s="201"/>
+      <c r="I2" s="202"/>
+      <c r="J2" s="198" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2827,7 +2830,7 @@
       <c r="I3" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="J3" s="185"/>
+      <c r="J3" s="199"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="107">
@@ -3428,73 +3431,73 @@
       </c>
     </row>
     <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="198" t="s">
+      <c r="C3" s="225" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="199"/>
-      <c r="E3" s="199"/>
-      <c r="F3" s="199"/>
-      <c r="G3" s="200"/>
-      <c r="H3" s="195" t="s">
+      <c r="D3" s="226"/>
+      <c r="E3" s="226"/>
+      <c r="F3" s="226"/>
+      <c r="G3" s="227"/>
+      <c r="H3" s="222" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="196"/>
-      <c r="J3" s="197"/>
-      <c r="K3" s="195" t="s">
+      <c r="I3" s="223"/>
+      <c r="J3" s="224"/>
+      <c r="K3" s="222" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="196"/>
-      <c r="M3" s="196"/>
-      <c r="N3" s="207" t="s">
+      <c r="L3" s="223"/>
+      <c r="M3" s="223"/>
+      <c r="N3" s="209" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="208"/>
-      <c r="P3" s="209"/>
+      <c r="O3" s="210"/>
+      <c r="P3" s="211"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="201" t="s">
+      <c r="S3" s="203" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="202"/>
-      <c r="U3" s="202"/>
-      <c r="V3" s="202"/>
-      <c r="W3" s="202"/>
-      <c r="X3" s="202"/>
-      <c r="Y3" s="202"/>
-      <c r="Z3" s="203"/>
-      <c r="AA3" s="204" t="s">
+      <c r="T3" s="204"/>
+      <c r="U3" s="204"/>
+      <c r="V3" s="204"/>
+      <c r="W3" s="204"/>
+      <c r="X3" s="204"/>
+      <c r="Y3" s="204"/>
+      <c r="Z3" s="205"/>
+      <c r="AA3" s="206" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="205"/>
-      <c r="AC3" s="205"/>
-      <c r="AD3" s="205"/>
-      <c r="AE3" s="205"/>
-      <c r="AF3" s="205"/>
-      <c r="AG3" s="205"/>
-      <c r="AH3" s="206"/>
+      <c r="AB3" s="207"/>
+      <c r="AC3" s="207"/>
+      <c r="AD3" s="207"/>
+      <c r="AE3" s="207"/>
+      <c r="AF3" s="207"/>
+      <c r="AG3" s="207"/>
+      <c r="AH3" s="208"/>
     </row>
     <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="B5" s="212" t="s">
+      <c r="B5" s="214" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="210" t="s">
+      <c r="C5" s="212" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="210"/>
-      <c r="E5" s="210"/>
-      <c r="F5" s="210"/>
-      <c r="G5" s="210"/>
-      <c r="H5" s="210"/>
-      <c r="I5" s="210"/>
-      <c r="J5" s="211"/>
+      <c r="D5" s="212"/>
+      <c r="E5" s="212"/>
+      <c r="F5" s="212"/>
+      <c r="G5" s="212"/>
+      <c r="H5" s="212"/>
+      <c r="I5" s="212"/>
+      <c r="J5" s="213"/>
     </row>
     <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="213"/>
+      <c r="B6" s="215"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3524,16 +3527,16 @@
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="189" t="s">
+      <c r="C7" s="216" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="190"/>
-      <c r="E7" s="190"/>
-      <c r="F7" s="190"/>
-      <c r="G7" s="190"/>
-      <c r="H7" s="190"/>
-      <c r="I7" s="190"/>
-      <c r="J7" s="191"/>
+      <c r="D7" s="217"/>
+      <c r="E7" s="217"/>
+      <c r="F7" s="217"/>
+      <c r="G7" s="217"/>
+      <c r="H7" s="217"/>
+      <c r="I7" s="217"/>
+      <c r="J7" s="218"/>
     </row>
     <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
@@ -3543,25 +3546,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="192" t="s">
+      <c r="G8" s="219" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="193"/>
-      <c r="I8" s="193"/>
-      <c r="J8" s="194"/>
+      <c r="H8" s="220"/>
+      <c r="I8" s="220"/>
+      <c r="J8" s="221"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="C3:G3"/>
     <mergeCell ref="S3:Z3"/>
     <mergeCell ref="AA3:AH3"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="C5:J5"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3584,29 +3587,29 @@
   <sheetData>
     <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="214" t="s">
+      <c r="B2" s="249" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="215"/>
-      <c r="D2" s="215"/>
-      <c r="E2" s="215"/>
-      <c r="F2" s="215"/>
-      <c r="G2" s="216"/>
-      <c r="H2" s="184" t="s">
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="198" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="184" t="s">
+      <c r="I2" s="198" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="214" t="s">
+      <c r="J2" s="249" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="215"/>
-      <c r="L2" s="215"/>
-      <c r="M2" s="184" t="s">
+      <c r="K2" s="250"/>
+      <c r="L2" s="250"/>
+      <c r="M2" s="198" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="184" t="s">
+      <c r="N2" s="198" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3629,8 +3632,8 @@
       <c r="G3" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="185"/>
-      <c r="I3" s="185"/>
+      <c r="H3" s="199"/>
+      <c r="I3" s="199"/>
       <c r="J3" s="49" t="s">
         <v>3</v>
       </c>
@@ -3640,8 +3643,8 @@
       <c r="L3" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="185"/>
-      <c r="N3" s="185"/>
+      <c r="M3" s="199"/>
+      <c r="N3" s="199"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="81">
@@ -3667,7 +3670,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="217" t="s">
+      <c r="H4" s="230" t="s">
         <v>45</v>
       </c>
       <c r="I4" s="68" t="s">
@@ -3713,7 +3716,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="218"/>
+      <c r="H5" s="229"/>
       <c r="I5" s="43" t="s">
         <v>3</v>
       </c>
@@ -3757,25 +3760,25 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="219" t="s">
+      <c r="H6" s="228" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="220" t="s">
+      <c r="J6" s="232" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="222" t="s">
+      <c r="K6" s="241" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="224" t="s">
+      <c r="L6" s="238" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="232" t="s">
+      <c r="M6" s="243" t="s">
         <v>113</v>
       </c>
-      <c r="N6" s="226" t="s">
+      <c r="N6" s="246" t="s">
         <v>71</v>
       </c>
     </row>
@@ -3803,15 +3806,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="219"/>
+      <c r="H7" s="228"/>
       <c r="I7" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="220"/>
-      <c r="K7" s="222"/>
-      <c r="L7" s="224"/>
-      <c r="M7" s="233"/>
-      <c r="N7" s="226"/>
+      <c r="J7" s="232"/>
+      <c r="K7" s="241"/>
+      <c r="L7" s="238"/>
+      <c r="M7" s="244"/>
+      <c r="N7" s="246"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="82">
@@ -3837,15 +3840,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="219"/>
+      <c r="H8" s="228"/>
       <c r="I8" s="91" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="220"/>
-      <c r="K8" s="222"/>
-      <c r="L8" s="224"/>
-      <c r="M8" s="233"/>
-      <c r="N8" s="226"/>
+      <c r="J8" s="232"/>
+      <c r="K8" s="241"/>
+      <c r="L8" s="238"/>
+      <c r="M8" s="244"/>
+      <c r="N8" s="246"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="82">
@@ -3871,15 +3874,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="219"/>
+      <c r="H9" s="228"/>
       <c r="I9" s="91" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="220"/>
-      <c r="K9" s="222"/>
-      <c r="L9" s="224"/>
-      <c r="M9" s="233"/>
-      <c r="N9" s="226"/>
+      <c r="J9" s="232"/>
+      <c r="K9" s="241"/>
+      <c r="L9" s="238"/>
+      <c r="M9" s="244"/>
+      <c r="N9" s="246"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="82">
@@ -3905,15 +3908,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="219"/>
+      <c r="H10" s="228"/>
       <c r="I10" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="220"/>
-      <c r="K10" s="222"/>
-      <c r="L10" s="224"/>
-      <c r="M10" s="233"/>
-      <c r="N10" s="226"/>
+      <c r="J10" s="232"/>
+      <c r="K10" s="241"/>
+      <c r="L10" s="238"/>
+      <c r="M10" s="244"/>
+      <c r="N10" s="246"/>
     </row>
     <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="83">
@@ -3939,15 +3942,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="218"/>
+      <c r="H11" s="229"/>
       <c r="I11" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="221"/>
-      <c r="K11" s="223"/>
-      <c r="L11" s="225"/>
-      <c r="M11" s="234"/>
-      <c r="N11" s="227"/>
+      <c r="J11" s="233"/>
+      <c r="K11" s="242"/>
+      <c r="L11" s="239"/>
+      <c r="M11" s="245"/>
+      <c r="N11" s="247"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="81">
@@ -3973,25 +3976,25 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="217" t="s">
+      <c r="H12" s="230" t="s">
         <v>55</v>
       </c>
       <c r="I12" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="228" t="s">
+      <c r="J12" s="231" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="229" t="s">
+      <c r="K12" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="230" t="s">
+      <c r="L12" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="217" t="s">
+      <c r="M12" s="230" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="231" t="s">
+      <c r="N12" s="248" t="s">
         <v>104</v>
       </c>
     </row>
@@ -4019,15 +4022,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="219"/>
+      <c r="H13" s="228"/>
       <c r="I13" s="91" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="220"/>
-      <c r="K13" s="222"/>
-      <c r="L13" s="224"/>
-      <c r="M13" s="219"/>
-      <c r="N13" s="226"/>
+      <c r="J13" s="232"/>
+      <c r="K13" s="241"/>
+      <c r="L13" s="238"/>
+      <c r="M13" s="228"/>
+      <c r="N13" s="246"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="82">
@@ -4053,15 +4056,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="219"/>
+      <c r="H14" s="228"/>
       <c r="I14" s="91" t="s">
         <v>102</v>
       </c>
-      <c r="J14" s="220"/>
-      <c r="K14" s="222"/>
-      <c r="L14" s="224"/>
-      <c r="M14" s="219"/>
-      <c r="N14" s="226"/>
+      <c r="J14" s="232"/>
+      <c r="K14" s="241"/>
+      <c r="L14" s="238"/>
+      <c r="M14" s="228"/>
+      <c r="N14" s="246"/>
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="83">
@@ -4087,15 +4090,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="218"/>
+      <c r="H15" s="229"/>
       <c r="I15" s="44" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="221"/>
-      <c r="K15" s="223"/>
-      <c r="L15" s="225"/>
-      <c r="M15" s="218"/>
-      <c r="N15" s="227"/>
+      <c r="J15" s="233"/>
+      <c r="K15" s="242"/>
+      <c r="L15" s="239"/>
+      <c r="M15" s="229"/>
+      <c r="N15" s="247"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="81">
@@ -4121,22 +4124,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="217" t="s">
+      <c r="H16" s="230" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="228" t="s">
+      <c r="J16" s="231" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="235" t="s">
+      <c r="K16" s="234" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="230" t="s">
+      <c r="L16" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M16" s="217" t="s">
+      <c r="M16" s="230" t="s">
         <v>114</v>
       </c>
       <c r="N16" s="76" t="s">
@@ -4167,14 +4170,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="219"/>
+      <c r="H17" s="228"/>
       <c r="I17" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="220"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="224"/>
-      <c r="M17" s="219"/>
+      <c r="J17" s="232"/>
+      <c r="K17" s="235"/>
+      <c r="L17" s="238"/>
+      <c r="M17" s="228"/>
       <c r="N17" s="75" t="s">
         <v>105</v>
       </c>
@@ -4203,14 +4206,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="219"/>
+      <c r="H18" s="228"/>
       <c r="I18" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="220"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="224"/>
-      <c r="M18" s="219"/>
+      <c r="J18" s="232"/>
+      <c r="K18" s="235"/>
+      <c r="L18" s="238"/>
+      <c r="M18" s="228"/>
       <c r="N18" s="75" t="s">
         <v>107</v>
       </c>
@@ -4239,14 +4242,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="218"/>
+      <c r="H19" s="229"/>
       <c r="I19" s="44" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="221"/>
-      <c r="K19" s="237"/>
-      <c r="L19" s="225"/>
-      <c r="M19" s="218"/>
+      <c r="J19" s="233"/>
+      <c r="K19" s="236"/>
+      <c r="L19" s="239"/>
+      <c r="M19" s="229"/>
       <c r="N19" s="45" t="s">
         <v>108</v>
       </c>
@@ -4276,22 +4279,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="217" t="s">
+      <c r="H20" s="230" t="s">
         <v>57</v>
       </c>
       <c r="I20" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="228" t="s">
+      <c r="J20" s="231" t="s">
         <v>16</v>
       </c>
-      <c r="K20" s="229" t="s">
+      <c r="K20" s="240" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="230" t="s">
+      <c r="L20" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="232" t="s">
+      <c r="M20" s="243" t="s">
         <v>113</v>
       </c>
       <c r="N20" s="42" t="s">
@@ -4322,14 +4325,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="219"/>
+      <c r="H21" s="228"/>
       <c r="I21" s="71" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="220"/>
-      <c r="K21" s="222"/>
-      <c r="L21" s="224"/>
-      <c r="M21" s="233"/>
+      <c r="J21" s="232"/>
+      <c r="K21" s="241"/>
+      <c r="L21" s="238"/>
+      <c r="M21" s="244"/>
       <c r="N21" s="75" t="s">
         <v>99</v>
       </c>
@@ -4358,14 +4361,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="219"/>
+      <c r="H22" s="228"/>
       <c r="I22" s="71" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="220"/>
-      <c r="K22" s="222"/>
-      <c r="L22" s="224"/>
-      <c r="M22" s="233"/>
+      <c r="J22" s="232"/>
+      <c r="K22" s="241"/>
+      <c r="L22" s="238"/>
+      <c r="M22" s="244"/>
       <c r="N22" s="75" t="s">
         <v>100</v>
       </c>
@@ -4394,14 +4397,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="218"/>
+      <c r="H23" s="229"/>
       <c r="I23" s="43" t="s">
         <v>21</v>
       </c>
-      <c r="J23" s="221"/>
-      <c r="K23" s="223"/>
-      <c r="L23" s="225"/>
-      <c r="M23" s="234"/>
+      <c r="J23" s="233"/>
+      <c r="K23" s="242"/>
+      <c r="L23" s="239"/>
+      <c r="M23" s="245"/>
       <c r="N23" s="42" t="s">
         <v>101</v>
       </c>
@@ -4430,7 +4433,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="217" t="s">
+      <c r="H24" s="230" t="s">
         <v>58</v>
       </c>
       <c r="I24" s="65" t="s">
@@ -4476,7 +4479,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="219"/>
+      <c r="H25" s="228"/>
       <c r="I25" s="71" t="s">
         <v>46</v>
       </c>
@@ -4520,7 +4523,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="219"/>
+      <c r="H26" s="228"/>
       <c r="I26" s="105"/>
       <c r="J26" s="139"/>
       <c r="K26" s="140"/>
@@ -4552,7 +4555,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="218"/>
+      <c r="H27" s="229"/>
       <c r="I27" s="98"/>
       <c r="J27" s="136"/>
       <c r="K27" s="137"/>
@@ -4584,7 +4587,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="217" t="s">
+      <c r="H28" s="230" t="s">
         <v>60</v>
       </c>
       <c r="I28" s="38" t="s">
@@ -4630,7 +4633,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="219"/>
+      <c r="H29" s="228"/>
       <c r="I29" s="71" t="s">
         <v>52</v>
       </c>
@@ -4674,7 +4677,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="219"/>
+      <c r="H30" s="228"/>
       <c r="I30" s="71" t="s">
         <v>53</v>
       </c>
@@ -4718,7 +4721,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="218"/>
+      <c r="H31" s="229"/>
       <c r="I31" s="92"/>
       <c r="J31" s="95"/>
       <c r="K31" s="96"/>
@@ -4750,7 +4753,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="219" t="s">
+      <c r="H32" s="228" t="s">
         <v>59</v>
       </c>
       <c r="I32" s="65" t="s">
@@ -4797,7 +4800,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="219"/>
+      <c r="H33" s="228"/>
       <c r="I33" s="71" t="s">
         <v>24</v>
       </c>
@@ -4842,7 +4845,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="218"/>
+      <c r="H34" s="229"/>
       <c r="I34" s="98"/>
       <c r="J34" s="95"/>
       <c r="K34" s="96"/>
@@ -4899,11 +4902,25 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="N6:N11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="N12:N15"/>
+    <mergeCell ref="M6:M11"/>
     <mergeCell ref="K16:K19"/>
     <mergeCell ref="L16:L19"/>
     <mergeCell ref="M16:M19"/>
@@ -4912,25 +4929,11 @@
     <mergeCell ref="K20:K23"/>
     <mergeCell ref="L20:L23"/>
     <mergeCell ref="M20:M23"/>
-    <mergeCell ref="N6:N11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="N12:N15"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4952,26 +4955,26 @@
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="214" t="s">
+      <c r="B2" s="249" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="215"/>
-      <c r="D2" s="215"/>
-      <c r="E2" s="215"/>
-      <c r="F2" s="215"/>
-      <c r="G2" s="216"/>
-      <c r="H2" s="184" t="s">
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="250"/>
+      <c r="G2" s="251"/>
+      <c r="H2" s="198" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="184" t="s">
+      <c r="I2" s="198" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="214" t="s">
+      <c r="J2" s="249" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="215"/>
-      <c r="L2" s="215"/>
-      <c r="M2" s="184" t="s">
+      <c r="K2" s="250"/>
+      <c r="L2" s="250"/>
+      <c r="M2" s="198" t="s">
         <v>33</v>
       </c>
     </row>
@@ -4994,8 +4997,8 @@
       <c r="G3" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="185"/>
-      <c r="I3" s="185"/>
+      <c r="H3" s="199"/>
+      <c r="I3" s="199"/>
       <c r="J3" s="49" t="s">
         <v>3</v>
       </c>
@@ -5005,7 +5008,7 @@
       <c r="L3" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="185"/>
+      <c r="M3" s="199"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="81">
@@ -5031,7 +5034,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="217" t="s">
+      <c r="H4" s="230" t="s">
         <v>45</v>
       </c>
       <c r="I4" s="68" t="s">
@@ -5074,7 +5077,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="218"/>
+      <c r="H5" s="229"/>
       <c r="I5" s="43" t="s">
         <v>3</v>
       </c>
@@ -5115,22 +5118,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="219" t="s">
+      <c r="H6" s="228" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="91" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="220" t="s">
+      <c r="J6" s="232" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="222" t="s">
+      <c r="K6" s="241" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="224" t="s">
+      <c r="L6" s="238" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="226" t="s">
+      <c r="M6" s="246" t="s">
         <v>71</v>
       </c>
     </row>
@@ -5158,12 +5161,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="219"/>
-      <c r="I7" s="238"/>
-      <c r="J7" s="220"/>
-      <c r="K7" s="222"/>
-      <c r="L7" s="224"/>
-      <c r="M7" s="226"/>
+      <c r="H7" s="228"/>
+      <c r="I7" s="252"/>
+      <c r="J7" s="232"/>
+      <c r="K7" s="241"/>
+      <c r="L7" s="238"/>
+      <c r="M7" s="246"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="82">
@@ -5189,12 +5192,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="219"/>
-      <c r="I8" s="239"/>
-      <c r="J8" s="220"/>
-      <c r="K8" s="222"/>
-      <c r="L8" s="224"/>
-      <c r="M8" s="226"/>
+      <c r="H8" s="228"/>
+      <c r="I8" s="265"/>
+      <c r="J8" s="232"/>
+      <c r="K8" s="241"/>
+      <c r="L8" s="238"/>
+      <c r="M8" s="246"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="82">
@@ -5220,12 +5223,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="219"/>
-      <c r="I9" s="240"/>
-      <c r="J9" s="220"/>
-      <c r="K9" s="222"/>
-      <c r="L9" s="224"/>
-      <c r="M9" s="226"/>
+      <c r="H9" s="228"/>
+      <c r="I9" s="266"/>
+      <c r="J9" s="232"/>
+      <c r="K9" s="241"/>
+      <c r="L9" s="238"/>
+      <c r="M9" s="246"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="82">
@@ -5251,14 +5254,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="219"/>
+      <c r="H10" s="228"/>
       <c r="I10" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="220"/>
-      <c r="K10" s="222"/>
-      <c r="L10" s="224"/>
-      <c r="M10" s="226"/>
+      <c r="J10" s="232"/>
+      <c r="K10" s="241"/>
+      <c r="L10" s="238"/>
+      <c r="M10" s="246"/>
     </row>
     <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="83">
@@ -5284,12 +5287,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="218"/>
+      <c r="H11" s="229"/>
       <c r="I11" s="105"/>
-      <c r="J11" s="221"/>
-      <c r="K11" s="223"/>
-      <c r="L11" s="225"/>
-      <c r="M11" s="227"/>
+      <c r="J11" s="233"/>
+      <c r="K11" s="242"/>
+      <c r="L11" s="239"/>
+      <c r="M11" s="247"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="81">
@@ -5315,22 +5318,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="217" t="s">
+      <c r="H12" s="230" t="s">
         <v>55</v>
       </c>
       <c r="I12" s="65" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="228" t="s">
+      <c r="J12" s="231" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="229" t="s">
+      <c r="K12" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="230" t="s">
+      <c r="L12" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="231" t="s">
+      <c r="M12" s="248" t="s">
         <v>104</v>
       </c>
     </row>
@@ -5358,12 +5361,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="219"/>
-      <c r="I13" s="238"/>
-      <c r="J13" s="220"/>
-      <c r="K13" s="222"/>
-      <c r="L13" s="224"/>
-      <c r="M13" s="226"/>
+      <c r="H13" s="228"/>
+      <c r="I13" s="252"/>
+      <c r="J13" s="232"/>
+      <c r="K13" s="241"/>
+      <c r="L13" s="238"/>
+      <c r="M13" s="246"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="82">
@@ -5389,12 +5392,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="219"/>
-      <c r="I14" s="239"/>
-      <c r="J14" s="220"/>
-      <c r="K14" s="222"/>
-      <c r="L14" s="224"/>
-      <c r="M14" s="226"/>
+      <c r="H14" s="228"/>
+      <c r="I14" s="265"/>
+      <c r="J14" s="232"/>
+      <c r="K14" s="241"/>
+      <c r="L14" s="238"/>
+      <c r="M14" s="246"/>
     </row>
     <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="83">
@@ -5420,12 +5423,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="218"/>
-      <c r="I15" s="241"/>
-      <c r="J15" s="221"/>
-      <c r="K15" s="223"/>
-      <c r="L15" s="225"/>
-      <c r="M15" s="227"/>
+      <c r="H15" s="229"/>
+      <c r="I15" s="253"/>
+      <c r="J15" s="233"/>
+      <c r="K15" s="242"/>
+      <c r="L15" s="239"/>
+      <c r="M15" s="247"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="81">
@@ -5451,19 +5454,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="217" t="s">
+      <c r="H16" s="230" t="s">
         <v>56</v>
       </c>
       <c r="I16" s="65" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="228" t="s">
+      <c r="J16" s="231" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="235" t="s">
+      <c r="K16" s="234" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="230" t="s">
+      <c r="L16" s="237" t="s">
         <v>66</v>
       </c>
       <c r="M16" s="76" t="s">
@@ -5494,13 +5497,13 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="219"/>
+      <c r="H17" s="228"/>
       <c r="I17" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="220"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="224"/>
+      <c r="J17" s="232"/>
+      <c r="K17" s="235"/>
+      <c r="L17" s="238"/>
       <c r="M17" s="75" t="s">
         <v>105</v>
       </c>
@@ -5529,12 +5532,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="219"/>
-      <c r="I18" s="238"/>
-      <c r="J18" s="220"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="224"/>
-      <c r="M18" s="238"/>
+      <c r="H18" s="228"/>
+      <c r="I18" s="252"/>
+      <c r="J18" s="232"/>
+      <c r="K18" s="235"/>
+      <c r="L18" s="238"/>
+      <c r="M18" s="252"/>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="83">
@@ -5560,12 +5563,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="218"/>
-      <c r="I19" s="241"/>
-      <c r="J19" s="221"/>
-      <c r="K19" s="237"/>
-      <c r="L19" s="225"/>
-      <c r="M19" s="241"/>
+      <c r="H19" s="229"/>
+      <c r="I19" s="253"/>
+      <c r="J19" s="233"/>
+      <c r="K19" s="236"/>
+      <c r="L19" s="239"/>
+      <c r="M19" s="253"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
@@ -5592,7 +5595,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="242" t="s">
+      <c r="H20" s="254" t="s">
         <v>179</v>
       </c>
       <c r="I20" s="180" t="s">
@@ -5635,7 +5638,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="243"/>
+      <c r="H21" s="255"/>
       <c r="I21" s="171"/>
       <c r="J21" s="173"/>
       <c r="K21" s="175"/>
@@ -5666,7 +5669,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="243"/>
+      <c r="H22" s="255"/>
       <c r="I22" s="171"/>
       <c r="J22" s="173"/>
       <c r="K22" s="175"/>
@@ -5697,7 +5700,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="244"/>
+      <c r="H23" s="256"/>
       <c r="I23" s="172"/>
       <c r="J23" s="174"/>
       <c r="K23" s="176"/>
@@ -5728,7 +5731,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="217" t="s">
+      <c r="H24" s="230" t="s">
         <v>58</v>
       </c>
       <c r="I24" s="65" t="s">
@@ -5771,7 +5774,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="219"/>
+      <c r="H25" s="228"/>
       <c r="I25" s="71" t="s">
         <v>46</v>
       </c>
@@ -5812,12 +5815,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="219"/>
-      <c r="I26" s="238"/>
-      <c r="J26" s="245"/>
-      <c r="K26" s="247"/>
-      <c r="L26" s="249"/>
-      <c r="M26" s="251"/>
+      <c r="H26" s="228"/>
+      <c r="I26" s="252"/>
+      <c r="J26" s="257"/>
+      <c r="K26" s="259"/>
+      <c r="L26" s="261"/>
+      <c r="M26" s="263"/>
     </row>
     <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="83">
@@ -5843,12 +5846,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="218"/>
-      <c r="I27" s="241"/>
-      <c r="J27" s="246"/>
-      <c r="K27" s="248"/>
-      <c r="L27" s="250"/>
-      <c r="M27" s="252"/>
+      <c r="H27" s="229"/>
+      <c r="I27" s="253"/>
+      <c r="J27" s="258"/>
+      <c r="K27" s="260"/>
+      <c r="L27" s="262"/>
+      <c r="M27" s="264"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="81">
@@ -5874,7 +5877,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="217" t="s">
+      <c r="H28" s="230" t="s">
         <v>167</v>
       </c>
       <c r="I28" s="38" t="s">
@@ -5917,7 +5920,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="219"/>
+      <c r="H29" s="228"/>
       <c r="I29" s="71" t="s">
         <v>52</v>
       </c>
@@ -5958,7 +5961,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="219"/>
+      <c r="H30" s="228"/>
       <c r="I30" s="71" t="s">
         <v>53</v>
       </c>
@@ -5999,7 +6002,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="218"/>
+      <c r="H31" s="229"/>
       <c r="I31" s="92"/>
       <c r="J31" s="166"/>
       <c r="K31" s="167"/>
@@ -6030,7 +6033,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="219" t="s">
+      <c r="H32" s="228" t="s">
         <v>168</v>
       </c>
       <c r="I32" s="38" t="s">
@@ -6074,7 +6077,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="219"/>
+      <c r="H33" s="228"/>
       <c r="I33" s="71" t="s">
         <v>52</v>
       </c>
@@ -6116,7 +6119,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="218"/>
+      <c r="H34" s="229"/>
       <c r="I34" s="71" t="s">
         <v>53</v>
       </c>
@@ -6179,6 +6182,24 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6194,24 +6215,6 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6228,13 +6231,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="214" t="s">
+      <c r="B2" s="249" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="215"/>
-      <c r="D2" s="215"/>
-      <c r="E2" s="216"/>
-      <c r="F2" s="184" t="s">
+      <c r="C2" s="250"/>
+      <c r="D2" s="250"/>
+      <c r="E2" s="251"/>
+      <c r="F2" s="198" t="s">
         <v>32</v>
       </c>
     </row>
@@ -6251,7 +6254,7 @@
       <c r="E3" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="185"/>
+      <c r="F3" s="199"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="13">
@@ -6432,30 +6435,30 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="184" t="s">
+      <c r="B2" s="198" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="262" t="s">
+      <c r="C2" s="276" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="263"/>
-      <c r="E2" s="263"/>
-      <c r="F2" s="263"/>
-      <c r="G2" s="263"/>
-      <c r="H2" s="263"/>
-      <c r="I2" s="263"/>
-      <c r="J2" s="263"/>
-      <c r="K2" s="263"/>
-      <c r="L2" s="263"/>
-      <c r="M2" s="263"/>
-      <c r="N2" s="263"/>
-      <c r="O2" s="263"/>
-      <c r="P2" s="263"/>
-      <c r="Q2" s="263"/>
-      <c r="R2" s="264"/>
+      <c r="D2" s="277"/>
+      <c r="E2" s="277"/>
+      <c r="F2" s="277"/>
+      <c r="G2" s="277"/>
+      <c r="H2" s="277"/>
+      <c r="I2" s="277"/>
+      <c r="J2" s="277"/>
+      <c r="K2" s="277"/>
+      <c r="L2" s="277"/>
+      <c r="M2" s="277"/>
+      <c r="N2" s="277"/>
+      <c r="O2" s="277"/>
+      <c r="P2" s="277"/>
+      <c r="Q2" s="277"/>
+      <c r="R2" s="278"/>
     </row>
     <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="185"/>
+      <c r="B3" s="199"/>
       <c r="C3" s="118">
         <v>15</v>
       </c>
@@ -6526,13 +6529,13 @@
       <c r="M4" s="69" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="256" t="s">
+      <c r="N4" s="270" t="s">
         <v>89</v>
       </c>
-      <c r="O4" s="256"/>
-      <c r="P4" s="256"/>
-      <c r="Q4" s="256"/>
-      <c r="R4" s="257"/>
+      <c r="O4" s="270"/>
+      <c r="P4" s="270"/>
+      <c r="Q4" s="270"/>
+      <c r="R4" s="271"/>
     </row>
     <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="89" t="s">
@@ -6546,16 +6549,16 @@
       <c r="H5" s="157"/>
       <c r="I5" s="157"/>
       <c r="J5" s="158"/>
-      <c r="K5" s="258" t="s">
+      <c r="K5" s="272" t="s">
         <v>85</v>
       </c>
-      <c r="L5" s="254"/>
-      <c r="M5" s="254"/>
-      <c r="N5" s="254"/>
-      <c r="O5" s="254"/>
-      <c r="P5" s="254"/>
-      <c r="Q5" s="254"/>
-      <c r="R5" s="255"/>
+      <c r="L5" s="268"/>
+      <c r="M5" s="268"/>
+      <c r="N5" s="268"/>
+      <c r="O5" s="268"/>
+      <c r="P5" s="268"/>
+      <c r="Q5" s="268"/>
+      <c r="R5" s="269"/>
     </row>
     <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="89" t="s">
@@ -6569,16 +6572,16 @@
       <c r="H6" s="157"/>
       <c r="I6" s="157"/>
       <c r="J6" s="158"/>
-      <c r="K6" s="258" t="s">
+      <c r="K6" s="272" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="254"/>
-      <c r="M6" s="254"/>
-      <c r="N6" s="254"/>
-      <c r="O6" s="254"/>
-      <c r="P6" s="254"/>
-      <c r="Q6" s="254"/>
-      <c r="R6" s="255"/>
+      <c r="L6" s="268"/>
+      <c r="M6" s="268"/>
+      <c r="N6" s="268"/>
+      <c r="O6" s="268"/>
+      <c r="P6" s="268"/>
+      <c r="Q6" s="268"/>
+      <c r="R6" s="269"/>
     </row>
     <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="89" t="s">
@@ -6592,39 +6595,39 @@
       <c r="H7" s="159"/>
       <c r="I7" s="159"/>
       <c r="J7" s="159"/>
-      <c r="K7" s="259" t="s">
+      <c r="K7" s="273" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="260"/>
-      <c r="M7" s="260"/>
-      <c r="N7" s="260"/>
-      <c r="O7" s="260"/>
-      <c r="P7" s="260"/>
-      <c r="Q7" s="260"/>
-      <c r="R7" s="261"/>
+      <c r="L7" s="274"/>
+      <c r="M7" s="274"/>
+      <c r="N7" s="274"/>
+      <c r="O7" s="274"/>
+      <c r="P7" s="274"/>
+      <c r="Q7" s="274"/>
+      <c r="R7" s="275"/>
     </row>
     <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="89" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="253" t="s">
+      <c r="C8" s="267" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="254"/>
-      <c r="E8" s="254"/>
-      <c r="F8" s="254"/>
-      <c r="G8" s="254"/>
-      <c r="H8" s="254"/>
-      <c r="I8" s="254"/>
-      <c r="J8" s="254"/>
-      <c r="K8" s="254"/>
-      <c r="L8" s="254"/>
-      <c r="M8" s="254"/>
-      <c r="N8" s="254"/>
-      <c r="O8" s="254"/>
-      <c r="P8" s="254"/>
-      <c r="Q8" s="254"/>
-      <c r="R8" s="255"/>
+      <c r="D8" s="268"/>
+      <c r="E8" s="268"/>
+      <c r="F8" s="268"/>
+      <c r="G8" s="268"/>
+      <c r="H8" s="268"/>
+      <c r="I8" s="268"/>
+      <c r="J8" s="268"/>
+      <c r="K8" s="268"/>
+      <c r="L8" s="268"/>
+      <c r="M8" s="268"/>
+      <c r="N8" s="268"/>
+      <c r="O8" s="268"/>
+      <c r="P8" s="268"/>
+      <c r="Q8" s="268"/>
+      <c r="R8" s="269"/>
     </row>
     <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="90" t="s">
@@ -6828,10 +6831,10 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="265" t="s">
+      <c r="B2" s="279" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="266"/>
+      <c r="C2" s="280"/>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6848,7 +6851,7 @@
       <c r="C4" s="133" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="267" t="s">
+      <c r="D4" s="281" t="s">
         <v>148</v>
       </c>
     </row>
@@ -6857,21 +6860,21 @@
       <c r="C5" s="134" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="268"/>
+      <c r="D5" s="282"/>
     </row>
     <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="136"/>
       <c r="C6" s="64" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="269"/>
+      <c r="D6" s="283"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="144" t="s">
         <v>143</v>
       </c>
       <c r="C7" s="145"/>
-      <c r="D7" s="270" t="s">
+      <c r="D7" s="284" t="s">
         <v>149</v>
       </c>
     </row>
@@ -6880,14 +6883,14 @@
         <v>142</v>
       </c>
       <c r="C8" s="146"/>
-      <c r="D8" s="271"/>
+      <c r="D8" s="285"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="41" t="s">
         <v>144</v>
       </c>
       <c r="C9" s="146"/>
-      <c r="D9" s="271"/>
+      <c r="D9" s="285"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="147" t="s">
@@ -6896,7 +6899,7 @@
       <c r="C10" s="148" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="271"/>
+      <c r="D10" s="285"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="41" t="s">
@@ -6905,7 +6908,7 @@
       <c r="C11" s="134" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="271"/>
+      <c r="D11" s="285"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6915,7 +6918,7 @@
       <c r="C12" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="D12" s="272"/>
+      <c r="D12" s="286"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6940,17 +6943,17 @@
       <c r="B2" s="287" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="285" t="s">
+      <c r="C2" s="289" t="s">
         <v>194</v>
       </c>
-      <c r="D2" s="286"/>
+      <c r="D2" s="290"/>
     </row>
     <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="288"/>
-      <c r="C3" s="289" t="s">
+      <c r="C3" s="189" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="290" t="s">
+      <c r="D3" s="190" t="s">
         <v>192</v>
       </c>
     </row>
@@ -6961,50 +6964,50 @@
       <c r="C4" s="147" t="s">
         <v>199</v>
       </c>
-      <c r="D4" s="230" t="s">
+      <c r="D4" s="237" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="273">
-        <v>1</v>
-      </c>
-      <c r="C5" s="294" t="s">
+      <c r="B5" s="181">
+        <v>1</v>
+      </c>
+      <c r="C5" s="194" t="s">
         <v>200</v>
       </c>
-      <c r="D5" s="277"/>
+      <c r="D5" s="291"/>
     </row>
     <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="89">
         <v>2</v>
       </c>
-      <c r="C6" s="275" t="s">
+      <c r="C6" s="293" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="280" t="s">
+      <c r="D6" s="292" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="273">
+      <c r="B7" s="181">
         <v>3</v>
       </c>
-      <c r="C7" s="220"/>
-      <c r="D7" s="224"/>
+      <c r="C7" s="232"/>
+      <c r="D7" s="238"/>
     </row>
     <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="89">
         <v>4</v>
       </c>
-      <c r="C8" s="276"/>
-      <c r="D8" s="277"/>
+      <c r="C8" s="294"/>
+      <c r="D8" s="291"/>
     </row>
     <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="273">
+      <c r="B9" s="181">
         <v>5</v>
       </c>
       <c r="C9" s="95"/>
-      <c r="D9" s="278"/>
+      <c r="D9" s="183"/>
     </row>
     <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="89">
@@ -7014,18 +7017,20 @@
       <c r="D10" s="146"/>
     </row>
     <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="274">
+      <c r="B11" s="182">
         <v>7</v>
       </c>
       <c r="C11" s="136"/>
-      <c r="D11" s="279"/>
+      <c r="D11" s="184" t="s">
+        <v>201</v>
+      </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="291" t="s">
+      <c r="B14" s="191" t="s">
         <v>197</v>
       </c>
-      <c r="C14" s="292" t="s">
+      <c r="C14" s="192" t="s">
         <v>196</v>
       </c>
     </row>
@@ -7038,10 +7043,10 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="273">
-        <v>1</v>
-      </c>
-      <c r="C16" s="281" t="s">
+      <c r="B16" s="181">
+        <v>1</v>
+      </c>
+      <c r="C16" s="185" t="s">
         <v>185</v>
       </c>
     </row>
@@ -7054,10 +7059,10 @@
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="273">
+      <c r="B18" s="181">
         <v>3</v>
       </c>
-      <c r="C18" s="281" t="s">
+      <c r="C18" s="185" t="s">
         <v>183</v>
       </c>
     </row>
@@ -7070,10 +7075,10 @@
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="273">
+      <c r="B20" s="181">
         <v>5</v>
       </c>
-      <c r="C20" s="281"/>
+      <c r="C20" s="185"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="89">
@@ -7082,10 +7087,10 @@
       <c r="C21" s="26"/>
     </row>
     <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="274">
+      <c r="B22" s="182">
         <v>7</v>
       </c>
-      <c r="C22" s="284"/>
+      <c r="C22" s="188"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
@@ -7094,10 +7099,10 @@
       <c r="B24" s="1"/>
     </row>
     <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="291" t="s">
+      <c r="B25" s="191" t="s">
         <v>197</v>
       </c>
-      <c r="C25" s="292" t="s">
+      <c r="C25" s="192" t="s">
         <v>189</v>
       </c>
     </row>
@@ -7110,10 +7115,10 @@
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="273">
-        <v>1</v>
-      </c>
-      <c r="C27" s="281" t="s">
+      <c r="B27" s="181">
+        <v>1</v>
+      </c>
+      <c r="C27" s="185" t="s">
         <v>187</v>
       </c>
     </row>
@@ -7126,19 +7131,19 @@
       </c>
     </row>
     <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="282">
+      <c r="B29" s="186">
         <v>3</v>
       </c>
-      <c r="C29" s="283" t="s">
+      <c r="C29" s="187" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="291" t="s">
+      <c r="B32" s="191" t="s">
         <v>197</v>
       </c>
-      <c r="C32" s="292" t="s">
+      <c r="C32" s="192" t="s">
         <v>193</v>
       </c>
     </row>
@@ -7151,10 +7156,10 @@
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="273">
-        <v>1</v>
-      </c>
-      <c r="C34" s="281" t="s">
+      <c r="B34" s="181">
+        <v>1</v>
+      </c>
+      <c r="C34" s="185" t="s">
         <v>158</v>
       </c>
     </row>
@@ -7167,10 +7172,10 @@
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B36" s="273">
+      <c r="B36" s="181">
         <v>3</v>
       </c>
-      <c r="C36" s="281" t="s">
+      <c r="C36" s="185" t="s">
         <v>121</v>
       </c>
     </row>
@@ -7183,10 +7188,10 @@
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="273">
+      <c r="B38" s="181">
         <v>5</v>
       </c>
-      <c r="C38" s="281" t="s">
+      <c r="C38" s="185" t="s">
         <v>46</v>
       </c>
     </row>
@@ -7194,15 +7199,15 @@
       <c r="B39" s="92">
         <v>6</v>
       </c>
-      <c r="C39" s="293" t="s">
+      <c r="C39" s="193" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="282">
+      <c r="B40" s="186">
         <v>7</v>
       </c>
-      <c r="C40" s="283" t="s">
+      <c r="C40" s="187" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Document stack pointer register
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEB2F67-9CC5-4F47-BB95-820EBA17111D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA779162-0020-4F05-96FC-DF67701F275C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="8" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="207">
   <si>
     <t>MODE B</t>
   </si>
@@ -651,6 +651,21 @@
   </si>
   <si>
     <t>reason</t>
+  </si>
+  <si>
+    <t>STPTR_0</t>
+  </si>
+  <si>
+    <t>STPTR_1</t>
+  </si>
+  <si>
+    <t>STPTR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bits 8..15 of the Stack Pointer </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bits 0..7 of the Stack Pointer </t>
   </si>
 </sst>
 </file>
@@ -1610,7 +1625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="295">
+  <cellXfs count="294">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1692,7 +1707,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="31" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="27" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1942,9 +1956,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="29" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2139,6 +2150,9 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="68" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2789,79 +2803,79 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="195" t="s">
+      <c r="B2" s="194" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="196"/>
-      <c r="D2" s="196"/>
-      <c r="E2" s="196"/>
-      <c r="F2" s="197"/>
-      <c r="G2" s="200" t="s">
+      <c r="C2" s="195"/>
+      <c r="D2" s="195"/>
+      <c r="E2" s="195"/>
+      <c r="F2" s="196"/>
+      <c r="G2" s="199" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="201"/>
-      <c r="I2" s="202"/>
-      <c r="J2" s="198" t="s">
+      <c r="H2" s="200"/>
+      <c r="I2" s="201"/>
+      <c r="J2" s="197" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="57" t="s">
+      <c r="B3" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="51" t="s">
         <v>37</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="F3" s="51" t="s">
+      <c r="F3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="G3" s="118" t="s">
+      <c r="G3" s="117" t="s">
         <v>52</v>
       </c>
-      <c r="H3" s="53" t="s">
+      <c r="H3" s="52" t="s">
         <v>53</v>
       </c>
-      <c r="I3" s="51" t="s">
+      <c r="I3" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="J3" s="199"/>
+      <c r="J3" s="198"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="107">
-        <v>0</v>
-      </c>
-      <c r="C4" s="58">
+      <c r="B4" s="106">
+        <v>0</v>
+      </c>
+      <c r="C4" s="57">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,3),1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="36">
+      <c r="D4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,2),1)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="36">
+      <c r="E4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,1),1)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="59">
+      <c r="F4" s="58">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,0),1)</f>
         <v>0</v>
       </c>
-      <c r="G4" s="119" t="s">
+      <c r="G4" s="118" t="s">
         <v>126</v>
       </c>
-      <c r="H4" s="126" t="s">
+      <c r="H4" s="124" t="s">
         <v>126</v>
       </c>
-      <c r="I4" s="110" t="s">
+      <c r="I4" s="109" t="s">
         <v>126</v>
       </c>
-      <c r="J4" s="108" t="s">
+      <c r="J4" s="107" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2869,7 +2883,7 @@
       <c r="B5" s="13">
         <v>1</v>
       </c>
-      <c r="C5" s="60">
+      <c r="C5" s="59">
         <f t="shared" ref="C5:C19" si="0">_xlfn.BITAND(_xlfn.BITRSHIFT($B5,3),1)</f>
         <v>0</v>
       </c>
@@ -2885,13 +2899,13 @@
         <f t="shared" ref="F5:F19" si="3">_xlfn.BITAND(_xlfn.BITRSHIFT($B5,0),1)</f>
         <v>1</v>
       </c>
-      <c r="G5" s="120" t="s">
+      <c r="G5" s="119" t="s">
         <v>127</v>
       </c>
-      <c r="H5" s="127" t="s">
+      <c r="H5" s="125" t="s">
         <v>127</v>
       </c>
-      <c r="I5" s="111" t="s">
+      <c r="I5" s="110" t="s">
         <v>127</v>
       </c>
       <c r="J5" s="26" t="s">
@@ -2902,7 +2916,7 @@
       <c r="B6" s="19">
         <v>2</v>
       </c>
-      <c r="C6" s="77">
+      <c r="C6" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2918,13 +2932,13 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G6" s="121" t="s">
+      <c r="G6" s="120" t="s">
         <v>128</v>
       </c>
-      <c r="H6" s="128" t="s">
+      <c r="H6" s="126" t="s">
         <v>128</v>
       </c>
-      <c r="I6" s="112" t="s">
+      <c r="I6" s="111" t="s">
         <v>128</v>
       </c>
       <c r="J6" s="28" t="s">
@@ -2935,7 +2949,7 @@
       <c r="B7" s="22">
         <v>3</v>
       </c>
-      <c r="C7" s="78">
+      <c r="C7" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2951,13 +2965,13 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G7" s="122" t="s">
+      <c r="G7" s="121" t="s">
         <v>129</v>
       </c>
-      <c r="H7" s="129" t="s">
+      <c r="H7" s="127" t="s">
         <v>129</v>
       </c>
-      <c r="I7" s="113" t="s">
+      <c r="I7" s="112" t="s">
         <v>129</v>
       </c>
       <c r="J7" s="30" t="s">
@@ -2968,7 +2982,7 @@
       <c r="B8" s="13">
         <v>4</v>
       </c>
-      <c r="C8" s="60">
+      <c r="C8" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2984,13 +2998,13 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G8" s="120" t="s">
+      <c r="G8" s="119" t="s">
         <v>130</v>
       </c>
-      <c r="H8" s="127" t="s">
+      <c r="H8" s="125" t="s">
         <v>130</v>
       </c>
-      <c r="I8" s="111" t="s">
+      <c r="I8" s="110" t="s">
         <v>130</v>
       </c>
       <c r="J8" s="26" t="s">
@@ -3001,7 +3015,7 @@
       <c r="B9" s="13">
         <v>5</v>
       </c>
-      <c r="C9" s="60">
+      <c r="C9" s="59">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3017,13 +3031,13 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G9" s="120" t="s">
+      <c r="G9" s="119" t="s">
         <v>131</v>
       </c>
-      <c r="H9" s="127" t="s">
+      <c r="H9" s="125" t="s">
         <v>131</v>
       </c>
-      <c r="I9" s="111" t="s">
+      <c r="I9" s="110" t="s">
         <v>131</v>
       </c>
       <c r="J9" s="26" t="s">
@@ -3034,7 +3048,7 @@
       <c r="B10" s="19">
         <v>6</v>
       </c>
-      <c r="C10" s="77">
+      <c r="C10" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3050,13 +3064,13 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G10" s="121" t="s">
+      <c r="G10" s="120" t="s">
         <v>132</v>
       </c>
-      <c r="H10" s="128" t="s">
+      <c r="H10" s="126" t="s">
         <v>132</v>
       </c>
-      <c r="I10" s="112" t="s">
+      <c r="I10" s="111" t="s">
         <v>132</v>
       </c>
       <c r="J10" s="28" t="s">
@@ -3067,7 +3081,7 @@
       <c r="B11" s="22">
         <v>7</v>
       </c>
-      <c r="C11" s="78">
+      <c r="C11" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -3083,13 +3097,13 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G11" s="122" t="s">
+      <c r="G11" s="121" t="s">
         <v>133</v>
       </c>
-      <c r="H11" s="129" t="s">
+      <c r="H11" s="127" t="s">
         <v>133</v>
       </c>
-      <c r="I11" s="113" t="s">
+      <c r="I11" s="112" t="s">
         <v>133</v>
       </c>
       <c r="J11" s="30" t="s">
@@ -3100,7 +3114,7 @@
       <c r="B12" s="13">
         <v>8</v>
       </c>
-      <c r="C12" s="60">
+      <c r="C12" s="59">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B12,3),1)</f>
         <v>1</v>
       </c>
@@ -3116,13 +3130,13 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G12" s="121" t="s">
+      <c r="G12" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="H12" s="151" t="s">
+      <c r="H12" s="149" t="s">
         <v>147</v>
       </c>
-      <c r="I12" s="116"/>
+      <c r="I12" s="115"/>
       <c r="J12" s="28" t="s">
         <v>39</v>
       </c>
@@ -3131,7 +3145,7 @@
       <c r="B13" s="13">
         <v>9</v>
       </c>
-      <c r="C13" s="60">
+      <c r="C13" s="59">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3147,11 +3161,11 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G13" s="120" t="s">
+      <c r="G13" s="119" t="s">
         <v>135</v>
       </c>
-      <c r="H13" s="152"/>
-      <c r="I13" s="115"/>
+      <c r="H13" s="150"/>
+      <c r="I13" s="114"/>
       <c r="J13" s="26" t="s">
         <v>40</v>
       </c>
@@ -3160,7 +3174,7 @@
       <c r="B14" s="19">
         <v>10</v>
       </c>
-      <c r="C14" s="77">
+      <c r="C14" s="76">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3176,16 +3190,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G14" s="124"/>
-      <c r="H14" s="130"/>
-      <c r="I14" s="116"/>
-      <c r="J14" s="32"/>
+      <c r="G14" s="122"/>
+      <c r="H14" s="128"/>
+      <c r="I14" s="115"/>
+      <c r="J14" s="31"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="22">
         <v>11</v>
       </c>
-      <c r="C15" s="78">
+      <c r="C15" s="77">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3201,13 +3215,13 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G15" s="122" t="s">
+      <c r="G15" s="121" t="s">
         <v>136</v>
       </c>
-      <c r="H15" s="142" t="s">
+      <c r="H15" s="140" t="s">
         <v>136</v>
       </c>
-      <c r="I15" s="114"/>
+      <c r="I15" s="113"/>
       <c r="J15" s="30" t="s">
         <v>137</v>
       </c>
@@ -3216,7 +3230,7 @@
       <c r="B16" s="13">
         <v>12</v>
       </c>
-      <c r="C16" s="60">
+      <c r="C16" s="59">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3232,16 +3246,22 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G16" s="123"/>
-      <c r="H16" s="131"/>
-      <c r="I16" s="115"/>
-      <c r="J16" s="31"/>
+      <c r="G16" s="119" t="s">
+        <v>202</v>
+      </c>
+      <c r="H16" s="193" t="s">
+        <v>204</v>
+      </c>
+      <c r="I16" s="114"/>
+      <c r="J16" s="26" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="13">
         <v>13</v>
       </c>
-      <c r="C17" s="60">
+      <c r="C17" s="59">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3257,16 +3277,20 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G17" s="123"/>
-      <c r="H17" s="131"/>
-      <c r="I17" s="115"/>
-      <c r="J17" s="31"/>
+      <c r="G17" s="119" t="s">
+        <v>203</v>
+      </c>
+      <c r="H17" s="129"/>
+      <c r="I17" s="114"/>
+      <c r="J17" s="26" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="19">
         <v>14</v>
       </c>
-      <c r="C18" s="77">
+      <c r="C18" s="76">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3282,16 +3306,16 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G18" s="124"/>
-      <c r="H18" s="130"/>
-      <c r="I18" s="116"/>
-      <c r="J18" s="32"/>
+      <c r="G18" s="122"/>
+      <c r="H18" s="128"/>
+      <c r="I18" s="115"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="19" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="16">
         <v>15</v>
       </c>
-      <c r="C19" s="61">
+      <c r="C19" s="60">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -3307,10 +3331,10 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="G19" s="125"/>
-      <c r="H19" s="132"/>
-      <c r="I19" s="117"/>
-      <c r="J19" s="109"/>
+      <c r="G19" s="123"/>
+      <c r="H19" s="130"/>
+      <c r="I19" s="116"/>
+      <c r="J19" s="108"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3431,73 +3455,73 @@
       </c>
     </row>
     <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="225" t="s">
+      <c r="C3" s="224" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="226"/>
-      <c r="E3" s="226"/>
-      <c r="F3" s="226"/>
-      <c r="G3" s="227"/>
-      <c r="H3" s="222" t="s">
+      <c r="D3" s="225"/>
+      <c r="E3" s="225"/>
+      <c r="F3" s="225"/>
+      <c r="G3" s="226"/>
+      <c r="H3" s="221" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="223"/>
-      <c r="J3" s="224"/>
-      <c r="K3" s="222" t="s">
+      <c r="I3" s="222"/>
+      <c r="J3" s="223"/>
+      <c r="K3" s="221" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="223"/>
-      <c r="M3" s="223"/>
-      <c r="N3" s="209" t="s">
+      <c r="L3" s="222"/>
+      <c r="M3" s="222"/>
+      <c r="N3" s="208" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="210"/>
-      <c r="P3" s="211"/>
+      <c r="O3" s="209"/>
+      <c r="P3" s="210"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="203" t="s">
+      <c r="S3" s="202" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="204"/>
-      <c r="U3" s="204"/>
-      <c r="V3" s="204"/>
-      <c r="W3" s="204"/>
-      <c r="X3" s="204"/>
-      <c r="Y3" s="204"/>
-      <c r="Z3" s="205"/>
-      <c r="AA3" s="206" t="s">
+      <c r="T3" s="203"/>
+      <c r="U3" s="203"/>
+      <c r="V3" s="203"/>
+      <c r="W3" s="203"/>
+      <c r="X3" s="203"/>
+      <c r="Y3" s="203"/>
+      <c r="Z3" s="204"/>
+      <c r="AA3" s="205" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="207"/>
-      <c r="AC3" s="207"/>
-      <c r="AD3" s="207"/>
-      <c r="AE3" s="207"/>
-      <c r="AF3" s="207"/>
-      <c r="AG3" s="207"/>
-      <c r="AH3" s="208"/>
+      <c r="AB3" s="206"/>
+      <c r="AC3" s="206"/>
+      <c r="AD3" s="206"/>
+      <c r="AE3" s="206"/>
+      <c r="AF3" s="206"/>
+      <c r="AG3" s="206"/>
+      <c r="AH3" s="207"/>
     </row>
     <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="B5" s="214" t="s">
+      <c r="B5" s="213" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="212" t="s">
+      <c r="C5" s="211" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="212"/>
-      <c r="E5" s="212"/>
-      <c r="F5" s="212"/>
-      <c r="G5" s="212"/>
-      <c r="H5" s="212"/>
-      <c r="I5" s="212"/>
-      <c r="J5" s="213"/>
+      <c r="D5" s="211"/>
+      <c r="E5" s="211"/>
+      <c r="F5" s="211"/>
+      <c r="G5" s="211"/>
+      <c r="H5" s="211"/>
+      <c r="I5" s="211"/>
+      <c r="J5" s="212"/>
     </row>
     <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="215"/>
+      <c r="B6" s="214"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3527,16 +3551,16 @@
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="216" t="s">
+      <c r="C7" s="215" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="217"/>
-      <c r="E7" s="217"/>
-      <c r="F7" s="217"/>
-      <c r="G7" s="217"/>
-      <c r="H7" s="217"/>
-      <c r="I7" s="217"/>
-      <c r="J7" s="218"/>
+      <c r="D7" s="216"/>
+      <c r="E7" s="216"/>
+      <c r="F7" s="216"/>
+      <c r="G7" s="216"/>
+      <c r="H7" s="216"/>
+      <c r="I7" s="216"/>
+      <c r="J7" s="217"/>
     </row>
     <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
@@ -3546,12 +3570,12 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="219" t="s">
+      <c r="G8" s="218" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="220"/>
-      <c r="I8" s="220"/>
-      <c r="J8" s="221"/>
+      <c r="H8" s="219"/>
+      <c r="I8" s="219"/>
+      <c r="J8" s="220"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -3587,113 +3611,113 @@
   <sheetData>
     <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="249" t="s">
+      <c r="B2" s="248" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="198" t="s">
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="197" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="198" t="s">
+      <c r="I2" s="197" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="249" t="s">
+      <c r="J2" s="248" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="250"/>
-      <c r="L2" s="250"/>
-      <c r="M2" s="198" t="s">
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="197" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="198" t="s">
+      <c r="N2" s="197" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="51" t="s">
+      <c r="G3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="199"/>
-      <c r="I3" s="199"/>
-      <c r="J3" s="49" t="s">
+      <c r="H3" s="198"/>
+      <c r="I3" s="198"/>
+      <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="53" t="s">
+      <c r="K3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="52" t="s">
+      <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="199"/>
-      <c r="N3" s="199"/>
+      <c r="M3" s="198"/>
+      <c r="N3" s="198"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B4" s="81">
-        <v>0</v>
-      </c>
-      <c r="C4" s="36">
+      <c r="B4" s="80">
+        <v>0</v>
+      </c>
+      <c r="C4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,4),1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="36">
+      <c r="D4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,3),1)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="36">
+      <c r="E4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="36">
+      <c r="F4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G4" s="79">
+      <c r="G4" s="78">
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="230" t="s">
+      <c r="H4" s="229" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="68" t="s">
+      <c r="I4" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="67" t="s">
+      <c r="K4" s="66" t="s">
         <v>115</v>
       </c>
-      <c r="L4" s="70" t="s">
+      <c r="L4" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="M4" s="70" t="s">
+      <c r="M4" s="69" t="s">
         <v>113</v>
       </c>
-      <c r="N4" s="76" t="s">
+      <c r="N4" s="75" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="83">
+      <c r="B5" s="82">
         <v>1</v>
       </c>
       <c r="C5" s="17">
@@ -3712,32 +3736,32 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B5,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="80">
+      <c r="G5" s="79">
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="229"/>
-      <c r="I5" s="43" t="s">
+      <c r="H5" s="228"/>
+      <c r="I5" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="J5" s="63" t="s">
+      <c r="J5" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="55" t="s">
+      <c r="K5" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="64" t="s">
+      <c r="L5" s="63" t="s">
         <v>66</v>
       </c>
-      <c r="M5" s="35" t="s">
+      <c r="M5" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="N5" s="45" t="s">
+      <c r="N5" s="44" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="82">
+      <c r="B6" s="81">
         <v>2</v>
       </c>
       <c r="C6" s="14">
@@ -3748,7 +3772,7 @@
         <f t="shared" ref="D6:D35" si="2">_xlfn.BITAND(_xlfn.BITRSHIFT($B6,3),1)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="60">
+      <c r="E6" s="59">
         <f t="shared" ref="E6:E35" si="3">_xlfn.BITAND(_xlfn.BITRSHIFT($B6,2),1)</f>
         <v>0</v>
       </c>
@@ -3760,30 +3784,30 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="228" t="s">
+      <c r="H6" s="227" t="s">
         <v>61</v>
       </c>
-      <c r="I6" s="65" t="s">
+      <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="232" t="s">
+      <c r="J6" s="231" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="241" t="s">
+      <c r="K6" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="238" t="s">
+      <c r="L6" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="243" t="s">
+      <c r="M6" s="242" t="s">
         <v>113</v>
       </c>
-      <c r="N6" s="246" t="s">
+      <c r="N6" s="245" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B7" s="82">
+      <c r="B7" s="81">
         <v>3</v>
       </c>
       <c r="C7" s="14">
@@ -3794,7 +3818,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E7" s="60">
+      <c r="E7" s="59">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -3806,18 +3830,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="228"/>
-      <c r="I7" s="71" t="s">
+      <c r="H7" s="227"/>
+      <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="232"/>
-      <c r="K7" s="241"/>
-      <c r="L7" s="238"/>
-      <c r="M7" s="244"/>
-      <c r="N7" s="246"/>
+      <c r="J7" s="231"/>
+      <c r="K7" s="240"/>
+      <c r="L7" s="237"/>
+      <c r="M7" s="243"/>
+      <c r="N7" s="245"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B8" s="82">
+      <c r="B8" s="81">
         <v>4</v>
       </c>
       <c r="C8" s="14">
@@ -3828,7 +3852,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E8" s="60">
+      <c r="E8" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -3840,18 +3864,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="228"/>
-      <c r="I8" s="91" t="s">
+      <c r="H8" s="227"/>
+      <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="232"/>
-      <c r="K8" s="241"/>
-      <c r="L8" s="238"/>
-      <c r="M8" s="244"/>
-      <c r="N8" s="246"/>
+      <c r="J8" s="231"/>
+      <c r="K8" s="240"/>
+      <c r="L8" s="237"/>
+      <c r="M8" s="243"/>
+      <c r="N8" s="245"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B9" s="82">
+      <c r="B9" s="81">
         <v>5</v>
       </c>
       <c r="C9" s="14">
@@ -3862,7 +3886,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E9" s="60">
+      <c r="E9" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -3874,18 +3898,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="228"/>
-      <c r="I9" s="91" t="s">
+      <c r="H9" s="227"/>
+      <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="232"/>
-      <c r="K9" s="241"/>
-      <c r="L9" s="238"/>
-      <c r="M9" s="244"/>
-      <c r="N9" s="246"/>
+      <c r="J9" s="231"/>
+      <c r="K9" s="240"/>
+      <c r="L9" s="237"/>
+      <c r="M9" s="243"/>
+      <c r="N9" s="245"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B10" s="82">
+      <c r="B10" s="81">
         <v>6</v>
       </c>
       <c r="C10" s="14">
@@ -3896,7 +3920,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E10" s="60">
+      <c r="E10" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -3908,18 +3932,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="228"/>
-      <c r="I10" s="91" t="s">
+      <c r="H10" s="227"/>
+      <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="232"/>
-      <c r="K10" s="241"/>
-      <c r="L10" s="238"/>
-      <c r="M10" s="244"/>
-      <c r="N10" s="246"/>
+      <c r="J10" s="231"/>
+      <c r="K10" s="240"/>
+      <c r="L10" s="237"/>
+      <c r="M10" s="243"/>
+      <c r="N10" s="245"/>
     </row>
     <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="83">
+      <c r="B11" s="82">
         <v>7</v>
       </c>
       <c r="C11" s="17">
@@ -3930,7 +3954,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E11" s="61">
+      <c r="E11" s="60">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -3942,64 +3966,64 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="229"/>
-      <c r="I11" s="44" t="s">
+      <c r="H11" s="228"/>
+      <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="233"/>
-      <c r="K11" s="242"/>
-      <c r="L11" s="239"/>
-      <c r="M11" s="245"/>
-      <c r="N11" s="247"/>
+      <c r="J11" s="232"/>
+      <c r="K11" s="241"/>
+      <c r="L11" s="238"/>
+      <c r="M11" s="244"/>
+      <c r="N11" s="246"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B12" s="81">
+      <c r="B12" s="80">
         <v>8</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="35">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F12" s="58">
+      <c r="F12" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G12" s="59">
+      <c r="G12" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="230" t="s">
+      <c r="H12" s="229" t="s">
         <v>55</v>
       </c>
-      <c r="I12" s="65" t="s">
+      <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="231" t="s">
+      <c r="J12" s="230" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="240" t="s">
+      <c r="K12" s="239" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="237" t="s">
+      <c r="L12" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="230" t="s">
+      <c r="M12" s="229" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="248" t="s">
+      <c r="N12" s="247" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B13" s="82">
+      <c r="B13" s="81">
         <v>9</v>
       </c>
       <c r="C13" s="14">
@@ -4014,7 +4038,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F13" s="60">
+      <c r="F13" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -4022,18 +4046,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="228"/>
-      <c r="I13" s="91" t="s">
+      <c r="H13" s="227"/>
+      <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="232"/>
-      <c r="K13" s="241"/>
-      <c r="L13" s="238"/>
-      <c r="M13" s="228"/>
-      <c r="N13" s="246"/>
+      <c r="J13" s="231"/>
+      <c r="K13" s="240"/>
+      <c r="L13" s="237"/>
+      <c r="M13" s="227"/>
+      <c r="N13" s="245"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B14" s="82">
+      <c r="B14" s="81">
         <v>10</v>
       </c>
       <c r="C14" s="14">
@@ -4048,7 +4072,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F14" s="60">
+      <c r="F14" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4056,18 +4080,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="228"/>
-      <c r="I14" s="91" t="s">
+      <c r="H14" s="227"/>
+      <c r="I14" s="90" t="s">
         <v>102</v>
       </c>
-      <c r="J14" s="232"/>
-      <c r="K14" s="241"/>
-      <c r="L14" s="238"/>
-      <c r="M14" s="228"/>
-      <c r="N14" s="246"/>
+      <c r="J14" s="231"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="237"/>
+      <c r="M14" s="227"/>
+      <c r="N14" s="245"/>
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="83">
+      <c r="B15" s="82">
         <v>11</v>
       </c>
       <c r="C15" s="17">
@@ -4082,7 +4106,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F15" s="61">
+      <c r="F15" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4090,64 +4114,64 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="229"/>
-      <c r="I15" s="44" t="s">
+      <c r="H15" s="228"/>
+      <c r="I15" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="233"/>
-      <c r="K15" s="242"/>
-      <c r="L15" s="239"/>
-      <c r="M15" s="229"/>
-      <c r="N15" s="247"/>
+      <c r="J15" s="232"/>
+      <c r="K15" s="241"/>
+      <c r="L15" s="238"/>
+      <c r="M15" s="228"/>
+      <c r="N15" s="246"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B16" s="81">
+      <c r="B16" s="80">
         <v>12</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="35">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D16" s="36">
+      <c r="D16" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F16" s="58">
+      <c r="F16" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G16" s="59">
+      <c r="G16" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="230" t="s">
+      <c r="H16" s="229" t="s">
         <v>56</v>
       </c>
-      <c r="I16" s="65" t="s">
+      <c r="I16" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="231" t="s">
+      <c r="J16" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="234" t="s">
+      <c r="K16" s="233" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="237" t="s">
+      <c r="L16" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M16" s="230" t="s">
+      <c r="M16" s="229" t="s">
         <v>114</v>
       </c>
-      <c r="N16" s="76" t="s">
+      <c r="N16" s="75" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B17" s="82">
+      <c r="B17" s="81">
         <v>13</v>
       </c>
       <c r="C17" s="14">
@@ -4162,7 +4186,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F17" s="60">
+      <c r="F17" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -4170,20 +4194,20 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="228"/>
-      <c r="I17" s="71" t="s">
+      <c r="H17" s="227"/>
+      <c r="I17" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="232"/>
-      <c r="K17" s="235"/>
-      <c r="L17" s="238"/>
-      <c r="M17" s="228"/>
-      <c r="N17" s="75" t="s">
+      <c r="J17" s="231"/>
+      <c r="K17" s="234"/>
+      <c r="L17" s="237"/>
+      <c r="M17" s="227"/>
+      <c r="N17" s="74" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B18" s="82">
+      <c r="B18" s="81">
         <v>14</v>
       </c>
       <c r="C18" s="14">
@@ -4198,7 +4222,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F18" s="60">
+      <c r="F18" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4206,20 +4230,20 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="228"/>
-      <c r="I18" s="71" t="s">
+      <c r="H18" s="227"/>
+      <c r="I18" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="232"/>
-      <c r="K18" s="235"/>
-      <c r="L18" s="238"/>
-      <c r="M18" s="228"/>
-      <c r="N18" s="75" t="s">
+      <c r="J18" s="231"/>
+      <c r="K18" s="234"/>
+      <c r="L18" s="237"/>
+      <c r="M18" s="227"/>
+      <c r="N18" s="74" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="19" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="83">
+      <c r="B19" s="82">
         <v>15</v>
       </c>
       <c r="C19" s="17">
@@ -4234,7 +4258,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F19" s="61">
+      <c r="F19" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4242,67 +4266,67 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="229"/>
-      <c r="I19" s="44" t="s">
+      <c r="H19" s="228"/>
+      <c r="I19" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="233"/>
-      <c r="K19" s="236"/>
-      <c r="L19" s="239"/>
-      <c r="M19" s="229"/>
-      <c r="N19" s="45" t="s">
+      <c r="J19" s="232"/>
+      <c r="K19" s="235"/>
+      <c r="L19" s="238"/>
+      <c r="M19" s="228"/>
+      <c r="N19" s="44" t="s">
         <v>108</v>
       </c>
       <c r="P19" s="1"/>
     </row>
     <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" s="81">
+      <c r="B20" s="80">
         <v>16</v>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D20" s="36">
+      <c r="D20" s="35">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G20" s="59">
+      <c r="G20" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="230" t="s">
+      <c r="H20" s="229" t="s">
         <v>57</v>
       </c>
-      <c r="I20" s="65" t="s">
+      <c r="I20" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="231" t="s">
+      <c r="J20" s="230" t="s">
         <v>16</v>
       </c>
-      <c r="K20" s="240" t="s">
+      <c r="K20" s="239" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="237" t="s">
+      <c r="L20" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="243" t="s">
+      <c r="M20" s="242" t="s">
         <v>113</v>
       </c>
-      <c r="N20" s="42" t="s">
+      <c r="N20" s="41" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" s="82">
+      <c r="B21" s="81">
         <v>17</v>
       </c>
       <c r="C21" s="14">
@@ -4317,7 +4341,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F21" s="60">
+      <c r="F21" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -4325,20 +4349,20 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="228"/>
-      <c r="I21" s="71" t="s">
+      <c r="H21" s="227"/>
+      <c r="I21" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="232"/>
-      <c r="K21" s="241"/>
-      <c r="L21" s="238"/>
-      <c r="M21" s="244"/>
-      <c r="N21" s="75" t="s">
+      <c r="J21" s="231"/>
+      <c r="K21" s="240"/>
+      <c r="L21" s="237"/>
+      <c r="M21" s="243"/>
+      <c r="N21" s="74" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" s="82">
+      <c r="B22" s="81">
         <v>18</v>
       </c>
       <c r="C22" s="14">
@@ -4353,7 +4377,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F22" s="60">
+      <c r="F22" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4361,20 +4385,20 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="228"/>
-      <c r="I22" s="71" t="s">
+      <c r="H22" s="227"/>
+      <c r="I22" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="232"/>
-      <c r="K22" s="241"/>
-      <c r="L22" s="238"/>
-      <c r="M22" s="244"/>
-      <c r="N22" s="75" t="s">
+      <c r="J22" s="231"/>
+      <c r="K22" s="240"/>
+      <c r="L22" s="237"/>
+      <c r="M22" s="243"/>
+      <c r="N22" s="74" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="82">
+      <c r="B23" s="81">
         <v>19</v>
       </c>
       <c r="C23" s="14">
@@ -4389,7 +4413,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F23" s="61">
+      <c r="F23" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4397,66 +4421,66 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="229"/>
-      <c r="I23" s="43" t="s">
+      <c r="H23" s="228"/>
+      <c r="I23" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="J23" s="233"/>
-      <c r="K23" s="242"/>
-      <c r="L23" s="239"/>
-      <c r="M23" s="245"/>
-      <c r="N23" s="42" t="s">
+      <c r="J23" s="232"/>
+      <c r="K23" s="241"/>
+      <c r="L23" s="238"/>
+      <c r="M23" s="244"/>
+      <c r="N23" s="41" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="81">
+      <c r="B24" s="80">
         <v>20</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C24" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D24" s="36">
+      <c r="D24" s="35">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F24" s="58">
+      <c r="F24" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G24" s="59">
+      <c r="G24" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="230" t="s">
+      <c r="H24" s="229" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="65" t="s">
+      <c r="I24" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="J24" s="67" t="s">
+      <c r="J24" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="K24" s="66" t="s">
+      <c r="K24" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="L24" s="68" t="s">
+      <c r="L24" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="M24" s="103" t="s">
+      <c r="M24" s="102" t="s">
         <v>113</v>
       </c>
-      <c r="N24" s="76" t="s">
+      <c r="N24" s="75" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B25" s="82">
+      <c r="B25" s="81">
         <v>21</v>
       </c>
       <c r="C25" s="14">
@@ -4471,7 +4495,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F25" s="60">
+      <c r="F25" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -4479,28 +4503,28 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="228"/>
-      <c r="I25" s="71" t="s">
+      <c r="H25" s="227"/>
+      <c r="I25" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="J25" s="101" t="s">
+      <c r="J25" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="K25" s="104" t="s">
+      <c r="K25" s="103" t="s">
         <v>16</v>
       </c>
-      <c r="L25" s="102" t="s">
+      <c r="L25" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M25" s="100" t="s">
+      <c r="M25" s="99" t="s">
         <v>113</v>
       </c>
-      <c r="N25" s="75" t="s">
+      <c r="N25" s="74" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B26" s="82">
+      <c r="B26" s="81">
         <v>22</v>
       </c>
       <c r="C26" s="14">
@@ -4515,7 +4539,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F26" s="60">
+      <c r="F26" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4523,16 +4547,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="228"/>
-      <c r="I26" s="105"/>
-      <c r="J26" s="139"/>
-      <c r="K26" s="140"/>
-      <c r="L26" s="141"/>
-      <c r="M26" s="106"/>
-      <c r="N26" s="106"/>
+      <c r="H26" s="227"/>
+      <c r="I26" s="104"/>
+      <c r="J26" s="137"/>
+      <c r="K26" s="138"/>
+      <c r="L26" s="139"/>
+      <c r="M26" s="105"/>
+      <c r="N26" s="105"/>
     </row>
     <row r="27" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="83">
+      <c r="B27" s="82">
         <v>23</v>
       </c>
       <c r="C27" s="14">
@@ -4547,7 +4571,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F27" s="61">
+      <c r="F27" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4555,62 +4579,62 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="229"/>
-      <c r="I27" s="98"/>
-      <c r="J27" s="136"/>
-      <c r="K27" s="137"/>
-      <c r="L27" s="138"/>
-      <c r="M27" s="135"/>
-      <c r="N27" s="135"/>
+      <c r="H27" s="228"/>
+      <c r="I27" s="97"/>
+      <c r="J27" s="134"/>
+      <c r="K27" s="135"/>
+      <c r="L27" s="136"/>
+      <c r="M27" s="133"/>
+      <c r="N27" s="133"/>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B28" s="81">
+      <c r="B28" s="80">
         <v>24</v>
       </c>
-      <c r="C28" s="36">
+      <c r="C28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,4),1)</f>
         <v>1</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,3),1)</f>
         <v>1</v>
       </c>
-      <c r="E28" s="36">
+      <c r="E28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="58">
+      <c r="F28" s="57">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="59">
+      <c r="G28" s="58">
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="230" t="s">
+      <c r="H28" s="229" t="s">
         <v>60</v>
       </c>
-      <c r="I28" s="38" t="s">
+      <c r="I28" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="J28" s="34" t="s">
+      <c r="J28" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="K28" s="54" t="s">
+      <c r="K28" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="L28" s="40" t="s">
+      <c r="L28" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="M28" s="99" t="s">
+      <c r="M28" s="98" t="s">
         <v>113</v>
       </c>
-      <c r="N28" s="39" t="s">
+      <c r="N28" s="38" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B29" s="82">
+      <c r="B29" s="81">
         <v>25</v>
       </c>
       <c r="C29" s="14">
@@ -4625,7 +4649,7 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B29,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="60">
+      <c r="F29" s="59">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B29,1),1)</f>
         <v>0</v>
       </c>
@@ -4633,28 +4657,28 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="228"/>
-      <c r="I29" s="71" t="s">
+      <c r="H29" s="227"/>
+      <c r="I29" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="J29" s="72" t="s">
+      <c r="J29" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="K29" s="73" t="s">
+      <c r="K29" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L29" s="74" t="s">
+      <c r="L29" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="M29" s="100" t="s">
+      <c r="M29" s="99" t="s">
         <v>113</v>
       </c>
-      <c r="N29" s="75" t="s">
+      <c r="N29" s="74" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B30" s="82">
+      <c r="B30" s="81">
         <v>26</v>
       </c>
       <c r="C30" s="14">
@@ -4669,7 +4693,7 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B30,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="60">
+      <c r="F30" s="59">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B30,1),1)</f>
         <v>1</v>
       </c>
@@ -4677,28 +4701,28 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="228"/>
-      <c r="I30" s="71" t="s">
+      <c r="H30" s="227"/>
+      <c r="I30" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="J30" s="101" t="s">
+      <c r="J30" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="K30" s="73" t="s">
+      <c r="K30" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L30" s="102" t="s">
+      <c r="L30" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M30" s="100" t="s">
+      <c r="M30" s="99" t="s">
         <v>113</v>
       </c>
-      <c r="N30" s="75" t="s">
+      <c r="N30" s="74" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="83">
+      <c r="B31" s="82">
         <v>27</v>
       </c>
       <c r="C31" s="17">
@@ -4713,7 +4737,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F31" s="61">
+      <c r="F31" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4721,63 +4745,63 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="229"/>
-      <c r="I31" s="92"/>
-      <c r="J31" s="95"/>
-      <c r="K31" s="96"/>
-      <c r="L31" s="97"/>
-      <c r="M31" s="97"/>
-      <c r="N31" s="94"/>
+      <c r="H31" s="228"/>
+      <c r="I31" s="91"/>
+      <c r="J31" s="94"/>
+      <c r="K31" s="95"/>
+      <c r="L31" s="96"/>
+      <c r="M31" s="96"/>
+      <c r="N31" s="93"/>
     </row>
     <row r="32" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B32" s="82">
+      <c r="B32" s="81">
         <v>28</v>
       </c>
-      <c r="C32" s="36">
+      <c r="C32" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D32" s="36">
+      <c r="D32" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E32" s="36">
+      <c r="E32" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F32" s="58">
+      <c r="F32" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G32" s="59">
+      <c r="G32" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="228" t="s">
+      <c r="H32" s="227" t="s">
         <v>59</v>
       </c>
-      <c r="I32" s="65" t="s">
+      <c r="I32" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="J32" s="67" t="s">
+      <c r="J32" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="K32" s="69" t="s">
+      <c r="K32" s="68" t="s">
         <v>68</v>
       </c>
-      <c r="L32" s="70" t="s">
+      <c r="L32" s="69" t="s">
         <v>44</v>
       </c>
-      <c r="M32" s="70" t="s">
+      <c r="M32" s="69" t="s">
         <v>113</v>
       </c>
-      <c r="N32" s="76" t="s">
+      <c r="N32" s="75" t="s">
         <v>109</v>
       </c>
       <c r="Q32" s="1"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B33" s="82">
+      <c r="B33" s="81">
         <v>29</v>
       </c>
       <c r="C33" s="14">
@@ -4792,7 +4816,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F33" s="60">
+      <c r="F33" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -4800,29 +4824,29 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="228"/>
-      <c r="I33" s="71" t="s">
+      <c r="H33" s="227"/>
+      <c r="I33" s="70" t="s">
         <v>24</v>
       </c>
-      <c r="J33" s="72" t="s">
+      <c r="J33" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="73" t="s">
+      <c r="K33" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L33" s="102" t="s">
+      <c r="L33" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M33" s="102" t="s">
+      <c r="M33" s="101" t="s">
         <v>113</v>
       </c>
-      <c r="N33" s="75" t="s">
+      <c r="N33" s="74" t="s">
         <v>110</v>
       </c>
       <c r="Q33" s="1"/>
     </row>
     <row r="34" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="82">
+      <c r="B34" s="81">
         <v>30</v>
       </c>
       <c r="C34" s="14">
@@ -4837,7 +4861,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F34" s="60">
+      <c r="F34" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -4845,58 +4869,58 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="229"/>
-      <c r="I34" s="98"/>
-      <c r="J34" s="95"/>
-      <c r="K34" s="96"/>
-      <c r="L34" s="97"/>
-      <c r="M34" s="97"/>
-      <c r="N34" s="94"/>
+      <c r="H34" s="228"/>
+      <c r="I34" s="97"/>
+      <c r="J34" s="94"/>
+      <c r="K34" s="95"/>
+      <c r="L34" s="96"/>
+      <c r="M34" s="96"/>
+      <c r="N34" s="93"/>
       <c r="Q34" s="1"/>
     </row>
     <row r="35" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="84">
+      <c r="B35" s="83">
         <v>31</v>
       </c>
-      <c r="C35" s="37">
+      <c r="C35" s="36">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D35" s="37">
+      <c r="D35" s="36">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E35" s="37">
+      <c r="E35" s="36">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F35" s="37">
+      <c r="F35" s="36">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="G35" s="62">
+      <c r="G35" s="61">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H35" s="46" t="s">
+      <c r="H35" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="46" t="s">
+      <c r="I35" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="J35" s="48" t="s">
+      <c r="J35" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="56" t="s">
+      <c r="K35" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="L35" s="33" t="s">
+      <c r="L35" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="M35" s="33" t="s">
+      <c r="M35" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="N35" s="47" t="s">
+      <c r="N35" s="46" t="s">
         <v>111</v>
       </c>
     </row>
@@ -4955,106 +4979,106 @@
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="249" t="s">
+      <c r="B2" s="248" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="250"/>
-      <c r="G2" s="251"/>
-      <c r="H2" s="198" t="s">
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="249"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="197" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="198" t="s">
+      <c r="I2" s="197" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="249" t="s">
+      <c r="J2" s="248" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="250"/>
-      <c r="L2" s="250"/>
-      <c r="M2" s="198" t="s">
+      <c r="K2" s="249"/>
+      <c r="L2" s="249"/>
+      <c r="M2" s="197" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="85" t="s">
+      <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="50" t="s">
+      <c r="C3" s="49" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>37</v>
       </c>
-      <c r="E3" s="50" t="s">
+      <c r="E3" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="50" t="s">
+      <c r="F3" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="51" t="s">
+      <c r="G3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="199"/>
-      <c r="I3" s="199"/>
-      <c r="J3" s="49" t="s">
+      <c r="H3" s="198"/>
+      <c r="I3" s="198"/>
+      <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="53" t="s">
+      <c r="K3" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="L3" s="52" t="s">
+      <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="199"/>
+      <c r="M3" s="198"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B4" s="81">
-        <v>0</v>
-      </c>
-      <c r="C4" s="36">
+      <c r="B4" s="80">
+        <v>0</v>
+      </c>
+      <c r="C4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,4),1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="36">
+      <c r="D4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,3),1)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="36">
+      <c r="E4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F4" s="36">
+      <c r="F4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G4" s="79">
+      <c r="G4" s="78">
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="230" t="s">
+      <c r="H4" s="229" t="s">
         <v>45</v>
       </c>
-      <c r="I4" s="68" t="s">
+      <c r="I4" s="67" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="K4" s="69" t="s">
+      <c r="K4" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="L4" s="67" t="s">
+      <c r="L4" s="66" t="s">
         <v>85</v>
       </c>
-      <c r="M4" s="76" t="s">
+      <c r="M4" s="75" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="5" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="83">
+      <c r="B5" s="82">
         <v>1</v>
       </c>
       <c r="C5" s="17">
@@ -5073,29 +5097,29 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B5,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="80">
+      <c r="G5" s="79">
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="229"/>
-      <c r="I5" s="43" t="s">
+      <c r="H5" s="228"/>
+      <c r="I5" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="J5" s="63" t="s">
+      <c r="J5" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="K5" s="55" t="s">
+      <c r="K5" s="54" t="s">
         <v>64</v>
       </c>
-      <c r="L5" s="64" t="s">
+      <c r="L5" s="63" t="s">
         <v>16</v>
       </c>
-      <c r="M5" s="45" t="s">
+      <c r="M5" s="44" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B6" s="82">
+      <c r="B6" s="81">
         <v>2</v>
       </c>
       <c r="C6" s="14">
@@ -5106,7 +5130,7 @@
         <f t="shared" ref="D6:D35" si="2">_xlfn.BITAND(_xlfn.BITRSHIFT($B6,3),1)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="60">
+      <c r="E6" s="59">
         <f t="shared" ref="E6:E35" si="3">_xlfn.BITAND(_xlfn.BITRSHIFT($B6,2),1)</f>
         <v>0</v>
       </c>
@@ -5118,27 +5142,27 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="228" t="s">
+      <c r="H6" s="227" t="s">
         <v>61</v>
       </c>
-      <c r="I6" s="91" t="s">
+      <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="232" t="s">
+      <c r="J6" s="231" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="241" t="s">
+      <c r="K6" s="240" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="238" t="s">
+      <c r="L6" s="237" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="246" t="s">
+      <c r="M6" s="245" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B7" s="82">
+      <c r="B7" s="81">
         <v>3</v>
       </c>
       <c r="C7" s="14">
@@ -5149,7 +5173,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E7" s="60">
+      <c r="E7" s="59">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -5161,15 +5185,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="228"/>
-      <c r="I7" s="252"/>
-      <c r="J7" s="232"/>
-      <c r="K7" s="241"/>
-      <c r="L7" s="238"/>
-      <c r="M7" s="246"/>
+      <c r="H7" s="227"/>
+      <c r="I7" s="251"/>
+      <c r="J7" s="231"/>
+      <c r="K7" s="240"/>
+      <c r="L7" s="237"/>
+      <c r="M7" s="245"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B8" s="82">
+      <c r="B8" s="81">
         <v>4</v>
       </c>
       <c r="C8" s="14">
@@ -5180,7 +5204,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E8" s="60">
+      <c r="E8" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -5192,15 +5216,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="228"/>
-      <c r="I8" s="265"/>
-      <c r="J8" s="232"/>
-      <c r="K8" s="241"/>
-      <c r="L8" s="238"/>
-      <c r="M8" s="246"/>
+      <c r="H8" s="227"/>
+      <c r="I8" s="264"/>
+      <c r="J8" s="231"/>
+      <c r="K8" s="240"/>
+      <c r="L8" s="237"/>
+      <c r="M8" s="245"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B9" s="82">
+      <c r="B9" s="81">
         <v>5</v>
       </c>
       <c r="C9" s="14">
@@ -5211,7 +5235,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E9" s="60">
+      <c r="E9" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -5223,15 +5247,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="228"/>
-      <c r="I9" s="266"/>
-      <c r="J9" s="232"/>
-      <c r="K9" s="241"/>
-      <c r="L9" s="238"/>
-      <c r="M9" s="246"/>
+      <c r="H9" s="227"/>
+      <c r="I9" s="265"/>
+      <c r="J9" s="231"/>
+      <c r="K9" s="240"/>
+      <c r="L9" s="237"/>
+      <c r="M9" s="245"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="82">
+      <c r="B10" s="81">
         <v>6</v>
       </c>
       <c r="C10" s="14">
@@ -5242,7 +5266,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E10" s="60">
+      <c r="E10" s="59">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -5254,17 +5278,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="228"/>
-      <c r="I10" s="91" t="s">
+      <c r="H10" s="227"/>
+      <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="232"/>
-      <c r="K10" s="241"/>
-      <c r="L10" s="238"/>
-      <c r="M10" s="246"/>
+      <c r="J10" s="231"/>
+      <c r="K10" s="240"/>
+      <c r="L10" s="237"/>
+      <c r="M10" s="245"/>
     </row>
     <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="83">
+      <c r="B11" s="82">
         <v>7</v>
       </c>
       <c r="C11" s="17">
@@ -5275,7 +5299,7 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E11" s="61">
+      <c r="E11" s="60">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
@@ -5287,58 +5311,58 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="229"/>
-      <c r="I11" s="105"/>
-      <c r="J11" s="233"/>
-      <c r="K11" s="242"/>
-      <c r="L11" s="239"/>
-      <c r="M11" s="247"/>
+      <c r="H11" s="228"/>
+      <c r="I11" s="104"/>
+      <c r="J11" s="232"/>
+      <c r="K11" s="241"/>
+      <c r="L11" s="238"/>
+      <c r="M11" s="246"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B12" s="81">
+      <c r="B12" s="80">
         <v>8</v>
       </c>
-      <c r="C12" s="36">
+      <c r="C12" s="35">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F12" s="58">
+      <c r="F12" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G12" s="59">
+      <c r="G12" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="230" t="s">
+      <c r="H12" s="229" t="s">
         <v>55</v>
       </c>
-      <c r="I12" s="65" t="s">
+      <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="231" t="s">
+      <c r="J12" s="230" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="240" t="s">
+      <c r="K12" s="239" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="237" t="s">
+      <c r="L12" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="248" t="s">
+      <c r="M12" s="247" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B13" s="82">
+      <c r="B13" s="81">
         <v>9</v>
       </c>
       <c r="C13" s="14">
@@ -5353,7 +5377,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F13" s="60">
+      <c r="F13" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -5361,15 +5385,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="228"/>
-      <c r="I13" s="252"/>
-      <c r="J13" s="232"/>
-      <c r="K13" s="241"/>
-      <c r="L13" s="238"/>
-      <c r="M13" s="246"/>
+      <c r="H13" s="227"/>
+      <c r="I13" s="251"/>
+      <c r="J13" s="231"/>
+      <c r="K13" s="240"/>
+      <c r="L13" s="237"/>
+      <c r="M13" s="245"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B14" s="82">
+      <c r="B14" s="81">
         <v>10</v>
       </c>
       <c r="C14" s="14">
@@ -5384,7 +5408,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F14" s="60">
+      <c r="F14" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5392,15 +5416,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="228"/>
-      <c r="I14" s="265"/>
-      <c r="J14" s="232"/>
-      <c r="K14" s="241"/>
-      <c r="L14" s="238"/>
-      <c r="M14" s="246"/>
+      <c r="H14" s="227"/>
+      <c r="I14" s="264"/>
+      <c r="J14" s="231"/>
+      <c r="K14" s="240"/>
+      <c r="L14" s="237"/>
+      <c r="M14" s="245"/>
     </row>
     <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="83">
+      <c r="B15" s="82">
         <v>11</v>
       </c>
       <c r="C15" s="17">
@@ -5415,7 +5439,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F15" s="61">
+      <c r="F15" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5423,58 +5447,58 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="229"/>
-      <c r="I15" s="253"/>
-      <c r="J15" s="233"/>
-      <c r="K15" s="242"/>
-      <c r="L15" s="239"/>
-      <c r="M15" s="247"/>
+      <c r="H15" s="228"/>
+      <c r="I15" s="252"/>
+      <c r="J15" s="232"/>
+      <c r="K15" s="241"/>
+      <c r="L15" s="238"/>
+      <c r="M15" s="246"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="81">
+      <c r="B16" s="80">
         <v>12</v>
       </c>
-      <c r="C16" s="36">
+      <c r="C16" s="35">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D16" s="36">
+      <c r="D16" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F16" s="58">
+      <c r="F16" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G16" s="59">
+      <c r="G16" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="230" t="s">
+      <c r="H16" s="229" t="s">
         <v>56</v>
       </c>
-      <c r="I16" s="65" t="s">
+      <c r="I16" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="231" t="s">
+      <c r="J16" s="230" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="234" t="s">
+      <c r="K16" s="233" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="237" t="s">
+      <c r="L16" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M16" s="76" t="s">
+      <c r="M16" s="75" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B17" s="82">
+      <c r="B17" s="81">
         <v>13</v>
       </c>
       <c r="C17" s="14">
@@ -5489,7 +5513,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F17" s="60">
+      <c r="F17" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -5497,19 +5521,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="228"/>
-      <c r="I17" s="71" t="s">
+      <c r="H17" s="227"/>
+      <c r="I17" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="232"/>
-      <c r="K17" s="235"/>
-      <c r="L17" s="238"/>
-      <c r="M17" s="75" t="s">
+      <c r="J17" s="231"/>
+      <c r="K17" s="234"/>
+      <c r="L17" s="237"/>
+      <c r="M17" s="74" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B18" s="82">
+      <c r="B18" s="81">
         <v>14</v>
       </c>
       <c r="C18" s="14">
@@ -5524,7 +5548,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F18" s="60">
+      <c r="F18" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5532,15 +5556,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="228"/>
-      <c r="I18" s="252"/>
-      <c r="J18" s="232"/>
-      <c r="K18" s="235"/>
-      <c r="L18" s="238"/>
-      <c r="M18" s="252"/>
+      <c r="H18" s="227"/>
+      <c r="I18" s="251"/>
+      <c r="J18" s="231"/>
+      <c r="K18" s="234"/>
+      <c r="L18" s="237"/>
+      <c r="M18" s="251"/>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="83">
+      <c r="B19" s="82">
         <v>15</v>
       </c>
       <c r="C19" s="17">
@@ -5555,7 +5579,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F19" s="61">
+      <c r="F19" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5563,59 +5587,59 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="229"/>
-      <c r="I19" s="253"/>
-      <c r="J19" s="233"/>
-      <c r="K19" s="236"/>
-      <c r="L19" s="239"/>
-      <c r="M19" s="253"/>
+      <c r="H19" s="228"/>
+      <c r="I19" s="252"/>
+      <c r="J19" s="232"/>
+      <c r="K19" s="235"/>
+      <c r="L19" s="238"/>
+      <c r="M19" s="252"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" s="81">
+      <c r="B20" s="80">
         <v>16</v>
       </c>
-      <c r="C20" s="36">
+      <c r="C20" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D20" s="36">
+      <c r="D20" s="35">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E20" s="36">
+      <c r="E20" s="35">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F20" s="58">
+      <c r="F20" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G20" s="59">
+      <c r="G20" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="254" t="s">
+      <c r="H20" s="253" t="s">
         <v>179</v>
       </c>
-      <c r="I20" s="180" t="s">
+      <c r="I20" s="178" t="s">
         <v>119</v>
       </c>
-      <c r="J20" s="67" t="s">
+      <c r="J20" s="66" t="s">
         <v>181</v>
       </c>
-      <c r="K20" s="66" t="s">
+      <c r="K20" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="L20" s="170" t="s">
+      <c r="L20" s="168" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="179" t="s">
+      <c r="M20" s="177" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B21" s="82">
+      <c r="B21" s="81">
         <v>17</v>
       </c>
       <c r="C21" s="14">
@@ -5630,7 +5654,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F21" s="60">
+      <c r="F21" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -5638,15 +5662,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="255"/>
-      <c r="I21" s="171"/>
-      <c r="J21" s="173"/>
-      <c r="K21" s="175"/>
-      <c r="L21" s="177"/>
-      <c r="M21" s="171"/>
+      <c r="H21" s="254"/>
+      <c r="I21" s="169"/>
+      <c r="J21" s="171"/>
+      <c r="K21" s="173"/>
+      <c r="L21" s="175"/>
+      <c r="M21" s="169"/>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B22" s="82">
+      <c r="B22" s="81">
         <v>18</v>
       </c>
       <c r="C22" s="14">
@@ -5661,7 +5685,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F22" s="60">
+      <c r="F22" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5669,15 +5693,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="255"/>
-      <c r="I22" s="171"/>
-      <c r="J22" s="173"/>
-      <c r="K22" s="175"/>
-      <c r="L22" s="177"/>
-      <c r="M22" s="171"/>
+      <c r="H22" s="254"/>
+      <c r="I22" s="169"/>
+      <c r="J22" s="171"/>
+      <c r="K22" s="173"/>
+      <c r="L22" s="175"/>
+      <c r="M22" s="169"/>
     </row>
     <row r="23" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="82">
+      <c r="B23" s="81">
         <v>19</v>
       </c>
       <c r="C23" s="14">
@@ -5692,7 +5716,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F23" s="61">
+      <c r="F23" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5700,58 +5724,58 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="256"/>
-      <c r="I23" s="172"/>
-      <c r="J23" s="174"/>
-      <c r="K23" s="176"/>
-      <c r="L23" s="178"/>
-      <c r="M23" s="172"/>
+      <c r="H23" s="255"/>
+      <c r="I23" s="170"/>
+      <c r="J23" s="172"/>
+      <c r="K23" s="174"/>
+      <c r="L23" s="176"/>
+      <c r="M23" s="170"/>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" s="81">
+      <c r="B24" s="80">
         <v>20</v>
       </c>
-      <c r="C24" s="36">
+      <c r="C24" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D24" s="36">
+      <c r="D24" s="35">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F24" s="58">
+      <c r="F24" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G24" s="59">
+      <c r="G24" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="230" t="s">
+      <c r="H24" s="229" t="s">
         <v>58</v>
       </c>
-      <c r="I24" s="65" t="s">
+      <c r="I24" s="64" t="s">
         <v>45</v>
       </c>
-      <c r="J24" s="67" t="s">
+      <c r="J24" s="66" t="s">
         <v>67</v>
       </c>
-      <c r="K24" s="66" t="s">
+      <c r="K24" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="L24" s="68" t="s">
+      <c r="L24" s="67" t="s">
         <v>16</v>
       </c>
-      <c r="M24" s="76" t="s">
+      <c r="M24" s="75" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B25" s="82">
+      <c r="B25" s="81">
         <v>21</v>
       </c>
       <c r="C25" s="14">
@@ -5766,7 +5790,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F25" s="60">
+      <c r="F25" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -5774,25 +5798,25 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="228"/>
-      <c r="I25" s="71" t="s">
+      <c r="H25" s="227"/>
+      <c r="I25" s="70" t="s">
         <v>46</v>
       </c>
-      <c r="J25" s="101" t="s">
+      <c r="J25" s="100" t="s">
         <v>67</v>
       </c>
-      <c r="K25" s="104" t="s">
+      <c r="K25" s="103" t="s">
         <v>16</v>
       </c>
-      <c r="L25" s="102" t="s">
+      <c r="L25" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M25" s="75" t="s">
+      <c r="M25" s="74" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B26" s="82">
+      <c r="B26" s="81">
         <v>22</v>
       </c>
       <c r="C26" s="14">
@@ -5807,7 +5831,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F26" s="60">
+      <c r="F26" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5815,15 +5839,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="228"/>
-      <c r="I26" s="252"/>
-      <c r="J26" s="257"/>
-      <c r="K26" s="259"/>
-      <c r="L26" s="261"/>
-      <c r="M26" s="263"/>
+      <c r="H26" s="227"/>
+      <c r="I26" s="251"/>
+      <c r="J26" s="256"/>
+      <c r="K26" s="258"/>
+      <c r="L26" s="260"/>
+      <c r="M26" s="262"/>
     </row>
     <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="83">
+      <c r="B27" s="82">
         <v>23</v>
       </c>
       <c r="C27" s="14">
@@ -5838,7 +5862,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F27" s="61">
+      <c r="F27" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -5846,58 +5870,58 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="229"/>
-      <c r="I27" s="253"/>
-      <c r="J27" s="258"/>
-      <c r="K27" s="260"/>
-      <c r="L27" s="262"/>
-      <c r="M27" s="264"/>
+      <c r="H27" s="228"/>
+      <c r="I27" s="252"/>
+      <c r="J27" s="257"/>
+      <c r="K27" s="259"/>
+      <c r="L27" s="261"/>
+      <c r="M27" s="263"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B28" s="81">
+      <c r="B28" s="80">
         <v>24</v>
       </c>
-      <c r="C28" s="36">
+      <c r="C28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,4),1)</f>
         <v>1</v>
       </c>
-      <c r="D28" s="36">
+      <c r="D28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,3),1)</f>
         <v>1</v>
       </c>
-      <c r="E28" s="36">
+      <c r="E28" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="58">
+      <c r="F28" s="57">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B28,1),1)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="59">
+      <c r="G28" s="58">
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="230" t="s">
+      <c r="H28" s="229" t="s">
         <v>167</v>
       </c>
-      <c r="I28" s="38" t="s">
+      <c r="I28" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="J28" s="34" t="s">
+      <c r="J28" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="K28" s="54" t="s">
+      <c r="K28" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="L28" s="40" t="s">
+      <c r="L28" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="M28" s="39" t="s">
+      <c r="M28" s="38" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B29" s="82">
+      <c r="B29" s="81">
         <v>25</v>
       </c>
       <c r="C29" s="14">
@@ -5912,7 +5936,7 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B29,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="60">
+      <c r="F29" s="59">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B29,1),1)</f>
         <v>0</v>
       </c>
@@ -5920,25 +5944,25 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="228"/>
-      <c r="I29" s="71" t="s">
+      <c r="H29" s="227"/>
+      <c r="I29" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="J29" s="72" t="s">
+      <c r="J29" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="K29" s="73" t="s">
+      <c r="K29" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L29" s="74" t="s">
+      <c r="L29" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="M29" s="75" t="s">
+      <c r="M29" s="74" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B30" s="82">
+      <c r="B30" s="81">
         <v>26</v>
       </c>
       <c r="C30" s="14">
@@ -5953,7 +5977,7 @@
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B30,2),1)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="60">
+      <c r="F30" s="59">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B30,1),1)</f>
         <v>1</v>
       </c>
@@ -5961,25 +5985,25 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="228"/>
-      <c r="I30" s="71" t="s">
+      <c r="H30" s="227"/>
+      <c r="I30" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="J30" s="101" t="s">
+      <c r="J30" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="K30" s="73" t="s">
+      <c r="K30" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L30" s="102" t="s">
+      <c r="L30" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M30" s="75" t="s">
+      <c r="M30" s="74" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="83">
+      <c r="B31" s="82">
         <v>27</v>
       </c>
       <c r="C31" s="17">
@@ -5994,7 +6018,7 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="F31" s="61">
+      <c r="F31" s="60">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -6002,59 +6026,59 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="229"/>
-      <c r="I31" s="92"/>
-      <c r="J31" s="166"/>
-      <c r="K31" s="167"/>
-      <c r="L31" s="168"/>
-      <c r="M31" s="94"/>
+      <c r="H31" s="228"/>
+      <c r="I31" s="91"/>
+      <c r="J31" s="164"/>
+      <c r="K31" s="165"/>
+      <c r="L31" s="166"/>
+      <c r="M31" s="93"/>
     </row>
     <row r="32" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B32" s="82">
+      <c r="B32" s="81">
         <v>28</v>
       </c>
-      <c r="C32" s="36">
+      <c r="C32" s="35">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D32" s="36">
+      <c r="D32" s="35">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E32" s="36">
+      <c r="E32" s="35">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F32" s="58">
+      <c r="F32" s="57">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G32" s="59">
+      <c r="G32" s="58">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="228" t="s">
+      <c r="H32" s="227" t="s">
         <v>168</v>
       </c>
-      <c r="I32" s="38" t="s">
+      <c r="I32" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="J32" s="34" t="s">
+      <c r="J32" s="33" t="s">
         <v>64</v>
       </c>
-      <c r="K32" s="54" t="s">
+      <c r="K32" s="53" t="s">
         <v>64</v>
       </c>
-      <c r="L32" s="40" t="s">
+      <c r="L32" s="39" t="s">
         <v>62</v>
       </c>
-      <c r="M32" s="39" t="s">
+      <c r="M32" s="38" t="s">
         <v>163</v>
       </c>
       <c r="P32" s="1"/>
     </row>
     <row r="33" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B33" s="82">
+      <c r="B33" s="81">
         <v>29</v>
       </c>
       <c r="C33" s="14">
@@ -6069,7 +6093,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F33" s="60">
+      <c r="F33" s="59">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -6077,26 +6101,26 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="228"/>
-      <c r="I33" s="71" t="s">
+      <c r="H33" s="227"/>
+      <c r="I33" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="J33" s="72" t="s">
+      <c r="J33" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="K33" s="73" t="s">
+      <c r="K33" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L33" s="74" t="s">
+      <c r="L33" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="M33" s="75" t="s">
+      <c r="M33" s="74" t="s">
         <v>164</v>
       </c>
       <c r="P33" s="1"/>
     </row>
     <row r="34" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="82">
+      <c r="B34" s="81">
         <v>30</v>
       </c>
       <c r="C34" s="14">
@@ -6111,7 +6135,7 @@
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F34" s="60">
+      <c r="F34" s="59">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
@@ -6119,64 +6143,64 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="229"/>
-      <c r="I34" s="71" t="s">
+      <c r="H34" s="228"/>
+      <c r="I34" s="70" t="s">
         <v>53</v>
       </c>
-      <c r="J34" s="101" t="s">
+      <c r="J34" s="100" t="s">
         <v>16</v>
       </c>
-      <c r="K34" s="73" t="s">
+      <c r="K34" s="72" t="s">
         <v>64</v>
       </c>
-      <c r="L34" s="102" t="s">
+      <c r="L34" s="101" t="s">
         <v>44</v>
       </c>
-      <c r="M34" s="75" t="s">
+      <c r="M34" s="74" t="s">
         <v>165</v>
       </c>
       <c r="P34" s="1"/>
     </row>
     <row r="35" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="84">
+      <c r="B35" s="83">
         <v>31</v>
       </c>
-      <c r="C35" s="37">
+      <c r="C35" s="36">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="D35" s="37">
+      <c r="D35" s="36">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="E35" s="37">
+      <c r="E35" s="36">
         <f t="shared" si="3"/>
         <v>1</v>
       </c>
-      <c r="F35" s="37">
+      <c r="F35" s="36">
         <f t="shared" si="4"/>
         <v>1</v>
       </c>
-      <c r="G35" s="62">
+      <c r="G35" s="61">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H35" s="46" t="s">
+      <c r="H35" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="I35" s="46" t="s">
+      <c r="I35" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="J35" s="48" t="s">
+      <c r="J35" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="K35" s="56" t="s">
+      <c r="K35" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="L35" s="169" t="s">
+      <c r="L35" s="167" t="s">
         <v>178</v>
       </c>
-      <c r="M35" s="47" t="s">
+      <c r="M35" s="46" t="s">
         <v>111</v>
       </c>
     </row>
@@ -6231,13 +6255,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="249" t="s">
+      <c r="B2" s="248" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="250"/>
-      <c r="D2" s="250"/>
-      <c r="E2" s="251"/>
-      <c r="F2" s="198" t="s">
+      <c r="C2" s="249"/>
+      <c r="D2" s="249"/>
+      <c r="E2" s="250"/>
+      <c r="F2" s="197" t="s">
         <v>32</v>
       </c>
     </row>
@@ -6245,30 +6269,30 @@
       <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="52" t="s">
+      <c r="C3" s="51" t="s">
         <v>36</v>
       </c>
-      <c r="D3" s="50" t="s">
+      <c r="D3" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E3" s="51" t="s">
+      <c r="E3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="199"/>
+      <c r="F3" s="198"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="13">
         <v>0</v>
       </c>
-      <c r="C4" s="58">
+      <c r="C4" s="57">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,2),1)</f>
         <v>0</v>
       </c>
-      <c r="D4" s="36">
+      <c r="D4" s="35">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,1),1)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="59">
+      <c r="E4" s="58">
         <f>_xlfn.BITAND(_xlfn.BITRSHIFT($B4,0),1)</f>
         <v>0</v>
       </c>
@@ -6280,7 +6304,7 @@
       <c r="B5" s="13">
         <v>1</v>
       </c>
-      <c r="C5" s="60">
+      <c r="C5" s="59">
         <f t="shared" ref="C5:C11" si="0">_xlfn.BITAND(_xlfn.BITRSHIFT($B5,2),1)</f>
         <v>0</v>
       </c>
@@ -6300,7 +6324,7 @@
       <c r="B6" s="19">
         <v>2</v>
       </c>
-      <c r="C6" s="77">
+      <c r="C6" s="76">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6320,7 +6344,7 @@
       <c r="B7" s="22">
         <v>3</v>
       </c>
-      <c r="C7" s="78">
+      <c r="C7" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6340,7 +6364,7 @@
       <c r="B8" s="13">
         <v>4</v>
       </c>
-      <c r="C8" s="60">
+      <c r="C8" s="59">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6360,7 +6384,7 @@
       <c r="B9" s="13">
         <v>5</v>
       </c>
-      <c r="C9" s="60">
+      <c r="C9" s="59">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6380,7 +6404,7 @@
       <c r="B10" s="19">
         <v>6</v>
       </c>
-      <c r="C10" s="77">
+      <c r="C10" s="76">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6400,7 +6424,7 @@
       <c r="B11" s="22">
         <v>7</v>
       </c>
-      <c r="C11" s="78">
+      <c r="C11" s="77">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -6435,202 +6459,202 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="198" t="s">
+      <c r="B2" s="197" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="276" t="s">
+      <c r="C2" s="275" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="277"/>
-      <c r="E2" s="277"/>
-      <c r="F2" s="277"/>
-      <c r="G2" s="277"/>
-      <c r="H2" s="277"/>
-      <c r="I2" s="277"/>
-      <c r="J2" s="277"/>
-      <c r="K2" s="277"/>
-      <c r="L2" s="277"/>
-      <c r="M2" s="277"/>
-      <c r="N2" s="277"/>
-      <c r="O2" s="277"/>
-      <c r="P2" s="277"/>
-      <c r="Q2" s="277"/>
-      <c r="R2" s="278"/>
+      <c r="D2" s="276"/>
+      <c r="E2" s="276"/>
+      <c r="F2" s="276"/>
+      <c r="G2" s="276"/>
+      <c r="H2" s="276"/>
+      <c r="I2" s="276"/>
+      <c r="J2" s="276"/>
+      <c r="K2" s="276"/>
+      <c r="L2" s="276"/>
+      <c r="M2" s="276"/>
+      <c r="N2" s="276"/>
+      <c r="O2" s="276"/>
+      <c r="P2" s="276"/>
+      <c r="Q2" s="276"/>
+      <c r="R2" s="277"/>
     </row>
     <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="199"/>
-      <c r="C3" s="118">
+      <c r="B3" s="198"/>
+      <c r="C3" s="117">
         <v>15</v>
       </c>
-      <c r="D3" s="86">
+      <c r="D3" s="85">
         <v>14</v>
       </c>
-      <c r="E3" s="86">
+      <c r="E3" s="85">
         <v>13</v>
       </c>
-      <c r="F3" s="86">
+      <c r="F3" s="85">
         <v>12</v>
       </c>
-      <c r="G3" s="86">
+      <c r="G3" s="85">
         <v>11</v>
       </c>
-      <c r="H3" s="86">
+      <c r="H3" s="85">
         <v>10</v>
       </c>
-      <c r="I3" s="86">
+      <c r="I3" s="85">
         <v>9</v>
       </c>
-      <c r="J3" s="86">
+      <c r="J3" s="85">
         <v>8</v>
       </c>
-      <c r="K3" s="86">
+      <c r="K3" s="85">
         <v>7</v>
       </c>
-      <c r="L3" s="86">
+      <c r="L3" s="85">
         <v>6</v>
       </c>
-      <c r="M3" s="86">
+      <c r="M3" s="85">
         <v>5</v>
       </c>
-      <c r="N3" s="86">
+      <c r="N3" s="85">
         <v>4</v>
       </c>
-      <c r="O3" s="86">
+      <c r="O3" s="85">
         <v>3</v>
       </c>
-      <c r="P3" s="86">
+      <c r="P3" s="85">
         <v>2</v>
       </c>
-      <c r="Q3" s="86">
-        <v>1</v>
-      </c>
-      <c r="R3" s="87">
+      <c r="Q3" s="85">
+        <v>1</v>
+      </c>
+      <c r="R3" s="86">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="88" t="s">
+      <c r="B4" s="87" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="155"/>
-      <c r="D4" s="155"/>
-      <c r="E4" s="155"/>
-      <c r="F4" s="155"/>
-      <c r="G4" s="155"/>
-      <c r="H4" s="155"/>
-      <c r="I4" s="155"/>
-      <c r="J4" s="155"/>
-      <c r="K4" s="69" t="s">
+      <c r="C4" s="153"/>
+      <c r="D4" s="153"/>
+      <c r="E4" s="153"/>
+      <c r="F4" s="153"/>
+      <c r="G4" s="153"/>
+      <c r="H4" s="153"/>
+      <c r="I4" s="153"/>
+      <c r="J4" s="153"/>
+      <c r="K4" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="L4" s="69" t="s">
+      <c r="L4" s="68" t="s">
         <v>87</v>
       </c>
-      <c r="M4" s="69" t="s">
+      <c r="M4" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="270" t="s">
+      <c r="N4" s="269" t="s">
         <v>89</v>
       </c>
-      <c r="O4" s="270"/>
-      <c r="P4" s="270"/>
-      <c r="Q4" s="270"/>
-      <c r="R4" s="271"/>
+      <c r="O4" s="269"/>
+      <c r="P4" s="269"/>
+      <c r="Q4" s="269"/>
+      <c r="R4" s="270"/>
     </row>
     <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="89" t="s">
+      <c r="B5" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="156"/>
-      <c r="D5" s="157"/>
-      <c r="E5" s="157"/>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
-      <c r="H5" s="157"/>
-      <c r="I5" s="157"/>
-      <c r="J5" s="158"/>
-      <c r="K5" s="272" t="s">
+      <c r="C5" s="154"/>
+      <c r="D5" s="155"/>
+      <c r="E5" s="155"/>
+      <c r="F5" s="155"/>
+      <c r="G5" s="155"/>
+      <c r="H5" s="155"/>
+      <c r="I5" s="155"/>
+      <c r="J5" s="156"/>
+      <c r="K5" s="271" t="s">
         <v>85</v>
       </c>
-      <c r="L5" s="268"/>
-      <c r="M5" s="268"/>
-      <c r="N5" s="268"/>
-      <c r="O5" s="268"/>
-      <c r="P5" s="268"/>
-      <c r="Q5" s="268"/>
-      <c r="R5" s="269"/>
+      <c r="L5" s="267"/>
+      <c r="M5" s="267"/>
+      <c r="N5" s="267"/>
+      <c r="O5" s="267"/>
+      <c r="P5" s="267"/>
+      <c r="Q5" s="267"/>
+      <c r="R5" s="268"/>
     </row>
     <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="89" t="s">
+      <c r="B6" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="156"/>
-      <c r="D6" s="157"/>
-      <c r="E6" s="157"/>
-      <c r="F6" s="157"/>
-      <c r="G6" s="157"/>
-      <c r="H6" s="157"/>
-      <c r="I6" s="157"/>
-      <c r="J6" s="158"/>
-      <c r="K6" s="272" t="s">
+      <c r="C6" s="154"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="155"/>
+      <c r="H6" s="155"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="156"/>
+      <c r="K6" s="271" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="268"/>
-      <c r="M6" s="268"/>
-      <c r="N6" s="268"/>
-      <c r="O6" s="268"/>
-      <c r="P6" s="268"/>
-      <c r="Q6" s="268"/>
-      <c r="R6" s="269"/>
+      <c r="L6" s="267"/>
+      <c r="M6" s="267"/>
+      <c r="N6" s="267"/>
+      <c r="O6" s="267"/>
+      <c r="P6" s="267"/>
+      <c r="Q6" s="267"/>
+      <c r="R6" s="268"/>
     </row>
     <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="89" t="s">
+      <c r="B7" s="88" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="159"/>
-      <c r="D7" s="159"/>
-      <c r="E7" s="159"/>
-      <c r="F7" s="159"/>
-      <c r="G7" s="159"/>
-      <c r="H7" s="159"/>
-      <c r="I7" s="159"/>
-      <c r="J7" s="159"/>
-      <c r="K7" s="273" t="s">
+      <c r="C7" s="157"/>
+      <c r="D7" s="157"/>
+      <c r="E7" s="157"/>
+      <c r="F7" s="157"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="157"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="272" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="274"/>
-      <c r="M7" s="274"/>
-      <c r="N7" s="274"/>
-      <c r="O7" s="274"/>
-      <c r="P7" s="274"/>
-      <c r="Q7" s="274"/>
-      <c r="R7" s="275"/>
+      <c r="L7" s="273"/>
+      <c r="M7" s="273"/>
+      <c r="N7" s="273"/>
+      <c r="O7" s="273"/>
+      <c r="P7" s="273"/>
+      <c r="Q7" s="273"/>
+      <c r="R7" s="274"/>
     </row>
     <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="89" t="s">
+      <c r="B8" s="88" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="267" t="s">
+      <c r="C8" s="266" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="268"/>
-      <c r="E8" s="268"/>
-      <c r="F8" s="268"/>
-      <c r="G8" s="268"/>
-      <c r="H8" s="268"/>
-      <c r="I8" s="268"/>
-      <c r="J8" s="268"/>
-      <c r="K8" s="268"/>
-      <c r="L8" s="268"/>
-      <c r="M8" s="268"/>
-      <c r="N8" s="268"/>
-      <c r="O8" s="268"/>
-      <c r="P8" s="268"/>
-      <c r="Q8" s="268"/>
-      <c r="R8" s="269"/>
+      <c r="D8" s="267"/>
+      <c r="E8" s="267"/>
+      <c r="F8" s="267"/>
+      <c r="G8" s="267"/>
+      <c r="H8" s="267"/>
+      <c r="I8" s="267"/>
+      <c r="J8" s="267"/>
+      <c r="K8" s="267"/>
+      <c r="L8" s="267"/>
+      <c r="M8" s="267"/>
+      <c r="N8" s="267"/>
+      <c r="O8" s="267"/>
+      <c r="P8" s="267"/>
+      <c r="Q8" s="267"/>
+      <c r="R8" s="268"/>
     </row>
     <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="90" t="s">
+      <c r="B9" s="89" t="s">
         <v>90</v>
       </c>
       <c r="C9" s="8"/>
@@ -6646,13 +6670,13 @@
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
-      <c r="P9" s="153" t="s">
+      <c r="P9" s="151" t="s">
         <v>88</v>
       </c>
-      <c r="Q9" s="153" t="s">
+      <c r="Q9" s="151" t="s">
         <v>92</v>
       </c>
-      <c r="R9" s="154" t="s">
+      <c r="R9" s="152" t="s">
         <v>91</v>
       </c>
     </row>
@@ -6683,136 +6707,136 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="160" t="s">
+      <c r="B2" s="158" t="s">
         <v>152</v>
       </c>
-      <c r="C2" s="162" t="s">
+      <c r="C2" s="160" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="161" t="s">
+      <c r="B3" s="159" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="38" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="163" t="s">
+      <c r="B4" s="161" t="s">
         <v>119</v>
       </c>
-      <c r="C4" s="75" t="s">
+      <c r="C4" s="74" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="161" t="s">
+      <c r="B5" s="159" t="s">
         <v>125</v>
       </c>
-      <c r="C5" s="42" t="s">
+      <c r="C5" s="41" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="163" t="s">
+      <c r="B6" s="161" t="s">
         <v>120</v>
       </c>
-      <c r="C6" s="75" t="s">
+      <c r="C6" s="74" t="s">
         <v>154</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="161" t="s">
+      <c r="B7" s="159" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="41" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="164" t="s">
+      <c r="B8" s="162" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="165" t="s">
+      <c r="C8" s="163" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="160" t="s">
+      <c r="B11" s="158" t="s">
         <v>152</v>
       </c>
-      <c r="C11" s="162" t="s">
+      <c r="C11" s="160" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="162" t="s">
+      <c r="D11" s="160" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="163" t="s">
+      <c r="B12" s="161" t="s">
         <v>156</v>
       </c>
-      <c r="C12" s="75" t="s">
+      <c r="C12" s="74" t="s">
         <v>157</v>
       </c>
-      <c r="D12" s="75" t="s">
+      <c r="D12" s="74" t="s">
         <v>175</v>
       </c>
     </row>
     <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="161" t="s">
+      <c r="B13" s="159" t="s">
         <v>158</v>
       </c>
-      <c r="C13" s="42" t="s">
+      <c r="C13" s="41" t="s">
         <v>159</v>
       </c>
-      <c r="D13" s="42" t="s">
+      <c r="D13" s="41" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="163" t="s">
+      <c r="B14" s="161" t="s">
         <v>160</v>
       </c>
-      <c r="C14" s="75" t="s">
+      <c r="C14" s="74" t="s">
         <v>161</v>
       </c>
-      <c r="D14" s="75" t="s">
+      <c r="D14" s="74" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="163" t="s">
+      <c r="B15" s="161" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="75" t="s">
+      <c r="C15" s="74" t="s">
         <v>166</v>
       </c>
-      <c r="D15" s="75" t="s">
+      <c r="D15" s="74" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="161" t="s">
+      <c r="B16" s="159" t="s">
         <v>169</v>
       </c>
-      <c r="C16" s="42" t="s">
+      <c r="C16" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="D16" s="42" t="s">
+      <c r="D16" s="41" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="164" t="s">
+      <c r="B17" s="162" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="165" t="s">
+      <c r="C17" s="163" t="s">
         <v>162</v>
       </c>
-      <c r="D17" s="165" t="s">
+      <c r="D17" s="163" t="s">
         <v>174</v>
       </c>
     </row>
@@ -6831,94 +6855,94 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="279" t="s">
+      <c r="B2" s="278" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="280"/>
+      <c r="C2" s="279"/>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="141" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="150" t="s">
+      <c r="C3" s="148" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="93"/>
-      <c r="C4" s="133" t="s">
+      <c r="B4" s="92"/>
+      <c r="C4" s="131" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="281" t="s">
+      <c r="D4" s="280" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="95"/>
-      <c r="C5" s="134" t="s">
+      <c r="B5" s="94"/>
+      <c r="C5" s="132" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="282"/>
+      <c r="D5" s="281"/>
     </row>
     <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="136"/>
-      <c r="C6" s="64" t="s">
+      <c r="B6" s="134"/>
+      <c r="C6" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="283"/>
+      <c r="D6" s="282"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="144" t="s">
+      <c r="B7" s="142" t="s">
         <v>143</v>
       </c>
-      <c r="C7" s="145"/>
-      <c r="D7" s="284" t="s">
+      <c r="C7" s="143"/>
+      <c r="D7" s="283" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="C8" s="146"/>
-      <c r="D8" s="285"/>
+      <c r="C8" s="144"/>
+      <c r="D8" s="284"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="C9" s="146"/>
-      <c r="D9" s="285"/>
+      <c r="C9" s="144"/>
+      <c r="D9" s="284"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="147" t="s">
+      <c r="B10" s="145" t="s">
         <v>145</v>
       </c>
-      <c r="C10" s="148" t="s">
+      <c r="C10" s="146" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="285"/>
+      <c r="D10" s="284"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="41" t="s">
+      <c r="B11" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="C11" s="134" t="s">
+      <c r="C11" s="132" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="285"/>
+      <c r="D11" s="284"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="149" t="s">
+      <c r="B12" s="147" t="s">
         <v>146</v>
       </c>
-      <c r="C12" s="64" t="s">
+      <c r="C12" s="63" t="s">
         <v>146</v>
       </c>
-      <c r="D12" s="286"/>
+      <c r="D12" s="285"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6940,102 +6964,102 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="287" t="s">
+      <c r="B2" s="286" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="289" t="s">
+      <c r="C2" s="288" t="s">
         <v>194</v>
       </c>
-      <c r="D2" s="290"/>
+      <c r="D2" s="289"/>
     </row>
     <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="288"/>
-      <c r="C3" s="189" t="s">
+      <c r="B3" s="287"/>
+      <c r="C3" s="187" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="190" t="s">
+      <c r="D3" s="188" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="89">
-        <v>0</v>
-      </c>
-      <c r="C4" s="147" t="s">
+      <c r="B4" s="88">
+        <v>0</v>
+      </c>
+      <c r="C4" s="145" t="s">
         <v>199</v>
       </c>
-      <c r="D4" s="237" t="s">
+      <c r="D4" s="236" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="181">
-        <v>1</v>
-      </c>
-      <c r="C5" s="194" t="s">
+      <c r="B5" s="179">
+        <v>1</v>
+      </c>
+      <c r="C5" s="192" t="s">
         <v>200</v>
       </c>
-      <c r="D5" s="291"/>
+      <c r="D5" s="290"/>
     </row>
     <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="89">
+      <c r="B6" s="88">
         <v>2</v>
       </c>
-      <c r="C6" s="293" t="s">
+      <c r="C6" s="292" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="292" t="s">
+      <c r="D6" s="291" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="181">
+      <c r="B7" s="179">
         <v>3</v>
       </c>
-      <c r="C7" s="232"/>
-      <c r="D7" s="238"/>
+      <c r="C7" s="231"/>
+      <c r="D7" s="237"/>
     </row>
     <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="89">
+      <c r="B8" s="88">
         <v>4</v>
       </c>
-      <c r="C8" s="294"/>
-      <c r="D8" s="291"/>
+      <c r="C8" s="293"/>
+      <c r="D8" s="290"/>
     </row>
     <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="181">
+      <c r="B9" s="179">
         <v>5</v>
       </c>
-      <c r="C9" s="95"/>
-      <c r="D9" s="183"/>
+      <c r="C9" s="94"/>
+      <c r="D9" s="181"/>
     </row>
     <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="89">
+      <c r="B10" s="88">
         <v>6</v>
       </c>
-      <c r="C10" s="139"/>
-      <c r="D10" s="146"/>
+      <c r="C10" s="137"/>
+      <c r="D10" s="144"/>
     </row>
     <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="182">
+      <c r="B11" s="180">
         <v>7</v>
       </c>
-      <c r="C11" s="136"/>
-      <c r="D11" s="184" t="s">
+      <c r="C11" s="134"/>
+      <c r="D11" s="182" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="191" t="s">
+      <c r="B14" s="189" t="s">
         <v>197</v>
       </c>
-      <c r="C14" s="192" t="s">
+      <c r="C14" s="190" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="89">
+      <c r="B15" s="88">
         <v>0</v>
       </c>
       <c r="C15" s="26" t="s">
@@ -7043,15 +7067,15 @@
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="181">
-        <v>1</v>
-      </c>
-      <c r="C16" s="185" t="s">
+      <c r="B16" s="179">
+        <v>1</v>
+      </c>
+      <c r="C16" s="183" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B17" s="89">
+      <c r="B17" s="88">
         <v>2</v>
       </c>
       <c r="C17" s="26" t="s">
@@ -7059,15 +7083,15 @@
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="181">
+      <c r="B18" s="179">
         <v>3</v>
       </c>
-      <c r="C18" s="185" t="s">
+      <c r="C18" s="183" t="s">
         <v>183</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B19" s="89">
+      <c r="B19" s="88">
         <v>4</v>
       </c>
       <c r="C19" s="26" t="s">
@@ -7075,22 +7099,22 @@
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="181">
+      <c r="B20" s="179">
         <v>5</v>
       </c>
-      <c r="C20" s="185"/>
+      <c r="C20" s="183"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B21" s="89">
+      <c r="B21" s="88">
         <v>6</v>
       </c>
       <c r="C21" s="26"/>
     </row>
     <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="182">
+      <c r="B22" s="180">
         <v>7</v>
       </c>
-      <c r="C22" s="188"/>
+      <c r="C22" s="186"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
@@ -7099,15 +7123,15 @@
       <c r="B24" s="1"/>
     </row>
     <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="191" t="s">
+      <c r="B25" s="189" t="s">
         <v>197</v>
       </c>
-      <c r="C25" s="192" t="s">
+      <c r="C25" s="190" t="s">
         <v>189</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B26" s="89">
+      <c r="B26" s="88">
         <v>0</v>
       </c>
       <c r="C26" s="26" t="s">
@@ -7115,15 +7139,15 @@
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="181">
-        <v>1</v>
-      </c>
-      <c r="C27" s="185" t="s">
+      <c r="B27" s="179">
+        <v>1</v>
+      </c>
+      <c r="C27" s="183" t="s">
         <v>187</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B28" s="89">
+      <c r="B28" s="88">
         <v>2</v>
       </c>
       <c r="C28" s="26" t="s">
@@ -7131,24 +7155,24 @@
       </c>
     </row>
     <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="186">
+      <c r="B29" s="184">
         <v>3</v>
       </c>
-      <c r="C29" s="187" t="s">
+      <c r="C29" s="185" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="191" t="s">
+      <c r="B32" s="189" t="s">
         <v>197</v>
       </c>
-      <c r="C32" s="192" t="s">
+      <c r="C32" s="190" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="89">
+      <c r="B33" s="88">
         <v>0</v>
       </c>
       <c r="C33" s="26" t="s">
@@ -7156,15 +7180,15 @@
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="181">
-        <v>1</v>
-      </c>
-      <c r="C34" s="185" t="s">
+      <c r="B34" s="179">
+        <v>1</v>
+      </c>
+      <c r="C34" s="183" t="s">
         <v>158</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B35" s="89">
+      <c r="B35" s="88">
         <v>2</v>
       </c>
       <c r="C35" s="26" t="s">
@@ -7172,15 +7196,15 @@
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B36" s="181">
+      <c r="B36" s="179">
         <v>3</v>
       </c>
-      <c r="C36" s="185" t="s">
+      <c r="C36" s="183" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B37" s="89">
+      <c r="B37" s="88">
         <v>4</v>
       </c>
       <c r="C37" s="26" t="s">
@@ -7188,26 +7212,26 @@
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="181">
+      <c r="B38" s="179">
         <v>5</v>
       </c>
-      <c r="C38" s="185" t="s">
+      <c r="C38" s="183" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B39" s="92">
+      <c r="B39" s="91">
         <v>6</v>
       </c>
-      <c r="C39" s="193" t="s">
+      <c r="C39" s="191" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="186">
+      <c r="B40" s="184">
         <v>7</v>
       </c>
-      <c r="C40" s="187" t="s">
+      <c r="C40" s="185" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix page write address
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA779162-0020-4F05-96FC-DF67701F275C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E505D9EE-13DD-4E62-AC93-B5A023966D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -1625,7 +1625,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="294">
+  <cellXfs count="293">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2009,9 +2009,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="50" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2178,6 +2175,42 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2217,94 +2250,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2313,19 +2292,43 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2364,12 +2367,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2456,7 +2453,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2477,7 +2474,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2794,32 +2791,32 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F30110-9AA6-4607-84AE-181659F51D05}">
   <dimension ref="B1:J19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="6" width="4.7109375" style="1" customWidth="1"/>
-    <col min="7" max="9" width="9.140625" customWidth="1"/>
-    <col min="10" max="10" width="34.28515625" customWidth="1"/>
+    <col min="3" max="6" width="4.73046875" style="1" customWidth="1"/>
+    <col min="7" max="9" width="9.1328125" customWidth="1"/>
+    <col min="10" max="10" width="34.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="194" t="s">
+    <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
+      <c r="B2" s="193" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="195"/>
-      <c r="D2" s="195"/>
-      <c r="E2" s="195"/>
-      <c r="F2" s="196"/>
-      <c r="G2" s="199" t="s">
+      <c r="C2" s="194"/>
+      <c r="D2" s="194"/>
+      <c r="E2" s="194"/>
+      <c r="F2" s="195"/>
+      <c r="G2" s="198" t="s">
         <v>32</v>
       </c>
-      <c r="H2" s="200"/>
-      <c r="I2" s="201"/>
-      <c r="J2" s="197" t="s">
+      <c r="H2" s="199"/>
+      <c r="I2" s="200"/>
+      <c r="J2" s="196" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="56" t="s">
         <v>16</v>
       </c>
@@ -2844,9 +2841,9 @@
       <c r="I3" s="50" t="s">
         <v>138</v>
       </c>
-      <c r="J3" s="198"/>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="J3" s="197"/>
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B4" s="106">
         <v>0</v>
       </c>
@@ -2879,7 +2876,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -2912,7 +2909,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -2945,7 +2942,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -2978,7 +2975,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -3011,7 +3008,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -3044,7 +3041,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -3077,7 +3074,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -3110,7 +3107,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B12" s="13">
         <v>8</v>
       </c>
@@ -3133,7 +3130,7 @@
       <c r="G12" s="120" t="s">
         <v>134</v>
       </c>
-      <c r="H12" s="149" t="s">
+      <c r="H12" s="148" t="s">
         <v>147</v>
       </c>
       <c r="I12" s="115"/>
@@ -3141,7 +3138,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B13" s="13">
         <v>9</v>
       </c>
@@ -3164,13 +3161,13 @@
       <c r="G13" s="119" t="s">
         <v>135</v>
       </c>
-      <c r="H13" s="150"/>
+      <c r="H13" s="149"/>
       <c r="I13" s="114"/>
       <c r="J13" s="26" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B14" s="19">
         <v>10</v>
       </c>
@@ -3191,11 +3188,13 @@
         <v>0</v>
       </c>
       <c r="G14" s="122"/>
-      <c r="H14" s="128"/>
+      <c r="H14" s="148" t="s">
+        <v>136</v>
+      </c>
       <c r="I14" s="115"/>
       <c r="J14" s="31"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B15" s="22">
         <v>11</v>
       </c>
@@ -3218,15 +3217,13 @@
       <c r="G15" s="121" t="s">
         <v>136</v>
       </c>
-      <c r="H15" s="140" t="s">
-        <v>136</v>
-      </c>
+      <c r="H15" s="149"/>
       <c r="I15" s="113"/>
       <c r="J15" s="30" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B16" s="13">
         <v>12</v>
       </c>
@@ -3249,7 +3246,7 @@
       <c r="G16" s="119" t="s">
         <v>202</v>
       </c>
-      <c r="H16" s="193" t="s">
+      <c r="H16" s="192" t="s">
         <v>204</v>
       </c>
       <c r="I16" s="114"/>
@@ -3257,7 +3254,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B17" s="13">
         <v>13</v>
       </c>
@@ -3286,7 +3283,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B18" s="19">
         <v>14</v>
       </c>
@@ -3311,7 +3308,7 @@
       <c r="I18" s="115"/>
       <c r="J18" s="31"/>
     </row>
-    <row r="19" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="16">
         <v>15</v>
       </c>
@@ -3350,13 +3347,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE0A35C-77D4-4A92-BE06-765002DB2402}">
   <dimension ref="B1:AH8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="34" width="7.7109375" customWidth="1"/>
+    <col min="3" max="34" width="7.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="C2" s="2">
         <v>31</v>
       </c>
@@ -3454,74 +3451,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="224" t="s">
+    <row r="3" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="C3" s="210" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="225"/>
-      <c r="E3" s="225"/>
-      <c r="F3" s="225"/>
-      <c r="G3" s="226"/>
-      <c r="H3" s="221" t="s">
+      <c r="D3" s="211"/>
+      <c r="E3" s="211"/>
+      <c r="F3" s="211"/>
+      <c r="G3" s="212"/>
+      <c r="H3" s="207" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="222"/>
-      <c r="J3" s="223"/>
-      <c r="K3" s="221" t="s">
+      <c r="I3" s="208"/>
+      <c r="J3" s="209"/>
+      <c r="K3" s="207" t="s">
         <v>96</v>
       </c>
-      <c r="L3" s="222"/>
-      <c r="M3" s="222"/>
-      <c r="N3" s="208" t="s">
+      <c r="L3" s="208"/>
+      <c r="M3" s="208"/>
+      <c r="N3" s="219" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="209"/>
-      <c r="P3" s="210"/>
+      <c r="O3" s="220"/>
+      <c r="P3" s="221"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="202" t="s">
+      <c r="S3" s="213" t="s">
         <v>28</v>
       </c>
-      <c r="T3" s="203"/>
-      <c r="U3" s="203"/>
-      <c r="V3" s="203"/>
-      <c r="W3" s="203"/>
-      <c r="X3" s="203"/>
-      <c r="Y3" s="203"/>
-      <c r="Z3" s="204"/>
-      <c r="AA3" s="205" t="s">
+      <c r="T3" s="214"/>
+      <c r="U3" s="214"/>
+      <c r="V3" s="214"/>
+      <c r="W3" s="214"/>
+      <c r="X3" s="214"/>
+      <c r="Y3" s="214"/>
+      <c r="Z3" s="215"/>
+      <c r="AA3" s="216" t="s">
         <v>29</v>
       </c>
-      <c r="AB3" s="206"/>
-      <c r="AC3" s="206"/>
-      <c r="AD3" s="206"/>
-      <c r="AE3" s="206"/>
-      <c r="AF3" s="206"/>
-      <c r="AG3" s="206"/>
-      <c r="AH3" s="207"/>
-    </row>
-    <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="B5" s="213" t="s">
+      <c r="AB3" s="217"/>
+      <c r="AC3" s="217"/>
+      <c r="AD3" s="217"/>
+      <c r="AE3" s="217"/>
+      <c r="AF3" s="217"/>
+      <c r="AG3" s="217"/>
+      <c r="AH3" s="218"/>
+    </row>
+    <row r="4" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="5" spans="2:34" x14ac:dyDescent="0.45">
+      <c r="B5" s="224" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="211" t="s">
+      <c r="C5" s="222" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="211"/>
-      <c r="E5" s="211"/>
-      <c r="F5" s="211"/>
-      <c r="G5" s="211"/>
-      <c r="H5" s="211"/>
-      <c r="I5" s="211"/>
-      <c r="J5" s="212"/>
-    </row>
-    <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="214"/>
+      <c r="D5" s="222"/>
+      <c r="E5" s="222"/>
+      <c r="F5" s="222"/>
+      <c r="G5" s="222"/>
+      <c r="H5" s="222"/>
+      <c r="I5" s="222"/>
+      <c r="J5" s="223"/>
+    </row>
+    <row r="6" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B6" s="225"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3547,22 +3544,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:34" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:34" x14ac:dyDescent="0.45">
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="215" t="s">
+      <c r="C7" s="201" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="216"/>
-      <c r="E7" s="216"/>
-      <c r="F7" s="216"/>
-      <c r="G7" s="216"/>
-      <c r="H7" s="216"/>
-      <c r="I7" s="216"/>
-      <c r="J7" s="217"/>
-    </row>
-    <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="202"/>
+      <c r="E7" s="202"/>
+      <c r="F7" s="202"/>
+      <c r="G7" s="202"/>
+      <c r="H7" s="202"/>
+      <c r="I7" s="202"/>
+      <c r="J7" s="203"/>
+    </row>
+    <row r="8" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="6">
         <v>1</v>
       </c>
@@ -3570,25 +3567,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="218" t="s">
+      <c r="G8" s="204" t="s">
         <v>27</v>
       </c>
-      <c r="H8" s="219"/>
-      <c r="I8" s="219"/>
-      <c r="J8" s="220"/>
+      <c r="H8" s="205"/>
+      <c r="I8" s="205"/>
+      <c r="J8" s="206"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="S3:Z3"/>
+    <mergeCell ref="AA3:AH3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:J7"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="S3:Z3"/>
-    <mergeCell ref="AA3:AH3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3598,46 +3595,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B20B11-9266-4E5E-A2B3-3496A1A10C3B}">
   <dimension ref="B1:Q35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="9.140625" style="1"/>
-    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.7109375" customWidth="1"/>
+    <col min="2" max="2" width="9.1328125" style="1"/>
+    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.73046875" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="90.28515625" customWidth="1"/>
+    <col min="14" max="14" width="90.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="248" t="s">
+    <row r="1" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="B2" s="226" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="197" t="s">
+      <c r="C2" s="227"/>
+      <c r="D2" s="227"/>
+      <c r="E2" s="227"/>
+      <c r="F2" s="227"/>
+      <c r="G2" s="228"/>
+      <c r="H2" s="196" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="197" t="s">
+      <c r="I2" s="196" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="248" t="s">
+      <c r="J2" s="226" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="249"/>
-      <c r="L2" s="249"/>
-      <c r="M2" s="197" t="s">
+      <c r="K2" s="227"/>
+      <c r="L2" s="227"/>
+      <c r="M2" s="196" t="s">
         <v>112</v>
       </c>
-      <c r="N2" s="197" t="s">
+      <c r="N2" s="196" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
@@ -3656,8 +3653,8 @@
       <c r="G3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="198"/>
-      <c r="I3" s="198"/>
+      <c r="H3" s="197"/>
+      <c r="I3" s="197"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -3667,10 +3664,10 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="198"/>
-      <c r="N3" s="198"/>
-    </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M3" s="197"/>
+      <c r="N3" s="197"/>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
         <v>0</v>
       </c>
@@ -3716,7 +3713,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B5" s="82">
         <v>1</v>
       </c>
@@ -3740,7 +3737,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="228"/>
+      <c r="H5" s="230"/>
       <c r="I5" s="42" t="s">
         <v>3</v>
       </c>
@@ -3760,7 +3757,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B6" s="81">
         <v>2</v>
       </c>
@@ -3784,29 +3781,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="227" t="s">
+      <c r="H6" s="231" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="231" t="s">
+      <c r="J6" s="232" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="240" t="s">
+      <c r="K6" s="234" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="237" t="s">
+      <c r="L6" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="242" t="s">
+      <c r="M6" s="244" t="s">
         <v>113</v>
       </c>
-      <c r="N6" s="245" t="s">
+      <c r="N6" s="238" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B7" s="81">
         <v>3</v>
       </c>
@@ -3830,17 +3827,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="227"/>
+      <c r="H7" s="231"/>
       <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="231"/>
-      <c r="K7" s="240"/>
-      <c r="L7" s="237"/>
-      <c r="M7" s="243"/>
-      <c r="N7" s="245"/>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J7" s="232"/>
+      <c r="K7" s="234"/>
+      <c r="L7" s="236"/>
+      <c r="M7" s="245"/>
+      <c r="N7" s="238"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B8" s="81">
         <v>4</v>
       </c>
@@ -3864,17 +3861,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="227"/>
+      <c r="H8" s="231"/>
       <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="231"/>
-      <c r="K8" s="240"/>
-      <c r="L8" s="237"/>
-      <c r="M8" s="243"/>
-      <c r="N8" s="245"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J8" s="232"/>
+      <c r="K8" s="234"/>
+      <c r="L8" s="236"/>
+      <c r="M8" s="245"/>
+      <c r="N8" s="238"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B9" s="81">
         <v>5</v>
       </c>
@@ -3898,17 +3895,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="227"/>
+      <c r="H9" s="231"/>
       <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="231"/>
-      <c r="K9" s="240"/>
-      <c r="L9" s="237"/>
-      <c r="M9" s="243"/>
-      <c r="N9" s="245"/>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J9" s="232"/>
+      <c r="K9" s="234"/>
+      <c r="L9" s="236"/>
+      <c r="M9" s="245"/>
+      <c r="N9" s="238"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B10" s="81">
         <v>6</v>
       </c>
@@ -3932,17 +3929,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="227"/>
+      <c r="H10" s="231"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="231"/>
-      <c r="K10" s="240"/>
-      <c r="L10" s="237"/>
-      <c r="M10" s="243"/>
-      <c r="N10" s="245"/>
-    </row>
-    <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J10" s="232"/>
+      <c r="K10" s="234"/>
+      <c r="L10" s="236"/>
+      <c r="M10" s="245"/>
+      <c r="N10" s="238"/>
+    </row>
+    <row r="11" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="82">
         <v>7</v>
       </c>
@@ -3966,17 +3963,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="228"/>
+      <c r="H11" s="230"/>
       <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="232"/>
-      <c r="K11" s="241"/>
-      <c r="L11" s="238"/>
-      <c r="M11" s="244"/>
-      <c r="N11" s="246"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J11" s="233"/>
+      <c r="K11" s="235"/>
+      <c r="L11" s="237"/>
+      <c r="M11" s="246"/>
+      <c r="N11" s="239"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B12" s="80">
         <v>8</v>
       </c>
@@ -4006,23 +4003,23 @@
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="230" t="s">
+      <c r="J12" s="240" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="239" t="s">
+      <c r="K12" s="241" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="236" t="s">
+      <c r="L12" s="242" t="s">
         <v>66</v>
       </c>
       <c r="M12" s="229" t="s">
         <v>114</v>
       </c>
-      <c r="N12" s="247" t="s">
+      <c r="N12" s="243" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B13" s="81">
         <v>9</v>
       </c>
@@ -4046,17 +4043,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="227"/>
+      <c r="H13" s="231"/>
       <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="231"/>
-      <c r="K13" s="240"/>
-      <c r="L13" s="237"/>
-      <c r="M13" s="227"/>
-      <c r="N13" s="245"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J13" s="232"/>
+      <c r="K13" s="234"/>
+      <c r="L13" s="236"/>
+      <c r="M13" s="231"/>
+      <c r="N13" s="238"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B14" s="81">
         <v>10</v>
       </c>
@@ -4080,17 +4077,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="227"/>
+      <c r="H14" s="231"/>
       <c r="I14" s="90" t="s">
         <v>102</v>
       </c>
-      <c r="J14" s="231"/>
-      <c r="K14" s="240"/>
-      <c r="L14" s="237"/>
-      <c r="M14" s="227"/>
-      <c r="N14" s="245"/>
-    </row>
-    <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J14" s="232"/>
+      <c r="K14" s="234"/>
+      <c r="L14" s="236"/>
+      <c r="M14" s="231"/>
+      <c r="N14" s="238"/>
+    </row>
+    <row r="15" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="82">
         <v>11</v>
       </c>
@@ -4114,17 +4111,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="228"/>
+      <c r="H15" s="230"/>
       <c r="I15" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="J15" s="232"/>
-      <c r="K15" s="241"/>
-      <c r="L15" s="238"/>
-      <c r="M15" s="228"/>
-      <c r="N15" s="246"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J15" s="233"/>
+      <c r="K15" s="235"/>
+      <c r="L15" s="237"/>
+      <c r="M15" s="230"/>
+      <c r="N15" s="239"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B16" s="80">
         <v>12</v>
       </c>
@@ -4154,13 +4151,13 @@
       <c r="I16" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="230" t="s">
+      <c r="J16" s="240" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="233" t="s">
+      <c r="K16" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="236" t="s">
+      <c r="L16" s="242" t="s">
         <v>66</v>
       </c>
       <c r="M16" s="229" t="s">
@@ -4170,7 +4167,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B17" s="81">
         <v>13</v>
       </c>
@@ -4194,19 +4191,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="227"/>
+      <c r="H17" s="231"/>
       <c r="I17" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="231"/>
-      <c r="K17" s="234"/>
-      <c r="L17" s="237"/>
-      <c r="M17" s="227"/>
+      <c r="J17" s="232"/>
+      <c r="K17" s="248"/>
+      <c r="L17" s="236"/>
+      <c r="M17" s="231"/>
       <c r="N17" s="74" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B18" s="81">
         <v>14</v>
       </c>
@@ -4230,19 +4227,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="227"/>
+      <c r="H18" s="231"/>
       <c r="I18" s="70" t="s">
         <v>49</v>
       </c>
-      <c r="J18" s="231"/>
-      <c r="K18" s="234"/>
-      <c r="L18" s="237"/>
-      <c r="M18" s="227"/>
+      <c r="J18" s="232"/>
+      <c r="K18" s="248"/>
+      <c r="L18" s="236"/>
+      <c r="M18" s="231"/>
       <c r="N18" s="74" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="82">
         <v>15</v>
       </c>
@@ -4266,20 +4263,20 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="228"/>
+      <c r="H19" s="230"/>
       <c r="I19" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="J19" s="232"/>
-      <c r="K19" s="235"/>
-      <c r="L19" s="238"/>
-      <c r="M19" s="228"/>
+      <c r="J19" s="233"/>
+      <c r="K19" s="249"/>
+      <c r="L19" s="237"/>
+      <c r="M19" s="230"/>
       <c r="N19" s="44" t="s">
         <v>108</v>
       </c>
       <c r="P19" s="1"/>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B20" s="80">
         <v>16</v>
       </c>
@@ -4309,23 +4306,23 @@
       <c r="I20" s="64" t="s">
         <v>17</v>
       </c>
-      <c r="J20" s="230" t="s">
+      <c r="J20" s="240" t="s">
         <v>16</v>
       </c>
-      <c r="K20" s="239" t="s">
+      <c r="K20" s="241" t="s">
         <v>18</v>
       </c>
-      <c r="L20" s="236" t="s">
+      <c r="L20" s="242" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="242" t="s">
+      <c r="M20" s="244" t="s">
         <v>113</v>
       </c>
       <c r="N20" s="41" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B21" s="81">
         <v>17</v>
       </c>
@@ -4349,19 +4346,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="227"/>
+      <c r="H21" s="231"/>
       <c r="I21" s="70" t="s">
         <v>19</v>
       </c>
-      <c r="J21" s="231"/>
-      <c r="K21" s="240"/>
-      <c r="L21" s="237"/>
-      <c r="M21" s="243"/>
+      <c r="J21" s="232"/>
+      <c r="K21" s="234"/>
+      <c r="L21" s="236"/>
+      <c r="M21" s="245"/>
       <c r="N21" s="74" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B22" s="81">
         <v>18</v>
       </c>
@@ -4385,19 +4382,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="227"/>
+      <c r="H22" s="231"/>
       <c r="I22" s="70" t="s">
         <v>20</v>
       </c>
-      <c r="J22" s="231"/>
-      <c r="K22" s="240"/>
-      <c r="L22" s="237"/>
-      <c r="M22" s="243"/>
+      <c r="J22" s="232"/>
+      <c r="K22" s="234"/>
+      <c r="L22" s="236"/>
+      <c r="M22" s="245"/>
       <c r="N22" s="74" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B23" s="81">
         <v>19</v>
       </c>
@@ -4421,19 +4418,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="228"/>
+      <c r="H23" s="230"/>
       <c r="I23" s="42" t="s">
         <v>21</v>
       </c>
-      <c r="J23" s="232"/>
-      <c r="K23" s="241"/>
-      <c r="L23" s="238"/>
-      <c r="M23" s="244"/>
+      <c r="J23" s="233"/>
+      <c r="K23" s="235"/>
+      <c r="L23" s="237"/>
+      <c r="M23" s="246"/>
       <c r="N23" s="41" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B24" s="80">
         <v>20</v>
       </c>
@@ -4479,7 +4476,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B25" s="81">
         <v>21</v>
       </c>
@@ -4503,7 +4500,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="227"/>
+      <c r="H25" s="231"/>
       <c r="I25" s="70" t="s">
         <v>46</v>
       </c>
@@ -4523,7 +4520,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B26" s="81">
         <v>22</v>
       </c>
@@ -4547,7 +4544,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="227"/>
+      <c r="H26" s="231"/>
       <c r="I26" s="104"/>
       <c r="J26" s="137"/>
       <c r="K26" s="138"/>
@@ -4555,7 +4552,7 @@
       <c r="M26" s="105"/>
       <c r="N26" s="105"/>
     </row>
-    <row r="27" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B27" s="82">
         <v>23</v>
       </c>
@@ -4579,7 +4576,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="228"/>
+      <c r="H27" s="230"/>
       <c r="I27" s="97"/>
       <c r="J27" s="134"/>
       <c r="K27" s="135"/>
@@ -4587,7 +4584,7 @@
       <c r="M27" s="133"/>
       <c r="N27" s="133"/>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B28" s="80">
         <v>24</v>
       </c>
@@ -4633,7 +4630,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B29" s="81">
         <v>25</v>
       </c>
@@ -4657,7 +4654,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="227"/>
+      <c r="H29" s="231"/>
       <c r="I29" s="70" t="s">
         <v>52</v>
       </c>
@@ -4677,7 +4674,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B30" s="81">
         <v>26</v>
       </c>
@@ -4701,7 +4698,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="227"/>
+      <c r="H30" s="231"/>
       <c r="I30" s="70" t="s">
         <v>53</v>
       </c>
@@ -4721,7 +4718,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B31" s="82">
         <v>27</v>
       </c>
@@ -4745,7 +4742,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="228"/>
+      <c r="H31" s="230"/>
       <c r="I31" s="91"/>
       <c r="J31" s="94"/>
       <c r="K31" s="95"/>
@@ -4753,7 +4750,7 @@
       <c r="M31" s="96"/>
       <c r="N31" s="93"/>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B32" s="81">
         <v>28</v>
       </c>
@@ -4777,7 +4774,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="227" t="s">
+      <c r="H32" s="231" t="s">
         <v>59</v>
       </c>
       <c r="I32" s="64" t="s">
@@ -4800,7 +4797,7 @@
       </c>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B33" s="81">
         <v>29</v>
       </c>
@@ -4824,7 +4821,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="227"/>
+      <c r="H33" s="231"/>
       <c r="I33" s="70" t="s">
         <v>24</v>
       </c>
@@ -4845,7 +4842,7 @@
       </c>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B34" s="81">
         <v>30</v>
       </c>
@@ -4869,7 +4866,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="228"/>
+      <c r="H34" s="230"/>
       <c r="I34" s="97"/>
       <c r="J34" s="94"/>
       <c r="K34" s="95"/>
@@ -4878,7 +4875,7 @@
       <c r="N34" s="93"/>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B35" s="83">
         <v>31</v>
       </c>
@@ -4926,17 +4923,19 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="J20:J23"/>
+    <mergeCell ref="K20:K23"/>
+    <mergeCell ref="L20:L23"/>
+    <mergeCell ref="M20:M23"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4945,19 +4944,17 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="J20:J23"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="M20:M23"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4967,42 +4964,42 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD788E61-AC5A-4E7F-9536-02553AF94143}">
   <dimension ref="B1:P35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9" style="1"/>
-    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.7109375" customWidth="1"/>
-    <col min="13" max="13" width="90.28515625" customWidth="1"/>
+    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.73046875" customWidth="1"/>
+    <col min="13" max="13" width="90.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="248" t="s">
+    <row r="1" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="B2" s="226" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="249"/>
-      <c r="G2" s="250"/>
-      <c r="H2" s="197" t="s">
+      <c r="C2" s="227"/>
+      <c r="D2" s="227"/>
+      <c r="E2" s="227"/>
+      <c r="F2" s="227"/>
+      <c r="G2" s="228"/>
+      <c r="H2" s="196" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="197" t="s">
+      <c r="I2" s="196" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="248" t="s">
+      <c r="J2" s="226" t="s">
         <v>43</v>
       </c>
-      <c r="K2" s="249"/>
-      <c r="L2" s="249"/>
-      <c r="M2" s="197" t="s">
+      <c r="K2" s="227"/>
+      <c r="L2" s="227"/>
+      <c r="M2" s="196" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
@@ -5021,8 +5018,8 @@
       <c r="G3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="198"/>
-      <c r="I3" s="198"/>
+      <c r="H3" s="197"/>
+      <c r="I3" s="197"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -5032,9 +5029,9 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="198"/>
-    </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="M3" s="197"/>
+    </row>
+    <row r="4" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
         <v>0</v>
       </c>
@@ -5077,7 +5074,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B5" s="82">
         <v>1</v>
       </c>
@@ -5101,7 +5098,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="228"/>
+      <c r="H5" s="230"/>
       <c r="I5" s="42" t="s">
         <v>3</v>
       </c>
@@ -5118,7 +5115,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B6" s="81">
         <v>2</v>
       </c>
@@ -5142,26 +5139,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="227" t="s">
+      <c r="H6" s="231" t="s">
         <v>61</v>
       </c>
       <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="231" t="s">
+      <c r="J6" s="232" t="s">
         <v>70</v>
       </c>
-      <c r="K6" s="240" t="s">
+      <c r="K6" s="234" t="s">
         <v>69</v>
       </c>
-      <c r="L6" s="237" t="s">
+      <c r="L6" s="236" t="s">
         <v>66</v>
       </c>
-      <c r="M6" s="245" t="s">
+      <c r="M6" s="238" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B7" s="81">
         <v>3</v>
       </c>
@@ -5185,14 +5182,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="227"/>
-      <c r="I7" s="251"/>
-      <c r="J7" s="231"/>
-      <c r="K7" s="240"/>
-      <c r="L7" s="237"/>
-      <c r="M7" s="245"/>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H7" s="231"/>
+      <c r="I7" s="250"/>
+      <c r="J7" s="232"/>
+      <c r="K7" s="234"/>
+      <c r="L7" s="236"/>
+      <c r="M7" s="238"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B8" s="81">
         <v>4</v>
       </c>
@@ -5216,14 +5213,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="227"/>
-      <c r="I8" s="264"/>
-      <c r="J8" s="231"/>
-      <c r="K8" s="240"/>
-      <c r="L8" s="237"/>
-      <c r="M8" s="245"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H8" s="231"/>
+      <c r="I8" s="251"/>
+      <c r="J8" s="232"/>
+      <c r="K8" s="234"/>
+      <c r="L8" s="236"/>
+      <c r="M8" s="238"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B9" s="81">
         <v>5</v>
       </c>
@@ -5247,14 +5244,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="227"/>
-      <c r="I9" s="265"/>
-      <c r="J9" s="231"/>
-      <c r="K9" s="240"/>
-      <c r="L9" s="237"/>
-      <c r="M9" s="245"/>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H9" s="231"/>
+      <c r="I9" s="252"/>
+      <c r="J9" s="232"/>
+      <c r="K9" s="234"/>
+      <c r="L9" s="236"/>
+      <c r="M9" s="238"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B10" s="81">
         <v>6</v>
       </c>
@@ -5278,16 +5275,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="227"/>
+      <c r="H10" s="231"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="231"/>
-      <c r="K10" s="240"/>
-      <c r="L10" s="237"/>
-      <c r="M10" s="245"/>
-    </row>
-    <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J10" s="232"/>
+      <c r="K10" s="234"/>
+      <c r="L10" s="236"/>
+      <c r="M10" s="238"/>
+    </row>
+    <row r="11" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="82">
         <v>7</v>
       </c>
@@ -5311,14 +5308,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="228"/>
+      <c r="H11" s="230"/>
       <c r="I11" s="104"/>
-      <c r="J11" s="232"/>
-      <c r="K11" s="241"/>
-      <c r="L11" s="238"/>
-      <c r="M11" s="246"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="J11" s="233"/>
+      <c r="K11" s="235"/>
+      <c r="L11" s="237"/>
+      <c r="M11" s="239"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B12" s="80">
         <v>8</v>
       </c>
@@ -5348,20 +5345,20 @@
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="230" t="s">
+      <c r="J12" s="240" t="s">
         <v>70</v>
       </c>
-      <c r="K12" s="239" t="s">
+      <c r="K12" s="241" t="s">
         <v>69</v>
       </c>
-      <c r="L12" s="236" t="s">
+      <c r="L12" s="242" t="s">
         <v>66</v>
       </c>
-      <c r="M12" s="247" t="s">
+      <c r="M12" s="243" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B13" s="81">
         <v>9</v>
       </c>
@@ -5385,14 +5382,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="227"/>
-      <c r="I13" s="251"/>
-      <c r="J13" s="231"/>
-      <c r="K13" s="240"/>
-      <c r="L13" s="237"/>
-      <c r="M13" s="245"/>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H13" s="231"/>
+      <c r="I13" s="250"/>
+      <c r="J13" s="232"/>
+      <c r="K13" s="234"/>
+      <c r="L13" s="236"/>
+      <c r="M13" s="238"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B14" s="81">
         <v>10</v>
       </c>
@@ -5416,14 +5413,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="227"/>
-      <c r="I14" s="264"/>
-      <c r="J14" s="231"/>
-      <c r="K14" s="240"/>
-      <c r="L14" s="237"/>
-      <c r="M14" s="245"/>
-    </row>
-    <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H14" s="231"/>
+      <c r="I14" s="251"/>
+      <c r="J14" s="232"/>
+      <c r="K14" s="234"/>
+      <c r="L14" s="236"/>
+      <c r="M14" s="238"/>
+    </row>
+    <row r="15" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="82">
         <v>11</v>
       </c>
@@ -5447,14 +5444,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="228"/>
-      <c r="I15" s="252"/>
-      <c r="J15" s="232"/>
-      <c r="K15" s="241"/>
-      <c r="L15" s="238"/>
-      <c r="M15" s="246"/>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="H15" s="230"/>
+      <c r="I15" s="253"/>
+      <c r="J15" s="233"/>
+      <c r="K15" s="235"/>
+      <c r="L15" s="237"/>
+      <c r="M15" s="239"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B16" s="80">
         <v>12</v>
       </c>
@@ -5484,20 +5481,20 @@
       <c r="I16" s="64" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="230" t="s">
+      <c r="J16" s="240" t="s">
         <v>65</v>
       </c>
-      <c r="K16" s="233" t="s">
+      <c r="K16" s="247" t="s">
         <v>64</v>
       </c>
-      <c r="L16" s="236" t="s">
+      <c r="L16" s="242" t="s">
         <v>66</v>
       </c>
       <c r="M16" s="75" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B17" s="81">
         <v>13</v>
       </c>
@@ -5521,18 +5518,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="227"/>
+      <c r="H17" s="231"/>
       <c r="I17" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="J17" s="231"/>
-      <c r="K17" s="234"/>
-      <c r="L17" s="237"/>
+      <c r="J17" s="232"/>
+      <c r="K17" s="248"/>
+      <c r="L17" s="236"/>
       <c r="M17" s="74" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B18" s="81">
         <v>14</v>
       </c>
@@ -5556,14 +5553,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="227"/>
-      <c r="I18" s="251"/>
-      <c r="J18" s="231"/>
-      <c r="K18" s="234"/>
-      <c r="L18" s="237"/>
-      <c r="M18" s="251"/>
-    </row>
-    <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H18" s="231"/>
+      <c r="I18" s="250"/>
+      <c r="J18" s="232"/>
+      <c r="K18" s="248"/>
+      <c r="L18" s="236"/>
+      <c r="M18" s="250"/>
+    </row>
+    <row r="19" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="82">
         <v>15</v>
       </c>
@@ -5587,15 +5584,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="228"/>
-      <c r="I19" s="252"/>
-      <c r="J19" s="232"/>
-      <c r="K19" s="235"/>
-      <c r="L19" s="238"/>
-      <c r="M19" s="252"/>
+      <c r="H19" s="230"/>
+      <c r="I19" s="253"/>
+      <c r="J19" s="233"/>
+      <c r="K19" s="249"/>
+      <c r="L19" s="237"/>
+      <c r="M19" s="253"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B20" s="80">
         <v>16</v>
       </c>
@@ -5619,10 +5616,10 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="253" t="s">
+      <c r="H20" s="254" t="s">
         <v>179</v>
       </c>
-      <c r="I20" s="178" t="s">
+      <c r="I20" s="177" t="s">
         <v>119</v>
       </c>
       <c r="J20" s="66" t="s">
@@ -5631,14 +5628,14 @@
       <c r="K20" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="L20" s="168" t="s">
+      <c r="L20" s="167" t="s">
         <v>66</v>
       </c>
-      <c r="M20" s="177" t="s">
+      <c r="M20" s="176" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B21" s="81">
         <v>17</v>
       </c>
@@ -5662,14 +5659,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="254"/>
-      <c r="I21" s="169"/>
-      <c r="J21" s="171"/>
-      <c r="K21" s="173"/>
-      <c r="L21" s="175"/>
-      <c r="M21" s="169"/>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H21" s="255"/>
+      <c r="I21" s="168"/>
+      <c r="J21" s="170"/>
+      <c r="K21" s="172"/>
+      <c r="L21" s="174"/>
+      <c r="M21" s="168"/>
+    </row>
+    <row r="22" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B22" s="81">
         <v>18</v>
       </c>
@@ -5693,14 +5690,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="254"/>
-      <c r="I22" s="169"/>
-      <c r="J22" s="171"/>
-      <c r="K22" s="173"/>
-      <c r="L22" s="175"/>
-      <c r="M22" s="169"/>
-    </row>
-    <row r="23" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H22" s="255"/>
+      <c r="I22" s="168"/>
+      <c r="J22" s="170"/>
+      <c r="K22" s="172"/>
+      <c r="L22" s="174"/>
+      <c r="M22" s="168"/>
+    </row>
+    <row r="23" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B23" s="81">
         <v>19</v>
       </c>
@@ -5724,14 +5721,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="255"/>
-      <c r="I23" s="170"/>
-      <c r="J23" s="172"/>
-      <c r="K23" s="174"/>
-      <c r="L23" s="176"/>
-      <c r="M23" s="170"/>
-    </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H23" s="256"/>
+      <c r="I23" s="169"/>
+      <c r="J23" s="171"/>
+      <c r="K23" s="173"/>
+      <c r="L23" s="175"/>
+      <c r="M23" s="169"/>
+    </row>
+    <row r="24" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B24" s="80">
         <v>20</v>
       </c>
@@ -5774,7 +5771,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B25" s="81">
         <v>21</v>
       </c>
@@ -5798,7 +5795,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="227"/>
+      <c r="H25" s="231"/>
       <c r="I25" s="70" t="s">
         <v>46</v>
       </c>
@@ -5815,7 +5812,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B26" s="81">
         <v>22</v>
       </c>
@@ -5839,14 +5836,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="227"/>
-      <c r="I26" s="251"/>
-      <c r="J26" s="256"/>
-      <c r="K26" s="258"/>
-      <c r="L26" s="260"/>
-      <c r="M26" s="262"/>
-    </row>
-    <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="H26" s="231"/>
+      <c r="I26" s="250"/>
+      <c r="J26" s="257"/>
+      <c r="K26" s="259"/>
+      <c r="L26" s="261"/>
+      <c r="M26" s="263"/>
+    </row>
+    <row r="27" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B27" s="82">
         <v>23</v>
       </c>
@@ -5870,14 +5867,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="228"/>
-      <c r="I27" s="252"/>
-      <c r="J27" s="257"/>
-      <c r="K27" s="259"/>
-      <c r="L27" s="261"/>
-      <c r="M27" s="263"/>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="H27" s="230"/>
+      <c r="I27" s="253"/>
+      <c r="J27" s="258"/>
+      <c r="K27" s="260"/>
+      <c r="L27" s="262"/>
+      <c r="M27" s="264"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B28" s="80">
         <v>24</v>
       </c>
@@ -5920,7 +5917,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B29" s="81">
         <v>25</v>
       </c>
@@ -5944,7 +5941,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="227"/>
+      <c r="H29" s="231"/>
       <c r="I29" s="70" t="s">
         <v>52</v>
       </c>
@@ -5961,7 +5958,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B30" s="81">
         <v>26</v>
       </c>
@@ -5985,7 +5982,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="227"/>
+      <c r="H30" s="231"/>
       <c r="I30" s="70" t="s">
         <v>53</v>
       </c>
@@ -6002,7 +5999,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B31" s="82">
         <v>27</v>
       </c>
@@ -6026,14 +6023,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="228"/>
+      <c r="H31" s="230"/>
       <c r="I31" s="91"/>
-      <c r="J31" s="164"/>
-      <c r="K31" s="165"/>
-      <c r="L31" s="166"/>
+      <c r="J31" s="163"/>
+      <c r="K31" s="164"/>
+      <c r="L31" s="165"/>
       <c r="M31" s="93"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B32" s="81">
         <v>28</v>
       </c>
@@ -6057,7 +6054,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="227" t="s">
+      <c r="H32" s="231" t="s">
         <v>168</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -6077,7 +6074,7 @@
       </c>
       <c r="P32" s="1"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B33" s="81">
         <v>29</v>
       </c>
@@ -6101,7 +6098,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="227"/>
+      <c r="H33" s="231"/>
       <c r="I33" s="70" t="s">
         <v>52</v>
       </c>
@@ -6119,7 +6116,7 @@
       </c>
       <c r="P33" s="1"/>
     </row>
-    <row r="34" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B34" s="81">
         <v>30</v>
       </c>
@@ -6143,7 +6140,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="228"/>
+      <c r="H34" s="230"/>
       <c r="I34" s="70" t="s">
         <v>53</v>
       </c>
@@ -6161,7 +6158,7 @@
       </c>
       <c r="P34" s="1"/>
     </row>
-    <row r="35" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B35" s="83">
         <v>31</v>
       </c>
@@ -6197,7 +6194,7 @@
       <c r="K35" s="55" t="s">
         <v>64</v>
       </c>
-      <c r="L35" s="167" t="s">
+      <c r="L35" s="166" t="s">
         <v>178</v>
       </c>
       <c r="M35" s="46" t="s">
@@ -6206,24 +6203,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6239,6 +6218,24 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6248,24 +6245,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4182B34D-1176-43D9-83DE-D8E7EA5C96ED}">
   <dimension ref="B1:F11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="5" width="4.7109375" customWidth="1"/>
+    <col min="3" max="5" width="4.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="248" t="s">
+    <row r="1" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
+      <c r="B2" s="226" t="s">
         <v>72</v>
       </c>
-      <c r="C2" s="249"/>
-      <c r="D2" s="249"/>
-      <c r="E2" s="250"/>
-      <c r="F2" s="197" t="s">
+      <c r="C2" s="227"/>
+      <c r="D2" s="227"/>
+      <c r="E2" s="228"/>
+      <c r="F2" s="196" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
@@ -6278,9 +6275,9 @@
       <c r="E3" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="198"/>
-    </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F3" s="197"/>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B4" s="13">
         <v>0</v>
       </c>
@@ -6300,7 +6297,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -6320,7 +6317,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -6340,7 +6337,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -6360,7 +6357,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -6380,7 +6377,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -6400,7 +6397,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -6420,7 +6417,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -6452,37 +6449,37 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{197DCCAF-E75B-41F9-A939-BF94359E828F}">
   <dimension ref="B1:R9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="14.28515625" customWidth="1"/>
+    <col min="2" max="2" width="14.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="197" t="s">
+    <row r="1" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:18" x14ac:dyDescent="0.45">
+      <c r="B2" s="196" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="275" t="s">
+      <c r="C2" s="274" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="276"/>
-      <c r="E2" s="276"/>
-      <c r="F2" s="276"/>
-      <c r="G2" s="276"/>
-      <c r="H2" s="276"/>
-      <c r="I2" s="276"/>
-      <c r="J2" s="276"/>
-      <c r="K2" s="276"/>
-      <c r="L2" s="276"/>
-      <c r="M2" s="276"/>
-      <c r="N2" s="276"/>
-      <c r="O2" s="276"/>
-      <c r="P2" s="276"/>
-      <c r="Q2" s="276"/>
-      <c r="R2" s="277"/>
-    </row>
-    <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="198"/>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="276"/>
+    </row>
+    <row r="3" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="197"/>
       <c r="C3" s="117">
         <v>15</v>
       </c>
@@ -6532,18 +6529,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="87" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="153"/>
-      <c r="D4" s="153"/>
-      <c r="E4" s="153"/>
-      <c r="F4" s="153"/>
-      <c r="G4" s="153"/>
-      <c r="H4" s="153"/>
-      <c r="I4" s="153"/>
-      <c r="J4" s="153"/>
+      <c r="C4" s="152"/>
+      <c r="D4" s="152"/>
+      <c r="E4" s="152"/>
+      <c r="F4" s="152"/>
+      <c r="G4" s="152"/>
+      <c r="H4" s="152"/>
+      <c r="I4" s="152"/>
+      <c r="J4" s="152"/>
       <c r="K4" s="68" t="s">
         <v>86</v>
       </c>
@@ -6553,107 +6550,107 @@
       <c r="M4" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="N4" s="269" t="s">
+      <c r="N4" s="268" t="s">
         <v>89</v>
       </c>
-      <c r="O4" s="269"/>
-      <c r="P4" s="269"/>
-      <c r="Q4" s="269"/>
-      <c r="R4" s="270"/>
-    </row>
-    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O4" s="268"/>
+      <c r="P4" s="268"/>
+      <c r="Q4" s="268"/>
+      <c r="R4" s="269"/>
+    </row>
+    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="154"/>
-      <c r="D5" s="155"/>
-      <c r="E5" s="155"/>
-      <c r="F5" s="155"/>
-      <c r="G5" s="155"/>
-      <c r="H5" s="155"/>
-      <c r="I5" s="155"/>
-      <c r="J5" s="156"/>
-      <c r="K5" s="271" t="s">
+      <c r="C5" s="153"/>
+      <c r="D5" s="154"/>
+      <c r="E5" s="154"/>
+      <c r="F5" s="154"/>
+      <c r="G5" s="154"/>
+      <c r="H5" s="154"/>
+      <c r="I5" s="154"/>
+      <c r="J5" s="155"/>
+      <c r="K5" s="270" t="s">
         <v>85</v>
       </c>
-      <c r="L5" s="267"/>
-      <c r="M5" s="267"/>
-      <c r="N5" s="267"/>
-      <c r="O5" s="267"/>
-      <c r="P5" s="267"/>
-      <c r="Q5" s="267"/>
-      <c r="R5" s="268"/>
-    </row>
-    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L5" s="266"/>
+      <c r="M5" s="266"/>
+      <c r="N5" s="266"/>
+      <c r="O5" s="266"/>
+      <c r="P5" s="266"/>
+      <c r="Q5" s="266"/>
+      <c r="R5" s="267"/>
+    </row>
+    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="154"/>
-      <c r="D6" s="155"/>
-      <c r="E6" s="155"/>
-      <c r="F6" s="155"/>
-      <c r="G6" s="155"/>
-      <c r="H6" s="155"/>
-      <c r="I6" s="155"/>
-      <c r="J6" s="156"/>
-      <c r="K6" s="271" t="s">
+      <c r="C6" s="153"/>
+      <c r="D6" s="154"/>
+      <c r="E6" s="154"/>
+      <c r="F6" s="154"/>
+      <c r="G6" s="154"/>
+      <c r="H6" s="154"/>
+      <c r="I6" s="154"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="270" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="267"/>
-      <c r="M6" s="267"/>
-      <c r="N6" s="267"/>
-      <c r="O6" s="267"/>
-      <c r="P6" s="267"/>
-      <c r="Q6" s="267"/>
-      <c r="R6" s="268"/>
-    </row>
-    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="266"/>
+      <c r="M6" s="266"/>
+      <c r="N6" s="266"/>
+      <c r="O6" s="266"/>
+      <c r="P6" s="266"/>
+      <c r="Q6" s="266"/>
+      <c r="R6" s="267"/>
+    </row>
+    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="88" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="157"/>
-      <c r="D7" s="157"/>
-      <c r="E7" s="157"/>
-      <c r="F7" s="157"/>
-      <c r="G7" s="157"/>
-      <c r="H7" s="157"/>
-      <c r="I7" s="157"/>
-      <c r="J7" s="157"/>
-      <c r="K7" s="272" t="s">
+      <c r="C7" s="156"/>
+      <c r="D7" s="156"/>
+      <c r="E7" s="156"/>
+      <c r="F7" s="156"/>
+      <c r="G7" s="156"/>
+      <c r="H7" s="156"/>
+      <c r="I7" s="156"/>
+      <c r="J7" s="156"/>
+      <c r="K7" s="271" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="273"/>
-      <c r="M7" s="273"/>
-      <c r="N7" s="273"/>
-      <c r="O7" s="273"/>
-      <c r="P7" s="273"/>
-      <c r="Q7" s="273"/>
-      <c r="R7" s="274"/>
-    </row>
-    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L7" s="272"/>
+      <c r="M7" s="272"/>
+      <c r="N7" s="272"/>
+      <c r="O7" s="272"/>
+      <c r="P7" s="272"/>
+      <c r="Q7" s="272"/>
+      <c r="R7" s="273"/>
+    </row>
+    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88" t="s">
         <v>84</v>
       </c>
-      <c r="C8" s="266" t="s">
+      <c r="C8" s="265" t="s">
         <v>150</v>
       </c>
-      <c r="D8" s="267"/>
-      <c r="E8" s="267"/>
-      <c r="F8" s="267"/>
-      <c r="G8" s="267"/>
-      <c r="H8" s="267"/>
-      <c r="I8" s="267"/>
-      <c r="J8" s="267"/>
-      <c r="K8" s="267"/>
-      <c r="L8" s="267"/>
-      <c r="M8" s="267"/>
-      <c r="N8" s="267"/>
-      <c r="O8" s="267"/>
-      <c r="P8" s="267"/>
-      <c r="Q8" s="267"/>
-      <c r="R8" s="268"/>
-    </row>
-    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="266"/>
+      <c r="E8" s="266"/>
+      <c r="F8" s="266"/>
+      <c r="G8" s="266"/>
+      <c r="H8" s="266"/>
+      <c r="I8" s="266"/>
+      <c r="J8" s="266"/>
+      <c r="K8" s="266"/>
+      <c r="L8" s="266"/>
+      <c r="M8" s="266"/>
+      <c r="N8" s="266"/>
+      <c r="O8" s="266"/>
+      <c r="P8" s="266"/>
+      <c r="Q8" s="266"/>
+      <c r="R8" s="267"/>
+    </row>
+    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9" s="89" t="s">
         <v>90</v>
       </c>
@@ -6670,13 +6667,13 @@
       <c r="M9" s="8"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
-      <c r="P9" s="151" t="s">
+      <c r="P9" s="150" t="s">
         <v>88</v>
       </c>
-      <c r="Q9" s="151" t="s">
+      <c r="Q9" s="150" t="s">
         <v>92</v>
       </c>
-      <c r="R9" s="152" t="s">
+      <c r="R9" s="151" t="s">
         <v>91</v>
       </c>
     </row>
@@ -6698,84 +6695,84 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
   <dimension ref="B1:D17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
-    <col min="3" max="3" width="82.28515625" customWidth="1"/>
+    <col min="2" max="2" width="21.1328125" customWidth="1"/>
+    <col min="3" max="3" width="82.265625" customWidth="1"/>
     <col min="4" max="4" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="158" t="s">
+    <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="157" t="s">
         <v>152</v>
       </c>
-      <c r="C2" s="160" t="s">
+      <c r="C2" s="159" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B3" s="159" t="s">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B3" s="158" t="s">
         <v>118</v>
       </c>
       <c r="C3" s="38" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="161" t="s">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B4" s="160" t="s">
         <v>119</v>
       </c>
       <c r="C4" s="74" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="159" t="s">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B5" s="158" t="s">
         <v>125</v>
       </c>
       <c r="C5" s="41" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="161" t="s">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B6" s="160" t="s">
         <v>120</v>
       </c>
       <c r="C6" s="74" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="159" t="s">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B7" s="158" t="s">
         <v>121</v>
       </c>
       <c r="C7" s="41" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="162" t="s">
+    <row r="8" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B8" s="161" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="163" t="s">
+      <c r="C8" s="162" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="158" t="s">
+    <row r="10" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="11" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B11" s="157" t="s">
         <v>152</v>
       </c>
-      <c r="C11" s="160" t="s">
+      <c r="C11" s="159" t="s">
         <v>153</v>
       </c>
-      <c r="D11" s="160" t="s">
+      <c r="D11" s="159" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="161" t="s">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B12" s="160" t="s">
         <v>156</v>
       </c>
       <c r="C12" s="74" t="s">
@@ -6785,8 +6782,8 @@
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="159" t="s">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B13" s="158" t="s">
         <v>158</v>
       </c>
       <c r="C13" s="41" t="s">
@@ -6796,8 +6793,8 @@
         <v>172</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B14" s="161" t="s">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B14" s="160" t="s">
         <v>160</v>
       </c>
       <c r="C14" s="74" t="s">
@@ -6807,8 +6804,8 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B15" s="161" t="s">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B15" s="160" t="s">
         <v>121</v>
       </c>
       <c r="C15" s="74" t="s">
@@ -6818,8 +6815,8 @@
         <v>176</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="159" t="s">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B16" s="158" t="s">
         <v>169</v>
       </c>
       <c r="C16" s="41" t="s">
@@ -6829,14 +6826,14 @@
         <v>177</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="162" t="s">
+    <row r="17" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B17" s="161" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="163" t="s">
+      <c r="C17" s="162" t="s">
         <v>162</v>
       </c>
-      <c r="D17" s="163" t="s">
+      <c r="D17" s="162" t="s">
         <v>174</v>
       </c>
     </row>
@@ -6848,101 +6845,101 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D036B2-790A-4A3D-BD75-883CE886D2D8}">
   <dimension ref="B1:E12"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="7.28515625" customWidth="1"/>
+    <col min="4" max="4" width="7.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="278" t="s">
+    <row r="1" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B2" s="277" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="279"/>
+      <c r="C2" s="278"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="141" t="s">
+    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="140" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="148" t="s">
+      <c r="C3" s="147" t="s">
         <v>140</v>
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B4" s="92"/>
       <c r="C4" s="131" t="s">
         <v>143</v>
       </c>
-      <c r="D4" s="280" t="s">
+      <c r="D4" s="279" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B5" s="94"/>
       <c r="C5" s="132" t="s">
         <v>142</v>
       </c>
-      <c r="D5" s="281"/>
-    </row>
-    <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="280"/>
+    </row>
+    <row r="6" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="134"/>
       <c r="C6" s="63" t="s">
         <v>144</v>
       </c>
-      <c r="D6" s="282"/>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="142" t="s">
+      <c r="D6" s="281"/>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B7" s="141" t="s">
         <v>143</v>
       </c>
-      <c r="C7" s="143"/>
-      <c r="D7" s="283" t="s">
+      <c r="C7" s="142"/>
+      <c r="D7" s="282" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B8" s="40" t="s">
         <v>142</v>
       </c>
-      <c r="C8" s="144"/>
-      <c r="D8" s="284"/>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C8" s="143"/>
+      <c r="D8" s="283"/>
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="C9" s="144"/>
-      <c r="D9" s="284"/>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="145" t="s">
+      <c r="C9" s="143"/>
+      <c r="D9" s="283"/>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B10" s="144" t="s">
         <v>145</v>
       </c>
-      <c r="C10" s="146" t="s">
+      <c r="C10" s="145" t="s">
         <v>145</v>
       </c>
-      <c r="D10" s="284"/>
-    </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="D10" s="283"/>
+    </row>
+    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" s="40" t="s">
         <v>142</v>
       </c>
       <c r="C11" s="132" t="s">
         <v>142</v>
       </c>
-      <c r="D11" s="284"/>
+      <c r="D11" s="283"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="147" t="s">
+    <row r="12" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B12" s="146" t="s">
         <v>146</v>
       </c>
       <c r="C12" s="63" t="s">
         <v>146</v>
       </c>
-      <c r="D12" s="285"/>
+      <c r="D12" s="284"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6957,108 +6954,108 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{728A29D2-349C-45CC-BF5A-2F605D047162}">
   <dimension ref="B1:D40"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="3" max="4" width="38.5703125" customWidth="1"/>
+    <col min="3" max="4" width="38.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="286" t="s">
+    <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B2" s="285" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="288" t="s">
+      <c r="C2" s="287" t="s">
         <v>194</v>
       </c>
-      <c r="D2" s="289"/>
-    </row>
-    <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="287"/>
-      <c r="C3" s="187" t="s">
+      <c r="D2" s="288"/>
+    </row>
+    <row r="3" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="286"/>
+      <c r="C3" s="186" t="s">
         <v>191</v>
       </c>
-      <c r="D3" s="188" t="s">
+      <c r="D3" s="187" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="88">
         <v>0</v>
       </c>
-      <c r="C4" s="145" t="s">
+      <c r="C4" s="144" t="s">
         <v>199</v>
       </c>
-      <c r="D4" s="236" t="s">
+      <c r="D4" s="242" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="179">
-        <v>1</v>
-      </c>
-      <c r="C5" s="192" t="s">
+    <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="178">
+        <v>1</v>
+      </c>
+      <c r="C5" s="191" t="s">
         <v>200</v>
       </c>
-      <c r="D5" s="290"/>
-    </row>
-    <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D5" s="289"/>
+    </row>
+    <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88">
         <v>2</v>
       </c>
-      <c r="C6" s="292" t="s">
+      <c r="C6" s="291" t="s">
         <v>196</v>
       </c>
-      <c r="D6" s="291" t="s">
+      <c r="D6" s="290" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="179">
+    <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B7" s="178">
         <v>3</v>
       </c>
-      <c r="C7" s="231"/>
-      <c r="D7" s="237"/>
-    </row>
-    <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="232"/>
+      <c r="D7" s="236"/>
+    </row>
+    <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88">
         <v>4</v>
       </c>
-      <c r="C8" s="293"/>
-      <c r="D8" s="290"/>
-    </row>
-    <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="179">
+      <c r="C8" s="292"/>
+      <c r="D8" s="289"/>
+    </row>
+    <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B9" s="178">
         <v>5</v>
       </c>
       <c r="C9" s="94"/>
-      <c r="D9" s="181"/>
-    </row>
-    <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D9" s="180"/>
+    </row>
+    <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B10" s="88">
         <v>6</v>
       </c>
       <c r="C10" s="137"/>
-      <c r="D10" s="144"/>
-    </row>
-    <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="180">
+      <c r="D10" s="143"/>
+    </row>
+    <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B11" s="179">
         <v>7</v>
       </c>
       <c r="C11" s="134"/>
-      <c r="D11" s="182" t="s">
+      <c r="D11" s="181" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="189" t="s">
+    <row r="13" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B14" s="188" t="s">
         <v>197</v>
       </c>
-      <c r="C14" s="190" t="s">
+      <c r="C14" s="189" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B15" s="88">
         <v>0</v>
       </c>
@@ -7066,15 +7063,15 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="179">
-        <v>1</v>
-      </c>
-      <c r="C16" s="183" t="s">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B16" s="178">
+        <v>1</v>
+      </c>
+      <c r="C16" s="182" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B17" s="88">
         <v>2</v>
       </c>
@@ -7082,15 +7079,15 @@
         <v>198</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B18" s="179">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B18" s="178">
         <v>3</v>
       </c>
-      <c r="C18" s="183" t="s">
+      <c r="C18" s="182" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B19" s="88">
         <v>4</v>
       </c>
@@ -7098,39 +7095,39 @@
         <v>184</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B20" s="179">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B20" s="178">
         <v>5</v>
       </c>
-      <c r="C20" s="183"/>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="182"/>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B21" s="88">
         <v>6</v>
       </c>
       <c r="C21" s="26"/>
     </row>
-    <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="180">
+    <row r="22" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B22" s="179">
         <v>7</v>
       </c>
-      <c r="C22" s="186"/>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="185"/>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="189" t="s">
+    <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B25" s="188" t="s">
         <v>197</v>
       </c>
-      <c r="C25" s="190" t="s">
+      <c r="C25" s="189" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B26" s="88">
         <v>0</v>
       </c>
@@ -7138,15 +7135,15 @@
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="179">
-        <v>1</v>
-      </c>
-      <c r="C27" s="183" t="s">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B27" s="178">
+        <v>1</v>
+      </c>
+      <c r="C27" s="182" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B28" s="88">
         <v>2</v>
       </c>
@@ -7154,24 +7151,24 @@
         <v>188</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="184">
+    <row r="29" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B29" s="183">
         <v>3</v>
       </c>
-      <c r="C29" s="185" t="s">
+      <c r="C29" s="184" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="189" t="s">
+    <row r="31" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B32" s="188" t="s">
         <v>197</v>
       </c>
-      <c r="C32" s="190" t="s">
+      <c r="C32" s="189" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B33" s="88">
         <v>0</v>
       </c>
@@ -7179,15 +7176,15 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B34" s="179">
-        <v>1</v>
-      </c>
-      <c r="C34" s="183" t="s">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B34" s="178">
+        <v>1</v>
+      </c>
+      <c r="C34" s="182" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B35" s="88">
         <v>2</v>
       </c>
@@ -7195,15 +7192,15 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B36" s="179">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B36" s="178">
         <v>3</v>
       </c>
-      <c r="C36" s="183" t="s">
+      <c r="C36" s="182" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B37" s="88">
         <v>4</v>
       </c>
@@ -7211,27 +7208,27 @@
         <v>169</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B38" s="179">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.45">
+      <c r="B38" s="178">
         <v>5</v>
       </c>
-      <c r="C38" s="183" t="s">
+      <c r="C38" s="182" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.45">
       <c r="B39" s="91">
         <v>6</v>
       </c>
-      <c r="C39" s="191" t="s">
+      <c r="C39" s="190" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="184">
+    <row r="40" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B40" s="183">
         <v>7</v>
       </c>
-      <c r="C40" s="185" t="s">
+      <c r="C40" s="184" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>

<commit_message>
ax08main decode and logic unit
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DD1E13-A5AE-4982-9FF9-4F0B30EF15F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E806F4-3C87-440B-B95E-7D6765473EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="2" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="191">
   <si>
     <t>MODE B</t>
   </si>
@@ -97,27 +97,9 @@
     <t>value</t>
   </si>
   <si>
-    <t>BIT GET</t>
-  </si>
-  <si>
-    <t>bit</t>
-  </si>
-  <si>
-    <t>BIT SET</t>
-  </si>
-  <si>
-    <t>BIT CLEAR</t>
-  </si>
-  <si>
-    <t>BIT TOGGLE</t>
-  </si>
-  <si>
     <t>BREAK</t>
   </si>
   <si>
-    <t>JUMP</t>
-  </si>
-  <si>
     <t>immediate value [0:7]</t>
   </si>
   <si>
@@ -211,9 +193,6 @@
     <t>SHIFT</t>
   </si>
   <si>
-    <t>BITWISE</t>
-  </si>
-  <si>
     <t>MEMORY</t>
   </si>
   <si>
@@ -323,18 +302,6 @@
   </si>
   <si>
     <t>CONDITION [0:2]</t>
-  </si>
-  <si>
-    <t>Returns 1 if the given bit of the given value is set otherwise 0. Also 0 if bit ∉ [0..7].</t>
-  </si>
-  <si>
-    <t>Takes the given value, sets the given bit to 1 and return the result. If bit ∉ [0..7] value is returned.</t>
-  </si>
-  <si>
-    <t>Takes the given value, clears the given bit to 0 and returns the result. If bit ∉ [0..7] value is returned.</t>
-  </si>
-  <si>
-    <t>Takes the given value, flips the given bit and returns the result. If bit ∉ [0..7] value is returned.</t>
   </si>
   <si>
     <t>A + B + C_in</t>
@@ -380,30 +347,12 @@
     <t>Writes the value to the output</t>
   </si>
   <si>
-    <t>FETCH</t>
-  </si>
-  <si>
     <t>DECODE</t>
   </si>
   <si>
-    <t>EXECUTE</t>
-  </si>
-  <si>
     <t>INCREMENT</t>
   </si>
   <si>
-    <t>Load next instruction at PC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Set A Immediate value / A address, B immediate value / B address, C address, output address, </t>
-  </si>
-  <si>
-    <t>Increment PC &amp; Buffer Output</t>
-  </si>
-  <si>
-    <t>CONDITION</t>
-  </si>
-  <si>
     <t>R0</t>
   </si>
   <si>
@@ -479,21 +428,12 @@
     <t>value [0..15]</t>
   </si>
   <si>
-    <t>Evaluates the condition</t>
-  </si>
-  <si>
     <t>STEP</t>
   </si>
   <si>
     <t>Description</t>
   </si>
   <si>
-    <t>Set OPCODE If condition is met</t>
-  </si>
-  <si>
-    <t>Write output to selected register if condition is met</t>
-  </si>
-  <si>
     <t>FREEZE WORD</t>
   </si>
   <si>
@@ -524,9 +464,6 @@
     <t>Writes the value to the UART unit.</t>
   </si>
   <si>
-    <t>Updates PC</t>
-  </si>
-  <si>
     <t>IO_0</t>
   </si>
   <si>
@@ -563,9 +500,6 @@
     <t>OVERRIDDEN</t>
   </si>
   <si>
-    <t>"""BITWISE"""</t>
-  </si>
-  <si>
     <t>Decodes Bit 0 - Bit 2 of input, upper bits unused.</t>
   </si>
   <si>
@@ -645,6 +579,46 @@
   </si>
   <si>
     <t xml:space="preserve">Bits 0..7 of the Stack Pointer </t>
+  </si>
+  <si>
+    <t>NDECODE</t>
+  </si>
+  <si>
+    <t>LOAD 2</t>
+  </si>
+  <si>
+    <t>Decodes Bit 0 - Bit 2 of input, upper bits unused. Output is active low</t>
+  </si>
+  <si>
+    <t>Decodes Bit 0 - Bit 2 of input, upper bits unused. Output is active high</t>
+  </si>
+  <si>
+    <t>Increments PC</t>
+  </si>
+  <si>
+    <t>Writes the combined 16bit value to the selected special function register</t>
+  </si>
+  <si>
+    <t>Writes the value to the selected output register</t>
+  </si>
+  <si>
+    <t>Performs the given arithmetic operation and returns the result. C_in is the state of the carry flag.
+The state of the carry flag is updated after the calculation</t>
+  </si>
+  <si>
+    <t>Stores the given value at the given memory address</t>
+  </si>
+  <si>
+    <t>Returns 1 if a new value is available from UART unit, otherwise returns 0</t>
+  </si>
+  <si>
+    <t>Copies the value from the UART unit and returns it</t>
+  </si>
+  <si>
+    <t>Writes the value to the UART unit</t>
+  </si>
+  <si>
+    <t>Causes the computer to enter a breakpoint</t>
   </si>
 </sst>
 </file>
@@ -748,7 +722,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="69">
+  <borders count="71">
     <border>
       <left/>
       <right/>
@@ -1600,11 +1574,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="292">
+  <cellXfs count="302">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2127,6 +2129,9 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2151,6 +2156,45 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2187,44 +2231,68 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2235,76 +2303,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2343,6 +2342,12 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2425,6 +2430,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2776,20 +2808,20 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B2" s="192" t="s">
+      <c r="B2" s="193" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="193"/>
-      <c r="D2" s="193"/>
-      <c r="E2" s="193"/>
-      <c r="F2" s="194"/>
-      <c r="G2" s="197" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="198"/>
-      <c r="I2" s="199"/>
-      <c r="J2" s="195" t="s">
-        <v>31</v>
+      <c r="C2" s="194"/>
+      <c r="D2" s="194"/>
+      <c r="E2" s="194"/>
+      <c r="F2" s="195"/>
+      <c r="G2" s="198" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="199"/>
+      <c r="I2" s="200"/>
+      <c r="J2" s="196" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -2797,27 +2829,27 @@
         <v>16</v>
       </c>
       <c r="C3" s="51" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E3" s="49" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F3" s="50" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H3" s="52" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="I3" s="50" t="s">
-        <v>131</v>
-      </c>
-      <c r="J3" s="196"/>
+        <v>114</v>
+      </c>
+      <c r="J3" s="197"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B4" s="105">
@@ -2840,16 +2872,16 @@
         <v>0</v>
       </c>
       <c r="G4" s="117" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="H4" s="123" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="I4" s="108" t="s">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="J4" s="106" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.45">
@@ -2873,16 +2905,16 @@
         <v>1</v>
       </c>
       <c r="G5" s="118" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="H5" s="124" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="I5" s="109" t="s">
-        <v>120</v>
+        <v>103</v>
       </c>
       <c r="J5" s="26" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.45">
@@ -2906,16 +2938,16 @@
         <v>0</v>
       </c>
       <c r="G6" s="119" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="H6" s="125" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="I6" s="110" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="J6" s="28" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.45">
@@ -2939,16 +2971,16 @@
         <v>1</v>
       </c>
       <c r="G7" s="120" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="H7" s="126" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="I7" s="111" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="J7" s="30" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.45">
@@ -2972,16 +3004,16 @@
         <v>0</v>
       </c>
       <c r="G8" s="118" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="H8" s="124" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="I8" s="109" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="J8" s="26" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="2:10" x14ac:dyDescent="0.45">
@@ -3005,16 +3037,16 @@
         <v>1</v>
       </c>
       <c r="G9" s="118" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="H9" s="124" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="I9" s="109" t="s">
-        <v>124</v>
+        <v>107</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.45">
@@ -3038,16 +3070,16 @@
         <v>0</v>
       </c>
       <c r="G10" s="119" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="H10" s="125" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="I10" s="110" t="s">
-        <v>125</v>
+        <v>108</v>
       </c>
       <c r="J10" s="28" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="2:10" x14ac:dyDescent="0.45">
@@ -3071,16 +3103,16 @@
         <v>1</v>
       </c>
       <c r="G11" s="120" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="H11" s="126" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="I11" s="111" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="J11" s="30" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.45">
@@ -3104,14 +3136,14 @@
         <v>0</v>
       </c>
       <c r="G12" s="119" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="H12" s="147" t="s">
-        <v>140</v>
+        <v>123</v>
       </c>
       <c r="I12" s="114"/>
       <c r="J12" s="28" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="2:10" x14ac:dyDescent="0.45">
@@ -3135,12 +3167,12 @@
         <v>1</v>
       </c>
       <c r="G13" s="118" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="H13" s="148"/>
       <c r="I13" s="113"/>
       <c r="J13" s="26" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.45">
@@ -3165,7 +3197,7 @@
       </c>
       <c r="G14" s="121"/>
       <c r="H14" s="147" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="I14" s="114"/>
       <c r="J14" s="31"/>
@@ -3191,12 +3223,12 @@
         <v>1</v>
       </c>
       <c r="G15" s="120" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="H15" s="148"/>
       <c r="I15" s="112"/>
       <c r="J15" s="30" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="2:10" x14ac:dyDescent="0.45">
@@ -3220,14 +3252,14 @@
         <v>0</v>
       </c>
       <c r="G16" s="118" t="s">
-        <v>195</v>
+        <v>173</v>
       </c>
       <c r="H16" s="191" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="I16" s="113"/>
       <c r="J16" s="26" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.45">
@@ -3251,12 +3283,12 @@
         <v>1</v>
       </c>
       <c r="G17" s="118" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="H17" s="128"/>
       <c r="I17" s="113"/>
       <c r="J17" s="26" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.45">
@@ -3428,73 +3460,73 @@
       </c>
     </row>
     <row r="3" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C3" s="209" t="s">
+      <c r="C3" s="223" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="210"/>
-      <c r="E3" s="210"/>
-      <c r="F3" s="210"/>
-      <c r="G3" s="211"/>
-      <c r="H3" s="206" t="s">
-        <v>92</v>
-      </c>
-      <c r="I3" s="207"/>
-      <c r="J3" s="208"/>
-      <c r="K3" s="206" t="s">
-        <v>91</v>
-      </c>
-      <c r="L3" s="207"/>
-      <c r="M3" s="207"/>
-      <c r="N3" s="218" t="s">
-        <v>90</v>
-      </c>
-      <c r="O3" s="219"/>
-      <c r="P3" s="220"/>
+      <c r="D3" s="224"/>
+      <c r="E3" s="224"/>
+      <c r="F3" s="224"/>
+      <c r="G3" s="225"/>
+      <c r="H3" s="220" t="s">
+        <v>85</v>
+      </c>
+      <c r="I3" s="221"/>
+      <c r="J3" s="222"/>
+      <c r="K3" s="220" t="s">
+        <v>84</v>
+      </c>
+      <c r="L3" s="221"/>
+      <c r="M3" s="221"/>
+      <c r="N3" s="207" t="s">
+        <v>83</v>
+      </c>
+      <c r="O3" s="208"/>
+      <c r="P3" s="209"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="212" t="s">
-        <v>26</v>
-      </c>
-      <c r="T3" s="213"/>
-      <c r="U3" s="213"/>
-      <c r="V3" s="213"/>
-      <c r="W3" s="213"/>
-      <c r="X3" s="213"/>
-      <c r="Y3" s="213"/>
-      <c r="Z3" s="214"/>
-      <c r="AA3" s="215" t="s">
-        <v>27</v>
-      </c>
-      <c r="AB3" s="216"/>
-      <c r="AC3" s="216"/>
-      <c r="AD3" s="216"/>
-      <c r="AE3" s="216"/>
-      <c r="AF3" s="216"/>
-      <c r="AG3" s="216"/>
-      <c r="AH3" s="217"/>
+      <c r="S3" s="201" t="s">
+        <v>20</v>
+      </c>
+      <c r="T3" s="202"/>
+      <c r="U3" s="202"/>
+      <c r="V3" s="202"/>
+      <c r="W3" s="202"/>
+      <c r="X3" s="202"/>
+      <c r="Y3" s="202"/>
+      <c r="Z3" s="203"/>
+      <c r="AA3" s="204" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB3" s="205"/>
+      <c r="AC3" s="205"/>
+      <c r="AD3" s="205"/>
+      <c r="AE3" s="205"/>
+      <c r="AF3" s="205"/>
+      <c r="AG3" s="205"/>
+      <c r="AH3" s="206"/>
     </row>
     <row r="4" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="5" spans="2:34" x14ac:dyDescent="0.45">
-      <c r="B5" s="223" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="221" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="221"/>
-      <c r="E5" s="221"/>
-      <c r="F5" s="221"/>
-      <c r="G5" s="221"/>
-      <c r="H5" s="221"/>
-      <c r="I5" s="221"/>
-      <c r="J5" s="222"/>
+      <c r="B5" s="212" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="210" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="210"/>
+      <c r="E5" s="210"/>
+      <c r="F5" s="210"/>
+      <c r="G5" s="210"/>
+      <c r="H5" s="210"/>
+      <c r="I5" s="210"/>
+      <c r="J5" s="211"/>
     </row>
     <row r="6" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="224"/>
+      <c r="B6" s="213"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3524,16 +3556,16 @@
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="200" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="201"/>
-      <c r="E7" s="201"/>
-      <c r="F7" s="201"/>
-      <c r="G7" s="201"/>
-      <c r="H7" s="201"/>
-      <c r="I7" s="201"/>
-      <c r="J7" s="202"/>
+      <c r="C7" s="214" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="215"/>
+      <c r="E7" s="215"/>
+      <c r="F7" s="215"/>
+      <c r="G7" s="215"/>
+      <c r="H7" s="215"/>
+      <c r="I7" s="215"/>
+      <c r="J7" s="216"/>
     </row>
     <row r="8" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="6">
@@ -3543,25 +3575,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="203" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8" s="204"/>
-      <c r="I8" s="204"/>
-      <c r="J8" s="205"/>
+      <c r="G8" s="217" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="218"/>
+      <c r="I8" s="218"/>
+      <c r="J8" s="219"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="C3:G3"/>
     <mergeCell ref="S3:Z3"/>
     <mergeCell ref="AA3:AH3"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="C5:J5"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3584,30 +3616,30 @@
   <sheetData>
     <row r="1" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B2" s="225" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="226"/>
-      <c r="D2" s="226"/>
-      <c r="E2" s="226"/>
-      <c r="F2" s="226"/>
-      <c r="G2" s="227"/>
-      <c r="H2" s="195" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="195" t="s">
+      <c r="B2" s="247" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="248"/>
+      <c r="D2" s="248"/>
+      <c r="E2" s="248"/>
+      <c r="F2" s="248"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="196" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="196" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="225" t="s">
-        <v>41</v>
-      </c>
-      <c r="K2" s="226"/>
-      <c r="L2" s="226"/>
-      <c r="M2" s="195" t="s">
-        <v>105</v>
-      </c>
-      <c r="N2" s="195" t="s">
-        <v>31</v>
+      <c r="J2" s="247" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="248"/>
+      <c r="L2" s="248"/>
+      <c r="M2" s="196" t="s">
+        <v>94</v>
+      </c>
+      <c r="N2" s="196" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -3615,22 +3647,22 @@
         <v>16</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" s="49" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G3" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="196"/>
-      <c r="I3" s="196"/>
+        <v>26</v>
+      </c>
+      <c r="H3" s="197"/>
+      <c r="I3" s="197"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -3640,8 +3672,8 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="196"/>
-      <c r="N3" s="196"/>
+      <c r="M3" s="197"/>
+      <c r="N3" s="197"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
@@ -3668,25 +3700,25 @@
         <v>0</v>
       </c>
       <c r="H4" s="228" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" s="66" t="s">
-        <v>80</v>
-      </c>
-      <c r="K4" s="66" t="s">
-        <v>108</v>
-      </c>
-      <c r="L4" s="69" t="s">
-        <v>42</v>
+        <v>179</v>
+      </c>
+      <c r="J4" s="300" t="s">
+        <v>73</v>
+      </c>
+      <c r="K4" s="301" t="s">
+        <v>97</v>
+      </c>
+      <c r="L4" s="235" t="s">
+        <v>16</v>
       </c>
       <c r="M4" s="69" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N4" s="75" t="s">
-        <v>109</v>
+        <v>183</v>
       </c>
     </row>
     <row r="5" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -3713,24 +3745,22 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="229"/>
+      <c r="H5" s="227"/>
       <c r="I5" s="42" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="J5" s="62" t="s">
         <v>16</v>
       </c>
       <c r="K5" s="54" t="s">
-        <v>60</v>
-      </c>
-      <c r="L5" s="63" t="s">
-        <v>62</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="L5" s="237"/>
       <c r="M5" s="34" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>110</v>
+        <v>184</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.45">
@@ -3757,26 +3787,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="230" t="s">
-        <v>57</v>
+      <c r="H6" s="226" t="s">
+        <v>50</v>
       </c>
       <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="231" t="s">
-        <v>65</v>
-      </c>
-      <c r="K6" s="233" t="s">
-        <v>64</v>
-      </c>
-      <c r="L6" s="235" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" s="243" t="s">
-        <v>106</v>
-      </c>
-      <c r="N6" s="237" t="s">
-        <v>66</v>
+      <c r="J6" s="230" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="239" t="s">
+        <v>57</v>
+      </c>
+      <c r="L6" s="236" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="241" t="s">
+        <v>95</v>
+      </c>
+      <c r="N6" s="244" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="2:14" x14ac:dyDescent="0.45">
@@ -3803,15 +3833,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="230"/>
+      <c r="H7" s="226"/>
       <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="231"/>
-      <c r="K7" s="233"/>
-      <c r="L7" s="235"/>
-      <c r="M7" s="244"/>
-      <c r="N7" s="237"/>
+      <c r="J7" s="230"/>
+      <c r="K7" s="239"/>
+      <c r="L7" s="236"/>
+      <c r="M7" s="242"/>
+      <c r="N7" s="244"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B8" s="81">
@@ -3837,15 +3867,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="230"/>
+      <c r="H8" s="226"/>
       <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="231"/>
-      <c r="K8" s="233"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="244"/>
-      <c r="N8" s="237"/>
+      <c r="J8" s="230"/>
+      <c r="K8" s="239"/>
+      <c r="L8" s="236"/>
+      <c r="M8" s="242"/>
+      <c r="N8" s="244"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B9" s="81">
@@ -3871,15 +3901,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="230"/>
+      <c r="H9" s="226"/>
       <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="231"/>
-      <c r="K9" s="233"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="244"/>
-      <c r="N9" s="237"/>
+      <c r="J9" s="230"/>
+      <c r="K9" s="239"/>
+      <c r="L9" s="236"/>
+      <c r="M9" s="242"/>
+      <c r="N9" s="244"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B10" s="81">
@@ -3905,15 +3935,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="230"/>
+      <c r="H10" s="226"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="231"/>
-      <c r="K10" s="233"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="244"/>
-      <c r="N10" s="237"/>
+      <c r="J10" s="230"/>
+      <c r="K10" s="239"/>
+      <c r="L10" s="236"/>
+      <c r="M10" s="242"/>
+      <c r="N10" s="244"/>
     </row>
     <row r="11" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="82">
@@ -3939,15 +3969,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="229"/>
+      <c r="H11" s="227"/>
       <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="232"/>
-      <c r="K11" s="234"/>
-      <c r="L11" s="236"/>
-      <c r="M11" s="245"/>
-      <c r="N11" s="238"/>
+      <c r="J11" s="231"/>
+      <c r="K11" s="240"/>
+      <c r="L11" s="237"/>
+      <c r="M11" s="243"/>
+      <c r="N11" s="245"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B12" s="80">
@@ -3974,25 +4004,25 @@
         <v>0</v>
       </c>
       <c r="H12" s="228" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="239" t="s">
-        <v>65</v>
-      </c>
-      <c r="K12" s="240" t="s">
-        <v>64</v>
-      </c>
-      <c r="L12" s="241" t="s">
-        <v>62</v>
+      <c r="J12" s="229" t="s">
+        <v>58</v>
+      </c>
+      <c r="K12" s="238" t="s">
+        <v>57</v>
+      </c>
+      <c r="L12" s="235" t="s">
+        <v>55</v>
       </c>
       <c r="M12" s="228" t="s">
-        <v>107</v>
-      </c>
-      <c r="N12" s="242" t="s">
-        <v>99</v>
+        <v>96</v>
+      </c>
+      <c r="N12" s="246" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.45">
@@ -4019,15 +4049,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="230"/>
+      <c r="H13" s="226"/>
       <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="231"/>
-      <c r="K13" s="233"/>
-      <c r="L13" s="235"/>
-      <c r="M13" s="230"/>
-      <c r="N13" s="237"/>
+      <c r="J13" s="230"/>
+      <c r="K13" s="239"/>
+      <c r="L13" s="236"/>
+      <c r="M13" s="226"/>
+      <c r="N13" s="244"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B14" s="81">
@@ -4053,15 +4083,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="230"/>
+      <c r="H14" s="226"/>
       <c r="I14" s="90" t="s">
-        <v>97</v>
-      </c>
-      <c r="J14" s="231"/>
-      <c r="K14" s="233"/>
-      <c r="L14" s="235"/>
-      <c r="M14" s="230"/>
-      <c r="N14" s="237"/>
+        <v>86</v>
+      </c>
+      <c r="J14" s="230"/>
+      <c r="K14" s="239"/>
+      <c r="L14" s="236"/>
+      <c r="M14" s="226"/>
+      <c r="N14" s="244"/>
     </row>
     <row r="15" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="82">
@@ -4087,15 +4117,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="229"/>
+      <c r="H15" s="227"/>
       <c r="I15" s="43" t="s">
-        <v>98</v>
-      </c>
-      <c r="J15" s="232"/>
-      <c r="K15" s="234"/>
-      <c r="L15" s="236"/>
-      <c r="M15" s="229"/>
-      <c r="N15" s="238"/>
+        <v>87</v>
+      </c>
+      <c r="J15" s="231"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="237"/>
+      <c r="M15" s="227"/>
+      <c r="N15" s="245"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B16" s="80">
@@ -4122,25 +4152,25 @@
         <v>0</v>
       </c>
       <c r="H16" s="228" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="J16" s="229" t="s">
         <v>54</v>
       </c>
-      <c r="I16" s="64" t="s">
-        <v>45</v>
-      </c>
-      <c r="J16" s="239" t="s">
-        <v>61</v>
-      </c>
-      <c r="K16" s="246" t="s">
-        <v>60</v>
-      </c>
-      <c r="L16" s="241" t="s">
-        <v>62</v>
+      <c r="K16" s="232" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="235" t="s">
+        <v>55</v>
       </c>
       <c r="M16" s="228" t="s">
-        <v>107</v>
+        <v>96</v>
       </c>
       <c r="N16" s="75" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.45">
@@ -4167,16 +4197,16 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="230"/>
+      <c r="H17" s="226"/>
       <c r="I17" s="70" t="s">
-        <v>46</v>
-      </c>
-      <c r="J17" s="231"/>
-      <c r="K17" s="247"/>
-      <c r="L17" s="235"/>
-      <c r="M17" s="230"/>
+        <v>40</v>
+      </c>
+      <c r="J17" s="230"/>
+      <c r="K17" s="233"/>
+      <c r="L17" s="236"/>
+      <c r="M17" s="226"/>
       <c r="N17" s="74" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="2:17" x14ac:dyDescent="0.45">
@@ -4203,16 +4233,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="230"/>
+      <c r="H18" s="226"/>
       <c r="I18" s="70" t="s">
-        <v>47</v>
-      </c>
-      <c r="J18" s="231"/>
-      <c r="K18" s="247"/>
-      <c r="L18" s="235"/>
-      <c r="M18" s="230"/>
+        <v>41</v>
+      </c>
+      <c r="J18" s="230"/>
+      <c r="K18" s="233"/>
+      <c r="L18" s="236"/>
+      <c r="M18" s="226"/>
       <c r="N18" s="74" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -4239,16 +4269,16 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="229"/>
+      <c r="H19" s="227"/>
       <c r="I19" s="43" t="s">
-        <v>48</v>
-      </c>
-      <c r="J19" s="232"/>
-      <c r="K19" s="248"/>
-      <c r="L19" s="236"/>
-      <c r="M19" s="229"/>
+        <v>42</v>
+      </c>
+      <c r="J19" s="231"/>
+      <c r="K19" s="234"/>
+      <c r="L19" s="237"/>
+      <c r="M19" s="227"/>
       <c r="N19" s="44" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="P19" s="1"/>
     </row>
@@ -4277,25 +4307,25 @@
         <v>0</v>
       </c>
       <c r="H20" s="228" t="s">
+        <v>100</v>
+      </c>
+      <c r="I20" s="192" t="s">
+        <v>178</v>
+      </c>
+      <c r="J20" s="140" t="s">
+        <v>152</v>
+      </c>
+      <c r="K20" s="232" t="s">
+        <v>53</v>
+      </c>
+      <c r="L20" s="296" t="s">
         <v>55</v>
       </c>
-      <c r="I20" s="64" t="s">
-        <v>17</v>
-      </c>
-      <c r="J20" s="239" t="s">
-        <v>16</v>
-      </c>
-      <c r="K20" s="240" t="s">
-        <v>18</v>
-      </c>
-      <c r="L20" s="241" t="s">
-        <v>62</v>
-      </c>
-      <c r="M20" s="243" t="s">
-        <v>106</v>
-      </c>
-      <c r="N20" s="41" t="s">
-        <v>93</v>
+      <c r="M20" s="241" t="s">
+        <v>95</v>
+      </c>
+      <c r="N20" s="298" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.45">
@@ -4322,16 +4352,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="230"/>
-      <c r="I21" s="70" t="s">
-        <v>19</v>
-      </c>
-      <c r="J21" s="231"/>
-      <c r="K21" s="233"/>
-      <c r="L21" s="235"/>
-      <c r="M21" s="244"/>
-      <c r="N21" s="74" t="s">
-        <v>94</v>
+      <c r="H21" s="226"/>
+      <c r="I21" s="293" t="s">
+        <v>100</v>
+      </c>
+      <c r="J21" s="99" t="s">
+        <v>152</v>
+      </c>
+      <c r="K21" s="295"/>
+      <c r="L21" s="297"/>
+      <c r="M21" s="294"/>
+      <c r="N21" s="299" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.45">
@@ -4358,17 +4390,13 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="230"/>
-      <c r="I22" s="70" t="s">
-        <v>20</v>
-      </c>
-      <c r="J22" s="231"/>
-      <c r="K22" s="233"/>
-      <c r="L22" s="235"/>
-      <c r="M22" s="244"/>
-      <c r="N22" s="74" t="s">
-        <v>95</v>
-      </c>
+      <c r="H22" s="226"/>
+      <c r="I22" s="103"/>
+      <c r="J22" s="136"/>
+      <c r="K22" s="137"/>
+      <c r="L22" s="138"/>
+      <c r="M22" s="104"/>
+      <c r="N22" s="104"/>
     </row>
     <row r="23" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B23" s="81">
@@ -4394,17 +4422,13 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="229"/>
-      <c r="I23" s="42" t="s">
-        <v>21</v>
-      </c>
-      <c r="J23" s="232"/>
-      <c r="K23" s="234"/>
-      <c r="L23" s="236"/>
-      <c r="M23" s="245"/>
-      <c r="N23" s="41" t="s">
-        <v>96</v>
-      </c>
+      <c r="H23" s="227"/>
+      <c r="I23" s="96"/>
+      <c r="J23" s="133"/>
+      <c r="K23" s="134"/>
+      <c r="L23" s="135"/>
+      <c r="M23" s="132"/>
+      <c r="N23" s="132"/>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.45">
       <c r="B24" s="80">
@@ -4431,25 +4455,25 @@
         <v>0</v>
       </c>
       <c r="H24" s="228" t="s">
+        <v>49</v>
+      </c>
+      <c r="I24" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="J24" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="I24" s="64" t="s">
-        <v>43</v>
-      </c>
-      <c r="J24" s="66" t="s">
-        <v>63</v>
-      </c>
       <c r="K24" s="65" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L24" s="67" t="s">
         <v>16</v>
       </c>
       <c r="M24" s="101" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N24" s="75" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.45">
@@ -4476,24 +4500,24 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="230"/>
+      <c r="H25" s="226"/>
       <c r="I25" s="70" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J25" s="99" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K25" s="102" t="s">
         <v>16</v>
       </c>
       <c r="L25" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M25" s="98" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N25" s="74" t="s">
-        <v>89</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.45">
@@ -4520,7 +4544,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="230"/>
+      <c r="H26" s="226"/>
       <c r="I26" s="103"/>
       <c r="J26" s="136"/>
       <c r="K26" s="137"/>
@@ -4552,7 +4576,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="229"/>
+      <c r="H27" s="227"/>
       <c r="I27" s="96"/>
       <c r="J27" s="133"/>
       <c r="K27" s="134"/>
@@ -4585,25 +4609,25 @@
         <v>0</v>
       </c>
       <c r="H28" s="228" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="J28" s="33" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K28" s="53" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L28" s="39" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="M28" s="97" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N28" s="38" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.45">
@@ -4630,24 +4654,24 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="230"/>
+      <c r="H29" s="226"/>
       <c r="I29" s="70" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J29" s="71" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K29" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L29" s="73" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="M29" s="98" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N29" s="74" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.45">
@@ -4674,24 +4698,24 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="230"/>
+      <c r="H30" s="226"/>
       <c r="I30" s="70" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J30" s="99" t="s">
         <v>16</v>
       </c>
       <c r="K30" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L30" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M30" s="98" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N30" s="74" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -4718,7 +4742,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="229"/>
+      <c r="H31" s="227"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -4750,26 +4774,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="230" t="s">
-        <v>161</v>
+      <c r="H32" s="226" t="s">
+        <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="J32" s="33" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K32" s="53" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L32" s="39" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="M32" s="69" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N32" s="38" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="Q32" s="1"/>
     </row>
@@ -4797,24 +4821,24 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="230"/>
+      <c r="H33" s="226"/>
       <c r="I33" s="70" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J33" s="71" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K33" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L33" s="73" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="M33" s="100" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N33" s="74" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
       <c r="Q33" s="1"/>
     </row>
@@ -4842,24 +4866,24 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="229"/>
+      <c r="H34" s="227"/>
       <c r="I34" s="70" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J34" s="99" t="s">
         <v>16</v>
       </c>
       <c r="K34" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L34" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M34" s="100" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N34" s="74" t="s">
-        <v>158</v>
+        <v>189</v>
       </c>
       <c r="Q34" s="1"/>
     </row>
@@ -4888,42 +4912,41 @@
         <v>1</v>
       </c>
       <c r="H35" s="45" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I35" s="45" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J35" s="47" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K35" s="55" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L35" s="32" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M35" s="32" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="N35" s="46" t="s">
-        <v>104</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="J20:J23"/>
-    <mergeCell ref="K20:K23"/>
-    <mergeCell ref="L20:L23"/>
-    <mergeCell ref="M20:M23"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="L4:L5"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4932,17 +4955,18 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="M20:M21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4964,27 +4988,27 @@
   <sheetData>
     <row r="1" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B2" s="225" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="226"/>
-      <c r="D2" s="226"/>
-      <c r="E2" s="226"/>
-      <c r="F2" s="226"/>
-      <c r="G2" s="227"/>
-      <c r="H2" s="195" t="s">
-        <v>52</v>
-      </c>
-      <c r="I2" s="195" t="s">
+      <c r="B2" s="247" t="s">
+        <v>33</v>
+      </c>
+      <c r="C2" s="248"/>
+      <c r="D2" s="248"/>
+      <c r="E2" s="248"/>
+      <c r="F2" s="248"/>
+      <c r="G2" s="249"/>
+      <c r="H2" s="196" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="196" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="225" t="s">
-        <v>41</v>
-      </c>
-      <c r="K2" s="226"/>
-      <c r="L2" s="226"/>
-      <c r="M2" s="195" t="s">
-        <v>31</v>
+      <c r="J2" s="247" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="248"/>
+      <c r="L2" s="248"/>
+      <c r="M2" s="196" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -4992,22 +5016,22 @@
         <v>16</v>
       </c>
       <c r="C3" s="49" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" s="49" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="F3" s="49" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G3" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="196"/>
-      <c r="I3" s="196"/>
+        <v>26</v>
+      </c>
+      <c r="H3" s="197"/>
+      <c r="I3" s="197"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -5017,7 +5041,7 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="196"/>
+      <c r="M3" s="197"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
@@ -5044,22 +5068,22 @@
         <v>0</v>
       </c>
       <c r="H4" s="228" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>23</v>
+        <v>179</v>
       </c>
       <c r="J4" s="66" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="K4" s="68" t="s">
-        <v>108</v>
+        <v>97</v>
       </c>
       <c r="L4" s="66" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="M4" s="75" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -5086,21 +5110,21 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="229"/>
+      <c r="H5" s="227"/>
       <c r="I5" s="42" t="s">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="J5" s="62" t="s">
         <v>16</v>
       </c>
       <c r="K5" s="54" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L5" s="63" t="s">
         <v>16</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.45">
@@ -5127,23 +5151,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="230" t="s">
-        <v>57</v>
+      <c r="H6" s="226" t="s">
+        <v>50</v>
       </c>
       <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="231" t="s">
-        <v>65</v>
-      </c>
-      <c r="K6" s="233" t="s">
-        <v>64</v>
-      </c>
-      <c r="L6" s="235" t="s">
-        <v>62</v>
-      </c>
-      <c r="M6" s="237" t="s">
-        <v>66</v>
+      <c r="J6" s="230" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" s="239" t="s">
+        <v>57</v>
+      </c>
+      <c r="L6" s="236" t="s">
+        <v>55</v>
+      </c>
+      <c r="M6" s="244" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.45">
@@ -5170,12 +5194,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="230"/>
-      <c r="I7" s="249"/>
-      <c r="J7" s="231"/>
-      <c r="K7" s="233"/>
-      <c r="L7" s="235"/>
-      <c r="M7" s="237"/>
+      <c r="H7" s="226"/>
+      <c r="I7" s="250"/>
+      <c r="J7" s="230"/>
+      <c r="K7" s="239"/>
+      <c r="L7" s="236"/>
+      <c r="M7" s="244"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B8" s="81">
@@ -5201,12 +5225,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="230"/>
-      <c r="I8" s="250"/>
-      <c r="J8" s="231"/>
-      <c r="K8" s="233"/>
-      <c r="L8" s="235"/>
-      <c r="M8" s="237"/>
+      <c r="H8" s="226"/>
+      <c r="I8" s="263"/>
+      <c r="J8" s="230"/>
+      <c r="K8" s="239"/>
+      <c r="L8" s="236"/>
+      <c r="M8" s="244"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B9" s="81">
@@ -5232,12 +5256,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="230"/>
-      <c r="I9" s="251"/>
-      <c r="J9" s="231"/>
-      <c r="K9" s="233"/>
-      <c r="L9" s="235"/>
-      <c r="M9" s="237"/>
+      <c r="H9" s="226"/>
+      <c r="I9" s="264"/>
+      <c r="J9" s="230"/>
+      <c r="K9" s="239"/>
+      <c r="L9" s="236"/>
+      <c r="M9" s="244"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B10" s="81">
@@ -5263,14 +5287,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="230"/>
+      <c r="H10" s="226"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="231"/>
-      <c r="K10" s="233"/>
-      <c r="L10" s="235"/>
-      <c r="M10" s="237"/>
+      <c r="J10" s="230"/>
+      <c r="K10" s="239"/>
+      <c r="L10" s="236"/>
+      <c r="M10" s="244"/>
     </row>
     <row r="11" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B11" s="82">
@@ -5296,12 +5320,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="229"/>
+      <c r="H11" s="227"/>
       <c r="I11" s="103"/>
-      <c r="J11" s="232"/>
-      <c r="K11" s="234"/>
-      <c r="L11" s="236"/>
-      <c r="M11" s="238"/>
+      <c r="J11" s="231"/>
+      <c r="K11" s="240"/>
+      <c r="L11" s="237"/>
+      <c r="M11" s="245"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B12" s="80">
@@ -5328,22 +5352,22 @@
         <v>0</v>
       </c>
       <c r="H12" s="228" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="239" t="s">
-        <v>65</v>
-      </c>
-      <c r="K12" s="240" t="s">
-        <v>64</v>
-      </c>
-      <c r="L12" s="241" t="s">
-        <v>62</v>
-      </c>
-      <c r="M12" s="242" t="s">
-        <v>99</v>
+      <c r="J12" s="229" t="s">
+        <v>58</v>
+      </c>
+      <c r="K12" s="238" t="s">
+        <v>57</v>
+      </c>
+      <c r="L12" s="235" t="s">
+        <v>55</v>
+      </c>
+      <c r="M12" s="246" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.45">
@@ -5370,12 +5394,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="230"/>
-      <c r="I13" s="249"/>
-      <c r="J13" s="231"/>
-      <c r="K13" s="233"/>
-      <c r="L13" s="235"/>
-      <c r="M13" s="237"/>
+      <c r="H13" s="226"/>
+      <c r="I13" s="250"/>
+      <c r="J13" s="230"/>
+      <c r="K13" s="239"/>
+      <c r="L13" s="236"/>
+      <c r="M13" s="244"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B14" s="81">
@@ -5401,12 +5425,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="230"/>
-      <c r="I14" s="250"/>
-      <c r="J14" s="231"/>
-      <c r="K14" s="233"/>
-      <c r="L14" s="235"/>
-      <c r="M14" s="237"/>
+      <c r="H14" s="226"/>
+      <c r="I14" s="263"/>
+      <c r="J14" s="230"/>
+      <c r="K14" s="239"/>
+      <c r="L14" s="236"/>
+      <c r="M14" s="244"/>
     </row>
     <row r="15" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B15" s="82">
@@ -5432,12 +5456,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="229"/>
-      <c r="I15" s="252"/>
-      <c r="J15" s="232"/>
-      <c r="K15" s="234"/>
-      <c r="L15" s="236"/>
-      <c r="M15" s="238"/>
+      <c r="H15" s="227"/>
+      <c r="I15" s="251"/>
+      <c r="J15" s="231"/>
+      <c r="K15" s="240"/>
+      <c r="L15" s="237"/>
+      <c r="M15" s="245"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B16" s="80">
@@ -5464,22 +5488,22 @@
         <v>0</v>
       </c>
       <c r="H16" s="228" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="64" t="s">
+        <v>39</v>
+      </c>
+      <c r="J16" s="229" t="s">
         <v>54</v>
       </c>
-      <c r="I16" s="64" t="s">
-        <v>45</v>
-      </c>
-      <c r="J16" s="239" t="s">
-        <v>61</v>
-      </c>
-      <c r="K16" s="246" t="s">
-        <v>60</v>
-      </c>
-      <c r="L16" s="241" t="s">
-        <v>62</v>
+      <c r="K16" s="232" t="s">
+        <v>53</v>
+      </c>
+      <c r="L16" s="235" t="s">
+        <v>55</v>
       </c>
       <c r="M16" s="75" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="2:16" x14ac:dyDescent="0.45">
@@ -5506,15 +5530,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="230"/>
+      <c r="H17" s="226"/>
       <c r="I17" s="70" t="s">
-        <v>46</v>
-      </c>
-      <c r="J17" s="231"/>
-      <c r="K17" s="247"/>
-      <c r="L17" s="235"/>
+        <v>40</v>
+      </c>
+      <c r="J17" s="230"/>
+      <c r="K17" s="233"/>
+      <c r="L17" s="236"/>
       <c r="M17" s="74" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="2:16" x14ac:dyDescent="0.45">
@@ -5541,12 +5565,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="230"/>
-      <c r="I18" s="249"/>
-      <c r="J18" s="231"/>
-      <c r="K18" s="247"/>
-      <c r="L18" s="235"/>
-      <c r="M18" s="249"/>
+      <c r="H18" s="226"/>
+      <c r="I18" s="250"/>
+      <c r="J18" s="230"/>
+      <c r="K18" s="233"/>
+      <c r="L18" s="236"/>
+      <c r="M18" s="250"/>
     </row>
     <row r="19" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="82">
@@ -5572,12 +5596,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="229"/>
-      <c r="I19" s="252"/>
-      <c r="J19" s="232"/>
-      <c r="K19" s="248"/>
-      <c r="L19" s="236"/>
-      <c r="M19" s="252"/>
+      <c r="H19" s="227"/>
+      <c r="I19" s="251"/>
+      <c r="J19" s="231"/>
+      <c r="K19" s="234"/>
+      <c r="L19" s="237"/>
+      <c r="M19" s="251"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.45">
@@ -5604,23 +5628,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="253" t="s">
-        <v>172</v>
+      <c r="H20" s="252" t="s">
+        <v>100</v>
       </c>
       <c r="I20" s="176" t="s">
-        <v>112</v>
+        <v>178</v>
       </c>
       <c r="J20" s="66" t="s">
-        <v>174</v>
+        <v>152</v>
       </c>
       <c r="K20" s="65" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L20" s="166" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="M20" s="175" t="s">
-        <v>173</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.45">
@@ -5647,7 +5671,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="254"/>
+      <c r="H21" s="253"/>
       <c r="I21" s="167"/>
       <c r="J21" s="169"/>
       <c r="K21" s="171"/>
@@ -5678,7 +5702,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="254"/>
+      <c r="H22" s="253"/>
       <c r="I22" s="167"/>
       <c r="J22" s="169"/>
       <c r="K22" s="171"/>
@@ -5709,7 +5733,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="255"/>
+      <c r="H23" s="254"/>
       <c r="I23" s="168"/>
       <c r="J23" s="170"/>
       <c r="K23" s="172"/>
@@ -5741,22 +5765,22 @@
         <v>0</v>
       </c>
       <c r="H24" s="228" t="s">
+        <v>49</v>
+      </c>
+      <c r="I24" s="64" t="s">
+        <v>37</v>
+      </c>
+      <c r="J24" s="66" t="s">
         <v>56</v>
       </c>
-      <c r="I24" s="64" t="s">
-        <v>43</v>
-      </c>
-      <c r="J24" s="66" t="s">
-        <v>63</v>
-      </c>
       <c r="K24" s="65" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L24" s="67" t="s">
         <v>16</v>
       </c>
       <c r="M24" s="75" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="2:16" x14ac:dyDescent="0.45">
@@ -5783,21 +5807,21 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="230"/>
+      <c r="H25" s="226"/>
       <c r="I25" s="70" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="J25" s="99" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="K25" s="102" t="s">
         <v>16</v>
       </c>
       <c r="L25" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M25" s="74" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.45">
@@ -5824,12 +5848,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="230"/>
-      <c r="I26" s="249"/>
-      <c r="J26" s="256"/>
-      <c r="K26" s="258"/>
-      <c r="L26" s="260"/>
-      <c r="M26" s="262"/>
+      <c r="H26" s="226"/>
+      <c r="I26" s="250"/>
+      <c r="J26" s="255"/>
+      <c r="K26" s="257"/>
+      <c r="L26" s="259"/>
+      <c r="M26" s="261"/>
     </row>
     <row r="27" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B27" s="82">
@@ -5855,12 +5879,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="229"/>
-      <c r="I27" s="252"/>
-      <c r="J27" s="257"/>
-      <c r="K27" s="259"/>
-      <c r="L27" s="261"/>
-      <c r="M27" s="263"/>
+      <c r="H27" s="227"/>
+      <c r="I27" s="251"/>
+      <c r="J27" s="256"/>
+      <c r="K27" s="258"/>
+      <c r="L27" s="260"/>
+      <c r="M27" s="262"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B28" s="80">
@@ -5887,22 +5911,22 @@
         <v>0</v>
       </c>
       <c r="H28" s="228" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="J28" s="33" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K28" s="53" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L28" s="39" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="M28" s="38" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
     </row>
     <row r="29" spans="2:16" x14ac:dyDescent="0.45">
@@ -5929,21 +5953,21 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="230"/>
+      <c r="H29" s="226"/>
       <c r="I29" s="70" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J29" s="71" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K29" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L29" s="73" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="M29" s="74" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" spans="2:16" x14ac:dyDescent="0.45">
@@ -5970,21 +5994,21 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="230"/>
+      <c r="H30" s="226"/>
       <c r="I30" s="70" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J30" s="99" t="s">
         <v>16</v>
       </c>
       <c r="K30" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L30" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M30" s="74" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
     </row>
     <row r="31" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -6011,7 +6035,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="229"/>
+      <c r="H31" s="227"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -6042,23 +6066,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="230" t="s">
-        <v>161</v>
+      <c r="H32" s="226" t="s">
+        <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="J32" s="33" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K32" s="53" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L32" s="39" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="M32" s="38" t="s">
-        <v>156</v>
+        <v>136</v>
       </c>
       <c r="P32" s="1"/>
     </row>
@@ -6086,21 +6110,21 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="230"/>
+      <c r="H33" s="226"/>
       <c r="I33" s="70" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J33" s="71" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K33" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L33" s="73" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="M33" s="74" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
       <c r="P33" s="1"/>
     </row>
@@ -6128,21 +6152,21 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="229"/>
+      <c r="H34" s="227"/>
       <c r="I34" s="70" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J34" s="99" t="s">
         <v>16</v>
       </c>
       <c r="K34" s="72" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L34" s="100" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="M34" s="74" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="P34" s="1"/>
     </row>
@@ -6171,26 +6195,44 @@
         <v>1</v>
       </c>
       <c r="H35" s="45" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I35" s="45" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="J35" s="47" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="K35" s="55" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="L35" s="165" t="s">
-        <v>171</v>
+        <v>150</v>
       </c>
       <c r="M35" s="46" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6206,24 +6248,6 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6240,14 +6264,14 @@
   <sheetData>
     <row r="1" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B2" s="225" t="s">
-        <v>67</v>
-      </c>
-      <c r="C2" s="226"/>
-      <c r="D2" s="226"/>
-      <c r="E2" s="227"/>
-      <c r="F2" s="195" t="s">
-        <v>30</v>
+      <c r="B2" s="247" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="248"/>
+      <c r="D2" s="248"/>
+      <c r="E2" s="249"/>
+      <c r="F2" s="196" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -6255,15 +6279,15 @@
         <v>16</v>
       </c>
       <c r="C3" s="51" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D3" s="49" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E3" s="50" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="196"/>
+        <v>26</v>
+      </c>
+      <c r="F3" s="197"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B4" s="13">
@@ -6282,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.45">
@@ -6302,7 +6326,7 @@
         <v>1</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="2:6" x14ac:dyDescent="0.45">
@@ -6322,7 +6346,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="27" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.45">
@@ -6342,7 +6366,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="29" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="2:6" x14ac:dyDescent="0.45">
@@ -6362,7 +6386,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="25" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:6" x14ac:dyDescent="0.45">
@@ -6382,7 +6406,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="25" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.45">
@@ -6402,7 +6426,7 @@
         <v>0</v>
       </c>
       <c r="F10" s="27" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.45">
@@ -6422,7 +6446,7 @@
         <v>1</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -6444,30 +6468,30 @@
   <sheetData>
     <row r="1" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.45">
-      <c r="B2" s="195" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="273" t="s">
-        <v>29</v>
-      </c>
-      <c r="D2" s="274"/>
-      <c r="E2" s="274"/>
-      <c r="F2" s="274"/>
-      <c r="G2" s="274"/>
-      <c r="H2" s="274"/>
-      <c r="I2" s="274"/>
-      <c r="J2" s="274"/>
-      <c r="K2" s="274"/>
-      <c r="L2" s="274"/>
-      <c r="M2" s="274"/>
-      <c r="N2" s="274"/>
-      <c r="O2" s="274"/>
-      <c r="P2" s="274"/>
-      <c r="Q2" s="274"/>
-      <c r="R2" s="275"/>
+      <c r="B2" s="196" t="s">
+        <v>69</v>
+      </c>
+      <c r="C2" s="274" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="275"/>
+      <c r="E2" s="275"/>
+      <c r="F2" s="275"/>
+      <c r="G2" s="275"/>
+      <c r="H2" s="275"/>
+      <c r="I2" s="275"/>
+      <c r="J2" s="275"/>
+      <c r="K2" s="275"/>
+      <c r="L2" s="275"/>
+      <c r="M2" s="275"/>
+      <c r="N2" s="275"/>
+      <c r="O2" s="275"/>
+      <c r="P2" s="275"/>
+      <c r="Q2" s="275"/>
+      <c r="R2" s="276"/>
     </row>
     <row r="3" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="196"/>
+      <c r="B3" s="197"/>
       <c r="C3" s="116">
         <v>15</v>
       </c>
@@ -6519,7 +6543,7 @@
     </row>
     <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B4" s="87" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C4" s="151"/>
       <c r="D4" s="151"/>
@@ -6530,21 +6554,21 @@
       <c r="I4" s="151"/>
       <c r="J4" s="151"/>
       <c r="K4" s="68" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="L4" s="68" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="M4" s="68" t="s">
-        <v>83</v>
-      </c>
-      <c r="N4" s="267" t="s">
-        <v>84</v>
-      </c>
-      <c r="O4" s="267"/>
-      <c r="P4" s="267"/>
-      <c r="Q4" s="267"/>
-      <c r="R4" s="268"/>
+        <v>76</v>
+      </c>
+      <c r="N4" s="268" t="s">
+        <v>77</v>
+      </c>
+      <c r="O4" s="268"/>
+      <c r="P4" s="268"/>
+      <c r="Q4" s="268"/>
+      <c r="R4" s="269"/>
     </row>
     <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="88" t="s">
@@ -6558,16 +6582,16 @@
       <c r="H5" s="153"/>
       <c r="I5" s="153"/>
       <c r="J5" s="154"/>
-      <c r="K5" s="269" t="s">
-        <v>80</v>
-      </c>
-      <c r="L5" s="265"/>
-      <c r="M5" s="265"/>
-      <c r="N5" s="265"/>
-      <c r="O5" s="265"/>
-      <c r="P5" s="265"/>
-      <c r="Q5" s="265"/>
-      <c r="R5" s="266"/>
+      <c r="K5" s="270" t="s">
+        <v>73</v>
+      </c>
+      <c r="L5" s="266"/>
+      <c r="M5" s="266"/>
+      <c r="N5" s="266"/>
+      <c r="O5" s="266"/>
+      <c r="P5" s="266"/>
+      <c r="Q5" s="266"/>
+      <c r="R5" s="267"/>
     </row>
     <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88" t="s">
@@ -6581,20 +6605,20 @@
       <c r="H6" s="153"/>
       <c r="I6" s="153"/>
       <c r="J6" s="154"/>
-      <c r="K6" s="269" t="s">
-        <v>80</v>
-      </c>
-      <c r="L6" s="265"/>
-      <c r="M6" s="265"/>
-      <c r="N6" s="265"/>
-      <c r="O6" s="265"/>
-      <c r="P6" s="265"/>
-      <c r="Q6" s="265"/>
-      <c r="R6" s="266"/>
+      <c r="K6" s="270" t="s">
+        <v>73</v>
+      </c>
+      <c r="L6" s="266"/>
+      <c r="M6" s="266"/>
+      <c r="N6" s="266"/>
+      <c r="O6" s="266"/>
+      <c r="P6" s="266"/>
+      <c r="Q6" s="266"/>
+      <c r="R6" s="267"/>
     </row>
     <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="88" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C7" s="155"/>
       <c r="D7" s="155"/>
@@ -6604,43 +6628,43 @@
       <c r="H7" s="155"/>
       <c r="I7" s="155"/>
       <c r="J7" s="155"/>
-      <c r="K7" s="270" t="s">
-        <v>80</v>
-      </c>
-      <c r="L7" s="271"/>
-      <c r="M7" s="271"/>
-      <c r="N7" s="271"/>
-      <c r="O7" s="271"/>
-      <c r="P7" s="271"/>
-      <c r="Q7" s="271"/>
-      <c r="R7" s="272"/>
+      <c r="K7" s="271" t="s">
+        <v>73</v>
+      </c>
+      <c r="L7" s="272"/>
+      <c r="M7" s="272"/>
+      <c r="N7" s="272"/>
+      <c r="O7" s="272"/>
+      <c r="P7" s="272"/>
+      <c r="Q7" s="272"/>
+      <c r="R7" s="273"/>
     </row>
     <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88" t="s">
-        <v>79</v>
-      </c>
-      <c r="C8" s="264" t="s">
-        <v>143</v>
-      </c>
-      <c r="D8" s="265"/>
-      <c r="E8" s="265"/>
-      <c r="F8" s="265"/>
-      <c r="G8" s="265"/>
-      <c r="H8" s="265"/>
-      <c r="I8" s="265"/>
-      <c r="J8" s="265"/>
-      <c r="K8" s="265"/>
-      <c r="L8" s="265"/>
-      <c r="M8" s="265"/>
-      <c r="N8" s="265"/>
-      <c r="O8" s="265"/>
-      <c r="P8" s="265"/>
-      <c r="Q8" s="265"/>
-      <c r="R8" s="266"/>
+        <v>72</v>
+      </c>
+      <c r="C8" s="265" t="s">
+        <v>126</v>
+      </c>
+      <c r="D8" s="266"/>
+      <c r="E8" s="266"/>
+      <c r="F8" s="266"/>
+      <c r="G8" s="266"/>
+      <c r="H8" s="266"/>
+      <c r="I8" s="266"/>
+      <c r="J8" s="266"/>
+      <c r="K8" s="266"/>
+      <c r="L8" s="266"/>
+      <c r="M8" s="266"/>
+      <c r="N8" s="266"/>
+      <c r="O8" s="266"/>
+      <c r="P8" s="266"/>
+      <c r="Q8" s="266"/>
+      <c r="R8" s="267"/>
     </row>
     <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9" s="89" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -6656,13 +6680,13 @@
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
       <c r="P9" s="149" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="Q9" s="149" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="R9" s="150" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -6682,7 +6706,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
-  <dimension ref="B1:D17"/>
+  <dimension ref="B1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="21.1328125" customWidth="1"/>
@@ -6691,138 +6715,81 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B2" s="156" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="158" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" s="158" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B3" s="159" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="74" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="74" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B4" s="157" t="s">
+        <v>131</v>
+      </c>
+      <c r="C4" s="41" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="41" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B5" s="159" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="74" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="74" t="s">
         <v>145</v>
-      </c>
-      <c r="C2" s="158" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B3" s="157" t="s">
-        <v>111</v>
-      </c>
-      <c r="C3" s="38" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B4" s="159" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="74" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B5" s="157" t="s">
-        <v>118</v>
-      </c>
-      <c r="C5" s="41" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B6" s="159" t="s">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="C6" s="74" t="s">
-        <v>147</v>
+        <v>182</v>
+      </c>
+      <c r="D6" s="74" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.45">
       <c r="B7" s="157" t="s">
-        <v>114</v>
+        <v>141</v>
       </c>
       <c r="C7" s="41" t="s">
-        <v>117</v>
+        <v>142</v>
+      </c>
+      <c r="D7" s="41" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="160" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C8" s="161" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="11" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B11" s="156" t="s">
-        <v>145</v>
-      </c>
-      <c r="C11" s="158" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="161" t="s">
         <v>146</v>
-      </c>
-      <c r="D11" s="158" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B12" s="159" t="s">
-        <v>149</v>
-      </c>
-      <c r="C12" s="74" t="s">
-        <v>150</v>
-      </c>
-      <c r="D12" s="74" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B13" s="157" t="s">
-        <v>151</v>
-      </c>
-      <c r="C13" s="41" t="s">
-        <v>152</v>
-      </c>
-      <c r="D13" s="41" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B14" s="159" t="s">
-        <v>153</v>
-      </c>
-      <c r="C14" s="74" t="s">
-        <v>154</v>
-      </c>
-      <c r="D14" s="74" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B15" s="159" t="s">
-        <v>114</v>
-      </c>
-      <c r="C15" s="74" t="s">
-        <v>159</v>
-      </c>
-      <c r="D15" s="74" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B16" s="157" t="s">
-        <v>162</v>
-      </c>
-      <c r="C16" s="41" t="s">
-        <v>163</v>
-      </c>
-      <c r="D16" s="41" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B17" s="160" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="161" t="s">
-        <v>155</v>
-      </c>
-      <c r="D17" s="161" t="s">
-        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -6840,94 +6807,94 @@
   <sheetData>
     <row r="1" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="276" t="s">
-        <v>134</v>
-      </c>
-      <c r="C2" s="277"/>
+      <c r="B2" s="277" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="278"/>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="139" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="C3" s="146" t="s">
-        <v>133</v>
+        <v>116</v>
       </c>
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B4" s="92"/>
       <c r="C4" s="130" t="s">
-        <v>136</v>
-      </c>
-      <c r="D4" s="278" t="s">
-        <v>141</v>
+        <v>119</v>
+      </c>
+      <c r="D4" s="279" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B5" s="94"/>
       <c r="C5" s="131" t="s">
-        <v>135</v>
-      </c>
-      <c r="D5" s="279"/>
+        <v>118</v>
+      </c>
+      <c r="D5" s="280"/>
     </row>
     <row r="6" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="133"/>
       <c r="C6" s="63" t="s">
-        <v>137</v>
-      </c>
-      <c r="D6" s="280"/>
+        <v>120</v>
+      </c>
+      <c r="D6" s="281"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B7" s="140" t="s">
-        <v>136</v>
+        <v>119</v>
       </c>
       <c r="C7" s="141"/>
-      <c r="D7" s="281" t="s">
-        <v>142</v>
+      <c r="D7" s="282" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B8" s="40" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="C8" s="142"/>
-      <c r="D8" s="282"/>
+      <c r="D8" s="283"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" s="40" t="s">
-        <v>137</v>
+        <v>120</v>
       </c>
       <c r="C9" s="142"/>
-      <c r="D9" s="282"/>
+      <c r="D9" s="283"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" s="143" t="s">
-        <v>138</v>
+        <v>121</v>
       </c>
       <c r="C10" s="144" t="s">
-        <v>138</v>
-      </c>
-      <c r="D10" s="282"/>
+        <v>121</v>
+      </c>
+      <c r="D10" s="283"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" s="40" t="s">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="C11" s="131" t="s">
-        <v>135</v>
-      </c>
-      <c r="D11" s="282"/>
+        <v>118</v>
+      </c>
+      <c r="D11" s="283"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="145" t="s">
-        <v>139</v>
+        <v>122</v>
       </c>
       <c r="C12" s="63" t="s">
-        <v>139</v>
-      </c>
-      <c r="D12" s="283"/>
+        <v>122</v>
+      </c>
+      <c r="D12" s="284"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6949,21 +6916,21 @@
   <sheetData>
     <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B2" s="284" t="s">
-        <v>188</v>
-      </c>
-      <c r="C2" s="286" t="s">
-        <v>187</v>
-      </c>
-      <c r="D2" s="287"/>
+      <c r="B2" s="285" t="s">
+        <v>166</v>
+      </c>
+      <c r="C2" s="287" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="288"/>
     </row>
     <row r="3" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="285"/>
+      <c r="B3" s="286"/>
       <c r="C3" s="185" t="s">
-        <v>184</v>
+        <v>162</v>
       </c>
       <c r="D3" s="186" t="s">
-        <v>185</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -6971,10 +6938,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="143" t="s">
-        <v>192</v>
-      </c>
-      <c r="D4" s="241" t="s">
-        <v>182</v>
+        <v>170</v>
+      </c>
+      <c r="D4" s="235" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -6982,34 +6949,34 @@
         <v>1</v>
       </c>
       <c r="C5" s="190" t="s">
-        <v>193</v>
-      </c>
-      <c r="D5" s="288"/>
+        <v>171</v>
+      </c>
+      <c r="D5" s="289"/>
     </row>
     <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88">
         <v>2</v>
       </c>
-      <c r="C6" s="290" t="s">
-        <v>189</v>
-      </c>
-      <c r="D6" s="289" t="s">
-        <v>186</v>
+      <c r="C6" s="291" t="s">
+        <v>167</v>
+      </c>
+      <c r="D6" s="290" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="177">
         <v>3</v>
       </c>
-      <c r="C7" s="231"/>
-      <c r="D7" s="235"/>
+      <c r="C7" s="230"/>
+      <c r="D7" s="236"/>
     </row>
     <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88">
         <v>4</v>
       </c>
-      <c r="C8" s="291"/>
-      <c r="D8" s="288"/>
+      <c r="C8" s="292"/>
+      <c r="D8" s="289"/>
     </row>
     <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="177">
@@ -7031,16 +6998,16 @@
       </c>
       <c r="C11" s="133"/>
       <c r="D11" s="180" t="s">
-        <v>194</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B14" s="187" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="C14" s="188" t="s">
-        <v>189</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.45">
@@ -7048,7 +7015,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>175</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.45">
@@ -7056,7 +7023,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="181" t="s">
-        <v>178</v>
+        <v>156</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.45">
@@ -7064,7 +7031,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>191</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.45">
@@ -7072,7 +7039,7 @@
         <v>3</v>
       </c>
       <c r="C18" s="181" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.45">
@@ -7080,7 +7047,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.45">
@@ -7109,10 +7076,10 @@
     </row>
     <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="187" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="C25" s="188" t="s">
-        <v>182</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.45">
@@ -7120,7 +7087,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>179</v>
+        <v>157</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.45">
@@ -7128,7 +7095,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="181" t="s">
-        <v>180</v>
+        <v>158</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.45">
@@ -7136,7 +7103,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>181</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -7144,16 +7111,16 @@
         <v>3</v>
       </c>
       <c r="C29" s="183" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B32" s="187" t="s">
-        <v>190</v>
+        <v>168</v>
       </c>
       <c r="C32" s="188" t="s">
-        <v>186</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.45">
@@ -7161,7 +7128,7 @@
         <v>0</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.45">
@@ -7169,7 +7136,7 @@
         <v>1</v>
       </c>
       <c r="C34" s="181" t="s">
-        <v>151</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.45">
@@ -7177,7 +7144,7 @@
         <v>2</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>153</v>
+        <v>133</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.45">
@@ -7185,7 +7152,7 @@
         <v>3</v>
       </c>
       <c r="C36" s="181" t="s">
-        <v>114</v>
+        <v>101</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.45">
@@ -7193,7 +7160,7 @@
         <v>4</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>162</v>
+        <v>141</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.45">
@@ -7201,7 +7168,7 @@
         <v>5</v>
       </c>
       <c r="C38" s="181" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.45">
@@ -7209,7 +7176,7 @@
         <v>6</v>
       </c>
       <c r="C39" s="189" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -7217,7 +7184,7 @@
         <v>7</v>
       </c>
       <c r="C40" s="183" t="s">
-        <v>183</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed ax08 sequencing issue (missing reset step)
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E806F4-3C87-440B-B95E-7D6765473EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85D925D-6599-475A-8E16-FAF41DE6C0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="2" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="6" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="193">
   <si>
     <t>MODE B</t>
   </si>
@@ -488,9 +488,6 @@
     <t>STORE ↑</t>
   </si>
   <si>
-    <t>FREEZE_WRD ↑, (STORE ↓)</t>
-  </si>
-  <si>
     <t>AD_RGSET_OVERRIDE ↑, (HOLD ↓)</t>
   </si>
   <si>
@@ -619,6 +616,15 @@
   </si>
   <si>
     <t>Causes the computer to enter a breakpoint</t>
+  </si>
+  <si>
+    <t>RESET</t>
+  </si>
+  <si>
+    <t>FREEZE_WRD ↑</t>
+  </si>
+  <si>
+    <t>STORE ↓ (all ↓)</t>
   </si>
 </sst>
 </file>
@@ -2132,6 +2138,21 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2156,6 +2177,42 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2195,94 +2252,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2291,19 +2297,52 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2342,12 +2381,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2430,33 +2463,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="69" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="70" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2808,19 +2814,19 @@
   <sheetData>
     <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.45">
-      <c r="B2" s="193" t="s">
+      <c r="B2" s="198" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="194"/>
-      <c r="D2" s="194"/>
-      <c r="E2" s="194"/>
-      <c r="F2" s="195"/>
-      <c r="G2" s="198" t="s">
+      <c r="C2" s="199"/>
+      <c r="D2" s="199"/>
+      <c r="E2" s="199"/>
+      <c r="F2" s="200"/>
+      <c r="G2" s="203" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="199"/>
-      <c r="I2" s="200"/>
-      <c r="J2" s="196" t="s">
+      <c r="H2" s="204"/>
+      <c r="I2" s="205"/>
+      <c r="J2" s="201" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2849,7 +2855,7 @@
       <c r="I3" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="J3" s="197"/>
+      <c r="J3" s="202"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.45">
       <c r="B4" s="105">
@@ -3252,14 +3258,14 @@
         <v>0</v>
       </c>
       <c r="G16" s="118" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H16" s="191" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="I16" s="113"/>
       <c r="J16" s="26" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.45">
@@ -3283,12 +3289,12 @@
         <v>1</v>
       </c>
       <c r="G17" s="118" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H17" s="128"/>
       <c r="I17" s="113"/>
       <c r="J17" s="26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.45">
@@ -3460,73 +3466,73 @@
       </c>
     </row>
     <row r="3" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C3" s="223" t="s">
+      <c r="C3" s="215" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="224"/>
-      <c r="E3" s="224"/>
-      <c r="F3" s="224"/>
-      <c r="G3" s="225"/>
-      <c r="H3" s="220" t="s">
+      <c r="D3" s="216"/>
+      <c r="E3" s="216"/>
+      <c r="F3" s="216"/>
+      <c r="G3" s="217"/>
+      <c r="H3" s="212" t="s">
         <v>85</v>
       </c>
-      <c r="I3" s="221"/>
-      <c r="J3" s="222"/>
-      <c r="K3" s="220" t="s">
+      <c r="I3" s="213"/>
+      <c r="J3" s="214"/>
+      <c r="K3" s="212" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="221"/>
-      <c r="M3" s="221"/>
-      <c r="N3" s="207" t="s">
+      <c r="L3" s="213"/>
+      <c r="M3" s="213"/>
+      <c r="N3" s="224" t="s">
         <v>83</v>
       </c>
-      <c r="O3" s="208"/>
-      <c r="P3" s="209"/>
+      <c r="O3" s="225"/>
+      <c r="P3" s="226"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="201" t="s">
+      <c r="S3" s="218" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="202"/>
-      <c r="U3" s="202"/>
-      <c r="V3" s="202"/>
-      <c r="W3" s="202"/>
-      <c r="X3" s="202"/>
-      <c r="Y3" s="202"/>
-      <c r="Z3" s="203"/>
-      <c r="AA3" s="204" t="s">
+      <c r="T3" s="219"/>
+      <c r="U3" s="219"/>
+      <c r="V3" s="219"/>
+      <c r="W3" s="219"/>
+      <c r="X3" s="219"/>
+      <c r="Y3" s="219"/>
+      <c r="Z3" s="220"/>
+      <c r="AA3" s="221" t="s">
         <v>21</v>
       </c>
-      <c r="AB3" s="205"/>
-      <c r="AC3" s="205"/>
-      <c r="AD3" s="205"/>
-      <c r="AE3" s="205"/>
-      <c r="AF3" s="205"/>
-      <c r="AG3" s="205"/>
-      <c r="AH3" s="206"/>
+      <c r="AB3" s="222"/>
+      <c r="AC3" s="222"/>
+      <c r="AD3" s="222"/>
+      <c r="AE3" s="222"/>
+      <c r="AF3" s="222"/>
+      <c r="AG3" s="222"/>
+      <c r="AH3" s="223"/>
     </row>
     <row r="4" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="5" spans="2:34" x14ac:dyDescent="0.45">
-      <c r="B5" s="212" t="s">
+      <c r="B5" s="229" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="210" t="s">
+      <c r="C5" s="227" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="210"/>
-      <c r="E5" s="210"/>
-      <c r="F5" s="210"/>
-      <c r="G5" s="210"/>
-      <c r="H5" s="210"/>
-      <c r="I5" s="210"/>
-      <c r="J5" s="211"/>
+      <c r="D5" s="227"/>
+      <c r="E5" s="227"/>
+      <c r="F5" s="227"/>
+      <c r="G5" s="227"/>
+      <c r="H5" s="227"/>
+      <c r="I5" s="227"/>
+      <c r="J5" s="228"/>
     </row>
     <row r="6" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="213"/>
+      <c r="B6" s="230"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3556,16 +3562,16 @@
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="214" t="s">
+      <c r="C7" s="206" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="215"/>
-      <c r="E7" s="215"/>
-      <c r="F7" s="215"/>
-      <c r="G7" s="215"/>
-      <c r="H7" s="215"/>
-      <c r="I7" s="215"/>
-      <c r="J7" s="216"/>
+      <c r="D7" s="207"/>
+      <c r="E7" s="207"/>
+      <c r="F7" s="207"/>
+      <c r="G7" s="207"/>
+      <c r="H7" s="207"/>
+      <c r="I7" s="207"/>
+      <c r="J7" s="208"/>
     </row>
     <row r="8" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B8" s="6">
@@ -3575,25 +3581,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="217" t="s">
+      <c r="G8" s="209" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="218"/>
-      <c r="I8" s="218"/>
-      <c r="J8" s="219"/>
+      <c r="H8" s="210"/>
+      <c r="I8" s="210"/>
+      <c r="J8" s="211"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="S3:Z3"/>
+    <mergeCell ref="AA3:AH3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:J7"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="S3:Z3"/>
-    <mergeCell ref="AA3:AH3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3616,29 +3622,29 @@
   <sheetData>
     <row r="1" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B2" s="247" t="s">
+      <c r="B2" s="231" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="248"/>
-      <c r="D2" s="248"/>
-      <c r="E2" s="248"/>
-      <c r="F2" s="248"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="196" t="s">
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="233"/>
+      <c r="H2" s="201" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="196" t="s">
+      <c r="I2" s="201" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="247" t="s">
+      <c r="J2" s="231" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="248"/>
-      <c r="L2" s="248"/>
-      <c r="M2" s="196" t="s">
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="M2" s="201" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="196" t="s">
+      <c r="N2" s="201" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3661,8 +3667,8 @@
       <c r="G3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="197"/>
-      <c r="I3" s="197"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -3672,8 +3678,8 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="197"/>
-      <c r="N3" s="197"/>
+      <c r="M3" s="202"/>
+      <c r="N3" s="202"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
@@ -3699,26 +3705,26 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="228" t="s">
+      <c r="H4" s="234" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>179</v>
-      </c>
-      <c r="J4" s="300" t="s">
+        <v>178</v>
+      </c>
+      <c r="J4" s="196" t="s">
         <v>73</v>
       </c>
-      <c r="K4" s="301" t="s">
+      <c r="K4" s="197" t="s">
         <v>97</v>
       </c>
-      <c r="L4" s="235" t="s">
+      <c r="L4" s="243" t="s">
         <v>16</v>
       </c>
       <c r="M4" s="69" t="s">
         <v>95</v>
       </c>
       <c r="N4" s="75" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -3745,7 +3751,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="227"/>
+      <c r="H5" s="235"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -3755,12 +3761,12 @@
       <c r="K5" s="54" t="s">
         <v>53</v>
       </c>
-      <c r="L5" s="237"/>
+      <c r="L5" s="242"/>
       <c r="M5" s="34" t="s">
         <v>95</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.45">
@@ -3787,22 +3793,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="226" t="s">
+      <c r="H6" s="236" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="230" t="s">
+      <c r="J6" s="237" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="239" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="236" t="s">
+      <c r="L6" s="241" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="241" t="s">
+      <c r="M6" s="249" t="s">
         <v>95</v>
       </c>
       <c r="N6" s="244" t="s">
@@ -3833,14 +3839,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="226"/>
+      <c r="H7" s="236"/>
       <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="230"/>
+      <c r="J7" s="237"/>
       <c r="K7" s="239"/>
-      <c r="L7" s="236"/>
-      <c r="M7" s="242"/>
+      <c r="L7" s="241"/>
+      <c r="M7" s="250"/>
       <c r="N7" s="244"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.45">
@@ -3867,14 +3873,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="226"/>
+      <c r="H8" s="236"/>
       <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="230"/>
+      <c r="J8" s="237"/>
       <c r="K8" s="239"/>
-      <c r="L8" s="236"/>
-      <c r="M8" s="242"/>
+      <c r="L8" s="241"/>
+      <c r="M8" s="250"/>
       <c r="N8" s="244"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.45">
@@ -3901,14 +3907,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="226"/>
+      <c r="H9" s="236"/>
       <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="230"/>
+      <c r="J9" s="237"/>
       <c r="K9" s="239"/>
-      <c r="L9" s="236"/>
-      <c r="M9" s="242"/>
+      <c r="L9" s="241"/>
+      <c r="M9" s="250"/>
       <c r="N9" s="244"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.45">
@@ -3935,14 +3941,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="226"/>
+      <c r="H10" s="236"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="230"/>
+      <c r="J10" s="237"/>
       <c r="K10" s="239"/>
-      <c r="L10" s="236"/>
-      <c r="M10" s="242"/>
+      <c r="L10" s="241"/>
+      <c r="M10" s="250"/>
       <c r="N10" s="244"/>
     </row>
     <row r="11" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -3969,14 +3975,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="227"/>
+      <c r="H11" s="235"/>
       <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="231"/>
+      <c r="J11" s="238"/>
       <c r="K11" s="240"/>
-      <c r="L11" s="237"/>
-      <c r="M11" s="243"/>
+      <c r="L11" s="242"/>
+      <c r="M11" s="251"/>
       <c r="N11" s="245"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.45">
@@ -4003,26 +4009,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="228" t="s">
+      <c r="H12" s="234" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="229" t="s">
+      <c r="J12" s="246" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="238" t="s">
+      <c r="K12" s="247" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="235" t="s">
+      <c r="L12" s="243" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="228" t="s">
+      <c r="M12" s="234" t="s">
         <v>96</v>
       </c>
-      <c r="N12" s="246" t="s">
-        <v>185</v>
+      <c r="N12" s="248" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.45">
@@ -4049,14 +4055,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="226"/>
+      <c r="H13" s="236"/>
       <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="230"/>
+      <c r="J13" s="237"/>
       <c r="K13" s="239"/>
-      <c r="L13" s="236"/>
-      <c r="M13" s="226"/>
+      <c r="L13" s="241"/>
+      <c r="M13" s="236"/>
       <c r="N13" s="244"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.45">
@@ -4083,14 +4089,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="226"/>
+      <c r="H14" s="236"/>
       <c r="I14" s="90" t="s">
         <v>86</v>
       </c>
-      <c r="J14" s="230"/>
+      <c r="J14" s="237"/>
       <c r="K14" s="239"/>
-      <c r="L14" s="236"/>
-      <c r="M14" s="226"/>
+      <c r="L14" s="241"/>
+      <c r="M14" s="236"/>
       <c r="N14" s="244"/>
     </row>
     <row r="15" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -4117,14 +4123,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="227"/>
+      <c r="H15" s="235"/>
       <c r="I15" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="J15" s="231"/>
+      <c r="J15" s="238"/>
       <c r="K15" s="240"/>
-      <c r="L15" s="237"/>
-      <c r="M15" s="227"/>
+      <c r="L15" s="242"/>
+      <c r="M15" s="235"/>
       <c r="N15" s="245"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.45">
@@ -4151,22 +4157,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="228" t="s">
+      <c r="H16" s="234" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="229" t="s">
+      <c r="J16" s="246" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="232" t="s">
+      <c r="K16" s="252" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="235" t="s">
+      <c r="L16" s="243" t="s">
         <v>55</v>
       </c>
-      <c r="M16" s="228" t="s">
+      <c r="M16" s="234" t="s">
         <v>96</v>
       </c>
       <c r="N16" s="75" t="s">
@@ -4197,14 +4203,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="226"/>
+      <c r="H17" s="236"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="230"/>
-      <c r="K17" s="233"/>
-      <c r="L17" s="236"/>
-      <c r="M17" s="226"/>
+      <c r="J17" s="237"/>
+      <c r="K17" s="253"/>
+      <c r="L17" s="241"/>
+      <c r="M17" s="236"/>
       <c r="N17" s="74" t="s">
         <v>89</v>
       </c>
@@ -4233,14 +4239,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="226"/>
+      <c r="H18" s="236"/>
       <c r="I18" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="J18" s="230"/>
-      <c r="K18" s="233"/>
-      <c r="L18" s="236"/>
-      <c r="M18" s="226"/>
+      <c r="J18" s="237"/>
+      <c r="K18" s="253"/>
+      <c r="L18" s="241"/>
+      <c r="M18" s="236"/>
       <c r="N18" s="74" t="s">
         <v>91</v>
       </c>
@@ -4269,14 +4275,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="227"/>
+      <c r="H19" s="235"/>
       <c r="I19" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="J19" s="231"/>
-      <c r="K19" s="234"/>
-      <c r="L19" s="237"/>
-      <c r="M19" s="227"/>
+      <c r="J19" s="238"/>
+      <c r="K19" s="254"/>
+      <c r="L19" s="242"/>
+      <c r="M19" s="235"/>
       <c r="N19" s="44" t="s">
         <v>92</v>
       </c>
@@ -4306,26 +4312,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="228" t="s">
+      <c r="H20" s="234" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="192" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J20" s="140" t="s">
-        <v>152</v>
-      </c>
-      <c r="K20" s="232" t="s">
+        <v>151</v>
+      </c>
+      <c r="K20" s="252" t="s">
         <v>53</v>
       </c>
-      <c r="L20" s="296" t="s">
+      <c r="L20" s="257" t="s">
         <v>55</v>
       </c>
-      <c r="M20" s="241" t="s">
+      <c r="M20" s="249" t="s">
         <v>95</v>
       </c>
-      <c r="N20" s="298" t="s">
-        <v>180</v>
+      <c r="N20" s="194" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.45">
@@ -4352,18 +4358,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="226"/>
-      <c r="I21" s="293" t="s">
+      <c r="H21" s="236"/>
+      <c r="I21" s="193" t="s">
         <v>100</v>
       </c>
       <c r="J21" s="99" t="s">
-        <v>152</v>
-      </c>
-      <c r="K21" s="295"/>
-      <c r="L21" s="297"/>
-      <c r="M21" s="294"/>
-      <c r="N21" s="299" t="s">
-        <v>181</v>
+        <v>151</v>
+      </c>
+      <c r="K21" s="256"/>
+      <c r="L21" s="258"/>
+      <c r="M21" s="255"/>
+      <c r="N21" s="195" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.45">
@@ -4390,7 +4396,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="226"/>
+      <c r="H22" s="236"/>
       <c r="I22" s="103"/>
       <c r="J22" s="136"/>
       <c r="K22" s="137"/>
@@ -4422,7 +4428,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="227"/>
+      <c r="H23" s="235"/>
       <c r="I23" s="96"/>
       <c r="J23" s="133"/>
       <c r="K23" s="134"/>
@@ -4454,7 +4460,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="228" t="s">
+      <c r="H24" s="234" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -4500,7 +4506,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="226"/>
+      <c r="H25" s="236"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -4517,7 +4523,7 @@
         <v>95</v>
       </c>
       <c r="N25" s="74" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.45">
@@ -4544,7 +4550,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="226"/>
+      <c r="H26" s="236"/>
       <c r="I26" s="103"/>
       <c r="J26" s="136"/>
       <c r="K26" s="137"/>
@@ -4576,7 +4582,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="227"/>
+      <c r="H27" s="235"/>
       <c r="I27" s="96"/>
       <c r="J27" s="133"/>
       <c r="K27" s="134"/>
@@ -4608,7 +4614,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="228" t="s">
+      <c r="H28" s="234" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -4627,7 +4633,7 @@
         <v>95</v>
       </c>
       <c r="N28" s="38" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.45">
@@ -4654,7 +4660,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="226"/>
+      <c r="H29" s="236"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -4671,7 +4677,7 @@
         <v>95</v>
       </c>
       <c r="N29" s="74" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.45">
@@ -4698,7 +4704,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="226"/>
+      <c r="H30" s="236"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -4715,7 +4721,7 @@
         <v>95</v>
       </c>
       <c r="N30" s="74" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -4742,7 +4748,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="227"/>
+      <c r="H31" s="235"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -4774,7 +4780,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="226" t="s">
+      <c r="H32" s="236" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -4793,7 +4799,7 @@
         <v>95</v>
       </c>
       <c r="N32" s="38" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="Q32" s="1"/>
     </row>
@@ -4821,7 +4827,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="226"/>
+      <c r="H33" s="236"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -4838,7 +4844,7 @@
         <v>95</v>
       </c>
       <c r="N33" s="74" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Q33" s="1"/>
     </row>
@@ -4866,7 +4872,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="227"/>
+      <c r="H34" s="235"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -4883,7 +4889,7 @@
         <v>95</v>
       </c>
       <c r="N34" s="74" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Q34" s="1"/>
     </row>
@@ -4930,23 +4936,23 @@
         <v>95</v>
       </c>
       <c r="N35" s="46" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="M20:M21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:L21"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4955,18 +4961,18 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="M20:M21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:L21"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4988,26 +4994,26 @@
   <sheetData>
     <row r="1" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B2" s="247" t="s">
+      <c r="B2" s="231" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="248"/>
-      <c r="D2" s="248"/>
-      <c r="E2" s="248"/>
-      <c r="F2" s="248"/>
-      <c r="G2" s="249"/>
-      <c r="H2" s="196" t="s">
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="232"/>
+      <c r="F2" s="232"/>
+      <c r="G2" s="233"/>
+      <c r="H2" s="201" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="196" t="s">
+      <c r="I2" s="201" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="247" t="s">
+      <c r="J2" s="231" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="248"/>
-      <c r="L2" s="248"/>
-      <c r="M2" s="196" t="s">
+      <c r="K2" s="232"/>
+      <c r="L2" s="232"/>
+      <c r="M2" s="201" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5030,8 +5036,8 @@
       <c r="G3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="197"/>
-      <c r="I3" s="197"/>
+      <c r="H3" s="202"/>
+      <c r="I3" s="202"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -5041,7 +5047,7 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="197"/>
+      <c r="M3" s="202"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.45">
       <c r="B4" s="80">
@@ -5067,11 +5073,11 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="228" t="s">
+      <c r="H4" s="234" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J4" s="66" t="s">
         <v>73</v>
@@ -5110,7 +5116,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="227"/>
+      <c r="H5" s="235"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -5151,19 +5157,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="226" t="s">
+      <c r="H6" s="236" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="230" t="s">
+      <c r="J6" s="237" t="s">
         <v>58</v>
       </c>
       <c r="K6" s="239" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="236" t="s">
+      <c r="L6" s="241" t="s">
         <v>55</v>
       </c>
       <c r="M6" s="244" t="s">
@@ -5194,11 +5200,11 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="226"/>
-      <c r="I7" s="250"/>
-      <c r="J7" s="230"/>
+      <c r="H7" s="236"/>
+      <c r="I7" s="259"/>
+      <c r="J7" s="237"/>
       <c r="K7" s="239"/>
-      <c r="L7" s="236"/>
+      <c r="L7" s="241"/>
       <c r="M7" s="244"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.45">
@@ -5225,11 +5231,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="226"/>
-      <c r="I8" s="263"/>
-      <c r="J8" s="230"/>
+      <c r="H8" s="236"/>
+      <c r="I8" s="260"/>
+      <c r="J8" s="237"/>
       <c r="K8" s="239"/>
-      <c r="L8" s="236"/>
+      <c r="L8" s="241"/>
       <c r="M8" s="244"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.45">
@@ -5256,11 +5262,11 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="226"/>
-      <c r="I9" s="264"/>
-      <c r="J9" s="230"/>
+      <c r="H9" s="236"/>
+      <c r="I9" s="261"/>
+      <c r="J9" s="237"/>
       <c r="K9" s="239"/>
-      <c r="L9" s="236"/>
+      <c r="L9" s="241"/>
       <c r="M9" s="244"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.45">
@@ -5287,13 +5293,13 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="226"/>
+      <c r="H10" s="236"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="230"/>
+      <c r="J10" s="237"/>
       <c r="K10" s="239"/>
-      <c r="L10" s="236"/>
+      <c r="L10" s="241"/>
       <c r="M10" s="244"/>
     </row>
     <row r="11" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -5320,11 +5326,11 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="227"/>
+      <c r="H11" s="235"/>
       <c r="I11" s="103"/>
-      <c r="J11" s="231"/>
+      <c r="J11" s="238"/>
       <c r="K11" s="240"/>
-      <c r="L11" s="237"/>
+      <c r="L11" s="242"/>
       <c r="M11" s="245"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.45">
@@ -5351,22 +5357,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="228" t="s">
+      <c r="H12" s="234" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="229" t="s">
+      <c r="J12" s="246" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="238" t="s">
+      <c r="K12" s="247" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="235" t="s">
+      <c r="L12" s="243" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="246" t="s">
+      <c r="M12" s="248" t="s">
         <v>88</v>
       </c>
     </row>
@@ -5394,11 +5400,11 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="226"/>
-      <c r="I13" s="250"/>
-      <c r="J13" s="230"/>
+      <c r="H13" s="236"/>
+      <c r="I13" s="259"/>
+      <c r="J13" s="237"/>
       <c r="K13" s="239"/>
-      <c r="L13" s="236"/>
+      <c r="L13" s="241"/>
       <c r="M13" s="244"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.45">
@@ -5425,11 +5431,11 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="226"/>
-      <c r="I14" s="263"/>
-      <c r="J14" s="230"/>
+      <c r="H14" s="236"/>
+      <c r="I14" s="260"/>
+      <c r="J14" s="237"/>
       <c r="K14" s="239"/>
-      <c r="L14" s="236"/>
+      <c r="L14" s="241"/>
       <c r="M14" s="244"/>
     </row>
     <row r="15" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -5456,11 +5462,11 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="227"/>
-      <c r="I15" s="251"/>
-      <c r="J15" s="231"/>
+      <c r="H15" s="235"/>
+      <c r="I15" s="262"/>
+      <c r="J15" s="238"/>
       <c r="K15" s="240"/>
-      <c r="L15" s="237"/>
+      <c r="L15" s="242"/>
       <c r="M15" s="245"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.45">
@@ -5487,19 +5493,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="228" t="s">
+      <c r="H16" s="234" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="229" t="s">
+      <c r="J16" s="246" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="232" t="s">
+      <c r="K16" s="252" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="235" t="s">
+      <c r="L16" s="243" t="s">
         <v>55</v>
       </c>
       <c r="M16" s="75" t="s">
@@ -5530,13 +5536,13 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="226"/>
+      <c r="H17" s="236"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="230"/>
-      <c r="K17" s="233"/>
-      <c r="L17" s="236"/>
+      <c r="J17" s="237"/>
+      <c r="K17" s="253"/>
+      <c r="L17" s="241"/>
       <c r="M17" s="74" t="s">
         <v>89</v>
       </c>
@@ -5565,12 +5571,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="226"/>
-      <c r="I18" s="250"/>
-      <c r="J18" s="230"/>
-      <c r="K18" s="233"/>
-      <c r="L18" s="236"/>
-      <c r="M18" s="250"/>
+      <c r="H18" s="236"/>
+      <c r="I18" s="259"/>
+      <c r="J18" s="237"/>
+      <c r="K18" s="253"/>
+      <c r="L18" s="241"/>
+      <c r="M18" s="259"/>
     </row>
     <row r="19" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B19" s="82">
@@ -5596,12 +5602,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="227"/>
-      <c r="I19" s="251"/>
-      <c r="J19" s="231"/>
-      <c r="K19" s="234"/>
-      <c r="L19" s="237"/>
-      <c r="M19" s="251"/>
+      <c r="H19" s="235"/>
+      <c r="I19" s="262"/>
+      <c r="J19" s="238"/>
+      <c r="K19" s="254"/>
+      <c r="L19" s="242"/>
+      <c r="M19" s="262"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.45">
@@ -5628,14 +5634,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="252" t="s">
+      <c r="H20" s="263" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="176" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J20" s="66" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K20" s="65" t="s">
         <v>53</v>
@@ -5644,7 +5650,7 @@
         <v>55</v>
       </c>
       <c r="M20" s="175" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.45">
@@ -5671,7 +5677,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="253"/>
+      <c r="H21" s="264"/>
       <c r="I21" s="167"/>
       <c r="J21" s="169"/>
       <c r="K21" s="171"/>
@@ -5702,7 +5708,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="253"/>
+      <c r="H22" s="264"/>
       <c r="I22" s="167"/>
       <c r="J22" s="169"/>
       <c r="K22" s="171"/>
@@ -5733,7 +5739,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="254"/>
+      <c r="H23" s="265"/>
       <c r="I23" s="168"/>
       <c r="J23" s="170"/>
       <c r="K23" s="172"/>
@@ -5764,7 +5770,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="228" t="s">
+      <c r="H24" s="234" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -5807,7 +5813,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="226"/>
+      <c r="H25" s="236"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -5848,12 +5854,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="226"/>
-      <c r="I26" s="250"/>
-      <c r="J26" s="255"/>
-      <c r="K26" s="257"/>
-      <c r="L26" s="259"/>
-      <c r="M26" s="261"/>
+      <c r="H26" s="236"/>
+      <c r="I26" s="259"/>
+      <c r="J26" s="266"/>
+      <c r="K26" s="268"/>
+      <c r="L26" s="270"/>
+      <c r="M26" s="272"/>
     </row>
     <row r="27" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B27" s="82">
@@ -5879,12 +5885,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="227"/>
-      <c r="I27" s="251"/>
-      <c r="J27" s="256"/>
-      <c r="K27" s="258"/>
-      <c r="L27" s="260"/>
-      <c r="M27" s="262"/>
+      <c r="H27" s="235"/>
+      <c r="I27" s="262"/>
+      <c r="J27" s="267"/>
+      <c r="K27" s="269"/>
+      <c r="L27" s="271"/>
+      <c r="M27" s="273"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.45">
       <c r="B28" s="80">
@@ -5910,7 +5916,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="228" t="s">
+      <c r="H28" s="234" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -5953,7 +5959,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="226"/>
+      <c r="H29" s="236"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -5994,7 +6000,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="226"/>
+      <c r="H30" s="236"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -6035,7 +6041,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="227"/>
+      <c r="H31" s="235"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -6066,7 +6072,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="226" t="s">
+      <c r="H32" s="236" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -6110,7 +6116,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="226"/>
+      <c r="H33" s="236"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -6152,7 +6158,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="227"/>
+      <c r="H34" s="235"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -6207,7 +6213,7 @@
         <v>53</v>
       </c>
       <c r="L35" s="165" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="M35" s="46" t="s">
         <v>93</v>
@@ -6215,24 +6221,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6248,6 +6236,24 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6264,13 +6270,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B2" s="247" t="s">
+      <c r="B2" s="231" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="248"/>
-      <c r="D2" s="248"/>
-      <c r="E2" s="249"/>
-      <c r="F2" s="196" t="s">
+      <c r="C2" s="232"/>
+      <c r="D2" s="232"/>
+      <c r="E2" s="233"/>
+      <c r="F2" s="201" t="s">
         <v>24</v>
       </c>
     </row>
@@ -6287,7 +6293,7 @@
       <c r="E3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="197"/>
+      <c r="F3" s="202"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.45">
       <c r="B4" s="13">
@@ -6468,30 +6474,30 @@
   <sheetData>
     <row r="1" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.45">
-      <c r="B2" s="196" t="s">
+      <c r="B2" s="201" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="274" t="s">
+      <c r="C2" s="283" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="275"/>
-      <c r="E2" s="275"/>
-      <c r="F2" s="275"/>
-      <c r="G2" s="275"/>
-      <c r="H2" s="275"/>
-      <c r="I2" s="275"/>
-      <c r="J2" s="275"/>
-      <c r="K2" s="275"/>
-      <c r="L2" s="275"/>
-      <c r="M2" s="275"/>
-      <c r="N2" s="275"/>
-      <c r="O2" s="275"/>
-      <c r="P2" s="275"/>
-      <c r="Q2" s="275"/>
-      <c r="R2" s="276"/>
+      <c r="D2" s="284"/>
+      <c r="E2" s="284"/>
+      <c r="F2" s="284"/>
+      <c r="G2" s="284"/>
+      <c r="H2" s="284"/>
+      <c r="I2" s="284"/>
+      <c r="J2" s="284"/>
+      <c r="K2" s="284"/>
+      <c r="L2" s="284"/>
+      <c r="M2" s="284"/>
+      <c r="N2" s="284"/>
+      <c r="O2" s="284"/>
+      <c r="P2" s="284"/>
+      <c r="Q2" s="284"/>
+      <c r="R2" s="285"/>
     </row>
     <row r="3" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="197"/>
+      <c r="B3" s="202"/>
       <c r="C3" s="116">
         <v>15</v>
       </c>
@@ -6562,13 +6568,13 @@
       <c r="M4" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="N4" s="268" t="s">
+      <c r="N4" s="277" t="s">
         <v>77</v>
       </c>
-      <c r="O4" s="268"/>
-      <c r="P4" s="268"/>
-      <c r="Q4" s="268"/>
-      <c r="R4" s="269"/>
+      <c r="O4" s="277"/>
+      <c r="P4" s="277"/>
+      <c r="Q4" s="277"/>
+      <c r="R4" s="278"/>
     </row>
     <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B5" s="88" t="s">
@@ -6582,16 +6588,16 @@
       <c r="H5" s="153"/>
       <c r="I5" s="153"/>
       <c r="J5" s="154"/>
-      <c r="K5" s="270" t="s">
+      <c r="K5" s="279" t="s">
         <v>73</v>
       </c>
-      <c r="L5" s="266"/>
-      <c r="M5" s="266"/>
-      <c r="N5" s="266"/>
-      <c r="O5" s="266"/>
-      <c r="P5" s="266"/>
-      <c r="Q5" s="266"/>
-      <c r="R5" s="267"/>
+      <c r="L5" s="275"/>
+      <c r="M5" s="275"/>
+      <c r="N5" s="275"/>
+      <c r="O5" s="275"/>
+      <c r="P5" s="275"/>
+      <c r="Q5" s="275"/>
+      <c r="R5" s="276"/>
     </row>
     <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88" t="s">
@@ -6605,16 +6611,16 @@
       <c r="H6" s="153"/>
       <c r="I6" s="153"/>
       <c r="J6" s="154"/>
-      <c r="K6" s="270" t="s">
+      <c r="K6" s="279" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="266"/>
-      <c r="M6" s="266"/>
-      <c r="N6" s="266"/>
-      <c r="O6" s="266"/>
-      <c r="P6" s="266"/>
-      <c r="Q6" s="266"/>
-      <c r="R6" s="267"/>
+      <c r="L6" s="275"/>
+      <c r="M6" s="275"/>
+      <c r="N6" s="275"/>
+      <c r="O6" s="275"/>
+      <c r="P6" s="275"/>
+      <c r="Q6" s="275"/>
+      <c r="R6" s="276"/>
     </row>
     <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="88" t="s">
@@ -6628,39 +6634,39 @@
       <c r="H7" s="155"/>
       <c r="I7" s="155"/>
       <c r="J7" s="155"/>
-      <c r="K7" s="271" t="s">
+      <c r="K7" s="280" t="s">
         <v>73</v>
       </c>
-      <c r="L7" s="272"/>
-      <c r="M7" s="272"/>
-      <c r="N7" s="272"/>
-      <c r="O7" s="272"/>
-      <c r="P7" s="272"/>
-      <c r="Q7" s="272"/>
-      <c r="R7" s="273"/>
+      <c r="L7" s="281"/>
+      <c r="M7" s="281"/>
+      <c r="N7" s="281"/>
+      <c r="O7" s="281"/>
+      <c r="P7" s="281"/>
+      <c r="Q7" s="281"/>
+      <c r="R7" s="282"/>
     </row>
     <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="265" t="s">
+      <c r="C8" s="274" t="s">
         <v>126</v>
       </c>
-      <c r="D8" s="266"/>
-      <c r="E8" s="266"/>
-      <c r="F8" s="266"/>
-      <c r="G8" s="266"/>
-      <c r="H8" s="266"/>
-      <c r="I8" s="266"/>
-      <c r="J8" s="266"/>
-      <c r="K8" s="266"/>
-      <c r="L8" s="266"/>
-      <c r="M8" s="266"/>
-      <c r="N8" s="266"/>
-      <c r="O8" s="266"/>
-      <c r="P8" s="266"/>
-      <c r="Q8" s="266"/>
-      <c r="R8" s="267"/>
+      <c r="D8" s="275"/>
+      <c r="E8" s="275"/>
+      <c r="F8" s="275"/>
+      <c r="G8" s="275"/>
+      <c r="H8" s="275"/>
+      <c r="I8" s="275"/>
+      <c r="J8" s="275"/>
+      <c r="K8" s="275"/>
+      <c r="L8" s="275"/>
+      <c r="M8" s="275"/>
+      <c r="N8" s="275"/>
+      <c r="O8" s="275"/>
+      <c r="P8" s="275"/>
+      <c r="Q8" s="275"/>
+      <c r="R8" s="276"/>
     </row>
     <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B9" s="89" t="s">
@@ -6706,7 +6712,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
-  <dimension ref="B1:D8"/>
+  <dimension ref="B1:D9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="21.1328125" customWidth="1"/>
@@ -6734,7 +6740,7 @@
         <v>130</v>
       </c>
       <c r="D3" s="74" t="s">
-        <v>147</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.45">
@@ -6764,32 +6770,43 @@
         <v>101</v>
       </c>
       <c r="C6" s="74" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D6" s="74" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B7" s="159" t="s">
+        <v>141</v>
+      </c>
+      <c r="C7" s="74" t="s">
+        <v>142</v>
+      </c>
+      <c r="D7" s="74" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B7" s="157" t="s">
-        <v>141</v>
-      </c>
-      <c r="C7" s="41" t="s">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B8" s="157" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="41" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B9" s="160" t="s">
+        <v>190</v>
+      </c>
+      <c r="C9" s="161" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="41" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B8" s="160" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="161" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="161" t="s">
-        <v>146</v>
+      <c r="D9" s="161" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -6807,10 +6824,10 @@
   <sheetData>
     <row r="1" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B2" s="277" t="s">
+      <c r="B2" s="286" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="278"/>
+      <c r="C2" s="287"/>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -6827,7 +6844,7 @@
       <c r="C4" s="130" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="279" t="s">
+      <c r="D4" s="288" t="s">
         <v>124</v>
       </c>
     </row>
@@ -6836,21 +6853,21 @@
       <c r="C5" s="131" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="280"/>
+      <c r="D5" s="289"/>
     </row>
     <row r="6" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="133"/>
       <c r="C6" s="63" t="s">
         <v>120</v>
       </c>
-      <c r="D6" s="281"/>
+      <c r="D6" s="290"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B7" s="140" t="s">
         <v>119</v>
       </c>
       <c r="C7" s="141"/>
-      <c r="D7" s="282" t="s">
+      <c r="D7" s="291" t="s">
         <v>125</v>
       </c>
     </row>
@@ -6859,14 +6876,14 @@
         <v>118</v>
       </c>
       <c r="C8" s="142"/>
-      <c r="D8" s="283"/>
+      <c r="D8" s="292"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" s="40" t="s">
         <v>120</v>
       </c>
       <c r="C9" s="142"/>
-      <c r="D9" s="283"/>
+      <c r="D9" s="292"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" s="143" t="s">
@@ -6875,7 +6892,7 @@
       <c r="C10" s="144" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="283"/>
+      <c r="D10" s="292"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" s="40" t="s">
@@ -6884,7 +6901,7 @@
       <c r="C11" s="131" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="283"/>
+      <c r="D11" s="292"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -6894,7 +6911,7 @@
       <c r="C12" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="284"/>
+      <c r="D12" s="293"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6916,21 +6933,21 @@
   <sheetData>
     <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.45">
-      <c r="B2" s="285" t="s">
-        <v>166</v>
-      </c>
-      <c r="C2" s="287" t="s">
+      <c r="B2" s="294" t="s">
         <v>165</v>
       </c>
-      <c r="D2" s="288"/>
+      <c r="C2" s="296" t="s">
+        <v>164</v>
+      </c>
+      <c r="D2" s="297"/>
     </row>
     <row r="3" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="286"/>
+      <c r="B3" s="295"/>
       <c r="C3" s="185" t="s">
+        <v>161</v>
+      </c>
+      <c r="D3" s="186" t="s">
         <v>162</v>
-      </c>
-      <c r="D3" s="186" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -6938,10 +6955,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="143" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" s="235" t="s">
-        <v>160</v>
+        <v>169</v>
+      </c>
+      <c r="D4" s="243" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
@@ -6949,34 +6966,34 @@
         <v>1</v>
       </c>
       <c r="C5" s="190" t="s">
-        <v>171</v>
-      </c>
-      <c r="D5" s="289"/>
+        <v>170</v>
+      </c>
+      <c r="D5" s="298"/>
     </row>
     <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B6" s="88">
         <v>2</v>
       </c>
-      <c r="C6" s="291" t="s">
-        <v>167</v>
-      </c>
-      <c r="D6" s="290" t="s">
-        <v>164</v>
+      <c r="C6" s="300" t="s">
+        <v>166</v>
+      </c>
+      <c r="D6" s="299" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B7" s="177">
         <v>3</v>
       </c>
-      <c r="C7" s="230"/>
-      <c r="D7" s="236"/>
+      <c r="C7" s="237"/>
+      <c r="D7" s="241"/>
     </row>
     <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B8" s="88">
         <v>4</v>
       </c>
-      <c r="C8" s="292"/>
-      <c r="D8" s="289"/>
+      <c r="C8" s="301"/>
+      <c r="D8" s="298"/>
     </row>
     <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B9" s="177">
@@ -6998,16 +7015,16 @@
       </c>
       <c r="C11" s="133"/>
       <c r="D11" s="180" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B14" s="187" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C14" s="188" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.45">
@@ -7015,7 +7032,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.45">
@@ -7023,7 +7040,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="181" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.45">
@@ -7031,7 +7048,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.45">
@@ -7039,7 +7056,7 @@
         <v>3</v>
       </c>
       <c r="C18" s="181" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.45">
@@ -7047,7 +7064,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.45">
@@ -7076,10 +7093,10 @@
     </row>
     <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B25" s="187" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C25" s="188" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.45">
@@ -7087,7 +7104,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.45">
@@ -7095,7 +7112,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="181" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.45">
@@ -7103,7 +7120,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -7111,16 +7128,16 @@
         <v>3</v>
       </c>
       <c r="C29" s="183" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B32" s="187" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C32" s="188" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.45">
@@ -7176,7 +7193,7 @@
         <v>6</v>
       </c>
       <c r="C39" s="189" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
@@ -7184,7 +7201,7 @@
         <v>7</v>
       </c>
       <c r="C40" s="183" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clear hold line when the opcode is freezed
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olive\Desktop\pc_project\rlpc\AX08-PC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B85D925D-6599-475A-8E16-FAF41DE6C0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD679EB-A19D-48CF-9A6B-3A922191C871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="6" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11835" activeTab="6" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="196">
   <si>
     <t>MODE B</t>
   </si>
@@ -625,6 +625,15 @@
   </si>
   <si>
     <t>STORE ↓ (all ↓)</t>
+  </si>
+  <si>
+    <t>FREEZE_OP ↑, (FREEZE_WRD ↓) (HOLD ↓)</t>
+  </si>
+  <si>
+    <t>AD_RGSET_OVERRIDE ↑,</t>
+  </si>
+  <si>
+    <t>Net action (firmware modules)</t>
   </si>
 </sst>
 </file>
@@ -2177,6 +2186,45 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2213,43 +2261,79 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2261,88 +2345,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2381,6 +2384,12 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2467,7 +2476,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2488,7 +2497,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2805,15 +2814,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F30110-9AA6-4607-84AE-181659F51D05}">
   <dimension ref="B1:J19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="6" width="4.73046875" style="1" customWidth="1"/>
-    <col min="7" max="9" width="9.1328125" customWidth="1"/>
-    <col min="10" max="10" width="34.265625" customWidth="1"/>
+    <col min="3" max="6" width="4.7109375" style="1" customWidth="1"/>
+    <col min="7" max="9" width="9.140625" customWidth="1"/>
+    <col min="10" max="10" width="34.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B2" s="198" t="s">
         <v>15</v>
       </c>
@@ -2830,7 +2839,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="56" t="s">
         <v>16</v>
       </c>
@@ -2857,7 +2866,7 @@
       </c>
       <c r="J3" s="202"/>
     </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="105">
         <v>0</v>
       </c>
@@ -2890,7 +2899,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -2923,7 +2932,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -2956,7 +2965,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -2989,7 +2998,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -3022,7 +3031,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -3055,7 +3064,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -3088,7 +3097,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -3121,7 +3130,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B12" s="13">
         <v>8</v>
       </c>
@@ -3152,7 +3161,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B13" s="13">
         <v>9</v>
       </c>
@@ -3181,7 +3190,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B14" s="19">
         <v>10</v>
       </c>
@@ -3208,7 +3217,7 @@
       <c r="I14" s="114"/>
       <c r="J14" s="31"/>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B15" s="22">
         <v>11</v>
       </c>
@@ -3237,7 +3246,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B16" s="13">
         <v>12</v>
       </c>
@@ -3268,7 +3277,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B17" s="13">
         <v>13</v>
       </c>
@@ -3297,7 +3306,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B18" s="19">
         <v>14</v>
       </c>
@@ -3322,7 +3331,7 @@
       <c r="I18" s="114"/>
       <c r="J18" s="31"/>
     </row>
-    <row r="19" spans="2:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="16">
         <v>15</v>
       </c>
@@ -3361,13 +3370,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADE0A35C-77D4-4A92-BE06-765002DB2402}">
   <dimension ref="B1:AH8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="34" width="7.73046875" customWidth="1"/>
+    <col min="3" max="34" width="7.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C2" s="2">
         <v>31</v>
       </c>
@@ -3465,74 +3474,74 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="C3" s="215" t="s">
+    <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="228" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="216"/>
-      <c r="E3" s="216"/>
-      <c r="F3" s="216"/>
-      <c r="G3" s="217"/>
-      <c r="H3" s="212" t="s">
+      <c r="D3" s="229"/>
+      <c r="E3" s="229"/>
+      <c r="F3" s="229"/>
+      <c r="G3" s="230"/>
+      <c r="H3" s="225" t="s">
         <v>85</v>
       </c>
-      <c r="I3" s="213"/>
-      <c r="J3" s="214"/>
-      <c r="K3" s="212" t="s">
+      <c r="I3" s="226"/>
+      <c r="J3" s="227"/>
+      <c r="K3" s="225" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="213"/>
-      <c r="M3" s="213"/>
-      <c r="N3" s="224" t="s">
+      <c r="L3" s="226"/>
+      <c r="M3" s="226"/>
+      <c r="N3" s="212" t="s">
         <v>83</v>
       </c>
-      <c r="O3" s="225"/>
-      <c r="P3" s="226"/>
+      <c r="O3" s="213"/>
+      <c r="P3" s="214"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="218" t="s">
+      <c r="S3" s="206" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="219"/>
-      <c r="U3" s="219"/>
-      <c r="V3" s="219"/>
-      <c r="W3" s="219"/>
-      <c r="X3" s="219"/>
-      <c r="Y3" s="219"/>
-      <c r="Z3" s="220"/>
-      <c r="AA3" s="221" t="s">
+      <c r="T3" s="207"/>
+      <c r="U3" s="207"/>
+      <c r="V3" s="207"/>
+      <c r="W3" s="207"/>
+      <c r="X3" s="207"/>
+      <c r="Y3" s="207"/>
+      <c r="Z3" s="208"/>
+      <c r="AA3" s="209" t="s">
         <v>21</v>
       </c>
-      <c r="AB3" s="222"/>
-      <c r="AC3" s="222"/>
-      <c r="AD3" s="222"/>
-      <c r="AE3" s="222"/>
-      <c r="AF3" s="222"/>
-      <c r="AG3" s="222"/>
-      <c r="AH3" s="223"/>
-    </row>
-    <row r="4" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="5" spans="2:34" x14ac:dyDescent="0.45">
-      <c r="B5" s="229" t="s">
+      <c r="AB3" s="210"/>
+      <c r="AC3" s="210"/>
+      <c r="AD3" s="210"/>
+      <c r="AE3" s="210"/>
+      <c r="AF3" s="210"/>
+      <c r="AG3" s="210"/>
+      <c r="AH3" s="211"/>
+    </row>
+    <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:34" x14ac:dyDescent="0.25">
+      <c r="B5" s="217" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="227" t="s">
+      <c r="C5" s="215" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="227"/>
-      <c r="E5" s="227"/>
-      <c r="F5" s="227"/>
-      <c r="G5" s="227"/>
-      <c r="H5" s="227"/>
-      <c r="I5" s="227"/>
-      <c r="J5" s="228"/>
-    </row>
-    <row r="6" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="230"/>
+      <c r="D5" s="215"/>
+      <c r="E5" s="215"/>
+      <c r="F5" s="215"/>
+      <c r="G5" s="215"/>
+      <c r="H5" s="215"/>
+      <c r="I5" s="215"/>
+      <c r="J5" s="216"/>
+    </row>
+    <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="218"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3558,22 +3567,22 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="2:34" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:34" x14ac:dyDescent="0.25">
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="206" t="s">
+      <c r="C7" s="219" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="207"/>
-      <c r="E7" s="207"/>
-      <c r="F7" s="207"/>
-      <c r="G7" s="207"/>
-      <c r="H7" s="207"/>
-      <c r="I7" s="207"/>
-      <c r="J7" s="208"/>
-    </row>
-    <row r="8" spans="2:34" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D7" s="220"/>
+      <c r="E7" s="220"/>
+      <c r="F7" s="220"/>
+      <c r="G7" s="220"/>
+      <c r="H7" s="220"/>
+      <c r="I7" s="220"/>
+      <c r="J7" s="221"/>
+    </row>
+    <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
         <v>1</v>
       </c>
@@ -3581,25 +3590,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="209" t="s">
+      <c r="G8" s="222" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="210"/>
-      <c r="I8" s="210"/>
-      <c r="J8" s="211"/>
+      <c r="H8" s="223"/>
+      <c r="I8" s="223"/>
+      <c r="J8" s="224"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="K3:M3"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="C3:G3"/>
     <mergeCell ref="S3:Z3"/>
     <mergeCell ref="AA3:AH3"/>
     <mergeCell ref="N3:P3"/>
     <mergeCell ref="C5:J5"/>
     <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="K3:M3"/>
-    <mergeCell ref="H3:J3"/>
-    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3609,38 +3618,38 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8B20B11-9266-4E5E-A2B3-3496A1A10C3B}">
   <dimension ref="B1:Q35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.1328125" style="1"/>
-    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.73046875" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="1"/>
+    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.7109375" customWidth="1"/>
     <col min="13" max="13" width="14" customWidth="1"/>
-    <col min="14" max="14" width="90.265625" customWidth="1"/>
+    <col min="14" max="14" width="90.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.45">
-      <c r="B2" s="231" t="s">
+    <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B2" s="256" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="233"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="258"/>
       <c r="H2" s="201" t="s">
         <v>46</v>
       </c>
       <c r="I2" s="201" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="231" t="s">
+      <c r="J2" s="256" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
       <c r="M2" s="201" t="s">
         <v>94</v>
       </c>
@@ -3648,7 +3657,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
@@ -3681,7 +3690,7 @@
       <c r="M3" s="202"/>
       <c r="N3" s="202"/>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="80">
         <v>0</v>
       </c>
@@ -3705,7 +3714,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="234" t="s">
+      <c r="H4" s="233" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
@@ -3717,7 +3726,7 @@
       <c r="K4" s="197" t="s">
         <v>97</v>
       </c>
-      <c r="L4" s="243" t="s">
+      <c r="L4" s="240" t="s">
         <v>16</v>
       </c>
       <c r="M4" s="69" t="s">
@@ -3727,7 +3736,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="82">
         <v>1</v>
       </c>
@@ -3751,7 +3760,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="235"/>
+      <c r="H5" s="232"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -3769,7 +3778,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="6" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B6" s="81">
         <v>2</v>
       </c>
@@ -3793,29 +3802,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="236" t="s">
+      <c r="H6" s="231" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="237" t="s">
+      <c r="J6" s="235" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="239" t="s">
+      <c r="K6" s="251" t="s">
         <v>57</v>
       </c>
       <c r="L6" s="241" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="249" t="s">
+      <c r="M6" s="243" t="s">
         <v>95</v>
       </c>
-      <c r="N6" s="244" t="s">
+      <c r="N6" s="248" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B7" s="81">
         <v>3</v>
       </c>
@@ -3839,17 +3848,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="236"/>
+      <c r="H7" s="231"/>
       <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="237"/>
-      <c r="K7" s="239"/>
+      <c r="J7" s="235"/>
+      <c r="K7" s="251"/>
       <c r="L7" s="241"/>
-      <c r="M7" s="250"/>
-      <c r="N7" s="244"/>
-    </row>
-    <row r="8" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M7" s="254"/>
+      <c r="N7" s="248"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="81">
         <v>4</v>
       </c>
@@ -3873,17 +3882,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="236"/>
+      <c r="H8" s="231"/>
       <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="237"/>
-      <c r="K8" s="239"/>
+      <c r="J8" s="235"/>
+      <c r="K8" s="251"/>
       <c r="L8" s="241"/>
-      <c r="M8" s="250"/>
-      <c r="N8" s="244"/>
-    </row>
-    <row r="9" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M8" s="254"/>
+      <c r="N8" s="248"/>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="81">
         <v>5</v>
       </c>
@@ -3907,17 +3916,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="236"/>
+      <c r="H9" s="231"/>
       <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="237"/>
-      <c r="K9" s="239"/>
+      <c r="J9" s="235"/>
+      <c r="K9" s="251"/>
       <c r="L9" s="241"/>
-      <c r="M9" s="250"/>
-      <c r="N9" s="244"/>
-    </row>
-    <row r="10" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M9" s="254"/>
+      <c r="N9" s="248"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="81">
         <v>6</v>
       </c>
@@ -3941,17 +3950,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="236"/>
+      <c r="H10" s="231"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="237"/>
-      <c r="K10" s="239"/>
+      <c r="J10" s="235"/>
+      <c r="K10" s="251"/>
       <c r="L10" s="241"/>
-      <c r="M10" s="250"/>
-      <c r="N10" s="244"/>
-    </row>
-    <row r="11" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M10" s="254"/>
+      <c r="N10" s="248"/>
+    </row>
+    <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="82">
         <v>7</v>
       </c>
@@ -3975,17 +3984,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="235"/>
+      <c r="H11" s="232"/>
       <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="238"/>
-      <c r="K11" s="240"/>
+      <c r="J11" s="236"/>
+      <c r="K11" s="252"/>
       <c r="L11" s="242"/>
-      <c r="M11" s="251"/>
-      <c r="N11" s="245"/>
-    </row>
-    <row r="12" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M11" s="255"/>
+      <c r="N11" s="249"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="80">
         <v>8</v>
       </c>
@@ -4009,29 +4018,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="234" t="s">
+      <c r="H12" s="233" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="246" t="s">
+      <c r="J12" s="234" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="247" t="s">
+      <c r="K12" s="250" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="243" t="s">
+      <c r="L12" s="240" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="234" t="s">
+      <c r="M12" s="233" t="s">
         <v>96</v>
       </c>
-      <c r="N12" s="248" t="s">
+      <c r="N12" s="253" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="13" spans="2:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B13" s="81">
         <v>9</v>
       </c>
@@ -4055,17 +4064,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="236"/>
+      <c r="H13" s="231"/>
       <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="237"/>
-      <c r="K13" s="239"/>
+      <c r="J13" s="235"/>
+      <c r="K13" s="251"/>
       <c r="L13" s="241"/>
-      <c r="M13" s="236"/>
-      <c r="N13" s="244"/>
-    </row>
-    <row r="14" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M13" s="231"/>
+      <c r="N13" s="248"/>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="81">
         <v>10</v>
       </c>
@@ -4089,17 +4098,17 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="236"/>
+      <c r="H14" s="231"/>
       <c r="I14" s="90" t="s">
         <v>86</v>
       </c>
-      <c r="J14" s="237"/>
-      <c r="K14" s="239"/>
+      <c r="J14" s="235"/>
+      <c r="K14" s="251"/>
       <c r="L14" s="241"/>
-      <c r="M14" s="236"/>
-      <c r="N14" s="244"/>
-    </row>
-    <row r="15" spans="2:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M14" s="231"/>
+      <c r="N14" s="248"/>
+    </row>
+    <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="82">
         <v>11</v>
       </c>
@@ -4123,17 +4132,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="235"/>
+      <c r="H15" s="232"/>
       <c r="I15" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="J15" s="238"/>
-      <c r="K15" s="240"/>
+      <c r="J15" s="236"/>
+      <c r="K15" s="252"/>
       <c r="L15" s="242"/>
-      <c r="M15" s="235"/>
-      <c r="N15" s="245"/>
-    </row>
-    <row r="16" spans="2:14" x14ac:dyDescent="0.45">
+      <c r="M15" s="232"/>
+      <c r="N15" s="249"/>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="80">
         <v>12</v>
       </c>
@@ -4157,29 +4166,29 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="234" t="s">
+      <c r="H16" s="233" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="246" t="s">
+      <c r="J16" s="234" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="252" t="s">
+      <c r="K16" s="237" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="243" t="s">
+      <c r="L16" s="240" t="s">
         <v>55</v>
       </c>
-      <c r="M16" s="234" t="s">
+      <c r="M16" s="233" t="s">
         <v>96</v>
       </c>
       <c r="N16" s="75" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="81">
         <v>13</v>
       </c>
@@ -4203,19 +4212,19 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="236"/>
+      <c r="H17" s="231"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="237"/>
-      <c r="K17" s="253"/>
+      <c r="J17" s="235"/>
+      <c r="K17" s="238"/>
       <c r="L17" s="241"/>
-      <c r="M17" s="236"/>
+      <c r="M17" s="231"/>
       <c r="N17" s="74" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B18" s="81">
         <v>14</v>
       </c>
@@ -4239,19 +4248,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="236"/>
+      <c r="H18" s="231"/>
       <c r="I18" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="J18" s="237"/>
-      <c r="K18" s="253"/>
+      <c r="J18" s="235"/>
+      <c r="K18" s="238"/>
       <c r="L18" s="241"/>
-      <c r="M18" s="236"/>
+      <c r="M18" s="231"/>
       <c r="N18" s="74" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="82">
         <v>15</v>
       </c>
@@ -4275,20 +4284,20 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="235"/>
+      <c r="H19" s="232"/>
       <c r="I19" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="J19" s="238"/>
-      <c r="K19" s="254"/>
+      <c r="J19" s="236"/>
+      <c r="K19" s="239"/>
       <c r="L19" s="242"/>
-      <c r="M19" s="235"/>
+      <c r="M19" s="232"/>
       <c r="N19" s="44" t="s">
         <v>92</v>
       </c>
       <c r="P19" s="1"/>
     </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B20" s="80">
         <v>16</v>
       </c>
@@ -4312,7 +4321,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="234" t="s">
+      <c r="H20" s="233" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="192" t="s">
@@ -4321,20 +4330,20 @@
       <c r="J20" s="140" t="s">
         <v>151</v>
       </c>
-      <c r="K20" s="252" t="s">
+      <c r="K20" s="237" t="s">
         <v>53</v>
       </c>
-      <c r="L20" s="257" t="s">
+      <c r="L20" s="246" t="s">
         <v>55</v>
       </c>
-      <c r="M20" s="249" t="s">
+      <c r="M20" s="243" t="s">
         <v>95</v>
       </c>
       <c r="N20" s="194" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B21" s="81">
         <v>17</v>
       </c>
@@ -4358,21 +4367,21 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="236"/>
+      <c r="H21" s="231"/>
       <c r="I21" s="193" t="s">
         <v>100</v>
       </c>
       <c r="J21" s="99" t="s">
         <v>151</v>
       </c>
-      <c r="K21" s="256"/>
-      <c r="L21" s="258"/>
-      <c r="M21" s="255"/>
+      <c r="K21" s="245"/>
+      <c r="L21" s="247"/>
+      <c r="M21" s="244"/>
       <c r="N21" s="195" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B22" s="81">
         <v>18</v>
       </c>
@@ -4396,7 +4405,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="236"/>
+      <c r="H22" s="231"/>
       <c r="I22" s="103"/>
       <c r="J22" s="136"/>
       <c r="K22" s="137"/>
@@ -4404,7 +4413,7 @@
       <c r="M22" s="104"/>
       <c r="N22" s="104"/>
     </row>
-    <row r="23" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="81">
         <v>19</v>
       </c>
@@ -4428,7 +4437,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="235"/>
+      <c r="H23" s="232"/>
       <c r="I23" s="96"/>
       <c r="J23" s="133"/>
       <c r="K23" s="134"/>
@@ -4436,7 +4445,7 @@
       <c r="M23" s="132"/>
       <c r="N23" s="132"/>
     </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B24" s="80">
         <v>20</v>
       </c>
@@ -4460,7 +4469,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="234" t="s">
+      <c r="H24" s="233" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -4482,7 +4491,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B25" s="81">
         <v>21</v>
       </c>
@@ -4506,7 +4515,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="236"/>
+      <c r="H25" s="231"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -4526,7 +4535,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B26" s="81">
         <v>22</v>
       </c>
@@ -4550,7 +4559,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="236"/>
+      <c r="H26" s="231"/>
       <c r="I26" s="103"/>
       <c r="J26" s="136"/>
       <c r="K26" s="137"/>
@@ -4558,7 +4567,7 @@
       <c r="M26" s="104"/>
       <c r="N26" s="104"/>
     </row>
-    <row r="27" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="27" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="82">
         <v>23</v>
       </c>
@@ -4582,7 +4591,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="235"/>
+      <c r="H27" s="232"/>
       <c r="I27" s="96"/>
       <c r="J27" s="133"/>
       <c r="K27" s="134"/>
@@ -4590,7 +4599,7 @@
       <c r="M27" s="132"/>
       <c r="N27" s="132"/>
     </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B28" s="80">
         <v>24</v>
       </c>
@@ -4614,7 +4623,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="234" t="s">
+      <c r="H28" s="233" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -4636,7 +4645,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B29" s="81">
         <v>25</v>
       </c>
@@ -4660,7 +4669,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="236"/>
+      <c r="H29" s="231"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -4680,7 +4689,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B30" s="81">
         <v>26</v>
       </c>
@@ -4704,7 +4713,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="236"/>
+      <c r="H30" s="231"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -4724,7 +4733,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="31" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="82">
         <v>27</v>
       </c>
@@ -4748,7 +4757,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="235"/>
+      <c r="H31" s="232"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -4756,7 +4765,7 @@
       <c r="M31" s="95"/>
       <c r="N31" s="93"/>
     </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B32" s="81">
         <v>28</v>
       </c>
@@ -4780,7 +4789,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="236" t="s">
+      <c r="H32" s="231" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -4803,7 +4812,7 @@
       </c>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B33" s="81">
         <v>29</v>
       </c>
@@ -4827,7 +4836,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="236"/>
+      <c r="H33" s="231"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -4848,7 +4857,7 @@
       </c>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="81">
         <v>30</v>
       </c>
@@ -4872,7 +4881,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="235"/>
+      <c r="H34" s="232"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -4893,7 +4902,7 @@
       </c>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35" spans="2:17" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="83">
         <v>31</v>
       </c>
@@ -4941,18 +4950,18 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="M20:M21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="L4:L5"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4961,18 +4970,18 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="M20:M21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:L21"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4982,42 +4991,42 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD788E61-AC5A-4E7F-9536-02553AF94143}">
   <dimension ref="B1:P35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="9" style="1"/>
-    <col min="3" max="7" width="4.73046875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="14.265625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="16.73046875" style="1" customWidth="1"/>
-    <col min="10" max="12" width="20.73046875" customWidth="1"/>
-    <col min="13" max="13" width="90.265625" customWidth="1"/>
+    <col min="3" max="7" width="4.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.28515625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16.7109375" style="1" customWidth="1"/>
+    <col min="10" max="12" width="20.7109375" customWidth="1"/>
+    <col min="13" max="13" width="90.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.45">
-      <c r="B2" s="231" t="s">
+    <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B2" s="256" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="232"/>
-      <c r="F2" s="232"/>
-      <c r="G2" s="233"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="257"/>
+      <c r="F2" s="257"/>
+      <c r="G2" s="258"/>
       <c r="H2" s="201" t="s">
         <v>46</v>
       </c>
       <c r="I2" s="201" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="231" t="s">
+      <c r="J2" s="256" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="232"/>
-      <c r="L2" s="232"/>
+      <c r="K2" s="257"/>
+      <c r="L2" s="257"/>
       <c r="M2" s="201" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="84" t="s">
         <v>16</v>
       </c>
@@ -5049,7 +5058,7 @@
       </c>
       <c r="M3" s="202"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="80">
         <v>0</v>
       </c>
@@ -5073,7 +5082,7 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="234" t="s">
+      <c r="H4" s="233" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
@@ -5092,7 +5101,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="82">
         <v>1</v>
       </c>
@@ -5116,7 +5125,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="235"/>
+      <c r="H5" s="232"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -5133,7 +5142,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B6" s="81">
         <v>2</v>
       </c>
@@ -5157,26 +5166,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="236" t="s">
+      <c r="H6" s="231" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="237" t="s">
+      <c r="J6" s="235" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="239" t="s">
+      <c r="K6" s="251" t="s">
         <v>57</v>
       </c>
       <c r="L6" s="241" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="244" t="s">
+      <c r="M6" s="248" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B7" s="81">
         <v>3</v>
       </c>
@@ -5200,14 +5209,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="236"/>
+      <c r="H7" s="231"/>
       <c r="I7" s="259"/>
-      <c r="J7" s="237"/>
-      <c r="K7" s="239"/>
+      <c r="J7" s="235"/>
+      <c r="K7" s="251"/>
       <c r="L7" s="241"/>
-      <c r="M7" s="244"/>
-    </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M7" s="248"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="81">
         <v>4</v>
       </c>
@@ -5231,14 +5240,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="236"/>
-      <c r="I8" s="260"/>
-      <c r="J8" s="237"/>
-      <c r="K8" s="239"/>
+      <c r="H8" s="231"/>
+      <c r="I8" s="272"/>
+      <c r="J8" s="235"/>
+      <c r="K8" s="251"/>
       <c r="L8" s="241"/>
-      <c r="M8" s="244"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M8" s="248"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="81">
         <v>5</v>
       </c>
@@ -5262,14 +5271,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="236"/>
-      <c r="I9" s="261"/>
-      <c r="J9" s="237"/>
-      <c r="K9" s="239"/>
+      <c r="H9" s="231"/>
+      <c r="I9" s="273"/>
+      <c r="J9" s="235"/>
+      <c r="K9" s="251"/>
       <c r="L9" s="241"/>
-      <c r="M9" s="244"/>
-    </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M9" s="248"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="81">
         <v>6</v>
       </c>
@@ -5293,16 +5302,16 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="236"/>
+      <c r="H10" s="231"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="237"/>
-      <c r="K10" s="239"/>
+      <c r="J10" s="235"/>
+      <c r="K10" s="251"/>
       <c r="L10" s="241"/>
-      <c r="M10" s="244"/>
-    </row>
-    <row r="11" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M10" s="248"/>
+    </row>
+    <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="82">
         <v>7</v>
       </c>
@@ -5326,14 +5335,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="235"/>
+      <c r="H11" s="232"/>
       <c r="I11" s="103"/>
-      <c r="J11" s="238"/>
-      <c r="K11" s="240"/>
+      <c r="J11" s="236"/>
+      <c r="K11" s="252"/>
       <c r="L11" s="242"/>
-      <c r="M11" s="245"/>
-    </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M11" s="249"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="80">
         <v>8</v>
       </c>
@@ -5357,26 +5366,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="234" t="s">
+      <c r="H12" s="233" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="246" t="s">
+      <c r="J12" s="234" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="247" t="s">
+      <c r="K12" s="250" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="243" t="s">
+      <c r="L12" s="240" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="248" t="s">
+      <c r="M12" s="253" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="2:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B13" s="81">
         <v>9</v>
       </c>
@@ -5400,14 +5409,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="236"/>
+      <c r="H13" s="231"/>
       <c r="I13" s="259"/>
-      <c r="J13" s="237"/>
-      <c r="K13" s="239"/>
+      <c r="J13" s="235"/>
+      <c r="K13" s="251"/>
       <c r="L13" s="241"/>
-      <c r="M13" s="244"/>
-    </row>
-    <row r="14" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M13" s="248"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="81">
         <v>10</v>
       </c>
@@ -5431,14 +5440,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="236"/>
-      <c r="I14" s="260"/>
-      <c r="J14" s="237"/>
-      <c r="K14" s="239"/>
+      <c r="H14" s="231"/>
+      <c r="I14" s="272"/>
+      <c r="J14" s="235"/>
+      <c r="K14" s="251"/>
       <c r="L14" s="241"/>
-      <c r="M14" s="244"/>
-    </row>
-    <row r="15" spans="2:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="M14" s="248"/>
+    </row>
+    <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="82">
         <v>11</v>
       </c>
@@ -5462,14 +5471,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="235"/>
-      <c r="I15" s="262"/>
-      <c r="J15" s="238"/>
-      <c r="K15" s="240"/>
+      <c r="H15" s="232"/>
+      <c r="I15" s="260"/>
+      <c r="J15" s="236"/>
+      <c r="K15" s="252"/>
       <c r="L15" s="242"/>
-      <c r="M15" s="245"/>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.45">
+      <c r="M15" s="249"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="80">
         <v>12</v>
       </c>
@@ -5493,26 +5502,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="234" t="s">
+      <c r="H16" s="233" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="246" t="s">
+      <c r="J16" s="234" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="252" t="s">
+      <c r="K16" s="237" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="243" t="s">
+      <c r="L16" s="240" t="s">
         <v>55</v>
       </c>
       <c r="M16" s="75" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B17" s="81">
         <v>13</v>
       </c>
@@ -5536,18 +5545,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="236"/>
+      <c r="H17" s="231"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="237"/>
-      <c r="K17" s="253"/>
+      <c r="J17" s="235"/>
+      <c r="K17" s="238"/>
       <c r="L17" s="241"/>
       <c r="M17" s="74" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B18" s="81">
         <v>14</v>
       </c>
@@ -5571,14 +5580,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="236"/>
+      <c r="H18" s="231"/>
       <c r="I18" s="259"/>
-      <c r="J18" s="237"/>
-      <c r="K18" s="253"/>
+      <c r="J18" s="235"/>
+      <c r="K18" s="238"/>
       <c r="L18" s="241"/>
       <c r="M18" s="259"/>
     </row>
-    <row r="19" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="82">
         <v>15</v>
       </c>
@@ -5602,15 +5611,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="235"/>
-      <c r="I19" s="262"/>
-      <c r="J19" s="238"/>
-      <c r="K19" s="254"/>
+      <c r="H19" s="232"/>
+      <c r="I19" s="260"/>
+      <c r="J19" s="236"/>
+      <c r="K19" s="239"/>
       <c r="L19" s="242"/>
-      <c r="M19" s="262"/>
+      <c r="M19" s="260"/>
       <c r="O19" s="1"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="80">
         <v>16</v>
       </c>
@@ -5634,7 +5643,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="263" t="s">
+      <c r="H20" s="261" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="176" t="s">
@@ -5653,7 +5662,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B21" s="81">
         <v>17</v>
       </c>
@@ -5677,14 +5686,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="264"/>
+      <c r="H21" s="262"/>
       <c r="I21" s="167"/>
       <c r="J21" s="169"/>
       <c r="K21" s="171"/>
       <c r="L21" s="173"/>
       <c r="M21" s="167"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="81">
         <v>18</v>
       </c>
@@ -5708,14 +5717,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="264"/>
+      <c r="H22" s="262"/>
       <c r="I22" s="167"/>
       <c r="J22" s="169"/>
       <c r="K22" s="171"/>
       <c r="L22" s="173"/>
       <c r="M22" s="167"/>
     </row>
-    <row r="23" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="23" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="81">
         <v>19</v>
       </c>
@@ -5739,14 +5748,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="265"/>
+      <c r="H23" s="263"/>
       <c r="I23" s="168"/>
       <c r="J23" s="170"/>
       <c r="K23" s="172"/>
       <c r="L23" s="174"/>
       <c r="M23" s="168"/>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B24" s="80">
         <v>20</v>
       </c>
@@ -5770,7 +5779,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="234" t="s">
+      <c r="H24" s="233" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -5789,7 +5798,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B25" s="81">
         <v>21</v>
       </c>
@@ -5813,7 +5822,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="236"/>
+      <c r="H25" s="231"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -5830,7 +5839,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B26" s="81">
         <v>22</v>
       </c>
@@ -5854,14 +5863,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="236"/>
+      <c r="H26" s="231"/>
       <c r="I26" s="259"/>
-      <c r="J26" s="266"/>
-      <c r="K26" s="268"/>
-      <c r="L26" s="270"/>
-      <c r="M26" s="272"/>
-    </row>
-    <row r="27" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="J26" s="264"/>
+      <c r="K26" s="266"/>
+      <c r="L26" s="268"/>
+      <c r="M26" s="270"/>
+    </row>
+    <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="82">
         <v>23</v>
       </c>
@@ -5885,14 +5894,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="235"/>
-      <c r="I27" s="262"/>
-      <c r="J27" s="267"/>
-      <c r="K27" s="269"/>
-      <c r="L27" s="271"/>
-      <c r="M27" s="273"/>
-    </row>
-    <row r="28" spans="2:16" x14ac:dyDescent="0.45">
+      <c r="H27" s="232"/>
+      <c r="I27" s="260"/>
+      <c r="J27" s="265"/>
+      <c r="K27" s="267"/>
+      <c r="L27" s="269"/>
+      <c r="M27" s="271"/>
+    </row>
+    <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="80">
         <v>24</v>
       </c>
@@ -5916,7 +5925,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="234" t="s">
+      <c r="H28" s="233" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -5935,7 +5944,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="29" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B29" s="81">
         <v>25</v>
       </c>
@@ -5959,7 +5968,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="236"/>
+      <c r="H29" s="231"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -5976,7 +5985,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="30" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B30" s="81">
         <v>26</v>
       </c>
@@ -6000,7 +6009,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="236"/>
+      <c r="H30" s="231"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -6017,7 +6026,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B31" s="82">
         <v>27</v>
       </c>
@@ -6041,14 +6050,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="235"/>
+      <c r="H31" s="232"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
       <c r="L31" s="164"/>
       <c r="M31" s="93"/>
     </row>
-    <row r="32" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B32" s="81">
         <v>28</v>
       </c>
@@ -6072,7 +6081,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="236" t="s">
+      <c r="H32" s="231" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -6092,7 +6101,7 @@
       </c>
       <c r="P32" s="1"/>
     </row>
-    <row r="33" spans="2:16" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B33" s="81">
         <v>29</v>
       </c>
@@ -6116,7 +6125,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="236"/>
+      <c r="H33" s="231"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -6134,7 +6143,7 @@
       </c>
       <c r="P33" s="1"/>
     </row>
-    <row r="34" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="34" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B34" s="81">
         <v>30</v>
       </c>
@@ -6158,7 +6167,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="235"/>
+      <c r="H34" s="232"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -6176,7 +6185,7 @@
       </c>
       <c r="P34" s="1"/>
     </row>
-    <row r="35" spans="2:16" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="35" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="83">
         <v>31</v>
       </c>
@@ -6221,6 +6230,24 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6236,24 +6263,6 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6263,24 +6272,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4182B34D-1176-43D9-83DE-D8E7EA5C96ED}">
   <dimension ref="B1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="5" width="4.73046875" customWidth="1"/>
+    <col min="3" max="5" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.45">
-      <c r="B2" s="231" t="s">
+    <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="256" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="232"/>
-      <c r="D2" s="232"/>
-      <c r="E2" s="233"/>
+      <c r="C2" s="257"/>
+      <c r="D2" s="257"/>
+      <c r="E2" s="258"/>
       <c r="F2" s="201" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="2:6" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
@@ -6295,7 +6304,7 @@
       </c>
       <c r="F3" s="202"/>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="13">
         <v>0</v>
       </c>
@@ -6315,7 +6324,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="13">
         <v>1</v>
       </c>
@@ -6335,7 +6344,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="19">
         <v>2</v>
       </c>
@@ -6355,7 +6364,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B7" s="22">
         <v>3</v>
       </c>
@@ -6375,7 +6384,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B8" s="13">
         <v>4</v>
       </c>
@@ -6395,7 +6404,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="13">
         <v>5</v>
       </c>
@@ -6415,7 +6424,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B10" s="19">
         <v>6</v>
       </c>
@@ -6435,7 +6444,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B11" s="22">
         <v>7</v>
       </c>
@@ -6467,13 +6476,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{197DCCAF-E75B-41F9-A939-BF94359E828F}">
   <dimension ref="B1:R9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="14.265625" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" s="201" t="s">
         <v>69</v>
       </c>
@@ -6496,7 +6505,7 @@
       <c r="Q2" s="284"/>
       <c r="R2" s="285"/>
     </row>
-    <row r="3" spans="2:18" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="202"/>
       <c r="C3" s="116">
         <v>15</v>
@@ -6547,7 +6556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="87" t="s">
         <v>70</v>
       </c>
@@ -6576,7 +6585,7 @@
       <c r="Q4" s="277"/>
       <c r="R4" s="278"/>
     </row>
-    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="88" t="s">
         <v>3</v>
       </c>
@@ -6599,7 +6608,7 @@
       <c r="Q5" s="275"/>
       <c r="R5" s="276"/>
     </row>
-    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="88" t="s">
         <v>2</v>
       </c>
@@ -6622,7 +6631,7 @@
       <c r="Q6" s="275"/>
       <c r="R6" s="276"/>
     </row>
-    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="88" t="s">
         <v>71</v>
       </c>
@@ -6645,7 +6654,7 @@
       <c r="Q7" s="281"/>
       <c r="R7" s="282"/>
     </row>
-    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="88" t="s">
         <v>72</v>
       </c>
@@ -6668,7 +6677,7 @@
       <c r="Q8" s="275"/>
       <c r="R8" s="276"/>
     </row>
-    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="89" t="s">
         <v>78</v>
       </c>
@@ -6712,16 +6721,16 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
-  <dimension ref="B1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="B1:E9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21.1328125" customWidth="1"/>
-    <col min="3" max="3" width="82.265625" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="3" max="3" width="82.28515625" customWidth="1"/>
+    <col min="4" max="5" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="156" t="s">
         <v>127</v>
       </c>
@@ -6731,8 +6740,11 @@
       <c r="D2" s="158" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E2" s="158" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B3" s="159" t="s">
         <v>129</v>
       </c>
@@ -6742,8 +6754,11 @@
       <c r="D3" s="74" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E3" s="74" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="157" t="s">
         <v>131</v>
       </c>
@@ -6753,8 +6768,11 @@
       <c r="D4" s="41" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E4" s="41" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="159" t="s">
         <v>133</v>
       </c>
@@ -6764,8 +6782,11 @@
       <c r="D5" s="74" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E5" s="74" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="159" t="s">
         <v>101</v>
       </c>
@@ -6775,8 +6796,11 @@
       <c r="D6" s="74" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E6" s="74" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="159" t="s">
         <v>141</v>
       </c>
@@ -6786,8 +6810,11 @@
       <c r="D7" s="74" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="E7" s="74" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="157" t="s">
         <v>38</v>
       </c>
@@ -6797,8 +6824,11 @@
       <c r="D8" s="41" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="9" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="E8" s="41" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="160" t="s">
         <v>190</v>
       </c>
@@ -6806,6 +6836,9 @@
         <v>142</v>
       </c>
       <c r="D9" s="161" t="s">
+        <v>192</v>
+      </c>
+      <c r="E9" s="161" t="s">
         <v>192</v>
       </c>
     </row>
@@ -6817,20 +6850,20 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7D036B2-790A-4A3D-BD75-883CE886D2D8}">
   <dimension ref="B1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="7.265625" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="286" t="s">
         <v>117</v>
       </c>
       <c r="C2" s="287"/>
       <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="139" t="s">
         <v>115</v>
       </c>
@@ -6839,7 +6872,7 @@
       </c>
       <c r="D3" s="1"/>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="92"/>
       <c r="C4" s="130" t="s">
         <v>119</v>
@@ -6848,21 +6881,21 @@
         <v>124</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="94"/>
       <c r="C5" s="131" t="s">
         <v>118</v>
       </c>
       <c r="D5" s="289"/>
     </row>
-    <row r="6" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="133"/>
       <c r="C6" s="63" t="s">
         <v>120</v>
       </c>
       <c r="D6" s="290"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="140" t="s">
         <v>119</v>
       </c>
@@ -6871,21 +6904,21 @@
         <v>125</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="40" t="s">
         <v>118</v>
       </c>
       <c r="C8" s="142"/>
       <c r="D8" s="292"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="40" t="s">
         <v>120</v>
       </c>
       <c r="C9" s="142"/>
       <c r="D9" s="292"/>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="143" t="s">
         <v>121</v>
       </c>
@@ -6894,7 +6927,7 @@
       </c>
       <c r="D10" s="292"/>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="40" t="s">
         <v>118</v>
       </c>
@@ -6904,7 +6937,7 @@
       <c r="D11" s="292"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="2:5" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="145" t="s">
         <v>122</v>
       </c>
@@ -6926,13 +6959,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{728A29D2-349C-45CC-BF5A-2F605D047162}">
   <dimension ref="B1:D40"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="4" width="38.59765625" customWidth="1"/>
+    <col min="3" max="4" width="38.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="294" t="s">
         <v>165</v>
       </c>
@@ -6941,7 +6974,7 @@
       </c>
       <c r="D2" s="297"/>
     </row>
-    <row r="3" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="295"/>
       <c r="C3" s="185" t="s">
         <v>161</v>
@@ -6950,18 +6983,18 @@
         <v>162</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="88">
         <v>0</v>
       </c>
       <c r="C4" s="143" t="s">
         <v>169</v>
       </c>
-      <c r="D4" s="243" t="s">
+      <c r="D4" s="240" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="177">
         <v>1</v>
       </c>
@@ -6970,7 +7003,7 @@
       </c>
       <c r="D5" s="298"/>
     </row>
-    <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="88">
         <v>2</v>
       </c>
@@ -6981,35 +7014,35 @@
         <v>163</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="177">
         <v>3</v>
       </c>
-      <c r="C7" s="237"/>
+      <c r="C7" s="235"/>
       <c r="D7" s="241"/>
     </row>
-    <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="88">
         <v>4</v>
       </c>
       <c r="C8" s="301"/>
       <c r="D8" s="298"/>
     </row>
-    <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="177">
         <v>5</v>
       </c>
       <c r="C9" s="94"/>
       <c r="D9" s="179"/>
     </row>
-    <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="88">
         <v>6</v>
       </c>
       <c r="C10" s="136"/>
       <c r="D10" s="142"/>
     </row>
-    <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="178">
         <v>7</v>
       </c>
@@ -7018,8 +7051,8 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="187" t="s">
         <v>167</v>
       </c>
@@ -7027,7 +7060,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="88">
         <v>0</v>
       </c>
@@ -7035,7 +7068,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.45">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="177">
         <v>1</v>
       </c>
@@ -7043,7 +7076,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="88">
         <v>2</v>
       </c>
@@ -7051,7 +7084,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="177">
         <v>3</v>
       </c>
@@ -7059,7 +7092,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="88">
         <v>4</v>
       </c>
@@ -7067,31 +7100,31 @@
         <v>154</v>
       </c>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" s="177">
         <v>5</v>
       </c>
       <c r="C20" s="181"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" s="88">
         <v>6</v>
       </c>
       <c r="C21" s="26"/>
     </row>
-    <row r="22" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="22" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="178">
         <v>7</v>
       </c>
       <c r="C22" s="184"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="24" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="187" t="s">
         <v>167</v>
       </c>
@@ -7099,7 +7132,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26" s="88">
         <v>0</v>
       </c>
@@ -7107,7 +7140,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27" s="177">
         <v>1</v>
       </c>
@@ -7115,7 +7148,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="88">
         <v>2</v>
       </c>
@@ -7123,7 +7156,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="29" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="182">
         <v>3</v>
       </c>
@@ -7131,8 +7164,8 @@
         <v>160</v>
       </c>
     </row>
-    <row r="31" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="187" t="s">
         <v>167</v>
       </c>
@@ -7140,7 +7173,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="88">
         <v>0</v>
       </c>
@@ -7148,7 +7181,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="177">
         <v>1</v>
       </c>
@@ -7156,7 +7189,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="88">
         <v>2</v>
       </c>
@@ -7164,7 +7197,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="36" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36" s="177">
         <v>3</v>
       </c>
@@ -7172,7 +7205,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37" s="88">
         <v>4</v>
       </c>
@@ -7180,7 +7213,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="177">
         <v>5</v>
       </c>
@@ -7188,7 +7221,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.45">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39" s="91">
         <v>6</v>
       </c>
@@ -7196,7 +7229,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="40" spans="2:3" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="182">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Sequencer ⏰ Revert changes to hold line and improve timings
This fixes a bug with the carry unit
</commit_message>
<xml_diff>
--- a/ax08.xlsx
+++ b/ax08.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projects\computer\ax08\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD679EB-A19D-48CF-9A6B-3A922191C871}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E74F170-AE22-4EF2-A897-36A6E73B7472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11835" activeTab="6" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="6" xr2:uid="{9E4BE3C4-600D-4A58-9D6E-A286F07640A8}"/>
   </bookViews>
   <sheets>
     <sheet name="registers" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="199">
   <si>
     <t>MODE B</t>
   </si>
@@ -482,13 +482,7 @@
     <t>FREEZE_OP ↑, (FREEZE_WRD ↓)</t>
   </si>
   <si>
-    <t>HOLD ↑, PC_SOURCE_INC ↑, (FREEZE_OP ↓)</t>
-  </si>
-  <si>
     <t>STORE ↑</t>
-  </si>
-  <si>
-    <t>AD_RGSET_OVERRIDE ↑, (HOLD ↓)</t>
   </si>
   <si>
     <t>PC_SOURCE_INC ↓, AD_RGSET_OVERRIDE ↓</t>
@@ -627,13 +621,28 @@
     <t>STORE ↓ (all ↓)</t>
   </si>
   <si>
-    <t>FREEZE_OP ↑, (FREEZE_WRD ↓) (HOLD ↓)</t>
-  </si>
-  <si>
     <t>AD_RGSET_OVERRIDE ↑,</t>
   </si>
   <si>
-    <t>Net action (firmware modules)</t>
+    <t>PRE INCREMENT</t>
+  </si>
+  <si>
+    <t>HOLD ↑, (FREEZE_OP ↓)</t>
+  </si>
+  <si>
+    <t>PC_SOURCE_INC ↑,  HOLD ↓</t>
+  </si>
+  <si>
+    <t>HOLD</t>
+  </si>
+  <si>
+    <t>PC_SOURCE_INC</t>
+  </si>
+  <si>
+    <t>AD_RGSET_OVERRIDE</t>
+  </si>
+  <si>
+    <t>FREEZE INSTR.</t>
   </si>
 </sst>
 </file>
@@ -1621,7 +1630,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="302">
+  <cellXfs count="314">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2163,6 +2172,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2186,6 +2204,42 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2225,91 +2279,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="42" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="45" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="46" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2318,34 +2324,52 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="41" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="38" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="56" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="44" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="67" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2384,12 +2408,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2474,6 +2492,15 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="66" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2823,19 +2850,19 @@
   <sheetData>
     <row r="1" spans="2:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="198" t="s">
+      <c r="B2" s="201" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="199"/>
-      <c r="D2" s="199"/>
-      <c r="E2" s="199"/>
-      <c r="F2" s="200"/>
-      <c r="G2" s="203" t="s">
+      <c r="C2" s="202"/>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="206" t="s">
         <v>24</v>
       </c>
-      <c r="H2" s="204"/>
-      <c r="I2" s="205"/>
-      <c r="J2" s="201" t="s">
+      <c r="H2" s="207"/>
+      <c r="I2" s="208"/>
+      <c r="J2" s="204" t="s">
         <v>25</v>
       </c>
     </row>
@@ -2864,7 +2891,7 @@
       <c r="I3" s="50" t="s">
         <v>114</v>
       </c>
-      <c r="J3" s="202"/>
+      <c r="J3" s="205"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B4" s="105">
@@ -3267,14 +3294,14 @@
         <v>0</v>
       </c>
       <c r="G16" s="118" t="s">
+        <v>170</v>
+      </c>
+      <c r="H16" s="191" t="s">
         <v>172</v>
-      </c>
-      <c r="H16" s="191" t="s">
-        <v>174</v>
       </c>
       <c r="I16" s="113"/>
       <c r="J16" s="26" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="2:10" x14ac:dyDescent="0.25">
@@ -3298,12 +3325,12 @@
         <v>1</v>
       </c>
       <c r="G17" s="118" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H17" s="128"/>
       <c r="I17" s="113"/>
       <c r="J17" s="26" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="18" spans="2:10" x14ac:dyDescent="0.25">
@@ -3475,73 +3502,73 @@
       </c>
     </row>
     <row r="3" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C3" s="228" t="s">
+      <c r="C3" s="218" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="229"/>
-      <c r="E3" s="229"/>
-      <c r="F3" s="229"/>
-      <c r="G3" s="230"/>
-      <c r="H3" s="225" t="s">
+      <c r="D3" s="219"/>
+      <c r="E3" s="219"/>
+      <c r="F3" s="219"/>
+      <c r="G3" s="220"/>
+      <c r="H3" s="215" t="s">
         <v>85</v>
       </c>
-      <c r="I3" s="226"/>
-      <c r="J3" s="227"/>
-      <c r="K3" s="225" t="s">
+      <c r="I3" s="216"/>
+      <c r="J3" s="217"/>
+      <c r="K3" s="215" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="226"/>
-      <c r="M3" s="226"/>
-      <c r="N3" s="212" t="s">
+      <c r="L3" s="216"/>
+      <c r="M3" s="216"/>
+      <c r="N3" s="227" t="s">
         <v>83</v>
       </c>
-      <c r="O3" s="213"/>
-      <c r="P3" s="214"/>
+      <c r="O3" s="228"/>
+      <c r="P3" s="229"/>
       <c r="Q3" s="11" t="s">
         <v>0</v>
       </c>
       <c r="R3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="206" t="s">
+      <c r="S3" s="221" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="207"/>
-      <c r="U3" s="207"/>
-      <c r="V3" s="207"/>
-      <c r="W3" s="207"/>
-      <c r="X3" s="207"/>
-      <c r="Y3" s="207"/>
-      <c r="Z3" s="208"/>
-      <c r="AA3" s="209" t="s">
+      <c r="T3" s="222"/>
+      <c r="U3" s="222"/>
+      <c r="V3" s="222"/>
+      <c r="W3" s="222"/>
+      <c r="X3" s="222"/>
+      <c r="Y3" s="222"/>
+      <c r="Z3" s="223"/>
+      <c r="AA3" s="224" t="s">
         <v>21</v>
       </c>
-      <c r="AB3" s="210"/>
-      <c r="AC3" s="210"/>
-      <c r="AD3" s="210"/>
-      <c r="AE3" s="210"/>
-      <c r="AF3" s="210"/>
-      <c r="AG3" s="210"/>
-      <c r="AH3" s="211"/>
+      <c r="AB3" s="225"/>
+      <c r="AC3" s="225"/>
+      <c r="AD3" s="225"/>
+      <c r="AE3" s="225"/>
+      <c r="AF3" s="225"/>
+      <c r="AG3" s="225"/>
+      <c r="AH3" s="226"/>
     </row>
     <row r="4" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:34" x14ac:dyDescent="0.25">
-      <c r="B5" s="217" t="s">
+      <c r="B5" s="232" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="215" t="s">
+      <c r="C5" s="230" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="215"/>
-      <c r="E5" s="215"/>
-      <c r="F5" s="215"/>
-      <c r="G5" s="215"/>
-      <c r="H5" s="215"/>
-      <c r="I5" s="215"/>
-      <c r="J5" s="216"/>
+      <c r="D5" s="230"/>
+      <c r="E5" s="230"/>
+      <c r="F5" s="230"/>
+      <c r="G5" s="230"/>
+      <c r="H5" s="230"/>
+      <c r="I5" s="230"/>
+      <c r="J5" s="231"/>
     </row>
     <row r="6" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="218"/>
+      <c r="B6" s="233"/>
       <c r="C6" s="7">
         <v>7</v>
       </c>
@@ -3571,16 +3598,16 @@
       <c r="B7" s="9">
         <v>0</v>
       </c>
-      <c r="C7" s="219" t="s">
+      <c r="C7" s="209" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="220"/>
-      <c r="E7" s="220"/>
-      <c r="F7" s="220"/>
-      <c r="G7" s="220"/>
-      <c r="H7" s="220"/>
-      <c r="I7" s="220"/>
-      <c r="J7" s="221"/>
+      <c r="D7" s="210"/>
+      <c r="E7" s="210"/>
+      <c r="F7" s="210"/>
+      <c r="G7" s="210"/>
+      <c r="H7" s="210"/>
+      <c r="I7" s="210"/>
+      <c r="J7" s="211"/>
     </row>
     <row r="8" spans="2:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="6">
@@ -3590,25 +3617,25 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="222" t="s">
+      <c r="G8" s="212" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="223"/>
-      <c r="I8" s="223"/>
-      <c r="J8" s="224"/>
+      <c r="H8" s="213"/>
+      <c r="I8" s="213"/>
+      <c r="J8" s="214"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="S3:Z3"/>
+    <mergeCell ref="AA3:AH3"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="C5:J5"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="C7:J7"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="C3:G3"/>
-    <mergeCell ref="S3:Z3"/>
-    <mergeCell ref="AA3:AH3"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="C5:J5"/>
-    <mergeCell ref="B5:B6"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3631,29 +3658,29 @@
   <sheetData>
     <row r="1" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="234" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="201" t="s">
+      <c r="C2" s="235"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
+      <c r="G2" s="236"/>
+      <c r="H2" s="204" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="201" t="s">
+      <c r="I2" s="204" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="256" t="s">
+      <c r="J2" s="234" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="257"/>
-      <c r="L2" s="257"/>
-      <c r="M2" s="201" t="s">
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
+      <c r="M2" s="204" t="s">
         <v>94</v>
       </c>
-      <c r="N2" s="201" t="s">
+      <c r="N2" s="204" t="s">
         <v>25</v>
       </c>
     </row>
@@ -3676,8 +3703,8 @@
       <c r="G3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="H3" s="205"/>
+      <c r="I3" s="205"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -3687,8 +3714,8 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="202"/>
-      <c r="N3" s="202"/>
+      <c r="M3" s="205"/>
+      <c r="N3" s="205"/>
     </row>
     <row r="4" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B4" s="80">
@@ -3714,11 +3741,11 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="233" t="s">
+      <c r="H4" s="237" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J4" s="196" t="s">
         <v>73</v>
@@ -3726,14 +3753,14 @@
       <c r="K4" s="197" t="s">
         <v>97</v>
       </c>
-      <c r="L4" s="240" t="s">
+      <c r="L4" s="246" t="s">
         <v>16</v>
       </c>
       <c r="M4" s="69" t="s">
         <v>95</v>
       </c>
       <c r="N4" s="75" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3760,7 +3787,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="232"/>
+      <c r="H5" s="238"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -3770,12 +3797,12 @@
       <c r="K5" s="54" t="s">
         <v>53</v>
       </c>
-      <c r="L5" s="242"/>
+      <c r="L5" s="245"/>
       <c r="M5" s="34" t="s">
         <v>95</v>
       </c>
       <c r="N5" s="44" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" spans="2:14" x14ac:dyDescent="0.25">
@@ -3802,25 +3829,25 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="231" t="s">
+      <c r="H6" s="239" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="64" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="240" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="251" t="s">
+      <c r="K6" s="242" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="241" t="s">
+      <c r="L6" s="244" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="243" t="s">
+      <c r="M6" s="252" t="s">
         <v>95</v>
       </c>
-      <c r="N6" s="248" t="s">
+      <c r="N6" s="247" t="s">
         <v>59</v>
       </c>
     </row>
@@ -3848,15 +3875,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="231"/>
+      <c r="H7" s="239"/>
       <c r="I7" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J7" s="235"/>
-      <c r="K7" s="251"/>
-      <c r="L7" s="241"/>
-      <c r="M7" s="254"/>
-      <c r="N7" s="248"/>
+      <c r="J7" s="240"/>
+      <c r="K7" s="242"/>
+      <c r="L7" s="244"/>
+      <c r="M7" s="253"/>
+      <c r="N7" s="247"/>
     </row>
     <row r="8" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B8" s="81">
@@ -3882,15 +3909,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="231"/>
+      <c r="H8" s="239"/>
       <c r="I8" s="90" t="s">
         <v>9</v>
       </c>
-      <c r="J8" s="235"/>
-      <c r="K8" s="251"/>
-      <c r="L8" s="241"/>
-      <c r="M8" s="254"/>
-      <c r="N8" s="248"/>
+      <c r="J8" s="240"/>
+      <c r="K8" s="242"/>
+      <c r="L8" s="244"/>
+      <c r="M8" s="253"/>
+      <c r="N8" s="247"/>
     </row>
     <row r="9" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B9" s="81">
@@ -3916,15 +3943,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="231"/>
+      <c r="H9" s="239"/>
       <c r="I9" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="J9" s="235"/>
-      <c r="K9" s="251"/>
-      <c r="L9" s="241"/>
-      <c r="M9" s="254"/>
-      <c r="N9" s="248"/>
+      <c r="J9" s="240"/>
+      <c r="K9" s="242"/>
+      <c r="L9" s="244"/>
+      <c r="M9" s="253"/>
+      <c r="N9" s="247"/>
     </row>
     <row r="10" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B10" s="81">
@@ -3950,15 +3977,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="231"/>
+      <c r="H10" s="239"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="235"/>
-      <c r="K10" s="251"/>
-      <c r="L10" s="241"/>
-      <c r="M10" s="254"/>
-      <c r="N10" s="248"/>
+      <c r="J10" s="240"/>
+      <c r="K10" s="242"/>
+      <c r="L10" s="244"/>
+      <c r="M10" s="253"/>
+      <c r="N10" s="247"/>
     </row>
     <row r="11" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="82">
@@ -3984,15 +4011,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="232"/>
+      <c r="H11" s="238"/>
       <c r="I11" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="J11" s="236"/>
-      <c r="K11" s="252"/>
-      <c r="L11" s="242"/>
-      <c r="M11" s="255"/>
-      <c r="N11" s="249"/>
+      <c r="J11" s="241"/>
+      <c r="K11" s="243"/>
+      <c r="L11" s="245"/>
+      <c r="M11" s="254"/>
+      <c r="N11" s="248"/>
     </row>
     <row r="12" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B12" s="80">
@@ -4018,26 +4045,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="233" t="s">
+      <c r="H12" s="237" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="234" t="s">
+      <c r="J12" s="249" t="s">
         <v>58</v>
       </c>
       <c r="K12" s="250" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="240" t="s">
+      <c r="L12" s="246" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="233" t="s">
+      <c r="M12" s="237" t="s">
         <v>96</v>
       </c>
-      <c r="N12" s="253" t="s">
-        <v>184</v>
+      <c r="N12" s="251" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="2:14" x14ac:dyDescent="0.25">
@@ -4064,15 +4091,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="231"/>
+      <c r="H13" s="239"/>
       <c r="I13" s="90" t="s">
         <v>14</v>
       </c>
-      <c r="J13" s="235"/>
-      <c r="K13" s="251"/>
-      <c r="L13" s="241"/>
-      <c r="M13" s="231"/>
-      <c r="N13" s="248"/>
+      <c r="J13" s="240"/>
+      <c r="K13" s="242"/>
+      <c r="L13" s="244"/>
+      <c r="M13" s="239"/>
+      <c r="N13" s="247"/>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B14" s="81">
@@ -4098,15 +4125,15 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="231"/>
+      <c r="H14" s="239"/>
       <c r="I14" s="90" t="s">
         <v>86</v>
       </c>
-      <c r="J14" s="235"/>
-      <c r="K14" s="251"/>
-      <c r="L14" s="241"/>
-      <c r="M14" s="231"/>
-      <c r="N14" s="248"/>
+      <c r="J14" s="240"/>
+      <c r="K14" s="242"/>
+      <c r="L14" s="244"/>
+      <c r="M14" s="239"/>
+      <c r="N14" s="247"/>
     </row>
     <row r="15" spans="2:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="82">
@@ -4132,15 +4159,15 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="232"/>
+      <c r="H15" s="238"/>
       <c r="I15" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="J15" s="236"/>
-      <c r="K15" s="252"/>
-      <c r="L15" s="242"/>
-      <c r="M15" s="232"/>
-      <c r="N15" s="249"/>
+      <c r="J15" s="241"/>
+      <c r="K15" s="243"/>
+      <c r="L15" s="245"/>
+      <c r="M15" s="238"/>
+      <c r="N15" s="248"/>
     </row>
     <row r="16" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B16" s="80">
@@ -4166,22 +4193,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="233" t="s">
+      <c r="H16" s="237" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="234" t="s">
+      <c r="J16" s="249" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="237" t="s">
+      <c r="K16" s="255" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="240" t="s">
+      <c r="L16" s="246" t="s">
         <v>55</v>
       </c>
-      <c r="M16" s="233" t="s">
+      <c r="M16" s="237" t="s">
         <v>96</v>
       </c>
       <c r="N16" s="75" t="s">
@@ -4212,14 +4239,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="231"/>
+      <c r="H17" s="239"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="235"/>
-      <c r="K17" s="238"/>
-      <c r="L17" s="241"/>
-      <c r="M17" s="231"/>
+      <c r="J17" s="240"/>
+      <c r="K17" s="256"/>
+      <c r="L17" s="244"/>
+      <c r="M17" s="239"/>
       <c r="N17" s="74" t="s">
         <v>89</v>
       </c>
@@ -4248,14 +4275,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="231"/>
+      <c r="H18" s="239"/>
       <c r="I18" s="70" t="s">
         <v>41</v>
       </c>
-      <c r="J18" s="235"/>
-      <c r="K18" s="238"/>
-      <c r="L18" s="241"/>
-      <c r="M18" s="231"/>
+      <c r="J18" s="240"/>
+      <c r="K18" s="256"/>
+      <c r="L18" s="244"/>
+      <c r="M18" s="239"/>
       <c r="N18" s="74" t="s">
         <v>91</v>
       </c>
@@ -4284,14 +4311,14 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="232"/>
+      <c r="H19" s="238"/>
       <c r="I19" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="J19" s="236"/>
-      <c r="K19" s="239"/>
-      <c r="L19" s="242"/>
-      <c r="M19" s="232"/>
+      <c r="J19" s="241"/>
+      <c r="K19" s="257"/>
+      <c r="L19" s="245"/>
+      <c r="M19" s="238"/>
       <c r="N19" s="44" t="s">
         <v>92</v>
       </c>
@@ -4321,26 +4348,26 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="233" t="s">
+      <c r="H20" s="237" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="192" t="s">
+        <v>175</v>
+      </c>
+      <c r="J20" s="140" t="s">
+        <v>149</v>
+      </c>
+      <c r="K20" s="255" t="s">
+        <v>53</v>
+      </c>
+      <c r="L20" s="260" t="s">
+        <v>55</v>
+      </c>
+      <c r="M20" s="252" t="s">
+        <v>95</v>
+      </c>
+      <c r="N20" s="194" t="s">
         <v>177</v>
-      </c>
-      <c r="J20" s="140" t="s">
-        <v>151</v>
-      </c>
-      <c r="K20" s="237" t="s">
-        <v>53</v>
-      </c>
-      <c r="L20" s="246" t="s">
-        <v>55</v>
-      </c>
-      <c r="M20" s="243" t="s">
-        <v>95</v>
-      </c>
-      <c r="N20" s="194" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="21" spans="2:17" x14ac:dyDescent="0.25">
@@ -4367,18 +4394,18 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="231"/>
+      <c r="H21" s="239"/>
       <c r="I21" s="193" t="s">
         <v>100</v>
       </c>
       <c r="J21" s="99" t="s">
-        <v>151</v>
-      </c>
-      <c r="K21" s="245"/>
-      <c r="L21" s="247"/>
-      <c r="M21" s="244"/>
+        <v>149</v>
+      </c>
+      <c r="K21" s="259"/>
+      <c r="L21" s="261"/>
+      <c r="M21" s="258"/>
       <c r="N21" s="195" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="22" spans="2:17" x14ac:dyDescent="0.25">
@@ -4405,7 +4432,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="231"/>
+      <c r="H22" s="239"/>
       <c r="I22" s="103"/>
       <c r="J22" s="136"/>
       <c r="K22" s="137"/>
@@ -4437,7 +4464,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="232"/>
+      <c r="H23" s="238"/>
       <c r="I23" s="96"/>
       <c r="J23" s="133"/>
       <c r="K23" s="134"/>
@@ -4469,7 +4496,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="233" t="s">
+      <c r="H24" s="237" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -4515,7 +4542,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="231"/>
+      <c r="H25" s="239"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -4532,7 +4559,7 @@
         <v>95</v>
       </c>
       <c r="N25" s="74" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="2:17" x14ac:dyDescent="0.25">
@@ -4559,7 +4586,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="231"/>
+      <c r="H26" s="239"/>
       <c r="I26" s="103"/>
       <c r="J26" s="136"/>
       <c r="K26" s="137"/>
@@ -4591,7 +4618,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="232"/>
+      <c r="H27" s="238"/>
       <c r="I27" s="96"/>
       <c r="J27" s="133"/>
       <c r="K27" s="134"/>
@@ -4623,7 +4650,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="233" t="s">
+      <c r="H28" s="237" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -4642,7 +4669,7 @@
         <v>95</v>
       </c>
       <c r="N28" s="38" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="29" spans="2:17" x14ac:dyDescent="0.25">
@@ -4669,7 +4696,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="231"/>
+      <c r="H29" s="239"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -4686,7 +4713,7 @@
         <v>95</v>
       </c>
       <c r="N29" s="74" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="30" spans="2:17" x14ac:dyDescent="0.25">
@@ -4713,7 +4740,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="231"/>
+      <c r="H30" s="239"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -4730,7 +4757,7 @@
         <v>95</v>
       </c>
       <c r="N30" s="74" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="31" spans="2:17" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4757,7 +4784,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="232"/>
+      <c r="H31" s="238"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -4789,7 +4816,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="231" t="s">
+      <c r="H32" s="239" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -4808,7 +4835,7 @@
         <v>95</v>
       </c>
       <c r="N32" s="38" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="Q32" s="1"/>
     </row>
@@ -4836,7 +4863,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="231"/>
+      <c r="H33" s="239"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -4853,7 +4880,7 @@
         <v>95</v>
       </c>
       <c r="N33" s="74" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="Q33" s="1"/>
     </row>
@@ -4881,7 +4908,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="232"/>
+      <c r="H34" s="238"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -4898,7 +4925,7 @@
         <v>95</v>
       </c>
       <c r="N34" s="74" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="Q34" s="1"/>
     </row>
@@ -4945,23 +4972,23 @@
         <v>95</v>
       </c>
       <c r="N35" s="46" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="H32:H34"/>
+    <mergeCell ref="H28:H31"/>
+    <mergeCell ref="H24:H27"/>
+    <mergeCell ref="H16:H19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="K16:K19"/>
+    <mergeCell ref="L16:L19"/>
+    <mergeCell ref="M16:M19"/>
+    <mergeCell ref="H20:H23"/>
+    <mergeCell ref="M20:M21"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:L21"/>
     <mergeCell ref="N6:N11"/>
     <mergeCell ref="H12:H15"/>
     <mergeCell ref="J12:J15"/>
@@ -4970,18 +4997,18 @@
     <mergeCell ref="M12:M15"/>
     <mergeCell ref="N12:N15"/>
     <mergeCell ref="M6:M11"/>
-    <mergeCell ref="K16:K19"/>
-    <mergeCell ref="L16:L19"/>
-    <mergeCell ref="M16:M19"/>
-    <mergeCell ref="H20:H23"/>
-    <mergeCell ref="M20:M21"/>
-    <mergeCell ref="K20:K21"/>
-    <mergeCell ref="L20:L21"/>
-    <mergeCell ref="H32:H34"/>
-    <mergeCell ref="H28:H31"/>
-    <mergeCell ref="H24:H27"/>
-    <mergeCell ref="H16:H19"/>
-    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="M2:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -5003,26 +5030,26 @@
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="234" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="257"/>
-      <c r="F2" s="257"/>
-      <c r="G2" s="258"/>
-      <c r="H2" s="201" t="s">
+      <c r="C2" s="235"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="235"/>
+      <c r="F2" s="235"/>
+      <c r="G2" s="236"/>
+      <c r="H2" s="204" t="s">
         <v>46</v>
       </c>
-      <c r="I2" s="201" t="s">
+      <c r="I2" s="204" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="256" t="s">
+      <c r="J2" s="234" t="s">
         <v>35</v>
       </c>
-      <c r="K2" s="257"/>
-      <c r="L2" s="257"/>
-      <c r="M2" s="201" t="s">
+      <c r="K2" s="235"/>
+      <c r="L2" s="235"/>
+      <c r="M2" s="204" t="s">
         <v>25</v>
       </c>
     </row>
@@ -5045,8 +5072,8 @@
       <c r="G3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
+      <c r="H3" s="205"/>
+      <c r="I3" s="205"/>
       <c r="J3" s="48" t="s">
         <v>3</v>
       </c>
@@ -5056,7 +5083,7 @@
       <c r="L3" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="202"/>
+      <c r="M3" s="205"/>
     </row>
     <row r="4" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B4" s="80">
@@ -5082,11 +5109,11 @@
         <f>_xlfn.BITAND($B4,1)</f>
         <v>0</v>
       </c>
-      <c r="H4" s="233" t="s">
+      <c r="H4" s="237" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="67" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J4" s="66" t="s">
         <v>73</v>
@@ -5125,7 +5152,7 @@
         <f t="shared" ref="G5:G35" si="0">_xlfn.BITAND($B5,1)</f>
         <v>1</v>
       </c>
-      <c r="H5" s="232"/>
+      <c r="H5" s="238"/>
       <c r="I5" s="42" t="s">
         <v>37</v>
       </c>
@@ -5166,22 +5193,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H6" s="231" t="s">
+      <c r="H6" s="239" t="s">
         <v>50</v>
       </c>
       <c r="I6" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="235" t="s">
+      <c r="J6" s="240" t="s">
         <v>58</v>
       </c>
-      <c r="K6" s="251" t="s">
+      <c r="K6" s="242" t="s">
         <v>57</v>
       </c>
-      <c r="L6" s="241" t="s">
+      <c r="L6" s="244" t="s">
         <v>55</v>
       </c>
-      <c r="M6" s="248" t="s">
+      <c r="M6" s="247" t="s">
         <v>59</v>
       </c>
     </row>
@@ -5209,12 +5236,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H7" s="231"/>
-      <c r="I7" s="259"/>
-      <c r="J7" s="235"/>
-      <c r="K7" s="251"/>
-      <c r="L7" s="241"/>
-      <c r="M7" s="248"/>
+      <c r="H7" s="239"/>
+      <c r="I7" s="262"/>
+      <c r="J7" s="240"/>
+      <c r="K7" s="242"/>
+      <c r="L7" s="244"/>
+      <c r="M7" s="247"/>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B8" s="81">
@@ -5240,12 +5267,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="231"/>
-      <c r="I8" s="272"/>
-      <c r="J8" s="235"/>
-      <c r="K8" s="251"/>
-      <c r="L8" s="241"/>
-      <c r="M8" s="248"/>
+      <c r="H8" s="239"/>
+      <c r="I8" s="263"/>
+      <c r="J8" s="240"/>
+      <c r="K8" s="242"/>
+      <c r="L8" s="244"/>
+      <c r="M8" s="247"/>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B9" s="81">
@@ -5271,12 +5298,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="231"/>
-      <c r="I9" s="273"/>
-      <c r="J9" s="235"/>
-      <c r="K9" s="251"/>
-      <c r="L9" s="241"/>
-      <c r="M9" s="248"/>
+      <c r="H9" s="239"/>
+      <c r="I9" s="264"/>
+      <c r="J9" s="240"/>
+      <c r="K9" s="242"/>
+      <c r="L9" s="244"/>
+      <c r="M9" s="247"/>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B10" s="81">
@@ -5302,14 +5329,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="231"/>
+      <c r="H10" s="239"/>
       <c r="I10" s="90" t="s">
         <v>11</v>
       </c>
-      <c r="J10" s="235"/>
-      <c r="K10" s="251"/>
-      <c r="L10" s="241"/>
-      <c r="M10" s="248"/>
+      <c r="J10" s="240"/>
+      <c r="K10" s="242"/>
+      <c r="L10" s="244"/>
+      <c r="M10" s="247"/>
     </row>
     <row r="11" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="82">
@@ -5335,12 +5362,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H11" s="232"/>
+      <c r="H11" s="238"/>
       <c r="I11" s="103"/>
-      <c r="J11" s="236"/>
-      <c r="K11" s="252"/>
-      <c r="L11" s="242"/>
-      <c r="M11" s="249"/>
+      <c r="J11" s="241"/>
+      <c r="K11" s="243"/>
+      <c r="L11" s="245"/>
+      <c r="M11" s="248"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="80">
@@ -5366,22 +5393,22 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="233" t="s">
+      <c r="H12" s="237" t="s">
         <v>47</v>
       </c>
       <c r="I12" s="64" t="s">
         <v>13</v>
       </c>
-      <c r="J12" s="234" t="s">
+      <c r="J12" s="249" t="s">
         <v>58</v>
       </c>
       <c r="K12" s="250" t="s">
         <v>57</v>
       </c>
-      <c r="L12" s="240" t="s">
+      <c r="L12" s="246" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="253" t="s">
+      <c r="M12" s="251" t="s">
         <v>88</v>
       </c>
     </row>
@@ -5409,12 +5436,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H13" s="231"/>
-      <c r="I13" s="259"/>
-      <c r="J13" s="235"/>
-      <c r="K13" s="251"/>
-      <c r="L13" s="241"/>
-      <c r="M13" s="248"/>
+      <c r="H13" s="239"/>
+      <c r="I13" s="262"/>
+      <c r="J13" s="240"/>
+      <c r="K13" s="242"/>
+      <c r="L13" s="244"/>
+      <c r="M13" s="247"/>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B14" s="81">
@@ -5440,12 +5467,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="231"/>
-      <c r="I14" s="272"/>
-      <c r="J14" s="235"/>
-      <c r="K14" s="251"/>
-      <c r="L14" s="241"/>
-      <c r="M14" s="248"/>
+      <c r="H14" s="239"/>
+      <c r="I14" s="263"/>
+      <c r="J14" s="240"/>
+      <c r="K14" s="242"/>
+      <c r="L14" s="244"/>
+      <c r="M14" s="247"/>
     </row>
     <row r="15" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="82">
@@ -5471,12 +5498,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H15" s="232"/>
-      <c r="I15" s="260"/>
-      <c r="J15" s="236"/>
-      <c r="K15" s="252"/>
-      <c r="L15" s="242"/>
-      <c r="M15" s="249"/>
+      <c r="H15" s="238"/>
+      <c r="I15" s="265"/>
+      <c r="J15" s="241"/>
+      <c r="K15" s="243"/>
+      <c r="L15" s="245"/>
+      <c r="M15" s="248"/>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B16" s="80">
@@ -5502,19 +5529,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="233" t="s">
+      <c r="H16" s="237" t="s">
         <v>48</v>
       </c>
       <c r="I16" s="64" t="s">
         <v>39</v>
       </c>
-      <c r="J16" s="234" t="s">
+      <c r="J16" s="249" t="s">
         <v>54</v>
       </c>
-      <c r="K16" s="237" t="s">
+      <c r="K16" s="255" t="s">
         <v>53</v>
       </c>
-      <c r="L16" s="240" t="s">
+      <c r="L16" s="246" t="s">
         <v>55</v>
       </c>
       <c r="M16" s="75" t="s">
@@ -5545,13 +5572,13 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H17" s="231"/>
+      <c r="H17" s="239"/>
       <c r="I17" s="70" t="s">
         <v>40</v>
       </c>
-      <c r="J17" s="235"/>
-      <c r="K17" s="238"/>
-      <c r="L17" s="241"/>
+      <c r="J17" s="240"/>
+      <c r="K17" s="256"/>
+      <c r="L17" s="244"/>
       <c r="M17" s="74" t="s">
         <v>89</v>
       </c>
@@ -5580,12 +5607,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="231"/>
-      <c r="I18" s="259"/>
-      <c r="J18" s="235"/>
-      <c r="K18" s="238"/>
-      <c r="L18" s="241"/>
-      <c r="M18" s="259"/>
+      <c r="H18" s="239"/>
+      <c r="I18" s="262"/>
+      <c r="J18" s="240"/>
+      <c r="K18" s="256"/>
+      <c r="L18" s="244"/>
+      <c r="M18" s="262"/>
     </row>
     <row r="19" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="82">
@@ -5611,12 +5638,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H19" s="232"/>
-      <c r="I19" s="260"/>
-      <c r="J19" s="236"/>
-      <c r="K19" s="239"/>
-      <c r="L19" s="242"/>
-      <c r="M19" s="260"/>
+      <c r="H19" s="238"/>
+      <c r="I19" s="265"/>
+      <c r="J19" s="241"/>
+      <c r="K19" s="257"/>
+      <c r="L19" s="245"/>
+      <c r="M19" s="265"/>
       <c r="O19" s="1"/>
     </row>
     <row r="20" spans="2:16" x14ac:dyDescent="0.25">
@@ -5643,14 +5670,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="261" t="s">
+      <c r="H20" s="266" t="s">
         <v>100</v>
       </c>
       <c r="I20" s="176" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="J20" s="66" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="K20" s="65" t="s">
         <v>53</v>
@@ -5659,7 +5686,7 @@
         <v>55</v>
       </c>
       <c r="M20" s="175" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21" spans="2:16" x14ac:dyDescent="0.25">
@@ -5686,7 +5713,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H21" s="262"/>
+      <c r="H21" s="267"/>
       <c r="I21" s="167"/>
       <c r="J21" s="169"/>
       <c r="K21" s="171"/>
@@ -5717,7 +5744,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H22" s="262"/>
+      <c r="H22" s="267"/>
       <c r="I22" s="167"/>
       <c r="J22" s="169"/>
       <c r="K22" s="171"/>
@@ -5748,7 +5775,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H23" s="263"/>
+      <c r="H23" s="268"/>
       <c r="I23" s="168"/>
       <c r="J23" s="170"/>
       <c r="K23" s="172"/>
@@ -5779,7 +5806,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H24" s="233" t="s">
+      <c r="H24" s="237" t="s">
         <v>49</v>
       </c>
       <c r="I24" s="64" t="s">
@@ -5822,7 +5849,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H25" s="231"/>
+      <c r="H25" s="239"/>
       <c r="I25" s="70" t="s">
         <v>38</v>
       </c>
@@ -5863,12 +5890,12 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H26" s="231"/>
-      <c r="I26" s="259"/>
-      <c r="J26" s="264"/>
-      <c r="K26" s="266"/>
-      <c r="L26" s="268"/>
-      <c r="M26" s="270"/>
+      <c r="H26" s="239"/>
+      <c r="I26" s="262"/>
+      <c r="J26" s="269"/>
+      <c r="K26" s="271"/>
+      <c r="L26" s="273"/>
+      <c r="M26" s="275"/>
     </row>
     <row r="27" spans="2:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="82">
@@ -5894,12 +5921,12 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H27" s="232"/>
-      <c r="I27" s="260"/>
-      <c r="J27" s="265"/>
-      <c r="K27" s="267"/>
-      <c r="L27" s="269"/>
-      <c r="M27" s="271"/>
+      <c r="H27" s="238"/>
+      <c r="I27" s="265"/>
+      <c r="J27" s="270"/>
+      <c r="K27" s="272"/>
+      <c r="L27" s="274"/>
+      <c r="M27" s="276"/>
     </row>
     <row r="28" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B28" s="80">
@@ -5925,7 +5952,7 @@
         <f>_xlfn.BITAND($B28,1)</f>
         <v>0</v>
       </c>
-      <c r="H28" s="233" t="s">
+      <c r="H28" s="237" t="s">
         <v>139</v>
       </c>
       <c r="I28" s="37" t="s">
@@ -5968,7 +5995,7 @@
         <f>_xlfn.BITAND($B29,1)</f>
         <v>1</v>
       </c>
-      <c r="H29" s="231"/>
+      <c r="H29" s="239"/>
       <c r="I29" s="70" t="s">
         <v>44</v>
       </c>
@@ -6009,7 +6036,7 @@
         <f>_xlfn.BITAND($B30,1)</f>
         <v>0</v>
       </c>
-      <c r="H30" s="231"/>
+      <c r="H30" s="239"/>
       <c r="I30" s="70" t="s">
         <v>45</v>
       </c>
@@ -6050,7 +6077,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H31" s="232"/>
+      <c r="H31" s="238"/>
       <c r="I31" s="91"/>
       <c r="J31" s="162"/>
       <c r="K31" s="163"/>
@@ -6081,7 +6108,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H32" s="231" t="s">
+      <c r="H32" s="239" t="s">
         <v>140</v>
       </c>
       <c r="I32" s="37" t="s">
@@ -6125,7 +6152,7 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H33" s="231"/>
+      <c r="H33" s="239"/>
       <c r="I33" s="70" t="s">
         <v>44</v>
       </c>
@@ -6167,7 +6194,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H34" s="232"/>
+      <c r="H34" s="238"/>
       <c r="I34" s="70" t="s">
         <v>45</v>
       </c>
@@ -6222,7 +6249,7 @@
         <v>53</v>
       </c>
       <c r="L35" s="165" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="M35" s="46" t="s">
         <v>93</v>
@@ -6230,24 +6257,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="H6:H11"/>
-    <mergeCell ref="J6:J11"/>
-    <mergeCell ref="K6:K11"/>
-    <mergeCell ref="L6:L11"/>
-    <mergeCell ref="I7:I9"/>
-    <mergeCell ref="M6:M11"/>
-    <mergeCell ref="H12:H15"/>
-    <mergeCell ref="J12:J15"/>
-    <mergeCell ref="K12:K15"/>
-    <mergeCell ref="L12:L15"/>
-    <mergeCell ref="M12:M15"/>
-    <mergeCell ref="I13:I15"/>
     <mergeCell ref="H32:H34"/>
     <mergeCell ref="I18:I19"/>
     <mergeCell ref="M18:M19"/>
@@ -6263,6 +6272,24 @@
     <mergeCell ref="M26:M27"/>
     <mergeCell ref="H24:H27"/>
     <mergeCell ref="H28:H31"/>
+    <mergeCell ref="M6:M11"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="J12:J15"/>
+    <mergeCell ref="K12:K15"/>
+    <mergeCell ref="L12:L15"/>
+    <mergeCell ref="M12:M15"/>
+    <mergeCell ref="I13:I15"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="H6:H11"/>
+    <mergeCell ref="J6:J11"/>
+    <mergeCell ref="K6:K11"/>
+    <mergeCell ref="L6:L11"/>
+    <mergeCell ref="I7:I9"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:L2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6279,13 +6306,13 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2" s="256" t="s">
+      <c r="B2" s="234" t="s">
         <v>60</v>
       </c>
-      <c r="C2" s="257"/>
-      <c r="D2" s="257"/>
-      <c r="E2" s="258"/>
-      <c r="F2" s="201" t="s">
+      <c r="C2" s="235"/>
+      <c r="D2" s="235"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="204" t="s">
         <v>24</v>
       </c>
     </row>
@@ -6302,7 +6329,7 @@
       <c r="E3" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="F3" s="202"/>
+      <c r="F3" s="205"/>
     </row>
     <row r="4" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="13">
@@ -6483,30 +6510,30 @@
   <sheetData>
     <row r="1" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B2" s="201" t="s">
+      <c r="B2" s="204" t="s">
         <v>69</v>
       </c>
-      <c r="C2" s="283" t="s">
+      <c r="C2" s="286" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="284"/>
-      <c r="E2" s="284"/>
-      <c r="F2" s="284"/>
-      <c r="G2" s="284"/>
-      <c r="H2" s="284"/>
-      <c r="I2" s="284"/>
-      <c r="J2" s="284"/>
-      <c r="K2" s="284"/>
-      <c r="L2" s="284"/>
-      <c r="M2" s="284"/>
-      <c r="N2" s="284"/>
-      <c r="O2" s="284"/>
-      <c r="P2" s="284"/>
-      <c r="Q2" s="284"/>
-      <c r="R2" s="285"/>
+      <c r="D2" s="287"/>
+      <c r="E2" s="287"/>
+      <c r="F2" s="287"/>
+      <c r="G2" s="287"/>
+      <c r="H2" s="287"/>
+      <c r="I2" s="287"/>
+      <c r="J2" s="287"/>
+      <c r="K2" s="287"/>
+      <c r="L2" s="287"/>
+      <c r="M2" s="287"/>
+      <c r="N2" s="287"/>
+      <c r="O2" s="287"/>
+      <c r="P2" s="287"/>
+      <c r="Q2" s="287"/>
+      <c r="R2" s="288"/>
     </row>
     <row r="3" spans="2:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="202"/>
+      <c r="B3" s="205"/>
       <c r="C3" s="116">
         <v>15</v>
       </c>
@@ -6577,13 +6604,13 @@
       <c r="M4" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="N4" s="277" t="s">
+      <c r="N4" s="280" t="s">
         <v>77</v>
       </c>
-      <c r="O4" s="277"/>
-      <c r="P4" s="277"/>
-      <c r="Q4" s="277"/>
-      <c r="R4" s="278"/>
+      <c r="O4" s="280"/>
+      <c r="P4" s="280"/>
+      <c r="Q4" s="280"/>
+      <c r="R4" s="281"/>
     </row>
     <row r="5" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="88" t="s">
@@ -6597,16 +6624,16 @@
       <c r="H5" s="153"/>
       <c r="I5" s="153"/>
       <c r="J5" s="154"/>
-      <c r="K5" s="279" t="s">
+      <c r="K5" s="282" t="s">
         <v>73</v>
       </c>
-      <c r="L5" s="275"/>
-      <c r="M5" s="275"/>
-      <c r="N5" s="275"/>
-      <c r="O5" s="275"/>
-      <c r="P5" s="275"/>
-      <c r="Q5" s="275"/>
-      <c r="R5" s="276"/>
+      <c r="L5" s="278"/>
+      <c r="M5" s="278"/>
+      <c r="N5" s="278"/>
+      <c r="O5" s="278"/>
+      <c r="P5" s="278"/>
+      <c r="Q5" s="278"/>
+      <c r="R5" s="279"/>
     </row>
     <row r="6" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="88" t="s">
@@ -6620,16 +6647,16 @@
       <c r="H6" s="153"/>
       <c r="I6" s="153"/>
       <c r="J6" s="154"/>
-      <c r="K6" s="279" t="s">
+      <c r="K6" s="282" t="s">
         <v>73</v>
       </c>
-      <c r="L6" s="275"/>
-      <c r="M6" s="275"/>
-      <c r="N6" s="275"/>
-      <c r="O6" s="275"/>
-      <c r="P6" s="275"/>
-      <c r="Q6" s="275"/>
-      <c r="R6" s="276"/>
+      <c r="L6" s="278"/>
+      <c r="M6" s="278"/>
+      <c r="N6" s="278"/>
+      <c r="O6" s="278"/>
+      <c r="P6" s="278"/>
+      <c r="Q6" s="278"/>
+      <c r="R6" s="279"/>
     </row>
     <row r="7" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="88" t="s">
@@ -6643,39 +6670,39 @@
       <c r="H7" s="155"/>
       <c r="I7" s="155"/>
       <c r="J7" s="155"/>
-      <c r="K7" s="280" t="s">
+      <c r="K7" s="283" t="s">
         <v>73</v>
       </c>
-      <c r="L7" s="281"/>
-      <c r="M7" s="281"/>
-      <c r="N7" s="281"/>
-      <c r="O7" s="281"/>
-      <c r="P7" s="281"/>
-      <c r="Q7" s="281"/>
-      <c r="R7" s="282"/>
+      <c r="L7" s="284"/>
+      <c r="M7" s="284"/>
+      <c r="N7" s="284"/>
+      <c r="O7" s="284"/>
+      <c r="P7" s="284"/>
+      <c r="Q7" s="284"/>
+      <c r="R7" s="285"/>
     </row>
     <row r="8" spans="2:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="88" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="274" t="s">
+      <c r="C8" s="277" t="s">
         <v>126</v>
       </c>
-      <c r="D8" s="275"/>
-      <c r="E8" s="275"/>
-      <c r="F8" s="275"/>
-      <c r="G8" s="275"/>
-      <c r="H8" s="275"/>
-      <c r="I8" s="275"/>
-      <c r="J8" s="275"/>
-      <c r="K8" s="275"/>
-      <c r="L8" s="275"/>
-      <c r="M8" s="275"/>
-      <c r="N8" s="275"/>
-      <c r="O8" s="275"/>
-      <c r="P8" s="275"/>
-      <c r="Q8" s="275"/>
-      <c r="R8" s="276"/>
+      <c r="D8" s="278"/>
+      <c r="E8" s="278"/>
+      <c r="F8" s="278"/>
+      <c r="G8" s="278"/>
+      <c r="H8" s="278"/>
+      <c r="I8" s="278"/>
+      <c r="J8" s="278"/>
+      <c r="K8" s="278"/>
+      <c r="L8" s="278"/>
+      <c r="M8" s="278"/>
+      <c r="N8" s="278"/>
+      <c r="O8" s="278"/>
+      <c r="P8" s="278"/>
+      <c r="Q8" s="278"/>
+      <c r="R8" s="279"/>
     </row>
     <row r="9" spans="2:18" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B9" s="89" t="s">
@@ -6721,16 +6748,17 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27FF78FE-3CCF-4749-B213-A95B9184CAE3}">
-  <dimension ref="B1:E9"/>
+  <dimension ref="B1:K10"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.140625" customWidth="1"/>
     <col min="3" max="3" width="82.28515625" customWidth="1"/>
-    <col min="4" max="5" width="44" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="6" max="11" width="14.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="156" t="s">
         <v>127</v>
       </c>
@@ -6740,11 +6768,26 @@
       <c r="D2" s="158" t="s">
         <v>143</v>
       </c>
-      <c r="E2" s="158" t="s">
+      <c r="F2" s="198" t="s">
+        <v>198</v>
+      </c>
+      <c r="G2" s="199" t="s">
+        <v>131</v>
+      </c>
+      <c r="H2" s="199" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="I2" s="199" t="s">
+        <v>196</v>
+      </c>
+      <c r="J2" s="199" t="s">
+        <v>197</v>
+      </c>
+      <c r="K2" s="200" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="159" t="s">
         <v>129</v>
       </c>
@@ -6752,13 +6795,16 @@
         <v>130</v>
       </c>
       <c r="D3" s="74" t="s">
-        <v>191</v>
-      </c>
-      <c r="E3" s="74" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+      <c r="F3" s="305"/>
+      <c r="G3" s="306"/>
+      <c r="H3" s="306"/>
+      <c r="I3" s="306"/>
+      <c r="J3" s="306"/>
+      <c r="K3" s="307"/>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="157" t="s">
         <v>131</v>
       </c>
@@ -6768,11 +6814,14 @@
       <c r="D4" s="41" t="s">
         <v>144</v>
       </c>
-      <c r="E4" s="41" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="308"/>
+      <c r="G4" s="309"/>
+      <c r="H4" s="306"/>
+      <c r="I4" s="306"/>
+      <c r="J4" s="306"/>
+      <c r="K4" s="307"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="159" t="s">
         <v>133</v>
       </c>
@@ -6780,67 +6829,97 @@
         <v>134</v>
       </c>
       <c r="D5" s="74" t="s">
+        <v>193</v>
+      </c>
+      <c r="F5" s="308"/>
+      <c r="G5" s="306"/>
+      <c r="H5" s="309"/>
+      <c r="I5" s="306"/>
+      <c r="J5" s="306"/>
+      <c r="K5" s="307"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B6" s="159" t="s">
+        <v>192</v>
+      </c>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" s="308"/>
+      <c r="G6" s="306"/>
+      <c r="H6" s="306"/>
+      <c r="I6" s="309"/>
+      <c r="J6" s="306"/>
+      <c r="K6" s="307"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B7" s="159" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="74" t="s">
+        <v>179</v>
+      </c>
+      <c r="D7" s="74" t="s">
+        <v>191</v>
+      </c>
+      <c r="F7" s="308"/>
+      <c r="G7" s="306"/>
+      <c r="H7" s="306"/>
+      <c r="I7" s="309"/>
+      <c r="J7" s="309"/>
+      <c r="K7" s="307"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B8" s="159" t="s">
+        <v>141</v>
+      </c>
+      <c r="C8" s="74" t="s">
+        <v>142</v>
+      </c>
+      <c r="D8" s="74" t="s">
+        <v>146</v>
+      </c>
+      <c r="F8" s="308"/>
+      <c r="G8" s="306"/>
+      <c r="H8" s="306"/>
+      <c r="I8" s="306"/>
+      <c r="J8" s="306"/>
+      <c r="K8" s="307"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B9" s="157" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="41" t="s">
+        <v>135</v>
+      </c>
+      <c r="D9" s="41" t="s">
         <v>145</v>
       </c>
-      <c r="E5" s="74" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="159" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="74" t="s">
-        <v>181</v>
-      </c>
-      <c r="D6" s="74" t="s">
-        <v>147</v>
-      </c>
-      <c r="E6" s="74" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="159" t="s">
-        <v>141</v>
-      </c>
-      <c r="C7" s="74" t="s">
+      <c r="F9" s="308"/>
+      <c r="G9" s="306"/>
+      <c r="H9" s="306"/>
+      <c r="I9" s="306"/>
+      <c r="J9" s="306"/>
+      <c r="K9" s="310"/>
+    </row>
+    <row r="10" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="160" t="s">
+        <v>188</v>
+      </c>
+      <c r="C10" s="161" t="s">
         <v>142</v>
       </c>
-      <c r="D7" s="74" t="s">
-        <v>148</v>
-      </c>
-      <c r="E7" s="74" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="157" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>135</v>
-      </c>
-      <c r="D8" s="41" t="s">
-        <v>146</v>
-      </c>
-      <c r="E8" s="41" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="9" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="160" t="s">
+      <c r="D10" s="161" t="s">
         <v>190</v>
       </c>
-      <c r="C9" s="161" t="s">
-        <v>142</v>
-      </c>
-      <c r="D9" s="161" t="s">
-        <v>192</v>
-      </c>
-      <c r="E9" s="161" t="s">
-        <v>192</v>
-      </c>
+      <c r="F10" s="311"/>
+      <c r="G10" s="312"/>
+      <c r="H10" s="312"/>
+      <c r="I10" s="312"/>
+      <c r="J10" s="312"/>
+      <c r="K10" s="313"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6857,10 +6936,10 @@
   <sheetData>
     <row r="1" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:5" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="286" t="s">
+      <c r="B2" s="289" t="s">
         <v>117</v>
       </c>
-      <c r="C2" s="287"/>
+      <c r="C2" s="290"/>
       <c r="D2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -6877,7 +6956,7 @@
       <c r="C4" s="130" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="288" t="s">
+      <c r="D4" s="291" t="s">
         <v>124</v>
       </c>
     </row>
@@ -6886,21 +6965,21 @@
       <c r="C5" s="131" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="289"/>
+      <c r="D5" s="292"/>
     </row>
     <row r="6" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="133"/>
       <c r="C6" s="63" t="s">
         <v>120</v>
       </c>
-      <c r="D6" s="290"/>
+      <c r="D6" s="293"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="140" t="s">
         <v>119</v>
       </c>
       <c r="C7" s="141"/>
-      <c r="D7" s="291" t="s">
+      <c r="D7" s="294" t="s">
         <v>125</v>
       </c>
     </row>
@@ -6909,14 +6988,14 @@
         <v>118</v>
       </c>
       <c r="C8" s="142"/>
-      <c r="D8" s="292"/>
+      <c r="D8" s="295"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="40" t="s">
         <v>120</v>
       </c>
       <c r="C9" s="142"/>
-      <c r="D9" s="292"/>
+      <c r="D9" s="295"/>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="143" t="s">
@@ -6925,7 +7004,7 @@
       <c r="C10" s="144" t="s">
         <v>121</v>
       </c>
-      <c r="D10" s="292"/>
+      <c r="D10" s="295"/>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="40" t="s">
@@ -6934,7 +7013,7 @@
       <c r="C11" s="131" t="s">
         <v>118</v>
       </c>
-      <c r="D11" s="292"/>
+      <c r="D11" s="295"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="2:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6944,7 +7023,7 @@
       <c r="C12" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="D12" s="293"/>
+      <c r="D12" s="296"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6966,21 +7045,21 @@
   <sheetData>
     <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B2" s="294" t="s">
-        <v>165</v>
-      </c>
-      <c r="C2" s="296" t="s">
-        <v>164</v>
-      </c>
-      <c r="D2" s="297"/>
+      <c r="B2" s="297" t="s">
+        <v>163</v>
+      </c>
+      <c r="C2" s="299" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" s="300"/>
     </row>
     <row r="3" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="295"/>
+      <c r="B3" s="298"/>
       <c r="C3" s="185" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D3" s="186" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6988,10 +7067,10 @@
         <v>0</v>
       </c>
       <c r="C4" s="143" t="s">
-        <v>169</v>
-      </c>
-      <c r="D4" s="240" t="s">
-        <v>159</v>
+        <v>167</v>
+      </c>
+      <c r="D4" s="246" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -6999,34 +7078,34 @@
         <v>1</v>
       </c>
       <c r="C5" s="190" t="s">
-        <v>170</v>
-      </c>
-      <c r="D5" s="298"/>
+        <v>168</v>
+      </c>
+      <c r="D5" s="301"/>
     </row>
     <row r="6" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="88">
         <v>2</v>
       </c>
-      <c r="C6" s="300" t="s">
-        <v>166</v>
-      </c>
-      <c r="D6" s="299" t="s">
-        <v>163</v>
+      <c r="C6" s="303" t="s">
+        <v>164</v>
+      </c>
+      <c r="D6" s="302" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="177">
         <v>3</v>
       </c>
-      <c r="C7" s="235"/>
-      <c r="D7" s="241"/>
+      <c r="C7" s="240"/>
+      <c r="D7" s="244"/>
     </row>
     <row r="8" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="88">
         <v>4</v>
       </c>
-      <c r="C8" s="301"/>
-      <c r="D8" s="298"/>
+      <c r="C8" s="304"/>
+      <c r="D8" s="301"/>
     </row>
     <row r="9" spans="2:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="177">
@@ -7048,16 +7127,16 @@
       </c>
       <c r="C11" s="133"/>
       <c r="D11" s="180" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="2:4" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="187" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C14" s="188" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.25">
@@ -7065,7 +7144,7 @@
         <v>0</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.25">
@@ -7073,7 +7152,7 @@
         <v>1</v>
       </c>
       <c r="C16" s="181" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
@@ -7081,7 +7160,7 @@
         <v>2</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
@@ -7089,7 +7168,7 @@
         <v>3</v>
       </c>
       <c r="C18" s="181" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
@@ -7097,7 +7176,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
@@ -7126,10 +7205,10 @@
     </row>
     <row r="25" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="187" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C25" s="188" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
@@ -7137,7 +7216,7 @@
         <v>0</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
@@ -7145,7 +7224,7 @@
         <v>1</v>
       </c>
       <c r="C27" s="181" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
@@ -7153,7 +7232,7 @@
         <v>2</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7161,16 +7240,16 @@
         <v>3</v>
       </c>
       <c r="C29" s="183" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="2:3" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="187" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C32" s="188" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
@@ -7226,7 +7305,7 @@
         <v>6</v>
       </c>
       <c r="C39" s="189" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="40" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7234,7 +7313,7 @@
         <v>7</v>
       </c>
       <c r="C40" s="183" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>